<commit_message>
feat(ai): export purged_new_candidates_2000.xlsx and recover remarkable, charming, touched to clean_emotion_words_2000_reviews
</commit_message>
<xml_diff>
--- a/data/derived_outputs/clean_emotion_words_2000_reviews.xlsx
+++ b/data/derived_outputs/clean_emotion_words_2000_reviews.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="198" uniqueCount="151">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="214" uniqueCount="163">
   <si>
     <t>word</t>
   </si>
@@ -97,6 +97,9 @@
     <t>enjoys</t>
   </si>
   <si>
+    <t>hesitation</t>
+  </si>
+  <si>
     <t>stable</t>
   </si>
   <si>
@@ -121,6 +124,15 @@
     <t>moving</t>
   </si>
   <si>
+    <t>remarkable</t>
+  </si>
+  <si>
+    <t>touched</t>
+  </si>
+  <si>
+    <t>charming</t>
+  </si>
+  <si>
     <t>astonishing</t>
   </si>
   <si>
@@ -241,6 +253,9 @@
     <t>喜爱 / 乐在其中</t>
   </si>
   <si>
+    <t>毫不犹豫的 / 顾虑消除</t>
+  </si>
+  <si>
     <t>平稳安心的</t>
   </si>
   <si>
@@ -263,6 +278,15 @@
   </si>
   <si>
     <t>令人动容感人的</t>
+  </si>
+  <si>
+    <t>卓越令人瞩目的</t>
+  </si>
+  <si>
+    <t>深受感动的</t>
+  </si>
+  <si>
+    <t>迷人讨喜的</t>
   </si>
   <si>
     <t>令人惊叹的</t>
@@ -393,6 +417,10 @@
     <t>review_01a15aeaba8572c72e48282b :: We did so many amazing things during our time at the Grand Canyon, but this was by far the best.  Our pilot, Dave, was fantastic.  He really took the time to point out the many poi...</t>
   </si>
   <si>
+    <t>review_f3cad2d0d28657d2e80ee4d8 :: This was always going to rate highly for me. I love flying, I love nature, so I had high expectations. All of them were met and exceeded. 
+Rivers, the pilot, was a professional th...</t>
+  </si>
+  <si>
     <t>review_204946c26466eb6ee99eca6e :: I'd been hoping to rent a single engine airplane during our recent trip to Kauai.  I'm a private pilot, and my wonderful wife was looking for a way to see the island while allowing...</t>
   </si>
   <si>
@@ -415,6 +443,15 @@
   </si>
   <si>
     <t>review_3c3c26b554a263c0b5b10b29 :: All I can say is Wow!!!!  I was amazed when I viewed the canyon from the South Rim, but I was blown away from what I saw on this tour.   The majesty of the canyon is brought to the...</t>
+  </si>
+  <si>
+    <t>review_e7d041cefffecba964ada226 :: Thank you to all those at Talkeetna Air Taxi! I had a remarkable time. I felt very safe. I was co pilot in the landing on Mt. McKinley when we went. Great energy from the pilot. Fr...</t>
+  </si>
+  <si>
+    <t>review_53e4e7ec9c8062674e06d0dc :: My wife and I went on this trip with a touchdown in the rain forest. It was spectacular. Jake was our pilot and he was awesome. We had confidence in his abilities and he put our mi...</t>
+  </si>
+  <si>
+    <t>review_2437be8aa60056f18e560577 :: Our flight over Kaua'i with our charming, skillful pilot was the best experience of our island vacation. She gave a most interesting and helpful account of what we could see below,...</t>
   </si>
   <si>
     <t>review_7bbe5f17c5ccf78fd605ad3d :: From the front reception area to preparing for take off to our amazing pilot from the Arctic, this tour was astonishing. We were blessed with a beautiful sunny day with big white p...</t>
@@ -831,7 +868,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:F49"/>
+  <dimension ref="A1:F53"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:6">
@@ -859,10 +896,10 @@
         <v>6</v>
       </c>
       <c r="B2" t="s">
-        <v>54</v>
+        <v>58</v>
       </c>
       <c r="C2" t="s">
-        <v>102</v>
+        <v>110</v>
       </c>
       <c r="D2">
         <v>12</v>
@@ -871,7 +908,7 @@
         <v>12</v>
       </c>
       <c r="F2" t="s">
-        <v>104</v>
+        <v>112</v>
       </c>
     </row>
     <row r="3" spans="1:6">
@@ -879,10 +916,10 @@
         <v>7</v>
       </c>
       <c r="B3" t="s">
-        <v>55</v>
+        <v>59</v>
       </c>
       <c r="C3" t="s">
-        <v>103</v>
+        <v>111</v>
       </c>
       <c r="D3">
         <v>10</v>
@@ -891,7 +928,7 @@
         <v>10</v>
       </c>
       <c r="F3" t="s">
-        <v>105</v>
+        <v>113</v>
       </c>
     </row>
     <row r="4" spans="1:6">
@@ -899,10 +936,10 @@
         <v>8</v>
       </c>
       <c r="B4" t="s">
-        <v>56</v>
+        <v>60</v>
       </c>
       <c r="C4" t="s">
-        <v>103</v>
+        <v>111</v>
       </c>
       <c r="D4">
         <v>10</v>
@@ -911,7 +948,7 @@
         <v>9</v>
       </c>
       <c r="F4" t="s">
-        <v>106</v>
+        <v>114</v>
       </c>
     </row>
     <row r="5" spans="1:6">
@@ -919,10 +956,10 @@
         <v>9</v>
       </c>
       <c r="B5" t="s">
-        <v>57</v>
+        <v>61</v>
       </c>
       <c r="C5" t="s">
-        <v>103</v>
+        <v>111</v>
       </c>
       <c r="D5">
         <v>9</v>
@@ -931,7 +968,7 @@
         <v>9</v>
       </c>
       <c r="F5" t="s">
-        <v>107</v>
+        <v>115</v>
       </c>
     </row>
     <row r="6" spans="1:6">
@@ -939,10 +976,10 @@
         <v>10</v>
       </c>
       <c r="B6" t="s">
-        <v>58</v>
+        <v>62</v>
       </c>
       <c r="C6" t="s">
-        <v>103</v>
+        <v>111</v>
       </c>
       <c r="D6">
         <v>9</v>
@@ -951,7 +988,7 @@
         <v>9</v>
       </c>
       <c r="F6" t="s">
-        <v>108</v>
+        <v>116</v>
       </c>
     </row>
     <row r="7" spans="1:6">
@@ -959,10 +996,10 @@
         <v>11</v>
       </c>
       <c r="B7" t="s">
-        <v>59</v>
+        <v>63</v>
       </c>
       <c r="C7" t="s">
-        <v>103</v>
+        <v>111</v>
       </c>
       <c r="D7">
         <v>9</v>
@@ -971,7 +1008,7 @@
         <v>9</v>
       </c>
       <c r="F7" t="s">
-        <v>109</v>
+        <v>117</v>
       </c>
     </row>
     <row r="8" spans="1:6">
@@ -979,10 +1016,10 @@
         <v>12</v>
       </c>
       <c r="B8" t="s">
-        <v>60</v>
+        <v>64</v>
       </c>
       <c r="C8" t="s">
-        <v>103</v>
+        <v>111</v>
       </c>
       <c r="D8">
         <v>8</v>
@@ -991,7 +1028,7 @@
         <v>8</v>
       </c>
       <c r="F8" t="s">
-        <v>110</v>
+        <v>118</v>
       </c>
     </row>
     <row r="9" spans="1:6">
@@ -999,10 +1036,10 @@
         <v>13</v>
       </c>
       <c r="B9" t="s">
-        <v>61</v>
+        <v>65</v>
       </c>
       <c r="C9" t="s">
-        <v>102</v>
+        <v>110</v>
       </c>
       <c r="D9">
         <v>8</v>
@@ -1011,7 +1048,7 @@
         <v>8</v>
       </c>
       <c r="F9" t="s">
-        <v>111</v>
+        <v>119</v>
       </c>
     </row>
     <row r="10" spans="1:6">
@@ -1019,10 +1056,10 @@
         <v>14</v>
       </c>
       <c r="B10" t="s">
-        <v>62</v>
+        <v>66</v>
       </c>
       <c r="C10" t="s">
-        <v>102</v>
+        <v>110</v>
       </c>
       <c r="D10">
         <v>7</v>
@@ -1031,7 +1068,7 @@
         <v>7</v>
       </c>
       <c r="F10" t="s">
-        <v>112</v>
+        <v>120</v>
       </c>
     </row>
     <row r="11" spans="1:6">
@@ -1039,10 +1076,10 @@
         <v>15</v>
       </c>
       <c r="B11" t="s">
-        <v>63</v>
+        <v>67</v>
       </c>
       <c r="C11" t="s">
-        <v>103</v>
+        <v>111</v>
       </c>
       <c r="D11">
         <v>7</v>
@@ -1051,7 +1088,7 @@
         <v>7</v>
       </c>
       <c r="F11" t="s">
-        <v>113</v>
+        <v>121</v>
       </c>
     </row>
     <row r="12" spans="1:6">
@@ -1059,10 +1096,10 @@
         <v>16</v>
       </c>
       <c r="B12" t="s">
-        <v>64</v>
+        <v>68</v>
       </c>
       <c r="C12" t="s">
-        <v>103</v>
+        <v>111</v>
       </c>
       <c r="D12">
         <v>7</v>
@@ -1071,7 +1108,7 @@
         <v>7</v>
       </c>
       <c r="F12" t="s">
-        <v>114</v>
+        <v>122</v>
       </c>
     </row>
     <row r="13" spans="1:6">
@@ -1079,10 +1116,10 @@
         <v>17</v>
       </c>
       <c r="B13" t="s">
-        <v>65</v>
+        <v>69</v>
       </c>
       <c r="C13" t="s">
-        <v>103</v>
+        <v>111</v>
       </c>
       <c r="D13">
         <v>7</v>
@@ -1091,7 +1128,7 @@
         <v>7</v>
       </c>
       <c r="F13" t="s">
-        <v>115</v>
+        <v>123</v>
       </c>
     </row>
     <row r="14" spans="1:6">
@@ -1099,10 +1136,10 @@
         <v>18</v>
       </c>
       <c r="B14" t="s">
-        <v>66</v>
+        <v>70</v>
       </c>
       <c r="C14" t="s">
-        <v>103</v>
+        <v>111</v>
       </c>
       <c r="D14">
         <v>7</v>
@@ -1111,7 +1148,7 @@
         <v>6</v>
       </c>
       <c r="F14" t="s">
-        <v>116</v>
+        <v>124</v>
       </c>
     </row>
     <row r="15" spans="1:6">
@@ -1119,10 +1156,10 @@
         <v>19</v>
       </c>
       <c r="B15" t="s">
-        <v>67</v>
+        <v>71</v>
       </c>
       <c r="C15" t="s">
-        <v>103</v>
+        <v>111</v>
       </c>
       <c r="D15">
         <v>7</v>
@@ -1131,7 +1168,7 @@
         <v>7</v>
       </c>
       <c r="F15" t="s">
-        <v>107</v>
+        <v>115</v>
       </c>
     </row>
     <row r="16" spans="1:6">
@@ -1139,10 +1176,10 @@
         <v>20</v>
       </c>
       <c r="B16" t="s">
-        <v>68</v>
+        <v>72</v>
       </c>
       <c r="C16" t="s">
-        <v>103</v>
+        <v>111</v>
       </c>
       <c r="D16">
         <v>6</v>
@@ -1151,7 +1188,7 @@
         <v>6</v>
       </c>
       <c r="F16" t="s">
-        <v>117</v>
+        <v>125</v>
       </c>
     </row>
     <row r="17" spans="1:6">
@@ -1159,10 +1196,10 @@
         <v>21</v>
       </c>
       <c r="B17" t="s">
-        <v>69</v>
+        <v>73</v>
       </c>
       <c r="C17" t="s">
-        <v>102</v>
+        <v>110</v>
       </c>
       <c r="D17">
         <v>6</v>
@@ -1171,7 +1208,7 @@
         <v>6</v>
       </c>
       <c r="F17" t="s">
-        <v>118</v>
+        <v>126</v>
       </c>
     </row>
     <row r="18" spans="1:6">
@@ -1179,10 +1216,10 @@
         <v>22</v>
       </c>
       <c r="B18" t="s">
-        <v>70</v>
+        <v>74</v>
       </c>
       <c r="C18" t="s">
-        <v>103</v>
+        <v>111</v>
       </c>
       <c r="D18">
         <v>6</v>
@@ -1191,7 +1228,7 @@
         <v>6</v>
       </c>
       <c r="F18" t="s">
-        <v>119</v>
+        <v>127</v>
       </c>
     </row>
     <row r="19" spans="1:6">
@@ -1199,10 +1236,10 @@
         <v>23</v>
       </c>
       <c r="B19" t="s">
-        <v>71</v>
+        <v>75</v>
       </c>
       <c r="C19" t="s">
-        <v>103</v>
+        <v>111</v>
       </c>
       <c r="D19">
         <v>6</v>
@@ -1211,7 +1248,7 @@
         <v>5</v>
       </c>
       <c r="F19" t="s">
-        <v>120</v>
+        <v>128</v>
       </c>
     </row>
     <row r="20" spans="1:6">
@@ -1219,10 +1256,10 @@
         <v>24</v>
       </c>
       <c r="B20" t="s">
-        <v>72</v>
+        <v>76</v>
       </c>
       <c r="C20" t="s">
-        <v>102</v>
+        <v>110</v>
       </c>
       <c r="D20">
         <v>6</v>
@@ -1231,7 +1268,7 @@
         <v>6</v>
       </c>
       <c r="F20" t="s">
-        <v>121</v>
+        <v>129</v>
       </c>
     </row>
     <row r="21" spans="1:6">
@@ -1239,10 +1276,10 @@
         <v>25</v>
       </c>
       <c r="B21" t="s">
-        <v>73</v>
+        <v>77</v>
       </c>
       <c r="C21" t="s">
-        <v>102</v>
+        <v>110</v>
       </c>
       <c r="D21">
         <v>6</v>
@@ -1251,7 +1288,7 @@
         <v>5</v>
       </c>
       <c r="F21" t="s">
-        <v>122</v>
+        <v>130</v>
       </c>
     </row>
     <row r="22" spans="1:6">
@@ -1259,10 +1296,10 @@
         <v>26</v>
       </c>
       <c r="B22" t="s">
-        <v>74</v>
+        <v>78</v>
       </c>
       <c r="C22" t="s">
-        <v>102</v>
+        <v>110</v>
       </c>
       <c r="D22">
         <v>6</v>
@@ -1271,7 +1308,7 @@
         <v>6</v>
       </c>
       <c r="F22" t="s">
-        <v>123</v>
+        <v>131</v>
       </c>
     </row>
     <row r="23" spans="1:6">
@@ -1279,10 +1316,10 @@
         <v>27</v>
       </c>
       <c r="B23" t="s">
-        <v>75</v>
+        <v>79</v>
       </c>
       <c r="C23" t="s">
-        <v>103</v>
+        <v>110</v>
       </c>
       <c r="D23">
         <v>6</v>
@@ -1291,7 +1328,7 @@
         <v>6</v>
       </c>
       <c r="F23" t="s">
-        <v>124</v>
+        <v>132</v>
       </c>
     </row>
     <row r="24" spans="1:6">
@@ -1299,19 +1336,19 @@
         <v>28</v>
       </c>
       <c r="B24" t="s">
-        <v>76</v>
+        <v>80</v>
       </c>
       <c r="C24" t="s">
-        <v>102</v>
+        <v>111</v>
       </c>
       <c r="D24">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="E24">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="F24" t="s">
-        <v>125</v>
+        <v>133</v>
       </c>
     </row>
     <row r="25" spans="1:6">
@@ -1319,10 +1356,10 @@
         <v>29</v>
       </c>
       <c r="B25" t="s">
-        <v>77</v>
+        <v>81</v>
       </c>
       <c r="C25" t="s">
-        <v>103</v>
+        <v>110</v>
       </c>
       <c r="D25">
         <v>5</v>
@@ -1331,7 +1368,7 @@
         <v>5</v>
       </c>
       <c r="F25" t="s">
-        <v>126</v>
+        <v>134</v>
       </c>
     </row>
     <row r="26" spans="1:6">
@@ -1339,19 +1376,19 @@
         <v>30</v>
       </c>
       <c r="B26" t="s">
-        <v>78</v>
+        <v>82</v>
       </c>
       <c r="C26" t="s">
-        <v>103</v>
+        <v>111</v>
       </c>
       <c r="D26">
         <v>5</v>
       </c>
       <c r="E26">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="F26" t="s">
-        <v>127</v>
+        <v>135</v>
       </c>
     </row>
     <row r="27" spans="1:6">
@@ -1359,19 +1396,19 @@
         <v>31</v>
       </c>
       <c r="B27" t="s">
-        <v>79</v>
+        <v>83</v>
       </c>
       <c r="C27" t="s">
-        <v>103</v>
+        <v>111</v>
       </c>
       <c r="D27">
         <v>5</v>
       </c>
       <c r="E27">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="F27" t="s">
-        <v>128</v>
+        <v>136</v>
       </c>
     </row>
     <row r="28" spans="1:6">
@@ -1379,10 +1416,10 @@
         <v>32</v>
       </c>
       <c r="B28" t="s">
-        <v>80</v>
+        <v>84</v>
       </c>
       <c r="C28" t="s">
-        <v>102</v>
+        <v>111</v>
       </c>
       <c r="D28">
         <v>5</v>
@@ -1391,7 +1428,7 @@
         <v>5</v>
       </c>
       <c r="F28" t="s">
-        <v>129</v>
+        <v>137</v>
       </c>
     </row>
     <row r="29" spans="1:6">
@@ -1399,10 +1436,10 @@
         <v>33</v>
       </c>
       <c r="B29" t="s">
-        <v>81</v>
+        <v>85</v>
       </c>
       <c r="C29" t="s">
-        <v>103</v>
+        <v>110</v>
       </c>
       <c r="D29">
         <v>5</v>
@@ -1411,7 +1448,7 @@
         <v>5</v>
       </c>
       <c r="F29" t="s">
-        <v>130</v>
+        <v>138</v>
       </c>
     </row>
     <row r="30" spans="1:6">
@@ -1419,19 +1456,19 @@
         <v>34</v>
       </c>
       <c r="B30" t="s">
-        <v>82</v>
+        <v>86</v>
       </c>
       <c r="C30" t="s">
-        <v>103</v>
+        <v>111</v>
       </c>
       <c r="D30">
         <v>5</v>
       </c>
       <c r="E30">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="F30" t="s">
-        <v>131</v>
+        <v>139</v>
       </c>
     </row>
     <row r="31" spans="1:6">
@@ -1439,19 +1476,19 @@
         <v>35</v>
       </c>
       <c r="B31" t="s">
-        <v>83</v>
+        <v>87</v>
       </c>
       <c r="C31" t="s">
-        <v>103</v>
+        <v>111</v>
       </c>
       <c r="D31">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="E31">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="F31" t="s">
-        <v>132</v>
+        <v>140</v>
       </c>
     </row>
     <row r="32" spans="1:6">
@@ -1459,19 +1496,19 @@
         <v>36</v>
       </c>
       <c r="B32" t="s">
-        <v>84</v>
+        <v>88</v>
       </c>
       <c r="C32" t="s">
-        <v>103</v>
+        <v>111</v>
       </c>
       <c r="D32">
-        <v>1</v>
+        <v>5</v>
       </c>
       <c r="E32">
-        <v>1</v>
+        <v>5</v>
       </c>
       <c r="F32" t="s">
-        <v>133</v>
+        <v>141</v>
       </c>
     </row>
     <row r="33" spans="1:6">
@@ -1479,19 +1516,19 @@
         <v>37</v>
       </c>
       <c r="B33" t="s">
-        <v>85</v>
+        <v>89</v>
       </c>
       <c r="C33" t="s">
-        <v>102</v>
+        <v>110</v>
       </c>
       <c r="D33">
-        <v>1</v>
+        <v>5</v>
       </c>
       <c r="E33">
-        <v>1</v>
+        <v>5</v>
       </c>
       <c r="F33" t="s">
-        <v>134</v>
+        <v>142</v>
       </c>
     </row>
     <row r="34" spans="1:6">
@@ -1499,19 +1536,19 @@
         <v>38</v>
       </c>
       <c r="B34" t="s">
-        <v>86</v>
+        <v>90</v>
       </c>
       <c r="C34" t="s">
-        <v>103</v>
+        <v>111</v>
       </c>
       <c r="D34">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="E34">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="F34" t="s">
-        <v>135</v>
+        <v>143</v>
       </c>
     </row>
     <row r="35" spans="1:6">
@@ -1519,19 +1556,19 @@
         <v>39</v>
       </c>
       <c r="B35" t="s">
-        <v>87</v>
+        <v>91</v>
       </c>
       <c r="C35" t="s">
-        <v>103</v>
+        <v>111</v>
       </c>
       <c r="D35">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="E35">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="F35" t="s">
-        <v>136</v>
+        <v>144</v>
       </c>
     </row>
     <row r="36" spans="1:6">
@@ -1539,10 +1576,10 @@
         <v>40</v>
       </c>
       <c r="B36" t="s">
-        <v>88</v>
+        <v>92</v>
       </c>
       <c r="C36" t="s">
-        <v>102</v>
+        <v>111</v>
       </c>
       <c r="D36">
         <v>1</v>
@@ -1551,7 +1588,7 @@
         <v>1</v>
       </c>
       <c r="F36" t="s">
-        <v>137</v>
+        <v>145</v>
       </c>
     </row>
     <row r="37" spans="1:6">
@@ -1559,10 +1596,10 @@
         <v>41</v>
       </c>
       <c r="B37" t="s">
-        <v>89</v>
+        <v>93</v>
       </c>
       <c r="C37" t="s">
-        <v>102</v>
+        <v>110</v>
       </c>
       <c r="D37">
         <v>1</v>
@@ -1571,7 +1608,7 @@
         <v>1</v>
       </c>
       <c r="F37" t="s">
-        <v>138</v>
+        <v>146</v>
       </c>
     </row>
     <row r="38" spans="1:6">
@@ -1579,10 +1616,10 @@
         <v>42</v>
       </c>
       <c r="B38" t="s">
-        <v>90</v>
+        <v>94</v>
       </c>
       <c r="C38" t="s">
-        <v>102</v>
+        <v>111</v>
       </c>
       <c r="D38">
         <v>1</v>
@@ -1591,7 +1628,7 @@
         <v>1</v>
       </c>
       <c r="F38" t="s">
-        <v>139</v>
+        <v>147</v>
       </c>
     </row>
     <row r="39" spans="1:6">
@@ -1599,10 +1636,10 @@
         <v>43</v>
       </c>
       <c r="B39" t="s">
-        <v>91</v>
+        <v>95</v>
       </c>
       <c r="C39" t="s">
-        <v>103</v>
+        <v>111</v>
       </c>
       <c r="D39">
         <v>1</v>
@@ -1611,7 +1648,7 @@
         <v>1</v>
       </c>
       <c r="F39" t="s">
-        <v>140</v>
+        <v>148</v>
       </c>
     </row>
     <row r="40" spans="1:6">
@@ -1619,10 +1656,10 @@
         <v>44</v>
       </c>
       <c r="B40" t="s">
-        <v>92</v>
+        <v>96</v>
       </c>
       <c r="C40" t="s">
-        <v>102</v>
+        <v>110</v>
       </c>
       <c r="D40">
         <v>1</v>
@@ -1631,7 +1668,7 @@
         <v>1</v>
       </c>
       <c r="F40" t="s">
-        <v>141</v>
+        <v>149</v>
       </c>
     </row>
     <row r="41" spans="1:6">
@@ -1639,10 +1676,10 @@
         <v>45</v>
       </c>
       <c r="B41" t="s">
-        <v>93</v>
+        <v>97</v>
       </c>
       <c r="C41" t="s">
-        <v>103</v>
+        <v>110</v>
       </c>
       <c r="D41">
         <v>1</v>
@@ -1651,7 +1688,7 @@
         <v>1</v>
       </c>
       <c r="F41" t="s">
-        <v>142</v>
+        <v>150</v>
       </c>
     </row>
     <row r="42" spans="1:6">
@@ -1659,10 +1696,10 @@
         <v>46</v>
       </c>
       <c r="B42" t="s">
-        <v>94</v>
+        <v>98</v>
       </c>
       <c r="C42" t="s">
-        <v>102</v>
+        <v>110</v>
       </c>
       <c r="D42">
         <v>1</v>
@@ -1671,7 +1708,7 @@
         <v>1</v>
       </c>
       <c r="F42" t="s">
-        <v>143</v>
+        <v>151</v>
       </c>
     </row>
     <row r="43" spans="1:6">
@@ -1679,10 +1716,10 @@
         <v>47</v>
       </c>
       <c r="B43" t="s">
-        <v>95</v>
+        <v>99</v>
       </c>
       <c r="C43" t="s">
-        <v>103</v>
+        <v>111</v>
       </c>
       <c r="D43">
         <v>1</v>
@@ -1691,7 +1728,7 @@
         <v>1</v>
       </c>
       <c r="F43" t="s">
-        <v>144</v>
+        <v>152</v>
       </c>
     </row>
     <row r="44" spans="1:6">
@@ -1699,10 +1736,10 @@
         <v>48</v>
       </c>
       <c r="B44" t="s">
-        <v>96</v>
+        <v>100</v>
       </c>
       <c r="C44" t="s">
-        <v>103</v>
+        <v>110</v>
       </c>
       <c r="D44">
         <v>1</v>
@@ -1711,7 +1748,7 @@
         <v>1</v>
       </c>
       <c r="F44" t="s">
-        <v>145</v>
+        <v>153</v>
       </c>
     </row>
     <row r="45" spans="1:6">
@@ -1719,10 +1756,10 @@
         <v>49</v>
       </c>
       <c r="B45" t="s">
-        <v>97</v>
+        <v>101</v>
       </c>
       <c r="C45" t="s">
-        <v>102</v>
+        <v>111</v>
       </c>
       <c r="D45">
         <v>1</v>
@@ -1731,7 +1768,7 @@
         <v>1</v>
       </c>
       <c r="F45" t="s">
-        <v>146</v>
+        <v>154</v>
       </c>
     </row>
     <row r="46" spans="1:6">
@@ -1739,10 +1776,10 @@
         <v>50</v>
       </c>
       <c r="B46" t="s">
-        <v>98</v>
+        <v>102</v>
       </c>
       <c r="C46" t="s">
-        <v>103</v>
+        <v>110</v>
       </c>
       <c r="D46">
         <v>1</v>
@@ -1751,7 +1788,7 @@
         <v>1</v>
       </c>
       <c r="F46" t="s">
-        <v>147</v>
+        <v>155</v>
       </c>
     </row>
     <row r="47" spans="1:6">
@@ -1759,10 +1796,10 @@
         <v>51</v>
       </c>
       <c r="B47" t="s">
-        <v>99</v>
+        <v>103</v>
       </c>
       <c r="C47" t="s">
-        <v>103</v>
+        <v>111</v>
       </c>
       <c r="D47">
         <v>1</v>
@@ -1771,7 +1808,7 @@
         <v>1</v>
       </c>
       <c r="F47" t="s">
-        <v>148</v>
+        <v>156</v>
       </c>
     </row>
     <row r="48" spans="1:6">
@@ -1779,10 +1816,10 @@
         <v>52</v>
       </c>
       <c r="B48" t="s">
-        <v>100</v>
+        <v>104</v>
       </c>
       <c r="C48" t="s">
-        <v>103</v>
+        <v>111</v>
       </c>
       <c r="D48">
         <v>1</v>
@@ -1791,7 +1828,7 @@
         <v>1</v>
       </c>
       <c r="F48" t="s">
-        <v>149</v>
+        <v>157</v>
       </c>
     </row>
     <row r="49" spans="1:6">
@@ -1799,10 +1836,10 @@
         <v>53</v>
       </c>
       <c r="B49" t="s">
-        <v>101</v>
+        <v>105</v>
       </c>
       <c r="C49" t="s">
-        <v>102</v>
+        <v>110</v>
       </c>
       <c r="D49">
         <v>1</v>
@@ -1811,7 +1848,87 @@
         <v>1</v>
       </c>
       <c r="F49" t="s">
-        <v>150</v>
+        <v>158</v>
+      </c>
+    </row>
+    <row r="50" spans="1:6">
+      <c r="A50" t="s">
+        <v>54</v>
+      </c>
+      <c r="B50" t="s">
+        <v>106</v>
+      </c>
+      <c r="C50" t="s">
+        <v>111</v>
+      </c>
+      <c r="D50">
+        <v>1</v>
+      </c>
+      <c r="E50">
+        <v>1</v>
+      </c>
+      <c r="F50" t="s">
+        <v>159</v>
+      </c>
+    </row>
+    <row r="51" spans="1:6">
+      <c r="A51" t="s">
+        <v>55</v>
+      </c>
+      <c r="B51" t="s">
+        <v>107</v>
+      </c>
+      <c r="C51" t="s">
+        <v>111</v>
+      </c>
+      <c r="D51">
+        <v>1</v>
+      </c>
+      <c r="E51">
+        <v>1</v>
+      </c>
+      <c r="F51" t="s">
+        <v>160</v>
+      </c>
+    </row>
+    <row r="52" spans="1:6">
+      <c r="A52" t="s">
+        <v>56</v>
+      </c>
+      <c r="B52" t="s">
+        <v>108</v>
+      </c>
+      <c r="C52" t="s">
+        <v>111</v>
+      </c>
+      <c r="D52">
+        <v>1</v>
+      </c>
+      <c r="E52">
+        <v>1</v>
+      </c>
+      <c r="F52" t="s">
+        <v>161</v>
+      </c>
+    </row>
+    <row r="53" spans="1:6">
+      <c r="A53" t="s">
+        <v>57</v>
+      </c>
+      <c r="B53" t="s">
+        <v>109</v>
+      </c>
+      <c r="C53" t="s">
+        <v>110</v>
+      </c>
+      <c r="D53">
+        <v>1</v>
+      </c>
+      <c r="E53">
+        <v>1</v>
+      </c>
+      <c r="F53" t="s">
+        <v>162</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
feat(ai): complete word-by-word adjudication of 2000 candidate terms into 137 pure emotion words and 771 purged non-emotion words
</commit_message>
<xml_diff>
--- a/data/derived_outputs/clean_emotion_words_2000_reviews.xlsx
+++ b/data/derived_outputs/clean_emotion_words_2000_reviews.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="214" uniqueCount="163">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="554" uniqueCount="412">
   <si>
     <t>word</t>
   </si>
@@ -133,27 +133,225 @@
     <t>charming</t>
   </si>
   <si>
+    <t>sad</t>
+  </si>
+  <si>
+    <t>splurge</t>
+  </si>
+  <si>
+    <t>stuck</t>
+  </si>
+  <si>
+    <t>suffer</t>
+  </si>
+  <si>
+    <t>thoughtful</t>
+  </si>
+  <si>
+    <t>unsafe</t>
+  </si>
+  <si>
+    <t>witty</t>
+  </si>
+  <si>
+    <t>wonderfully</t>
+  </si>
+  <si>
+    <t>adventurous</t>
+  </si>
+  <si>
+    <t>anxious</t>
+  </si>
+  <si>
     <t>astonishing</t>
   </si>
   <si>
+    <t>cherish</t>
+  </si>
+  <si>
+    <t>discomfort</t>
+  </si>
+  <si>
+    <t>safest</t>
+  </si>
+  <si>
+    <t>sensational</t>
+  </si>
+  <si>
+    <t>superbly</t>
+  </si>
+  <si>
+    <t>worthy</t>
+  </si>
+  <si>
+    <t>amusing</t>
+  </si>
+  <si>
+    <t>apologetic</t>
+  </si>
+  <si>
+    <t>astounding</t>
+  </si>
+  <si>
+    <t>awestruck</t>
+  </si>
+  <si>
+    <t>bummed</t>
+  </si>
+  <si>
+    <t>bummer</t>
+  </si>
+  <si>
+    <t>calmed</t>
+  </si>
+  <si>
+    <t>captivated</t>
+  </si>
+  <si>
+    <t>cordial</t>
+  </si>
+  <si>
+    <t>curiosity</t>
+  </si>
+  <si>
+    <t>discouraged</t>
+  </si>
+  <si>
+    <t>dizziness</t>
+  </si>
+  <si>
+    <t>exhausted</t>
+  </si>
+  <si>
+    <t>faultless</t>
+  </si>
+  <si>
+    <t>glowing</t>
+  </si>
+  <si>
+    <t>happiness</t>
+  </si>
+  <si>
+    <t>horrible</t>
+  </si>
+  <si>
+    <t>hospitable</t>
+  </si>
+  <si>
+    <t>joyful</t>
+  </si>
+  <si>
+    <t>peacefully</t>
+  </si>
+  <si>
+    <t>precious</t>
+  </si>
+  <si>
+    <t>raving</t>
+  </si>
+  <si>
+    <t>refreshing</t>
+  </si>
+  <si>
+    <t>romantic</t>
+  </si>
+  <si>
+    <t>ruined</t>
+  </si>
+  <si>
+    <t>satisfying</t>
+  </si>
+  <si>
+    <t>scare</t>
+  </si>
+  <si>
+    <t>seamless</t>
+  </si>
+  <si>
+    <t>seasick</t>
+  </si>
+  <si>
+    <t>unstable</t>
+  </si>
+  <si>
+    <t>vibrant</t>
+  </si>
+  <si>
     <t>bothering</t>
   </si>
   <si>
+    <t>calmer</t>
+  </si>
+  <si>
+    <t>carefree</t>
+  </si>
+  <si>
+    <t>cheerfully</t>
+  </si>
+  <si>
+    <t>classy</t>
+  </si>
+  <si>
+    <t>claustrophobic</t>
+  </si>
+  <si>
+    <t>clever</t>
+  </si>
+  <si>
+    <t>curious</t>
+  </si>
+  <si>
+    <t>desperate</t>
+  </si>
+  <si>
+    <t>embarrassed</t>
+  </si>
+  <si>
+    <t>enthralled</t>
+  </si>
+  <si>
+    <t>enthusiastically</t>
+  </si>
+  <si>
     <t>exhilaration</t>
   </si>
   <si>
     <t>frightening</t>
   </si>
   <si>
+    <t>hilarious</t>
+  </si>
+  <si>
     <t>intimidating</t>
   </si>
   <si>
+    <t>inviting</t>
+  </si>
+  <si>
     <t>irritated</t>
   </si>
   <si>
+    <t>jealous</t>
+  </si>
+  <si>
+    <t>jovial</t>
+  </si>
+  <si>
+    <t>marvelously</t>
+  </si>
+  <si>
+    <t>nauseated</t>
+  </si>
+  <si>
+    <t>nervousness</t>
+  </si>
+  <si>
     <t>overwhelmed</t>
   </si>
   <si>
+    <t>overwhelmingly</t>
+  </si>
+  <si>
     <t>pumped</t>
   </si>
   <si>
@@ -169,9 +367,66 @@
     <t>relieved</t>
   </si>
   <si>
+    <t>rewarding</t>
+  </si>
+  <si>
+    <t>screaming</t>
+  </si>
+  <si>
+    <t>shaking</t>
+  </si>
+  <si>
     <t>soothing</t>
   </si>
   <si>
+    <t>spellbinding</t>
+  </si>
+  <si>
+    <t>splendor</t>
+  </si>
+  <si>
+    <t>spoil</t>
+  </si>
+  <si>
+    <t>spoiled</t>
+  </si>
+  <si>
+    <t>squeamish</t>
+  </si>
+  <si>
+    <t>suffered</t>
+  </si>
+  <si>
+    <t>suffering</t>
+  </si>
+  <si>
+    <t>superlative</t>
+  </si>
+  <si>
+    <t>threaten</t>
+  </si>
+  <si>
+    <t>touching</t>
+  </si>
+  <si>
+    <t>trustworthy</t>
+  </si>
+  <si>
+    <t>uneasy</t>
+  </si>
+  <si>
+    <t>unnerving</t>
+  </si>
+  <si>
+    <t>unpleasant</t>
+  </si>
+  <si>
+    <t>unspoiled</t>
+  </si>
+  <si>
+    <t>warmest</t>
+  </si>
+  <si>
     <t>weird</t>
   </si>
   <si>
@@ -289,27 +544,225 @@
     <t>迷人讨喜的</t>
   </si>
   <si>
+    <t>悲伤的 / 遗憾痛心的</t>
+  </si>
+  <si>
+    <t>挥霍犒赏自己（特别体验）</t>
+  </si>
+  <si>
+    <t>卡住被困的（焦虑）</t>
+  </si>
+  <si>
+    <t>遭受痛苦/晕机</t>
+  </si>
+  <si>
+    <t>贴心周到的</t>
+  </si>
+  <si>
+    <t>感觉不安全的 / 担惊受怕的</t>
+  </si>
+  <si>
+    <t>风趣幽默的</t>
+  </si>
+  <si>
+    <t>极其出色绝妙地</t>
+  </si>
+  <si>
+    <t>充满冒险刺激感的</t>
+  </si>
+  <si>
+    <t>焦虑不安的 / 挂虑的</t>
+  </si>
+  <si>
     <t>令人惊叹的</t>
   </si>
   <si>
+    <t>珍视 / 珍惜铭记</t>
+  </si>
+  <si>
+    <t>身体/心理不适感</t>
+  </si>
+  <si>
+    <t>最安全平稳的</t>
+  </si>
+  <si>
+    <t>绝佳轰动震撼的</t>
+  </si>
+  <si>
+    <t>出类拔萃完美地</t>
+  </si>
+  <si>
+    <t>非常值的 / 值得的</t>
+  </si>
+  <si>
+    <t>风趣风趣令人发笑的</t>
+  </si>
+  <si>
+    <t>诚恳抱歉致歉的</t>
+  </si>
+  <si>
+    <t>令人无比震撼惊叹的</t>
+  </si>
+  <si>
+    <t>充满敬畏震撼的</t>
+  </si>
+  <si>
+    <t>感到扫兴遗憾失落的</t>
+  </si>
+  <si>
+    <t>令人扫兴扫兴的事</t>
+  </si>
+  <si>
+    <t>心情平静安稳下来的</t>
+  </si>
+  <si>
+    <t>被深深吸引着迷的</t>
+  </si>
+  <si>
+    <t>热情亲切礼貌的</t>
+  </si>
+  <si>
+    <t>好奇心 / 探索欲</t>
+  </si>
+  <si>
+    <t>感到灰心气馁的</t>
+  </si>
+  <si>
+    <t>头晕目眩不适</t>
+  </si>
+  <si>
+    <t>精疲力竭极为疲惫的</t>
+  </si>
+  <si>
+    <t>无可挑剔完美的</t>
+  </si>
+  <si>
+    <t>极度赞赏口碑极佳的</t>
+  </si>
+  <si>
+    <t>幸福快乐感</t>
+  </si>
+  <si>
+    <t>极度糟糕可怕的</t>
+  </si>
+  <si>
+    <t>殷勤好客的</t>
+  </si>
+  <si>
+    <t>充满喜悦欢快的</t>
+  </si>
+  <si>
+    <t>宁静和平地</t>
+  </si>
+  <si>
+    <t>弥足珍贵的 memory</t>
+  </si>
+  <si>
+    <t>赞不绝口极力推荐的</t>
+  </si>
+  <si>
+    <t>令人神清气爽耳目一新的</t>
+  </si>
+  <si>
+    <t>浪漫惬意的</t>
+  </si>
+  <si>
+    <t>毁掉行程的 / 扫兴糟心的</t>
+  </si>
+  <si>
+    <t>令人称心满意的</t>
+  </si>
+  <si>
+    <t>吓人 / 引发恐慌的</t>
+  </si>
+  <si>
+    <t>流畅无缝无摩擦的</t>
+  </si>
+  <si>
+    <t>晕船 / 晕眩恶心的</t>
+  </si>
+  <si>
+    <t>不稳定摇晃令人担心的</t>
+  </si>
+  <si>
+    <t>生机勃勃色彩斑斓的</t>
+  </si>
+  <si>
     <t>打扰令人烦心的</t>
   </si>
   <si>
+    <t>更平静安心的</t>
+  </si>
+  <si>
+    <t>无忧无虑自在的</t>
+  </si>
+  <si>
+    <t>欢快愉悦地</t>
+  </si>
+  <si>
+    <t>高端优雅的</t>
+  </si>
+  <si>
+    <t>感到幽闭恐惧压抑的</t>
+  </si>
+  <si>
+    <t>聪明睿智的</t>
+  </si>
+  <si>
+    <t>好奇求知的</t>
+  </si>
+  <si>
+    <t>感到绝望迫切的</t>
+  </si>
+  <si>
+    <t>感到尴尬难堪的</t>
+  </si>
+  <si>
+    <t>被深深吸引迷住的</t>
+  </si>
+  <si>
+    <t>热情高涨地</t>
+  </si>
+  <si>
     <t>极度兴奋快感</t>
   </si>
   <si>
     <t>令人惊恐吓人的</t>
   </si>
   <si>
+    <t>爆笑幽默搞笑的</t>
+  </si>
+  <si>
     <t>令人胆怯令人畏惧的</t>
   </si>
   <si>
+    <t>引人入胜令人愉悦的</t>
+  </si>
+  <si>
     <t>感到恼火烦躁的</t>
   </si>
   <si>
+    <t>令人羡慕嫉妒的</t>
+  </si>
+  <si>
+    <t>欢快风趣的</t>
+  </si>
+  <si>
+    <t>奇妙极其出色地</t>
+  </si>
+  <si>
+    <t>感到恶心反胃不适的</t>
+  </si>
+  <si>
+    <t>紧张不安的情绪</t>
+  </si>
+  <si>
     <t>被震撼/感动深深淹没的</t>
   </si>
   <si>
+    <t>压倒性震撼地</t>
+  </si>
+  <si>
     <t>兴奋激动的 / 跃跃欲试</t>
   </si>
   <si>
@@ -325,9 +778,66 @@
     <t>宽慰的 / 松了一口气</t>
   </si>
   <si>
+    <t>非常有成就感/物超所值的</t>
+  </si>
+  <si>
+    <t>惊恐尖叫的</t>
+  </si>
+  <si>
+    <t>吓得发抖颤抖的</t>
+  </si>
+  <si>
     <t>舒缓抚慰人心的</t>
   </si>
   <si>
+    <t>扣人心弦迷人的</t>
+  </si>
+  <si>
+    <t>壮丽辉煌的奇观</t>
+  </si>
+  <si>
+    <t>破坏 / 毁掉（好心情）</t>
+  </si>
+  <si>
+    <t>好心情被破坏毁掉的</t>
+  </si>
+  <si>
+    <t>胆怯恶心体质易受惊的</t>
+  </si>
+  <si>
+    <t>遭受身体/晕眩痛苦</t>
+  </si>
+  <si>
+    <t>受苦受难不适</t>
+  </si>
+  <si>
+    <t>顶级极致赞赏的</t>
+  </si>
+  <si>
+    <t>受到威胁/令人不安的</t>
+  </si>
+  <si>
+    <t>令人动容流泪的</t>
+  </si>
+  <si>
+    <t>值得信赖靠谱的</t>
+  </si>
+  <si>
+    <t>心神不宁感到不安的</t>
+  </si>
+  <si>
+    <t>令人发慌不安吓人的</t>
+  </si>
+  <si>
+    <t>令人不快令人难受的</t>
+  </si>
+  <si>
+    <t>未经破坏原始纯粹的</t>
+  </si>
+  <si>
+    <t>最暖心亲切的</t>
+  </si>
+  <si>
     <t>古怪令人不安的</t>
   </si>
   <si>
@@ -350,6 +860,9 @@
   </si>
   <si>
     <t>E2_Appraisal (Stimulus/Service Attribute)</t>
+  </si>
+  <si>
+    <t>E1_E2_Polysemous (State &amp; Appraisal)</t>
   </si>
   <si>
     <t>review_5f25933d61b76b7852dc85ff :: We booked Seawind on the cruise dock since we were uncertain about the weather.  We were assured the views would be good at Misty Fiords, so off we went!  The shuttle to and from t...</t>
@@ -454,43 +967,289 @@
     <t>review_2437be8aa60056f18e560577 :: Our flight over Kaua'i with our charming, skillful pilot was the best experience of our island vacation. She gave a most interesting and helpful account of what we could see below,...</t>
   </si>
   <si>
+    <t>review_641866daade55fe429557808 :: Unfortunately Denali was socked in with weather. Also the glaciers had degraded to the point of no landings. We were very sad. K2 offered us an option to Knik. It was UNBELIEVABLE!...</t>
+  </si>
+  <si>
+    <t>review_eda1a4bce0aac45015172f03 :: We heard so much about how beautiful Kauai was, but after driving around the entire island, we weren't that impressed. Mind you, we had just seen all the major sights of Maui, so w...</t>
+  </si>
+  <si>
+    <t>review_6df5ede0e4f38741f16273cc :: A fantastic flyover of the island.  A beautiful land with mountains, waterfalls, plantations, golf courses and the Napali Coast.  JT, the pilot was excellent and provided insight t...</t>
+  </si>
+  <si>
+    <t>review_5b5f5f21f1453f7f0c8229bf :: We did Wings Over Kauai on our first day on the island.  Bruce was an excellent pilot and shared lots of interesting information about Kauai.  The clouds passing over allowing the ...</t>
+  </si>
+  <si>
+    <t>review_afe3c66ee7b7c941929e9cfa :: In June 2010 4 of us took the Grand Denali Tour.  Booking this tour on our own separate from the cruise line was a bit tricky but saved us a great deal.  Elaine from K2 was most pl...</t>
+  </si>
+  <si>
+    <t>review_9fa767c0524e34fd96ef3ff4 :: Not a typical I loved it review. But I was very impressed with K2 and the way they run their business. We were booked for a glacier landing tour today but unfortunately the weather...</t>
+  </si>
+  <si>
+    <t>review_85b8dedf61096ea65b0cf853 :: We took our six children on this flight, and Dan was not just a good pilot. He was knowledgeable, had a witty personality, and educated us a lot about the landscapes, logging, and ...</t>
+  </si>
+  <si>
+    <t>review_4a7f3da7f6659561289690b5 :: Although we had to re-schedule our original reservation because of constant rainfall after having driven an hour to the destination, we were accommodated with a different date and ...</t>
+  </si>
+  <si>
+    <t>review_433ee9cdb612a1be49d51792 :: Wow! A must do when you are even near the Miami area. I moved to Miami in 1984 and I now live about 90 miles north of Miami. This is a must do and do yourself a favor and take the ...</t>
+  </si>
+  <si>
+    <t>review_74168f066a91714dc278f85e :: Amazing views of Denali- we were fortunate to have a clear day. Leighan, our pilot, was amazing. The flight was smooth, landing on the glacier was awe-inspiring, and her commentary...</t>
+  </si>
+  <si>
     <t>review_7bbe5f17c5ccf78fd605ad3d :: From the front reception area to preparing for take off to our amazing pilot from the Arctic, this tour was astonishing. We were blessed with a beautiful sunny day with big white p...</t>
   </si>
   <si>
+    <t>review_20bafb242eb918bb14d9309d :: We really enjoyed our tour! Staff were very friendly and our pilot, Doug, provided us with a safe, interesting and enjoyable flight. We would definitely recommend Wings Over Kauai....</t>
+  </si>
+  <si>
+    <t>review_b3611bb117be728e25d5ddec :: We had booked the 11 am tour online even before we reached Kauai. We called ahead and the person who answered told us we could come by 10:45 am or so. We reached round about then o...</t>
+  </si>
+  <si>
+    <t>review_fe566c581798d89f19f642e5 :: My husband and I were rained or otherwise "bad-weathered" out of every adventure we planned on Kauai.  Couldn't hike Kalalau due to the river crossing being flooded. 
+Couldn't kaya...</t>
+  </si>
+  <si>
+    <t>review_69b44dac34b50350cfb373aa :: Steve, our pilot was sensational.   We were greeted by name, promptness, and courtesy.  They took our bags and explained the flight procedure.   Steve pointed out areas of interest...</t>
+  </si>
+  <si>
+    <t>review_bcedc98e43ad7edec05befa8 :: There isn't much to say here, except the experience was fantastic. Seeing the landscape from the air was breathtaking, and landing and taking off from the glacier was a hoot. Our p...</t>
+  </si>
+  <si>
+    <t>review_d38fb233c92c34b779e4871c :: Wow - what an experience! I had the opportunity to take two separate flights - one in their Cessna and one in their incredible cherry red biplane (the only one on the island). 
+On...</t>
+  </si>
+  <si>
+    <t>review_c953e7d03bf994fca6d74d5d :: A helicopter trip is the best way to really appreciate the scale of the Grand Canyon and Maverick are a very professional outfit. Our pilot, Mike, was friendly, amusing, knowledgab...</t>
+  </si>
+  <si>
+    <t>review_8bf531e554f4eb9eb061f4ee :: We booked a Denali flight, and when we arrived in Talkeetna by Alaska Rail from Anchorage, the weather was so bad that they canceled it.  They were very professional and apologetic...</t>
+  </si>
+  <si>
+    <t>review_bfd57d15a7e6de7e1824ebd8 :: The wife and I would rate this experience was one of our all time bests. Air Ventures is very professional and appreciative and treats everyone like royalty. We did a helicopter to...</t>
+  </si>
+  <si>
+    <t>review_f85c9d7aa58920de9855549a :: Our entire experience was fabulous!  From Austin, our shuttle driver who took great care of us and our backpacks to and from their site (and had us laughing with his jokes), to our...</t>
+  </si>
+  <si>
+    <t>review_f5388b1e976e59c78115bdce :: We came for a flight seeing tour of Denali but due to weather weren’t able to fly that day. I wish I had known to check my email on the morning of the trip, it would have saved me ...</t>
+  </si>
+  <si>
+    <t>review_63c95c18f52ebddff67df7b4 :: We had a wonderful experience flying with Chuck when we were in Ketchikan. He calmed our nerves and we could tell he was very experienced. His plane was absolutely perfect. He gave...</t>
+  </si>
+  <si>
+    <t>review_53fcd6e518ab4f8fb6d54d7d :: Unforgettable!  Views stunning, excellent pilot. We were captivated by all of it...views of Denali and surrounding mountains, glaciers, moose, sheep, trumpet swans. Landing on glac...</t>
+  </si>
+  <si>
+    <t>review_a6425ff1171e21e3392aa88c :: The personnel at Air Ventures cordial, helpful and polite.  I would recommend their services to anyone wanting to get a great aerial view of the Island of Kawaii.
+Our pilot, rob, ...</t>
+  </si>
+  <si>
+    <t>review_49cf9647abacf6af128bd5f4 :: Everything about Talkeetna Air Taxi oozes experience and professionalism.  From the initial decision process on which flight to take, to the actual flight itself, I could not have ...</t>
+  </si>
+  <si>
+    <t>review_8fc23fecb45ba0ee94242f62 :: We are a family with 4 children ages 12 to 19 and spent a week on Kauai.  We really wanted to do an air tour with our kids but the cost of a helicopter flight would have been well ...</t>
+  </si>
+  <si>
+    <t>review_1639755de3ddcfd10c619c0b :: We originally scheduled the flight in Talkeetna. But due to the weather, our flight got cancelled. The people in the office were very patient and tried to help us to re-schedule. T...</t>
+  </si>
+  <si>
+    <t>review_1fe7b796395cf2ecac91e147 :: Our family of 4 booked this trip due to limited time during our vacation to see the Grand Canyon.  I thought it would the perfect solution and sounded like fun.  I have two girls, ...</t>
+  </si>
+  <si>
+    <t>review_77341391cb13d175af149c1d :: My wife is not a good flyer, even on a 767, let alone a little Cessna or the like. There was no way I could get her on a helicopter tour, so the doors off experience wasn't going t...</t>
+  </si>
+  <si>
+    <t>review_b5268b40d3aafe7496fcb498 :: If you are visiting the Grand Canyon, the only way to take in it's full majesty is to do it by Helicopter. Maverick Helicopter were fantastic. You must take a flight with them, wel...</t>
+  </si>
+  <si>
+    <t>review_c8c04aed9cd305332764808f :: I encouraged my husband to take the biplane flight/tour. I had no intention of going. My husband and the pilot Mark encouraged me to go along. The front seat holds two. I decided t...</t>
+  </si>
+  <si>
+    <t>review_ebb70b11c29e696fbd1d4b9d :: Both K2 and Talkeetna Air Taxi (TAT) get my highest recommendation. Follow along with the bouncing ball, kids, as our tale unfolds:
+Pre-booked directly with TAT about a month befo...</t>
+  </si>
+  <si>
+    <t>review_1a8c661361e1a55ed4a0ed52 :: The service provided by the Wings Over Kauai tours was very well done.  Ellen was very hospitable while waiting for our scheduled flight.  Capt. Josh has a very clear passion for a...</t>
+  </si>
+  <si>
+    <t>review_27ee31e44dec37dd44a492ba :: Eric, the pilot, is a amazing guy doing a great job! He said we are sharing his dream, actually he was making my dream come true by letting my little girl driving a little bit! Sou...</t>
+  </si>
+  <si>
+    <t>review_09687f3c5332ab59381de30a :: It was perfect and we would go again with this same company. A small fixed wing plane seating a pilot and 2 riders. Things to keep in mind if you pick this small plane-If you are v...</t>
+  </si>
+  <si>
+    <t>review_02d9b6799d194eb3a407125d :: Just got back from Kauai - went on a 1 hour airplane tour over Kauai - very nice experience over the island of Kauai - pilot tells you the sites that you are going over; at the end...</t>
+  </si>
+  <si>
+    <t>review_1758d760d6f52438c4d85cce :: Bruce the pilot was great with our 2 nervous flyers.  He gave a great talk while we were flying and patiently answered any/all questions.  All of us were raving about the tour long...</t>
+  </si>
+  <si>
+    <t>review_8343a9e5e6828bbdfdd832af :: We are 'local' (Anchorage) and had scheduled a trip on Saturday. Friday's trip to Talkeetna was beautiful....Denali visible from our home all the way to Talkeetna. Sarah worked wit...</t>
+  </si>
+  <si>
+    <t>review_ec2216c5191fd0c8ebfb9e1d :: amazing experience thanks a lot.
+highly recommended 
+max was amazing 
+very romantic 
+the view was perfect...</t>
+  </si>
+  <si>
+    <t>review_2d3f2a00e6ef98ca5161d902 :: The pilots are excellent, friendly, knowledgeable, and skilled. 
+But, don’t get your weight estimate wrong or Keith at the front desk will talk down to you as if you lied on purpo...</t>
+  </si>
+  <si>
+    <t>review_10fbd937c93c8e5b1ea0bd58 :: I traveled to Alaska for my 50th birthday and my experience with K2 sits on the top of my list and we did ALOT. We flew around Denali Mtn. on the 2 hour glacier landing trip. I lov...</t>
+  </si>
+  <si>
+    <t>review_5d94a7bb9a8a4324e9b57891 :: We chose the South face Tour with Glacier Landing. The check in was fast and easy. The staff was super nice. You have to weigh yourself and your belongings and they determine how t...</t>
+  </si>
+  <si>
+    <t>review_0f34dc86f2887a73f98dad09 :: We were 2 couples traveling on the Pride of America. Pilot Marcus took us on a spectacular flight over Kauai. It was a highlight of our cruise. His commentary was very interesting ...</t>
+  </si>
+  <si>
+    <t>review_b4defed8dabe04d3de367e4c :: Awesome service. Our pilot, Bruce, made a point to keep track of all our names and interacted with each of us by name throughout the flight. A very nice touch. We actually flew thr...</t>
+  </si>
+  <si>
+    <t>review_905ea7ae4640bfc3d91b8080 :: This trip around Mt Denali was breath taking and our pilot was awsome on knowledge and making sure we all had great views for pictures. The sky around the mountain was clear but th...</t>
+  </si>
+  <si>
     <t>review_4527b031d210aa6a5f73a0b7 :: There are 2 companies side by side that offer this, we went with Air Adventures do to availability (the other co I found first but they were booked .. this co was rated exactly the...</t>
   </si>
   <si>
+    <t>review_86bd6193f824d794bcf2deb5 :: When you pick an aerial solution to fly over Kauai, you have basically two choices - helicopters or fixed wing aircraft.
+Air ventures represents the best solution on Kauai for the...</t>
+  </si>
+  <si>
+    <t>review_e79cf3a7f8937f62d92afb5c :: A full day adventure visiting the west side of the Grand Canyon. Ryan, our pilot and guide, was very knowledgeable and super nice. Seeing a part of Arizona from above was interesti...</t>
+  </si>
+  <si>
+    <t>review_0eb891565b48a8217c71c654 :: K-2 Aviation is the best.   They are friendly and fun, while being professional at the same time.  Making a reservation was easy, and I called back a couple of times to confirm, si...</t>
+  </si>
+  <si>
+    <t>review_666e1f42eced3751f3747622 :: 5STARS ALL THE WAY: once in a lifetime moment! OK but so this is really a response to another  4 star review that honestly I had a problem with reading because everyone is such a c...</t>
+  </si>
+  <si>
+    <t>review_aa13884aeefdbbcacd63a44a :: We were scheduled to do a different tour and ended up not being able to do it.  (Due to bad knees).  We came across a brochure for Wings Over Kauai Air Tours.  We decided to try it...</t>
+  </si>
+  <si>
+    <t>review_bb3a9cb8ec67e136fcaefc32 :: Had a great time! Cool vintage plane! Perfect amount of time and narration. Oren was a clever guide. Highly recommend. Our teenager loved it....</t>
+  </si>
+  <si>
+    <t>review_5d9eea119504a77b7f64c33f :: So the BF and I were debating whether to view the Na Pali Coast by water or air.  I made the executive decision to do both.  We did the cheaper sunset cruise with Captain Andy's th...</t>
+  </si>
+  <si>
+    <t>review_93002c7973ba2bb5ce9edb94 :: My husband and I were desperate to take a flight over Kauai but were concerned we wouldn't be able to because of our children being so young (3yrs and 1yr). We stumbled across Wing...</t>
+  </si>
+  <si>
+    <t>review_46ddfd4445283a6a81911504 :: Booked the Grand Canyon Discovery Tour and very unimpressed with how short the flight time was (less than ten minutes total) with a short photo op stop on a ridge in the canyon.  O...</t>
+  </si>
+  <si>
+    <t>review_eb0c2bb6de3d5ffa9eac3e15 :: We took the around Denali flight over an hour on a beautiful day. Perfect weather ,great pilot "Nick". When we got there there were some questions as to if we should take this more...</t>
+  </si>
+  <si>
+    <t>review_8294fe79e0415f552542ed94 :: The flight was enjoyable but not earth shattering like promoted! Pilot Patrick was doing a job not actively enthusiastically participating so I’d rate that part as average. Without...</t>
+  </si>
+  <si>
     <t>review_23bc28108b7fc9fb77931ab6 :: From the shuttle driver the book..In procedure to the professionalism of the pilot and the beautiful scenery and the exhilaration of landing on the glacier this is a must do tour...</t>
   </si>
   <si>
     <t>review_ad4c129d7431549c0c82f1a8 :: Three of us signed up for the plane ride about a month in advance. There were really high winds that day (40 mph+), but the company didn't cancel so we went for the ride. 15 minute...</t>
   </si>
   <si>
+    <t>review_af9c2e4c708b6ef1ddffbdef :: We booked this as part of a Viator package to see Alcatraz and it completely blew us away.  We were a party of 4 - two adults, a ten year old and a 4 year old.  Despite a total fea...</t>
+  </si>
+  <si>
     <t>review_366a0217246d209bb9329b77 :: How do you describe something that takes your words away and leaves you speechless?  This was meant to be a Floatplane and Alaskan Bear excursion.  We definitely saw the floatplane...</t>
   </si>
   <si>
+    <t>review_39496617c0521efe63e69b0a :: Our trip was a blast! The Pilot was knowledgeable about the area and made the whole experience fun! The flight was smooth and the scenes were beautiful! The office gals were friend...</t>
+  </si>
+  <si>
     <t>review_b226b58865dcbe2109b81484 :: We recently took a flight seeing trip to Misty Fjords with Taquan Air.  We chose this company because of the B1G1 free coupon offered in the Toursaver coupon book.  I really didn't...</t>
   </si>
   <si>
+    <t>review_21f52836b887ea5e81a636ac :: Everyone that does the open door helicopter tour will tell you to DO IT. I am telling you try something different and do the BIPLANE. It was fantastic. The tour lasted longer than ...</t>
+  </si>
+  <si>
+    <t>review_e5850680238945a96a3caa96 :: This flightseeing tour with subsequent glacier landing was one of the coolest things I have ever done in my life, and one of the few activities where the views and experience is wo...</t>
+  </si>
+  <si>
+    <t>review_8b9e0dc5c5d87b98d2a06acb :: Great professionalism and unsurpassed scenery.  Pay the extra fee for the glacier landing. I grew up in Alaska and have visited Denali Park at least 30 times. Nevertheless, I'd nev...</t>
+  </si>
+  <si>
+    <t>review_ff282b470223120e69c6a4b8 :: This flightseeing trip was the pinnacle of 2 weeks of amazing experiences.  Words and pictures fail to convey what a flight around McKinley is like. I thought that upon landing my ...</t>
+  </si>
+  <si>
     <t>review_b0feded8c30b74f0a67e42f9 :: We absolutely loved our sunset trip. I was overwhelmed with how much the lady was willing to help me set up our trip. I had lots of scheduling issues and they saved the day!...</t>
   </si>
   <si>
+    <t>review_b5b0e8c69a1888eb640268f9 :: The folks at Talkeetna Air Taxi made our entire experience very enjoyable.  The weather had been overcast for days prior to our flight and the staff was very patient and understand...</t>
+  </si>
+  <si>
     <t>review_ed11136814c2ac8d48de6594 :: My husband and I were so pumped with our private Cessna adventure with Kevin as our pilot!  The flight was beautiful and informative and a super value - probably our favorite excur...</t>
   </si>
   <si>
     <t>review_6b17f5b0218c6e596e18af08 :: Took a noon flight to Friday harbor. Great flight great views!!  Smooth ride.  Friday harbor was lovely.  Quaint shops and restaurants. Took an afternoon flight back.  Also great f...</t>
   </si>
   <si>
-    <t>review_f5388b1e976e59c78115bdce :: We came for a flight seeing tour of Denali but due to weather weren’t able to fly that day. I wish I had known to check my email on the morning of the trip, it would have saved me ...</t>
-  </si>
-  <si>
     <t>review_aa76425694a5e2a07140dc28 :: We were scheduled to fly over Denali, but weather did not cooperate and pilots had to regrettably cancel flights.  The folks at K2 were very apologetic and understood our disappoin...</t>
   </si>
   <si>
     <t>review_0fd62b59dfddedcc4ce37b1b :: We arrived in good time and after  paying and being weighed for the correct distribution within the helicopter, we sat and waited for the 3 other passengers. The area you sit and w...</t>
   </si>
   <si>
+    <t>review_20a5d0a4abc1952fcfbb43d0 :: Had a flight seeing tour with K2. We couldn't do the glacier landing due to weather conditions but nevermind, we still very much enjoyed that our. We saw dramatic landscape, glacie...</t>
+  </si>
+  <si>
+    <t>review_326f19457a589d42a33ff874 :: Can't express how amazing this flightseeing was!! We did Mt. McKinley base camp with glacier landing. During the flight, I was just screaming (nobody could hear me as everyone wore...</t>
+  </si>
+  <si>
     <t>review_06c317e4d5d8ceacebdaa76d :: The scenery was amazing!  There is so much natural beauty in Kauai and this is a great and special way to see it.  Some of the interior parts of Kauai are only visible by air, as t...</t>
+  </si>
+  <si>
+    <t>review_8d4ddb6f94926e611f27073f :: I took the 30 minute San Francisco Bay tour on August 28th at 3:15.  It was a spectacular day with some fog around the Golden Gate Bridge.  We flew around and over every major tour...</t>
+  </si>
+  <si>
+    <t>review_60729dc12e183107376e19e8 :: We did the 1.5 hour flight with the glacier landing.  Words cannot explain the beauty and splendor of  Mount McKinley up close and personal like this.  It was truly amazing.  Our p...</t>
+  </si>
+  <si>
+    <t>review_38c140061a79f5dc4b034f30 :: Well.. I suppose we were really lucky ducks. ..
+Booked month in advance from downunder..flew specially over from our holiday stay on Waikiki for this trip.
+On arrival our booking w...</t>
+  </si>
+  <si>
+    <t>review_be8faf48d8d937ed7f366e98 :: K2 Aviation is a super friendly and well-run organization. Views were amazing. So glad my teenage kids got to really see a glacier for what it is. We'd talked about them so much on...</t>
+  </si>
+  <si>
+    <t>review_b0217b73fa2d49d7679ca1b5 :: We took the flight and I realized that I should have done this the first day of our vacation.  We waited a week for our relatives and they got the benefit of the overview that woul...</t>
+  </si>
+  <si>
+    <t>review_4002b14844a9fdb69e609624 :: The staff are cordial and warm. They called us in advance to warn us about inclement weather and cancellation of the tour on the day in question. The day of the tour , we arrived t...</t>
+  </si>
+  <si>
+    <t>review_ce23c1ddd00fe162177658fe :: To be fair, I want to say upfront that this review focuses not only on the provider but also on Trip Advisor (based on the comments of the owner/vendor that Trip Advisor is horribl...</t>
+  </si>
+  <si>
+    <t>review_65f6eeef22d6baf1636ca70e :: I have travelled to many parts of the world but this 2 hour flight with TAT is THEE BEST experience I can ever recall. They are seasoned professionals that will greatly exceed your...</t>
+  </si>
+  <si>
+    <t>review_d579c7ce2ec144775d909031 :: My family and I booked a package tour with Friday Harbor Seaplanes and Western Prince Explorer Whale Watching. We all had a great and comfortable time on the flight, which felt saf...</t>
+  </si>
+  <si>
+    <t>review_28c726804d0b55cac4d79f6a :: The staff is great and it's a great way to see the entire Island which you can't do with a car... However, if you are at all uneasy about flying, you should think twice about going...</t>
+  </si>
+  <si>
+    <t>review_25a5df0aa1c4c82bb9d30e47 :: This was a treat!  I've taken a helicopter tour, which was cool, but sometimes a little unnerving.  If you want a little more metal around your seat area, do this flight.  The ride...</t>
+  </si>
+  <si>
+    <t>review_7cd1afc1532ba6ca69afe686 :: This company deserves to be given the golden buzzer award for being the worst company in Miami. We paid double the price to reach to the airport, we were left waiting with no one t...</t>
+  </si>
+  <si>
+    <t>review_94adaa49f35fc20844991ace :: We took the flight tour of the Misty Fjords Wilderness when our cruise ship was in Ketchikan.  Lesley and her husband who own the business are wonderful to deal with.  They are bot...</t>
+  </si>
+  <si>
+    <t>review_95ec6a711bfc4f4d25ea7e38 :: We had a brilliant time on our Cessna tour, we're still talking about it in awe. From the moment we arrived and received the warmest welcome and smoothest check-in with the lovely ...</t>
   </si>
   <si>
     <t>review_25709817e43e27ba434614d8 :: Beautiful views from a perspective we hadn’t seen before. Pilot was great, especially with the weird winds that day. Staff helpful and friendly....</t>
@@ -868,7 +1627,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:F53"/>
+  <dimension ref="A1:F138"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:6">
@@ -896,10 +1655,10 @@
         <v>6</v>
       </c>
       <c r="B2" t="s">
-        <v>58</v>
+        <v>143</v>
       </c>
       <c r="C2" t="s">
-        <v>110</v>
+        <v>280</v>
       </c>
       <c r="D2">
         <v>12</v>
@@ -908,7 +1667,7 @@
         <v>12</v>
       </c>
       <c r="F2" t="s">
-        <v>112</v>
+        <v>283</v>
       </c>
     </row>
     <row r="3" spans="1:6">
@@ -916,10 +1675,10 @@
         <v>7</v>
       </c>
       <c r="B3" t="s">
-        <v>59</v>
+        <v>144</v>
       </c>
       <c r="C3" t="s">
-        <v>111</v>
+        <v>281</v>
       </c>
       <c r="D3">
         <v>10</v>
@@ -928,7 +1687,7 @@
         <v>10</v>
       </c>
       <c r="F3" t="s">
-        <v>113</v>
+        <v>284</v>
       </c>
     </row>
     <row r="4" spans="1:6">
@@ -936,10 +1695,10 @@
         <v>8</v>
       </c>
       <c r="B4" t="s">
-        <v>60</v>
+        <v>145</v>
       </c>
       <c r="C4" t="s">
-        <v>111</v>
+        <v>281</v>
       </c>
       <c r="D4">
         <v>10</v>
@@ -948,7 +1707,7 @@
         <v>9</v>
       </c>
       <c r="F4" t="s">
-        <v>114</v>
+        <v>285</v>
       </c>
     </row>
     <row r="5" spans="1:6">
@@ -956,10 +1715,10 @@
         <v>9</v>
       </c>
       <c r="B5" t="s">
-        <v>61</v>
+        <v>146</v>
       </c>
       <c r="C5" t="s">
-        <v>111</v>
+        <v>281</v>
       </c>
       <c r="D5">
         <v>9</v>
@@ -968,7 +1727,7 @@
         <v>9</v>
       </c>
       <c r="F5" t="s">
-        <v>115</v>
+        <v>286</v>
       </c>
     </row>
     <row r="6" spans="1:6">
@@ -976,10 +1735,10 @@
         <v>10</v>
       </c>
       <c r="B6" t="s">
-        <v>62</v>
+        <v>147</v>
       </c>
       <c r="C6" t="s">
-        <v>111</v>
+        <v>281</v>
       </c>
       <c r="D6">
         <v>9</v>
@@ -988,7 +1747,7 @@
         <v>9</v>
       </c>
       <c r="F6" t="s">
-        <v>116</v>
+        <v>287</v>
       </c>
     </row>
     <row r="7" spans="1:6">
@@ -996,10 +1755,10 @@
         <v>11</v>
       </c>
       <c r="B7" t="s">
-        <v>63</v>
+        <v>148</v>
       </c>
       <c r="C7" t="s">
-        <v>111</v>
+        <v>281</v>
       </c>
       <c r="D7">
         <v>9</v>
@@ -1008,7 +1767,7 @@
         <v>9</v>
       </c>
       <c r="F7" t="s">
-        <v>117</v>
+        <v>288</v>
       </c>
     </row>
     <row r="8" spans="1:6">
@@ -1016,10 +1775,10 @@
         <v>12</v>
       </c>
       <c r="B8" t="s">
-        <v>64</v>
+        <v>149</v>
       </c>
       <c r="C8" t="s">
-        <v>111</v>
+        <v>281</v>
       </c>
       <c r="D8">
         <v>8</v>
@@ -1028,7 +1787,7 @@
         <v>8</v>
       </c>
       <c r="F8" t="s">
-        <v>118</v>
+        <v>289</v>
       </c>
     </row>
     <row r="9" spans="1:6">
@@ -1036,10 +1795,10 @@
         <v>13</v>
       </c>
       <c r="B9" t="s">
-        <v>65</v>
+        <v>150</v>
       </c>
       <c r="C9" t="s">
-        <v>110</v>
+        <v>280</v>
       </c>
       <c r="D9">
         <v>8</v>
@@ -1048,7 +1807,7 @@
         <v>8</v>
       </c>
       <c r="F9" t="s">
-        <v>119</v>
+        <v>290</v>
       </c>
     </row>
     <row r="10" spans="1:6">
@@ -1056,10 +1815,10 @@
         <v>14</v>
       </c>
       <c r="B10" t="s">
-        <v>66</v>
+        <v>151</v>
       </c>
       <c r="C10" t="s">
-        <v>110</v>
+        <v>280</v>
       </c>
       <c r="D10">
         <v>7</v>
@@ -1068,7 +1827,7 @@
         <v>7</v>
       </c>
       <c r="F10" t="s">
-        <v>120</v>
+        <v>291</v>
       </c>
     </row>
     <row r="11" spans="1:6">
@@ -1076,10 +1835,10 @@
         <v>15</v>
       </c>
       <c r="B11" t="s">
-        <v>67</v>
+        <v>152</v>
       </c>
       <c r="C11" t="s">
-        <v>111</v>
+        <v>281</v>
       </c>
       <c r="D11">
         <v>7</v>
@@ -1088,7 +1847,7 @@
         <v>7</v>
       </c>
       <c r="F11" t="s">
-        <v>121</v>
+        <v>292</v>
       </c>
     </row>
     <row r="12" spans="1:6">
@@ -1096,10 +1855,10 @@
         <v>16</v>
       </c>
       <c r="B12" t="s">
-        <v>68</v>
+        <v>153</v>
       </c>
       <c r="C12" t="s">
-        <v>111</v>
+        <v>281</v>
       </c>
       <c r="D12">
         <v>7</v>
@@ -1108,7 +1867,7 @@
         <v>7</v>
       </c>
       <c r="F12" t="s">
-        <v>122</v>
+        <v>293</v>
       </c>
     </row>
     <row r="13" spans="1:6">
@@ -1116,10 +1875,10 @@
         <v>17</v>
       </c>
       <c r="B13" t="s">
-        <v>69</v>
+        <v>154</v>
       </c>
       <c r="C13" t="s">
-        <v>111</v>
+        <v>281</v>
       </c>
       <c r="D13">
         <v>7</v>
@@ -1128,7 +1887,7 @@
         <v>7</v>
       </c>
       <c r="F13" t="s">
-        <v>123</v>
+        <v>294</v>
       </c>
     </row>
     <row r="14" spans="1:6">
@@ -1136,10 +1895,10 @@
         <v>18</v>
       </c>
       <c r="B14" t="s">
-        <v>70</v>
+        <v>155</v>
       </c>
       <c r="C14" t="s">
-        <v>111</v>
+        <v>281</v>
       </c>
       <c r="D14">
         <v>7</v>
@@ -1148,7 +1907,7 @@
         <v>6</v>
       </c>
       <c r="F14" t="s">
-        <v>124</v>
+        <v>295</v>
       </c>
     </row>
     <row r="15" spans="1:6">
@@ -1156,10 +1915,10 @@
         <v>19</v>
       </c>
       <c r="B15" t="s">
-        <v>71</v>
+        <v>156</v>
       </c>
       <c r="C15" t="s">
-        <v>111</v>
+        <v>281</v>
       </c>
       <c r="D15">
         <v>7</v>
@@ -1168,7 +1927,7 @@
         <v>7</v>
       </c>
       <c r="F15" t="s">
-        <v>115</v>
+        <v>286</v>
       </c>
     </row>
     <row r="16" spans="1:6">
@@ -1176,10 +1935,10 @@
         <v>20</v>
       </c>
       <c r="B16" t="s">
-        <v>72</v>
+        <v>157</v>
       </c>
       <c r="C16" t="s">
-        <v>111</v>
+        <v>281</v>
       </c>
       <c r="D16">
         <v>6</v>
@@ -1188,7 +1947,7 @@
         <v>6</v>
       </c>
       <c r="F16" t="s">
-        <v>125</v>
+        <v>296</v>
       </c>
     </row>
     <row r="17" spans="1:6">
@@ -1196,10 +1955,10 @@
         <v>21</v>
       </c>
       <c r="B17" t="s">
-        <v>73</v>
+        <v>158</v>
       </c>
       <c r="C17" t="s">
-        <v>110</v>
+        <v>280</v>
       </c>
       <c r="D17">
         <v>6</v>
@@ -1208,7 +1967,7 @@
         <v>6</v>
       </c>
       <c r="F17" t="s">
-        <v>126</v>
+        <v>297</v>
       </c>
     </row>
     <row r="18" spans="1:6">
@@ -1216,10 +1975,10 @@
         <v>22</v>
       </c>
       <c r="B18" t="s">
-        <v>74</v>
+        <v>159</v>
       </c>
       <c r="C18" t="s">
-        <v>111</v>
+        <v>281</v>
       </c>
       <c r="D18">
         <v>6</v>
@@ -1228,7 +1987,7 @@
         <v>6</v>
       </c>
       <c r="F18" t="s">
-        <v>127</v>
+        <v>298</v>
       </c>
     </row>
     <row r="19" spans="1:6">
@@ -1236,10 +1995,10 @@
         <v>23</v>
       </c>
       <c r="B19" t="s">
-        <v>75</v>
+        <v>160</v>
       </c>
       <c r="C19" t="s">
-        <v>111</v>
+        <v>281</v>
       </c>
       <c r="D19">
         <v>6</v>
@@ -1248,7 +2007,7 @@
         <v>5</v>
       </c>
       <c r="F19" t="s">
-        <v>128</v>
+        <v>299</v>
       </c>
     </row>
     <row r="20" spans="1:6">
@@ -1256,10 +2015,10 @@
         <v>24</v>
       </c>
       <c r="B20" t="s">
-        <v>76</v>
+        <v>161</v>
       </c>
       <c r="C20" t="s">
-        <v>110</v>
+        <v>280</v>
       </c>
       <c r="D20">
         <v>6</v>
@@ -1268,7 +2027,7 @@
         <v>6</v>
       </c>
       <c r="F20" t="s">
-        <v>129</v>
+        <v>300</v>
       </c>
     </row>
     <row r="21" spans="1:6">
@@ -1276,10 +2035,10 @@
         <v>25</v>
       </c>
       <c r="B21" t="s">
-        <v>77</v>
+        <v>162</v>
       </c>
       <c r="C21" t="s">
-        <v>110</v>
+        <v>280</v>
       </c>
       <c r="D21">
         <v>6</v>
@@ -1288,7 +2047,7 @@
         <v>5</v>
       </c>
       <c r="F21" t="s">
-        <v>130</v>
+        <v>301</v>
       </c>
     </row>
     <row r="22" spans="1:6">
@@ -1296,10 +2055,10 @@
         <v>26</v>
       </c>
       <c r="B22" t="s">
-        <v>78</v>
+        <v>163</v>
       </c>
       <c r="C22" t="s">
-        <v>110</v>
+        <v>280</v>
       </c>
       <c r="D22">
         <v>6</v>
@@ -1308,7 +2067,7 @@
         <v>6</v>
       </c>
       <c r="F22" t="s">
-        <v>131</v>
+        <v>302</v>
       </c>
     </row>
     <row r="23" spans="1:6">
@@ -1316,10 +2075,10 @@
         <v>27</v>
       </c>
       <c r="B23" t="s">
-        <v>79</v>
+        <v>164</v>
       </c>
       <c r="C23" t="s">
-        <v>110</v>
+        <v>280</v>
       </c>
       <c r="D23">
         <v>6</v>
@@ -1328,7 +2087,7 @@
         <v>6</v>
       </c>
       <c r="F23" t="s">
-        <v>132</v>
+        <v>303</v>
       </c>
     </row>
     <row r="24" spans="1:6">
@@ -1336,10 +2095,10 @@
         <v>28</v>
       </c>
       <c r="B24" t="s">
-        <v>80</v>
+        <v>165</v>
       </c>
       <c r="C24" t="s">
-        <v>111</v>
+        <v>281</v>
       </c>
       <c r="D24">
         <v>6</v>
@@ -1348,7 +2107,7 @@
         <v>6</v>
       </c>
       <c r="F24" t="s">
-        <v>133</v>
+        <v>304</v>
       </c>
     </row>
     <row r="25" spans="1:6">
@@ -1356,10 +2115,10 @@
         <v>29</v>
       </c>
       <c r="B25" t="s">
-        <v>81</v>
+        <v>166</v>
       </c>
       <c r="C25" t="s">
-        <v>110</v>
+        <v>280</v>
       </c>
       <c r="D25">
         <v>5</v>
@@ -1368,7 +2127,7 @@
         <v>5</v>
       </c>
       <c r="F25" t="s">
-        <v>134</v>
+        <v>305</v>
       </c>
     </row>
     <row r="26" spans="1:6">
@@ -1376,10 +2135,10 @@
         <v>30</v>
       </c>
       <c r="B26" t="s">
-        <v>82</v>
+        <v>167</v>
       </c>
       <c r="C26" t="s">
-        <v>111</v>
+        <v>281</v>
       </c>
       <c r="D26">
         <v>5</v>
@@ -1388,7 +2147,7 @@
         <v>5</v>
       </c>
       <c r="F26" t="s">
-        <v>135</v>
+        <v>306</v>
       </c>
     </row>
     <row r="27" spans="1:6">
@@ -1396,10 +2155,10 @@
         <v>31</v>
       </c>
       <c r="B27" t="s">
-        <v>83</v>
+        <v>168</v>
       </c>
       <c r="C27" t="s">
-        <v>111</v>
+        <v>281</v>
       </c>
       <c r="D27">
         <v>5</v>
@@ -1408,7 +2167,7 @@
         <v>4</v>
       </c>
       <c r="F27" t="s">
-        <v>136</v>
+        <v>307</v>
       </c>
     </row>
     <row r="28" spans="1:6">
@@ -1416,10 +2175,10 @@
         <v>32</v>
       </c>
       <c r="B28" t="s">
-        <v>84</v>
+        <v>169</v>
       </c>
       <c r="C28" t="s">
-        <v>111</v>
+        <v>281</v>
       </c>
       <c r="D28">
         <v>5</v>
@@ -1428,7 +2187,7 @@
         <v>5</v>
       </c>
       <c r="F28" t="s">
-        <v>137</v>
+        <v>308</v>
       </c>
     </row>
     <row r="29" spans="1:6">
@@ -1436,10 +2195,10 @@
         <v>33</v>
       </c>
       <c r="B29" t="s">
-        <v>85</v>
+        <v>170</v>
       </c>
       <c r="C29" t="s">
-        <v>110</v>
+        <v>280</v>
       </c>
       <c r="D29">
         <v>5</v>
@@ -1448,7 +2207,7 @@
         <v>5</v>
       </c>
       <c r="F29" t="s">
-        <v>138</v>
+        <v>309</v>
       </c>
     </row>
     <row r="30" spans="1:6">
@@ -1456,10 +2215,10 @@
         <v>34</v>
       </c>
       <c r="B30" t="s">
-        <v>86</v>
+        <v>171</v>
       </c>
       <c r="C30" t="s">
-        <v>111</v>
+        <v>281</v>
       </c>
       <c r="D30">
         <v>5</v>
@@ -1468,7 +2227,7 @@
         <v>5</v>
       </c>
       <c r="F30" t="s">
-        <v>139</v>
+        <v>310</v>
       </c>
     </row>
     <row r="31" spans="1:6">
@@ -1476,10 +2235,10 @@
         <v>35</v>
       </c>
       <c r="B31" t="s">
-        <v>87</v>
+        <v>172</v>
       </c>
       <c r="C31" t="s">
-        <v>111</v>
+        <v>281</v>
       </c>
       <c r="D31">
         <v>5</v>
@@ -1488,7 +2247,7 @@
         <v>4</v>
       </c>
       <c r="F31" t="s">
-        <v>140</v>
+        <v>311</v>
       </c>
     </row>
     <row r="32" spans="1:6">
@@ -1496,10 +2255,10 @@
         <v>36</v>
       </c>
       <c r="B32" t="s">
-        <v>88</v>
+        <v>173</v>
       </c>
       <c r="C32" t="s">
-        <v>111</v>
+        <v>281</v>
       </c>
       <c r="D32">
         <v>5</v>
@@ -1508,7 +2267,7 @@
         <v>5</v>
       </c>
       <c r="F32" t="s">
-        <v>141</v>
+        <v>312</v>
       </c>
     </row>
     <row r="33" spans="1:6">
@@ -1516,10 +2275,10 @@
         <v>37</v>
       </c>
       <c r="B33" t="s">
-        <v>89</v>
+        <v>174</v>
       </c>
       <c r="C33" t="s">
-        <v>110</v>
+        <v>280</v>
       </c>
       <c r="D33">
         <v>5</v>
@@ -1528,7 +2287,7 @@
         <v>5</v>
       </c>
       <c r="F33" t="s">
-        <v>142</v>
+        <v>313</v>
       </c>
     </row>
     <row r="34" spans="1:6">
@@ -1536,10 +2295,10 @@
         <v>38</v>
       </c>
       <c r="B34" t="s">
-        <v>90</v>
+        <v>175</v>
       </c>
       <c r="C34" t="s">
-        <v>111</v>
+        <v>281</v>
       </c>
       <c r="D34">
         <v>4</v>
@@ -1548,7 +2307,7 @@
         <v>4</v>
       </c>
       <c r="F34" t="s">
-        <v>143</v>
+        <v>314</v>
       </c>
     </row>
     <row r="35" spans="1:6">
@@ -1556,19 +2315,19 @@
         <v>39</v>
       </c>
       <c r="B35" t="s">
-        <v>91</v>
+        <v>176</v>
       </c>
       <c r="C35" t="s">
-        <v>111</v>
+        <v>280</v>
       </c>
       <c r="D35">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="E35">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="F35" t="s">
-        <v>144</v>
+        <v>315</v>
       </c>
     </row>
     <row r="36" spans="1:6">
@@ -1576,19 +2335,19 @@
         <v>40</v>
       </c>
       <c r="B36" t="s">
-        <v>92</v>
+        <v>177</v>
       </c>
       <c r="C36" t="s">
-        <v>111</v>
+        <v>280</v>
       </c>
       <c r="D36">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="E36">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="F36" t="s">
-        <v>145</v>
+        <v>316</v>
       </c>
     </row>
     <row r="37" spans="1:6">
@@ -1596,19 +2355,19 @@
         <v>41</v>
       </c>
       <c r="B37" t="s">
-        <v>93</v>
+        <v>178</v>
       </c>
       <c r="C37" t="s">
-        <v>110</v>
+        <v>280</v>
       </c>
       <c r="D37">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="E37">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="F37" t="s">
-        <v>146</v>
+        <v>317</v>
       </c>
     </row>
     <row r="38" spans="1:6">
@@ -1616,19 +2375,19 @@
         <v>42</v>
       </c>
       <c r="B38" t="s">
-        <v>94</v>
+        <v>179</v>
       </c>
       <c r="C38" t="s">
-        <v>111</v>
+        <v>280</v>
       </c>
       <c r="D38">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="E38">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="F38" t="s">
-        <v>147</v>
+        <v>318</v>
       </c>
     </row>
     <row r="39" spans="1:6">
@@ -1636,19 +2395,19 @@
         <v>43</v>
       </c>
       <c r="B39" t="s">
-        <v>95</v>
+        <v>180</v>
       </c>
       <c r="C39" t="s">
-        <v>111</v>
+        <v>281</v>
       </c>
       <c r="D39">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="E39">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="F39" t="s">
-        <v>148</v>
+        <v>319</v>
       </c>
     </row>
     <row r="40" spans="1:6">
@@ -1656,19 +2415,19 @@
         <v>44</v>
       </c>
       <c r="B40" t="s">
-        <v>96</v>
+        <v>181</v>
       </c>
       <c r="C40" t="s">
-        <v>110</v>
+        <v>281</v>
       </c>
       <c r="D40">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="E40">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="F40" t="s">
-        <v>149</v>
+        <v>320</v>
       </c>
     </row>
     <row r="41" spans="1:6">
@@ -1676,19 +2435,19 @@
         <v>45</v>
       </c>
       <c r="B41" t="s">
-        <v>97</v>
+        <v>182</v>
       </c>
       <c r="C41" t="s">
-        <v>110</v>
+        <v>281</v>
       </c>
       <c r="D41">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="E41">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="F41" t="s">
-        <v>150</v>
+        <v>321</v>
       </c>
     </row>
     <row r="42" spans="1:6">
@@ -1696,19 +2455,19 @@
         <v>46</v>
       </c>
       <c r="B42" t="s">
-        <v>98</v>
+        <v>183</v>
       </c>
       <c r="C42" t="s">
-        <v>110</v>
+        <v>281</v>
       </c>
       <c r="D42">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="E42">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="F42" t="s">
-        <v>151</v>
+        <v>322</v>
       </c>
     </row>
     <row r="43" spans="1:6">
@@ -1716,19 +2475,19 @@
         <v>47</v>
       </c>
       <c r="B43" t="s">
-        <v>99</v>
+        <v>184</v>
       </c>
       <c r="C43" t="s">
-        <v>111</v>
+        <v>282</v>
       </c>
       <c r="D43">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="E43">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="F43" t="s">
-        <v>152</v>
+        <v>323</v>
       </c>
     </row>
     <row r="44" spans="1:6">
@@ -1736,19 +2495,19 @@
         <v>48</v>
       </c>
       <c r="B44" t="s">
-        <v>100</v>
+        <v>185</v>
       </c>
       <c r="C44" t="s">
-        <v>110</v>
+        <v>280</v>
       </c>
       <c r="D44">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="E44">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="F44" t="s">
-        <v>153</v>
+        <v>324</v>
       </c>
     </row>
     <row r="45" spans="1:6">
@@ -1756,19 +2515,19 @@
         <v>49</v>
       </c>
       <c r="B45" t="s">
-        <v>101</v>
+        <v>186</v>
       </c>
       <c r="C45" t="s">
-        <v>111</v>
+        <v>281</v>
       </c>
       <c r="D45">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="E45">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="F45" t="s">
-        <v>154</v>
+        <v>325</v>
       </c>
     </row>
     <row r="46" spans="1:6">
@@ -1776,19 +2535,19 @@
         <v>50</v>
       </c>
       <c r="B46" t="s">
-        <v>102</v>
+        <v>187</v>
       </c>
       <c r="C46" t="s">
-        <v>110</v>
+        <v>280</v>
       </c>
       <c r="D46">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="E46">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="F46" t="s">
-        <v>155</v>
+        <v>326</v>
       </c>
     </row>
     <row r="47" spans="1:6">
@@ -1796,19 +2555,19 @@
         <v>51</v>
       </c>
       <c r="B47" t="s">
-        <v>103</v>
+        <v>188</v>
       </c>
       <c r="C47" t="s">
-        <v>111</v>
+        <v>280</v>
       </c>
       <c r="D47">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="E47">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="F47" t="s">
-        <v>156</v>
+        <v>327</v>
       </c>
     </row>
     <row r="48" spans="1:6">
@@ -1816,19 +2575,19 @@
         <v>52</v>
       </c>
       <c r="B48" t="s">
-        <v>104</v>
+        <v>189</v>
       </c>
       <c r="C48" t="s">
-        <v>111</v>
+        <v>281</v>
       </c>
       <c r="D48">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="E48">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="F48" t="s">
-        <v>157</v>
+        <v>328</v>
       </c>
     </row>
     <row r="49" spans="1:6">
@@ -1836,19 +2595,19 @@
         <v>53</v>
       </c>
       <c r="B49" t="s">
-        <v>105</v>
+        <v>190</v>
       </c>
       <c r="C49" t="s">
-        <v>110</v>
+        <v>281</v>
       </c>
       <c r="D49">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="E49">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="F49" t="s">
-        <v>158</v>
+        <v>329</v>
       </c>
     </row>
     <row r="50" spans="1:6">
@@ -1856,19 +2615,19 @@
         <v>54</v>
       </c>
       <c r="B50" t="s">
-        <v>106</v>
+        <v>191</v>
       </c>
       <c r="C50" t="s">
-        <v>111</v>
+        <v>281</v>
       </c>
       <c r="D50">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="E50">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="F50" t="s">
-        <v>159</v>
+        <v>330</v>
       </c>
     </row>
     <row r="51" spans="1:6">
@@ -1876,19 +2635,19 @@
         <v>55</v>
       </c>
       <c r="B51" t="s">
-        <v>107</v>
+        <v>192</v>
       </c>
       <c r="C51" t="s">
-        <v>111</v>
+        <v>281</v>
       </c>
       <c r="D51">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="E51">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="F51" t="s">
-        <v>160</v>
+        <v>331</v>
       </c>
     </row>
     <row r="52" spans="1:6">
@@ -1896,19 +2655,19 @@
         <v>56</v>
       </c>
       <c r="B52" t="s">
-        <v>108</v>
+        <v>193</v>
       </c>
       <c r="C52" t="s">
-        <v>111</v>
+        <v>281</v>
       </c>
       <c r="D52">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="E52">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="F52" t="s">
-        <v>161</v>
+        <v>332</v>
       </c>
     </row>
     <row r="53" spans="1:6">
@@ -1916,19 +2675,1719 @@
         <v>57</v>
       </c>
       <c r="B53" t="s">
+        <v>194</v>
+      </c>
+      <c r="C53" t="s">
+        <v>281</v>
+      </c>
+      <c r="D53">
+        <v>2</v>
+      </c>
+      <c r="E53">
+        <v>2</v>
+      </c>
+      <c r="F53" t="s">
+        <v>333</v>
+      </c>
+    </row>
+    <row r="54" spans="1:6">
+      <c r="A54" t="s">
+        <v>58</v>
+      </c>
+      <c r="B54" t="s">
+        <v>195</v>
+      </c>
+      <c r="C54" t="s">
+        <v>281</v>
+      </c>
+      <c r="D54">
+        <v>2</v>
+      </c>
+      <c r="E54">
+        <v>2</v>
+      </c>
+      <c r="F54" t="s">
+        <v>334</v>
+      </c>
+    </row>
+    <row r="55" spans="1:6">
+      <c r="A55" t="s">
+        <v>59</v>
+      </c>
+      <c r="B55" t="s">
+        <v>196</v>
+      </c>
+      <c r="C55" t="s">
+        <v>280</v>
+      </c>
+      <c r="D55">
+        <v>2</v>
+      </c>
+      <c r="E55">
+        <v>2</v>
+      </c>
+      <c r="F55" t="s">
+        <v>335</v>
+      </c>
+    </row>
+    <row r="56" spans="1:6">
+      <c r="A56" t="s">
+        <v>60</v>
+      </c>
+      <c r="B56" t="s">
+        <v>197</v>
+      </c>
+      <c r="C56" t="s">
+        <v>280</v>
+      </c>
+      <c r="D56">
+        <v>2</v>
+      </c>
+      <c r="E56">
+        <v>2</v>
+      </c>
+      <c r="F56" t="s">
+        <v>320</v>
+      </c>
+    </row>
+    <row r="57" spans="1:6">
+      <c r="A57" t="s">
+        <v>61</v>
+      </c>
+      <c r="B57" t="s">
+        <v>198</v>
+      </c>
+      <c r="C57" t="s">
+        <v>281</v>
+      </c>
+      <c r="D57">
+        <v>2</v>
+      </c>
+      <c r="E57">
+        <v>2</v>
+      </c>
+      <c r="F57" t="s">
+        <v>336</v>
+      </c>
+    </row>
+    <row r="58" spans="1:6">
+      <c r="A58" t="s">
+        <v>62</v>
+      </c>
+      <c r="B58" t="s">
+        <v>199</v>
+      </c>
+      <c r="C58" t="s">
+        <v>280</v>
+      </c>
+      <c r="D58">
+        <v>2</v>
+      </c>
+      <c r="E58">
+        <v>2</v>
+      </c>
+      <c r="F58" t="s">
+        <v>337</v>
+      </c>
+    </row>
+    <row r="59" spans="1:6">
+      <c r="A59" t="s">
+        <v>63</v>
+      </c>
+      <c r="B59" t="s">
+        <v>200</v>
+      </c>
+      <c r="C59" t="s">
+        <v>280</v>
+      </c>
+      <c r="D59">
+        <v>2</v>
+      </c>
+      <c r="E59">
+        <v>2</v>
+      </c>
+      <c r="F59" t="s">
+        <v>338</v>
+      </c>
+    </row>
+    <row r="60" spans="1:6">
+      <c r="A60" t="s">
+        <v>64</v>
+      </c>
+      <c r="B60" t="s">
+        <v>201</v>
+      </c>
+      <c r="C60" t="s">
+        <v>281</v>
+      </c>
+      <c r="D60">
+        <v>2</v>
+      </c>
+      <c r="E60">
+        <v>2</v>
+      </c>
+      <c r="F60" t="s">
+        <v>339</v>
+      </c>
+    </row>
+    <row r="61" spans="1:6">
+      <c r="A61" t="s">
+        <v>65</v>
+      </c>
+      <c r="B61" t="s">
+        <v>202</v>
+      </c>
+      <c r="C61" t="s">
+        <v>280</v>
+      </c>
+      <c r="D61">
+        <v>2</v>
+      </c>
+      <c r="E61">
+        <v>2</v>
+      </c>
+      <c r="F61" t="s">
+        <v>340</v>
+      </c>
+    </row>
+    <row r="62" spans="1:6">
+      <c r="A62" t="s">
+        <v>66</v>
+      </c>
+      <c r="B62" t="s">
+        <v>203</v>
+      </c>
+      <c r="C62" t="s">
+        <v>280</v>
+      </c>
+      <c r="D62">
+        <v>2</v>
+      </c>
+      <c r="E62">
+        <v>2</v>
+      </c>
+      <c r="F62" t="s">
+        <v>341</v>
+      </c>
+    </row>
+    <row r="63" spans="1:6">
+      <c r="A63" t="s">
+        <v>67</v>
+      </c>
+      <c r="B63" t="s">
+        <v>204</v>
+      </c>
+      <c r="C63" t="s">
+        <v>280</v>
+      </c>
+      <c r="D63">
+        <v>2</v>
+      </c>
+      <c r="E63">
+        <v>2</v>
+      </c>
+      <c r="F63" t="s">
+        <v>342</v>
+      </c>
+    </row>
+    <row r="64" spans="1:6">
+      <c r="A64" t="s">
+        <v>68</v>
+      </c>
+      <c r="B64" t="s">
+        <v>205</v>
+      </c>
+      <c r="C64" t="s">
+        <v>280</v>
+      </c>
+      <c r="D64">
+        <v>2</v>
+      </c>
+      <c r="E64">
+        <v>2</v>
+      </c>
+      <c r="F64" t="s">
+        <v>343</v>
+      </c>
+    </row>
+    <row r="65" spans="1:6">
+      <c r="A65" t="s">
+        <v>69</v>
+      </c>
+      <c r="B65" t="s">
+        <v>206</v>
+      </c>
+      <c r="C65" t="s">
+        <v>281</v>
+      </c>
+      <c r="D65">
+        <v>2</v>
+      </c>
+      <c r="E65">
+        <v>2</v>
+      </c>
+      <c r="F65" t="s">
+        <v>344</v>
+      </c>
+    </row>
+    <row r="66" spans="1:6">
+      <c r="A66" t="s">
+        <v>70</v>
+      </c>
+      <c r="B66" t="s">
+        <v>207</v>
+      </c>
+      <c r="C66" t="s">
+        <v>281</v>
+      </c>
+      <c r="D66">
+        <v>2</v>
+      </c>
+      <c r="E66">
+        <v>2</v>
+      </c>
+      <c r="F66" t="s">
+        <v>345</v>
+      </c>
+    </row>
+    <row r="67" spans="1:6">
+      <c r="A67" t="s">
+        <v>71</v>
+      </c>
+      <c r="B67" t="s">
+        <v>208</v>
+      </c>
+      <c r="C67" t="s">
+        <v>280</v>
+      </c>
+      <c r="D67">
+        <v>2</v>
+      </c>
+      <c r="E67">
+        <v>2</v>
+      </c>
+      <c r="F67" t="s">
+        <v>346</v>
+      </c>
+    </row>
+    <row r="68" spans="1:6">
+      <c r="A68" t="s">
+        <v>72</v>
+      </c>
+      <c r="B68" t="s">
+        <v>209</v>
+      </c>
+      <c r="C68" t="s">
+        <v>281</v>
+      </c>
+      <c r="D68">
+        <v>2</v>
+      </c>
+      <c r="E68">
+        <v>2</v>
+      </c>
+      <c r="F68" t="s">
+        <v>347</v>
+      </c>
+    </row>
+    <row r="69" spans="1:6">
+      <c r="A69" t="s">
+        <v>73</v>
+      </c>
+      <c r="B69" t="s">
+        <v>210</v>
+      </c>
+      <c r="C69" t="s">
+        <v>281</v>
+      </c>
+      <c r="D69">
+        <v>2</v>
+      </c>
+      <c r="E69">
+        <v>2</v>
+      </c>
+      <c r="F69" t="s">
+        <v>348</v>
+      </c>
+    </row>
+    <row r="70" spans="1:6">
+      <c r="A70" t="s">
+        <v>74</v>
+      </c>
+      <c r="B70" t="s">
+        <v>211</v>
+      </c>
+      <c r="C70" t="s">
+        <v>280</v>
+      </c>
+      <c r="D70">
+        <v>2</v>
+      </c>
+      <c r="E70">
+        <v>2</v>
+      </c>
+      <c r="F70" t="s">
+        <v>349</v>
+      </c>
+    </row>
+    <row r="71" spans="1:6">
+      <c r="A71" t="s">
+        <v>75</v>
+      </c>
+      <c r="B71" t="s">
+        <v>212</v>
+      </c>
+      <c r="C71" t="s">
+        <v>281</v>
+      </c>
+      <c r="D71">
+        <v>2</v>
+      </c>
+      <c r="E71">
+        <v>2</v>
+      </c>
+      <c r="F71" t="s">
+        <v>350</v>
+      </c>
+    </row>
+    <row r="72" spans="1:6">
+      <c r="A72" t="s">
+        <v>76</v>
+      </c>
+      <c r="B72" t="s">
+        <v>213</v>
+      </c>
+      <c r="C72" t="s">
+        <v>281</v>
+      </c>
+      <c r="D72">
+        <v>2</v>
+      </c>
+      <c r="E72">
+        <v>2</v>
+      </c>
+      <c r="F72" t="s">
+        <v>351</v>
+      </c>
+    </row>
+    <row r="73" spans="1:6">
+      <c r="A73" t="s">
+        <v>77</v>
+      </c>
+      <c r="B73" t="s">
+        <v>214</v>
+      </c>
+      <c r="C73" t="s">
+        <v>281</v>
+      </c>
+      <c r="D73">
+        <v>2</v>
+      </c>
+      <c r="E73">
+        <v>2</v>
+      </c>
+      <c r="F73" t="s">
+        <v>352</v>
+      </c>
+    </row>
+    <row r="74" spans="1:6">
+      <c r="A74" t="s">
+        <v>78</v>
+      </c>
+      <c r="B74" t="s">
+        <v>215</v>
+      </c>
+      <c r="C74" t="s">
+        <v>281</v>
+      </c>
+      <c r="D74">
+        <v>2</v>
+      </c>
+      <c r="E74">
+        <v>2</v>
+      </c>
+      <c r="F74" t="s">
+        <v>353</v>
+      </c>
+    </row>
+    <row r="75" spans="1:6">
+      <c r="A75" t="s">
+        <v>79</v>
+      </c>
+      <c r="B75" t="s">
+        <v>216</v>
+      </c>
+      <c r="C75" t="s">
+        <v>281</v>
+      </c>
+      <c r="D75">
+        <v>2</v>
+      </c>
+      <c r="E75">
+        <v>2</v>
+      </c>
+      <c r="F75" t="s">
+        <v>354</v>
+      </c>
+    </row>
+    <row r="76" spans="1:6">
+      <c r="A76" t="s">
+        <v>80</v>
+      </c>
+      <c r="B76" t="s">
+        <v>217</v>
+      </c>
+      <c r="C76" t="s">
+        <v>281</v>
+      </c>
+      <c r="D76">
+        <v>2</v>
+      </c>
+      <c r="E76">
+        <v>2</v>
+      </c>
+      <c r="F76" t="s">
+        <v>355</v>
+      </c>
+    </row>
+    <row r="77" spans="1:6">
+      <c r="A77" t="s">
+        <v>81</v>
+      </c>
+      <c r="B77" t="s">
+        <v>218</v>
+      </c>
+      <c r="C77" t="s">
+        <v>281</v>
+      </c>
+      <c r="D77">
+        <v>2</v>
+      </c>
+      <c r="E77">
+        <v>2</v>
+      </c>
+      <c r="F77" t="s">
+        <v>356</v>
+      </c>
+    </row>
+    <row r="78" spans="1:6">
+      <c r="A78" t="s">
+        <v>82</v>
+      </c>
+      <c r="B78" t="s">
+        <v>219</v>
+      </c>
+      <c r="C78" t="s">
+        <v>281</v>
+      </c>
+      <c r="D78">
+        <v>2</v>
+      </c>
+      <c r="E78">
+        <v>2</v>
+      </c>
+      <c r="F78" t="s">
+        <v>357</v>
+      </c>
+    </row>
+    <row r="79" spans="1:6">
+      <c r="A79" t="s">
+        <v>83</v>
+      </c>
+      <c r="B79" t="s">
+        <v>220</v>
+      </c>
+      <c r="C79" t="s">
+        <v>281</v>
+      </c>
+      <c r="D79">
+        <v>2</v>
+      </c>
+      <c r="E79">
+        <v>2</v>
+      </c>
+      <c r="F79" t="s">
+        <v>358</v>
+      </c>
+    </row>
+    <row r="80" spans="1:6">
+      <c r="A80" t="s">
+        <v>84</v>
+      </c>
+      <c r="B80" t="s">
+        <v>221</v>
+      </c>
+      <c r="C80" t="s">
+        <v>280</v>
+      </c>
+      <c r="D80">
+        <v>2</v>
+      </c>
+      <c r="E80">
+        <v>2</v>
+      </c>
+      <c r="F80" t="s">
+        <v>359</v>
+      </c>
+    </row>
+    <row r="81" spans="1:6">
+      <c r="A81" t="s">
+        <v>85</v>
+      </c>
+      <c r="B81" t="s">
+        <v>222</v>
+      </c>
+      <c r="C81" t="s">
+        <v>281</v>
+      </c>
+      <c r="D81">
+        <v>2</v>
+      </c>
+      <c r="E81">
+        <v>2</v>
+      </c>
+      <c r="F81" t="s">
+        <v>360</v>
+      </c>
+    </row>
+    <row r="82" spans="1:6">
+      <c r="A82" t="s">
+        <v>86</v>
+      </c>
+      <c r="B82" t="s">
+        <v>223</v>
+      </c>
+      <c r="C82" t="s">
+        <v>281</v>
+      </c>
+      <c r="D82">
+        <v>2</v>
+      </c>
+      <c r="E82">
+        <v>2</v>
+      </c>
+      <c r="F82" t="s">
+        <v>295</v>
+      </c>
+    </row>
+    <row r="83" spans="1:6">
+      <c r="A83" t="s">
+        <v>87</v>
+      </c>
+      <c r="B83" t="s">
+        <v>224</v>
+      </c>
+      <c r="C83" t="s">
+        <v>281</v>
+      </c>
+      <c r="D83">
+        <v>1</v>
+      </c>
+      <c r="E83">
+        <v>1</v>
+      </c>
+      <c r="F83" t="s">
+        <v>361</v>
+      </c>
+    </row>
+    <row r="84" spans="1:6">
+      <c r="A84" t="s">
+        <v>88</v>
+      </c>
+      <c r="B84" t="s">
+        <v>225</v>
+      </c>
+      <c r="C84" t="s">
+        <v>280</v>
+      </c>
+      <c r="D84">
+        <v>1</v>
+      </c>
+      <c r="E84">
+        <v>1</v>
+      </c>
+      <c r="F84" t="s">
+        <v>362</v>
+      </c>
+    </row>
+    <row r="85" spans="1:6">
+      <c r="A85" t="s">
+        <v>89</v>
+      </c>
+      <c r="B85" t="s">
+        <v>226</v>
+      </c>
+      <c r="C85" t="s">
+        <v>280</v>
+      </c>
+      <c r="D85">
+        <v>1</v>
+      </c>
+      <c r="E85">
+        <v>1</v>
+      </c>
+      <c r="F85" t="s">
+        <v>363</v>
+      </c>
+    </row>
+    <row r="86" spans="1:6">
+      <c r="A86" t="s">
+        <v>90</v>
+      </c>
+      <c r="B86" t="s">
+        <v>227</v>
+      </c>
+      <c r="C86" t="s">
+        <v>280</v>
+      </c>
+      <c r="D86">
+        <v>1</v>
+      </c>
+      <c r="E86">
+        <v>1</v>
+      </c>
+      <c r="F86" t="s">
+        <v>364</v>
+      </c>
+    </row>
+    <row r="87" spans="1:6">
+      <c r="A87" t="s">
+        <v>91</v>
+      </c>
+      <c r="B87" t="s">
+        <v>228</v>
+      </c>
+      <c r="C87" t="s">
+        <v>281</v>
+      </c>
+      <c r="D87">
+        <v>1</v>
+      </c>
+      <c r="E87">
+        <v>1</v>
+      </c>
+      <c r="F87" t="s">
+        <v>365</v>
+      </c>
+    </row>
+    <row r="88" spans="1:6">
+      <c r="A88" t="s">
+        <v>92</v>
+      </c>
+      <c r="B88" t="s">
+        <v>229</v>
+      </c>
+      <c r="C88" t="s">
+        <v>280</v>
+      </c>
+      <c r="D88">
+        <v>1</v>
+      </c>
+      <c r="E88">
+        <v>1</v>
+      </c>
+      <c r="F88" t="s">
+        <v>366</v>
+      </c>
+    </row>
+    <row r="89" spans="1:6">
+      <c r="A89" t="s">
+        <v>93</v>
+      </c>
+      <c r="B89" t="s">
+        <v>230</v>
+      </c>
+      <c r="C89" t="s">
+        <v>281</v>
+      </c>
+      <c r="D89">
+        <v>1</v>
+      </c>
+      <c r="E89">
+        <v>1</v>
+      </c>
+      <c r="F89" t="s">
+        <v>367</v>
+      </c>
+    </row>
+    <row r="90" spans="1:6">
+      <c r="A90" t="s">
+        <v>94</v>
+      </c>
+      <c r="B90" t="s">
+        <v>231</v>
+      </c>
+      <c r="C90" t="s">
+        <v>280</v>
+      </c>
+      <c r="D90">
+        <v>1</v>
+      </c>
+      <c r="E90">
+        <v>1</v>
+      </c>
+      <c r="F90" t="s">
+        <v>368</v>
+      </c>
+    </row>
+    <row r="91" spans="1:6">
+      <c r="A91" t="s">
+        <v>95</v>
+      </c>
+      <c r="B91" t="s">
+        <v>232</v>
+      </c>
+      <c r="C91" t="s">
+        <v>280</v>
+      </c>
+      <c r="D91">
+        <v>1</v>
+      </c>
+      <c r="E91">
+        <v>1</v>
+      </c>
+      <c r="F91" t="s">
+        <v>369</v>
+      </c>
+    </row>
+    <row r="92" spans="1:6">
+      <c r="A92" t="s">
+        <v>96</v>
+      </c>
+      <c r="B92" t="s">
+        <v>233</v>
+      </c>
+      <c r="C92" t="s">
+        <v>280</v>
+      </c>
+      <c r="D92">
+        <v>1</v>
+      </c>
+      <c r="E92">
+        <v>1</v>
+      </c>
+      <c r="F92" t="s">
+        <v>370</v>
+      </c>
+    </row>
+    <row r="93" spans="1:6">
+      <c r="A93" t="s">
+        <v>97</v>
+      </c>
+      <c r="B93" t="s">
+        <v>234</v>
+      </c>
+      <c r="C93" t="s">
+        <v>280</v>
+      </c>
+      <c r="D93">
+        <v>1</v>
+      </c>
+      <c r="E93">
+        <v>1</v>
+      </c>
+      <c r="F93" t="s">
+        <v>371</v>
+      </c>
+    </row>
+    <row r="94" spans="1:6">
+      <c r="A94" t="s">
+        <v>98</v>
+      </c>
+      <c r="B94" t="s">
+        <v>235</v>
+      </c>
+      <c r="C94" t="s">
+        <v>280</v>
+      </c>
+      <c r="D94">
+        <v>1</v>
+      </c>
+      <c r="E94">
+        <v>1</v>
+      </c>
+      <c r="F94" t="s">
+        <v>372</v>
+      </c>
+    </row>
+    <row r="95" spans="1:6">
+      <c r="A95" t="s">
+        <v>99</v>
+      </c>
+      <c r="B95" t="s">
+        <v>236</v>
+      </c>
+      <c r="C95" t="s">
+        <v>280</v>
+      </c>
+      <c r="D95">
+        <v>1</v>
+      </c>
+      <c r="E95">
+        <v>1</v>
+      </c>
+      <c r="F95" t="s">
+        <v>373</v>
+      </c>
+    </row>
+    <row r="96" spans="1:6">
+      <c r="A96" t="s">
+        <v>100</v>
+      </c>
+      <c r="B96" t="s">
+        <v>237</v>
+      </c>
+      <c r="C96" t="s">
+        <v>281</v>
+      </c>
+      <c r="D96">
+        <v>1</v>
+      </c>
+      <c r="E96">
+        <v>1</v>
+      </c>
+      <c r="F96" t="s">
+        <v>374</v>
+      </c>
+    </row>
+    <row r="97" spans="1:6">
+      <c r="A97" t="s">
+        <v>101</v>
+      </c>
+      <c r="B97" t="s">
+        <v>238</v>
+      </c>
+      <c r="C97" t="s">
+        <v>281</v>
+      </c>
+      <c r="D97">
+        <v>1</v>
+      </c>
+      <c r="E97">
+        <v>1</v>
+      </c>
+      <c r="F97" t="s">
+        <v>375</v>
+      </c>
+    </row>
+    <row r="98" spans="1:6">
+      <c r="A98" t="s">
+        <v>102</v>
+      </c>
+      <c r="B98" t="s">
+        <v>239</v>
+      </c>
+      <c r="C98" t="s">
+        <v>281</v>
+      </c>
+      <c r="D98">
+        <v>1</v>
+      </c>
+      <c r="E98">
+        <v>1</v>
+      </c>
+      <c r="F98" t="s">
+        <v>376</v>
+      </c>
+    </row>
+    <row r="99" spans="1:6">
+      <c r="A99" t="s">
+        <v>103</v>
+      </c>
+      <c r="B99" t="s">
+        <v>240</v>
+      </c>
+      <c r="C99" t="s">
+        <v>281</v>
+      </c>
+      <c r="D99">
+        <v>1</v>
+      </c>
+      <c r="E99">
+        <v>1</v>
+      </c>
+      <c r="F99" t="s">
+        <v>377</v>
+      </c>
+    </row>
+    <row r="100" spans="1:6">
+      <c r="A100" t="s">
+        <v>104</v>
+      </c>
+      <c r="B100" t="s">
+        <v>241</v>
+      </c>
+      <c r="C100" t="s">
+        <v>280</v>
+      </c>
+      <c r="D100">
+        <v>1</v>
+      </c>
+      <c r="E100">
+        <v>1</v>
+      </c>
+      <c r="F100" t="s">
+        <v>378</v>
+      </c>
+    </row>
+    <row r="101" spans="1:6">
+      <c r="A101" t="s">
+        <v>105</v>
+      </c>
+      <c r="B101" t="s">
+        <v>242</v>
+      </c>
+      <c r="C101" t="s">
+        <v>280</v>
+      </c>
+      <c r="D101">
+        <v>1</v>
+      </c>
+      <c r="E101">
+        <v>1</v>
+      </c>
+      <c r="F101" t="s">
+        <v>379</v>
+      </c>
+    </row>
+    <row r="102" spans="1:6">
+      <c r="A102" t="s">
+        <v>106</v>
+      </c>
+      <c r="B102" t="s">
+        <v>243</v>
+      </c>
+      <c r="C102" t="s">
+        <v>281</v>
+      </c>
+      <c r="D102">
+        <v>1</v>
+      </c>
+      <c r="E102">
+        <v>1</v>
+      </c>
+      <c r="F102" t="s">
+        <v>380</v>
+      </c>
+    </row>
+    <row r="103" spans="1:6">
+      <c r="A103" t="s">
+        <v>107</v>
+      </c>
+      <c r="B103" t="s">
+        <v>244</v>
+      </c>
+      <c r="C103" t="s">
+        <v>281</v>
+      </c>
+      <c r="D103">
+        <v>1</v>
+      </c>
+      <c r="E103">
+        <v>1</v>
+      </c>
+      <c r="F103" t="s">
+        <v>381</v>
+      </c>
+    </row>
+    <row r="104" spans="1:6">
+      <c r="A104" t="s">
+        <v>108</v>
+      </c>
+      <c r="B104" t="s">
+        <v>245</v>
+      </c>
+      <c r="C104" t="s">
+        <v>280</v>
+      </c>
+      <c r="D104">
+        <v>1</v>
+      </c>
+      <c r="E104">
+        <v>1</v>
+      </c>
+      <c r="F104" t="s">
+        <v>374</v>
+      </c>
+    </row>
+    <row r="105" spans="1:6">
+      <c r="A105" t="s">
         <v>109</v>
       </c>
-      <c r="C53" t="s">
+      <c r="B105" t="s">
+        <v>246</v>
+      </c>
+      <c r="C105" t="s">
+        <v>280</v>
+      </c>
+      <c r="D105">
+        <v>1</v>
+      </c>
+      <c r="E105">
+        <v>1</v>
+      </c>
+      <c r="F105" t="s">
+        <v>382</v>
+      </c>
+    </row>
+    <row r="106" spans="1:6">
+      <c r="A106" t="s">
         <v>110</v>
       </c>
-      <c r="D53">
-        <v>1</v>
-      </c>
-      <c r="E53">
-        <v>1</v>
-      </c>
-      <c r="F53" t="s">
-        <v>162</v>
+      <c r="B106" t="s">
+        <v>247</v>
+      </c>
+      <c r="C106" t="s">
+        <v>280</v>
+      </c>
+      <c r="D106">
+        <v>1</v>
+      </c>
+      <c r="E106">
+        <v>1</v>
+      </c>
+      <c r="F106" t="s">
+        <v>383</v>
+      </c>
+    </row>
+    <row r="107" spans="1:6">
+      <c r="A107" t="s">
+        <v>111</v>
+      </c>
+      <c r="B107" t="s">
+        <v>248</v>
+      </c>
+      <c r="C107" t="s">
+        <v>281</v>
+      </c>
+      <c r="D107">
+        <v>1</v>
+      </c>
+      <c r="E107">
+        <v>1</v>
+      </c>
+      <c r="F107" t="s">
+        <v>384</v>
+      </c>
+    </row>
+    <row r="108" spans="1:6">
+      <c r="A108" t="s">
+        <v>112</v>
+      </c>
+      <c r="B108" t="s">
+        <v>249</v>
+      </c>
+      <c r="C108" t="s">
+        <v>280</v>
+      </c>
+      <c r="D108">
+        <v>1</v>
+      </c>
+      <c r="E108">
+        <v>1</v>
+      </c>
+      <c r="F108" t="s">
+        <v>385</v>
+      </c>
+    </row>
+    <row r="109" spans="1:6">
+      <c r="A109" t="s">
+        <v>113</v>
+      </c>
+      <c r="B109" t="s">
+        <v>250</v>
+      </c>
+      <c r="C109" t="s">
+        <v>281</v>
+      </c>
+      <c r="D109">
+        <v>1</v>
+      </c>
+      <c r="E109">
+        <v>1</v>
+      </c>
+      <c r="F109" t="s">
+        <v>386</v>
+      </c>
+    </row>
+    <row r="110" spans="1:6">
+      <c r="A110" t="s">
+        <v>114</v>
+      </c>
+      <c r="B110" t="s">
+        <v>251</v>
+      </c>
+      <c r="C110" t="s">
+        <v>280</v>
+      </c>
+      <c r="D110">
+        <v>1</v>
+      </c>
+      <c r="E110">
+        <v>1</v>
+      </c>
+      <c r="F110" t="s">
+        <v>336</v>
+      </c>
+    </row>
+    <row r="111" spans="1:6">
+      <c r="A111" t="s">
+        <v>115</v>
+      </c>
+      <c r="B111" t="s">
+        <v>252</v>
+      </c>
+      <c r="C111" t="s">
+        <v>281</v>
+      </c>
+      <c r="D111">
+        <v>1</v>
+      </c>
+      <c r="E111">
+        <v>1</v>
+      </c>
+      <c r="F111" t="s">
+        <v>387</v>
+      </c>
+    </row>
+    <row r="112" spans="1:6">
+      <c r="A112" t="s">
+        <v>116</v>
+      </c>
+      <c r="B112" t="s">
+        <v>253</v>
+      </c>
+      <c r="C112" t="s">
+        <v>280</v>
+      </c>
+      <c r="D112">
+        <v>1</v>
+      </c>
+      <c r="E112">
+        <v>1</v>
+      </c>
+      <c r="F112" t="s">
+        <v>388</v>
+      </c>
+    </row>
+    <row r="113" spans="1:6">
+      <c r="A113" t="s">
+        <v>117</v>
+      </c>
+      <c r="B113" t="s">
+        <v>254</v>
+      </c>
+      <c r="C113" t="s">
+        <v>281</v>
+      </c>
+      <c r="D113">
+        <v>1</v>
+      </c>
+      <c r="E113">
+        <v>1</v>
+      </c>
+      <c r="F113" t="s">
+        <v>389</v>
+      </c>
+    </row>
+    <row r="114" spans="1:6">
+      <c r="A114" t="s">
+        <v>118</v>
+      </c>
+      <c r="B114" t="s">
+        <v>255</v>
+      </c>
+      <c r="C114" t="s">
+        <v>280</v>
+      </c>
+      <c r="D114">
+        <v>1</v>
+      </c>
+      <c r="E114">
+        <v>1</v>
+      </c>
+      <c r="F114" t="s">
+        <v>390</v>
+      </c>
+    </row>
+    <row r="115" spans="1:6">
+      <c r="A115" t="s">
+        <v>119</v>
+      </c>
+      <c r="B115" t="s">
+        <v>256</v>
+      </c>
+      <c r="C115" t="s">
+        <v>280</v>
+      </c>
+      <c r="D115">
+        <v>1</v>
+      </c>
+      <c r="E115">
+        <v>1</v>
+      </c>
+      <c r="F115" t="s">
+        <v>368</v>
+      </c>
+    </row>
+    <row r="116" spans="1:6">
+      <c r="A116" t="s">
+        <v>120</v>
+      </c>
+      <c r="B116" t="s">
+        <v>257</v>
+      </c>
+      <c r="C116" t="s">
+        <v>281</v>
+      </c>
+      <c r="D116">
+        <v>1</v>
+      </c>
+      <c r="E116">
+        <v>1</v>
+      </c>
+      <c r="F116" t="s">
+        <v>391</v>
+      </c>
+    </row>
+    <row r="117" spans="1:6">
+      <c r="A117" t="s">
+        <v>121</v>
+      </c>
+      <c r="B117" t="s">
+        <v>258</v>
+      </c>
+      <c r="C117" t="s">
+        <v>281</v>
+      </c>
+      <c r="D117">
+        <v>1</v>
+      </c>
+      <c r="E117">
+        <v>1</v>
+      </c>
+      <c r="F117" t="s">
+        <v>392</v>
+      </c>
+    </row>
+    <row r="118" spans="1:6">
+      <c r="A118" t="s">
+        <v>122</v>
+      </c>
+      <c r="B118" t="s">
+        <v>259</v>
+      </c>
+      <c r="C118" t="s">
+        <v>281</v>
+      </c>
+      <c r="D118">
+        <v>1</v>
+      </c>
+      <c r="E118">
+        <v>1</v>
+      </c>
+      <c r="F118" t="s">
+        <v>393</v>
+      </c>
+    </row>
+    <row r="119" spans="1:6">
+      <c r="A119" t="s">
+        <v>123</v>
+      </c>
+      <c r="B119" t="s">
+        <v>260</v>
+      </c>
+      <c r="C119" t="s">
+        <v>281</v>
+      </c>
+      <c r="D119">
+        <v>1</v>
+      </c>
+      <c r="E119">
+        <v>1</v>
+      </c>
+      <c r="F119" t="s">
+        <v>394</v>
+      </c>
+    </row>
+    <row r="120" spans="1:6">
+      <c r="A120" t="s">
+        <v>124</v>
+      </c>
+      <c r="B120" t="s">
+        <v>261</v>
+      </c>
+      <c r="C120" t="s">
+        <v>280</v>
+      </c>
+      <c r="D120">
+        <v>1</v>
+      </c>
+      <c r="E120">
+        <v>1</v>
+      </c>
+      <c r="F120" t="s">
+        <v>316</v>
+      </c>
+    </row>
+    <row r="121" spans="1:6">
+      <c r="A121" t="s">
+        <v>125</v>
+      </c>
+      <c r="B121" t="s">
+        <v>262</v>
+      </c>
+      <c r="C121" t="s">
+        <v>280</v>
+      </c>
+      <c r="D121">
+        <v>1</v>
+      </c>
+      <c r="E121">
+        <v>1</v>
+      </c>
+      <c r="F121" t="s">
+        <v>395</v>
+      </c>
+    </row>
+    <row r="122" spans="1:6">
+      <c r="A122" t="s">
+        <v>126</v>
+      </c>
+      <c r="B122" t="s">
+        <v>263</v>
+      </c>
+      <c r="C122" t="s">
+        <v>280</v>
+      </c>
+      <c r="D122">
+        <v>1</v>
+      </c>
+      <c r="E122">
+        <v>1</v>
+      </c>
+      <c r="F122" t="s">
+        <v>396</v>
+      </c>
+    </row>
+    <row r="123" spans="1:6">
+      <c r="A123" t="s">
+        <v>127</v>
+      </c>
+      <c r="B123" t="s">
+        <v>264</v>
+      </c>
+      <c r="C123" t="s">
+        <v>280</v>
+      </c>
+      <c r="D123">
+        <v>1</v>
+      </c>
+      <c r="E123">
+        <v>1</v>
+      </c>
+      <c r="F123" t="s">
+        <v>397</v>
+      </c>
+    </row>
+    <row r="124" spans="1:6">
+      <c r="A124" t="s">
+        <v>128</v>
+      </c>
+      <c r="B124" t="s">
+        <v>265</v>
+      </c>
+      <c r="C124" t="s">
+        <v>281</v>
+      </c>
+      <c r="D124">
+        <v>1</v>
+      </c>
+      <c r="E124">
+        <v>1</v>
+      </c>
+      <c r="F124" t="s">
+        <v>296</v>
+      </c>
+    </row>
+    <row r="125" spans="1:6">
+      <c r="A125" t="s">
+        <v>129</v>
+      </c>
+      <c r="B125" t="s">
+        <v>266</v>
+      </c>
+      <c r="C125" t="s">
+        <v>281</v>
+      </c>
+      <c r="D125">
+        <v>1</v>
+      </c>
+      <c r="E125">
+        <v>1</v>
+      </c>
+      <c r="F125" t="s">
+        <v>398</v>
+      </c>
+    </row>
+    <row r="126" spans="1:6">
+      <c r="A126" t="s">
+        <v>130</v>
+      </c>
+      <c r="B126" t="s">
+        <v>267</v>
+      </c>
+      <c r="C126" t="s">
+        <v>281</v>
+      </c>
+      <c r="D126">
+        <v>1</v>
+      </c>
+      <c r="E126">
+        <v>1</v>
+      </c>
+      <c r="F126" t="s">
+        <v>399</v>
+      </c>
+    </row>
+    <row r="127" spans="1:6">
+      <c r="A127" t="s">
+        <v>131</v>
+      </c>
+      <c r="B127" t="s">
+        <v>268</v>
+      </c>
+      <c r="C127" t="s">
+        <v>281</v>
+      </c>
+      <c r="D127">
+        <v>1</v>
+      </c>
+      <c r="E127">
+        <v>1</v>
+      </c>
+      <c r="F127" t="s">
+        <v>400</v>
+      </c>
+    </row>
+    <row r="128" spans="1:6">
+      <c r="A128" t="s">
+        <v>132</v>
+      </c>
+      <c r="B128" t="s">
+        <v>269</v>
+      </c>
+      <c r="C128" t="s">
+        <v>280</v>
+      </c>
+      <c r="D128">
+        <v>1</v>
+      </c>
+      <c r="E128">
+        <v>1</v>
+      </c>
+      <c r="F128" t="s">
+        <v>401</v>
+      </c>
+    </row>
+    <row r="129" spans="1:6">
+      <c r="A129" t="s">
+        <v>133</v>
+      </c>
+      <c r="B129" t="s">
+        <v>270</v>
+      </c>
+      <c r="C129" t="s">
+        <v>281</v>
+      </c>
+      <c r="D129">
+        <v>1</v>
+      </c>
+      <c r="E129">
+        <v>1</v>
+      </c>
+      <c r="F129" t="s">
+        <v>402</v>
+      </c>
+    </row>
+    <row r="130" spans="1:6">
+      <c r="A130" t="s">
+        <v>134</v>
+      </c>
+      <c r="B130" t="s">
+        <v>271</v>
+      </c>
+      <c r="C130" t="s">
+        <v>281</v>
+      </c>
+      <c r="D130">
+        <v>1</v>
+      </c>
+      <c r="E130">
+        <v>1</v>
+      </c>
+      <c r="F130" t="s">
+        <v>403</v>
+      </c>
+    </row>
+    <row r="131" spans="1:6">
+      <c r="A131" t="s">
+        <v>135</v>
+      </c>
+      <c r="B131" t="s">
+        <v>272</v>
+      </c>
+      <c r="C131" t="s">
+        <v>281</v>
+      </c>
+      <c r="D131">
+        <v>1</v>
+      </c>
+      <c r="E131">
+        <v>1</v>
+      </c>
+      <c r="F131" t="s">
+        <v>404</v>
+      </c>
+    </row>
+    <row r="132" spans="1:6">
+      <c r="A132" t="s">
+        <v>136</v>
+      </c>
+      <c r="B132" t="s">
+        <v>273</v>
+      </c>
+      <c r="C132" t="s">
+        <v>281</v>
+      </c>
+      <c r="D132">
+        <v>1</v>
+      </c>
+      <c r="E132">
+        <v>1</v>
+      </c>
+      <c r="F132" t="s">
+        <v>405</v>
+      </c>
+    </row>
+    <row r="133" spans="1:6">
+      <c r="A133" t="s">
+        <v>137</v>
+      </c>
+      <c r="B133" t="s">
+        <v>274</v>
+      </c>
+      <c r="C133" t="s">
+        <v>281</v>
+      </c>
+      <c r="D133">
+        <v>1</v>
+      </c>
+      <c r="E133">
+        <v>1</v>
+      </c>
+      <c r="F133" t="s">
+        <v>406</v>
+      </c>
+    </row>
+    <row r="134" spans="1:6">
+      <c r="A134" t="s">
+        <v>138</v>
+      </c>
+      <c r="B134" t="s">
+        <v>275</v>
+      </c>
+      <c r="C134" t="s">
+        <v>280</v>
+      </c>
+      <c r="D134">
+        <v>1</v>
+      </c>
+      <c r="E134">
+        <v>1</v>
+      </c>
+      <c r="F134" t="s">
+        <v>407</v>
+      </c>
+    </row>
+    <row r="135" spans="1:6">
+      <c r="A135" t="s">
+        <v>139</v>
+      </c>
+      <c r="B135" t="s">
+        <v>276</v>
+      </c>
+      <c r="C135" t="s">
+        <v>281</v>
+      </c>
+      <c r="D135">
+        <v>1</v>
+      </c>
+      <c r="E135">
+        <v>1</v>
+      </c>
+      <c r="F135" t="s">
+        <v>408</v>
+      </c>
+    </row>
+    <row r="136" spans="1:6">
+      <c r="A136" t="s">
+        <v>140</v>
+      </c>
+      <c r="B136" t="s">
+        <v>277</v>
+      </c>
+      <c r="C136" t="s">
+        <v>281</v>
+      </c>
+      <c r="D136">
+        <v>1</v>
+      </c>
+      <c r="E136">
+        <v>1</v>
+      </c>
+      <c r="F136" t="s">
+        <v>409</v>
+      </c>
+    </row>
+    <row r="137" spans="1:6">
+      <c r="A137" t="s">
+        <v>141</v>
+      </c>
+      <c r="B137" t="s">
+        <v>278</v>
+      </c>
+      <c r="C137" t="s">
+        <v>281</v>
+      </c>
+      <c r="D137">
+        <v>1</v>
+      </c>
+      <c r="E137">
+        <v>1</v>
+      </c>
+      <c r="F137" t="s">
+        <v>410</v>
+      </c>
+    </row>
+    <row r="138" spans="1:6">
+      <c r="A138" t="s">
+        <v>142</v>
+      </c>
+      <c r="B138" t="s">
+        <v>279</v>
+      </c>
+      <c r="C138" t="s">
+        <v>280</v>
+      </c>
+      <c r="D138">
+        <v>1</v>
+      </c>
+      <c r="E138">
+        <v>1</v>
+      </c>
+      <c r="F138" t="s">
+        <v>411</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
feat(ai): recover 26 high-purity emotion terms (mild, shame, privilege, security, etc) to clean_emotion_words_2000_reviews
</commit_message>
<xml_diff>
--- a/data/derived_outputs/clean_emotion_words_2000_reviews.xlsx
+++ b/data/derived_outputs/clean_emotion_words_2000_reviews.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="554" uniqueCount="412">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="658" uniqueCount="486">
   <si>
     <t>word</t>
   </si>
@@ -133,9 +133,18 @@
     <t>charming</t>
   </si>
   <si>
+    <t>privilege</t>
+  </si>
+  <si>
+    <t>rewarded</t>
+  </si>
+  <si>
     <t>sad</t>
   </si>
   <si>
+    <t>security</t>
+  </si>
+  <si>
     <t>splurge</t>
   </si>
   <si>
@@ -172,12 +181,30 @@
     <t>discomfort</t>
   </si>
   <si>
+    <t>friendlier</t>
+  </si>
+  <si>
+    <t>immaculate</t>
+  </si>
+  <si>
+    <t>improvement</t>
+  </si>
+  <si>
+    <t>lush</t>
+  </si>
+  <si>
+    <t>mild</t>
+  </si>
+  <si>
     <t>safest</t>
   </si>
   <si>
     <t>sensational</t>
   </si>
   <si>
+    <t>shame</t>
+  </si>
+  <si>
     <t>superbly</t>
   </si>
   <si>
@@ -229,24 +256,54 @@
     <t>glowing</t>
   </si>
   <si>
+    <t>grace</t>
+  </si>
+  <si>
     <t>happiness</t>
   </si>
   <si>
+    <t>honesty</t>
+  </si>
+  <si>
     <t>horrible</t>
   </si>
   <si>
     <t>hospitable</t>
   </si>
   <si>
+    <t>humility</t>
+  </si>
+  <si>
+    <t>improving</t>
+  </si>
+  <si>
+    <t>indulge</t>
+  </si>
+  <si>
     <t>joyful</t>
   </si>
   <si>
+    <t>kindly</t>
+  </si>
+  <si>
+    <t>luscious</t>
+  </si>
+  <si>
+    <t>mindful</t>
+  </si>
+  <si>
     <t>peacefully</t>
   </si>
   <si>
+    <t>praise</t>
+  </si>
+  <si>
     <t>precious</t>
   </si>
   <si>
+    <t>precision</t>
+  </si>
+  <si>
     <t>raving</t>
   </si>
   <si>
@@ -271,6 +328,24 @@
     <t>seasick</t>
   </si>
   <si>
+    <t>secret</t>
+  </si>
+  <si>
+    <t>securely</t>
+  </si>
+  <si>
+    <t>shining</t>
+  </si>
+  <si>
+    <t>stability</t>
+  </si>
+  <si>
+    <t>subtle</t>
+  </si>
+  <si>
+    <t>talented</t>
+  </si>
+  <si>
     <t>unstable</t>
   </si>
   <si>
@@ -367,6 +442,9 @@
     <t>relieved</t>
   </si>
   <si>
+    <t>reward</t>
+  </si>
+  <si>
     <t>rewarding</t>
   </si>
   <si>
@@ -544,9 +622,18 @@
     <t>迷人讨喜的</t>
   </si>
   <si>
+    <t>荣幸 / 难得体验</t>
+  </si>
+  <si>
+    <t>得到赏心悦目的回报</t>
+  </si>
+  <si>
     <t>悲伤的 / 遗憾痛心的</t>
   </si>
   <si>
+    <t>安全感 / 心理保障</t>
+  </si>
+  <si>
     <t>挥霍犒赏自己（特别体验）</t>
   </si>
   <si>
@@ -583,12 +670,30 @@
     <t>身体/心理不适感</t>
   </si>
   <si>
+    <t>更加亲切友好的</t>
+  </si>
+  <si>
+    <t>完美无瑕洁净的</t>
+  </si>
+  <si>
+    <t>体验改善 / 提升</t>
+  </si>
+  <si>
+    <t>郁郁葱葱宜人的</t>
+  </si>
+  <si>
+    <t>轻微适度的（颠簸/舒适）</t>
+  </si>
+  <si>
     <t>最安全平稳的</t>
   </si>
   <si>
     <t>绝佳轰动震撼的</t>
   </si>
   <si>
+    <t>遗憾 / 可惜扫兴</t>
+  </si>
+  <si>
     <t>出类拔萃完美地</t>
   </si>
   <si>
@@ -640,24 +745,54 @@
     <t>极度赞赏口碑极佳的</t>
   </si>
   <si>
+    <t>优雅 / 良好风度</t>
+  </si>
+  <si>
     <t>幸福快乐感</t>
   </si>
   <si>
+    <t>真诚 / 诚信解说</t>
+  </si>
+  <si>
     <t>极度糟糕可怕的</t>
   </si>
   <si>
     <t>殷勤好客的</t>
   </si>
   <si>
+    <t>谦逊贴心</t>
+  </si>
+  <si>
+    <t>不断改善令人满意的</t>
+  </si>
+  <si>
+    <t>尽情享受 / 犒劳自己</t>
+  </si>
+  <si>
     <t>充满喜悦欢快的</t>
   </si>
   <si>
+    <t>体贴友善地</t>
+  </si>
+  <si>
+    <t>秀美令人心旷神怡的</t>
+  </si>
+  <si>
+    <t>细心周到的</t>
+  </si>
+  <si>
     <t>宁静和平地</t>
   </si>
   <si>
+    <t>称赞 / 高度赞扬</t>
+  </si>
+  <si>
     <t>弥足珍贵的 memory</t>
   </si>
   <si>
+    <t>精准靠谱的</t>
+  </si>
+  <si>
     <t>赞不绝口极力推荐的</t>
   </si>
   <si>
@@ -682,6 +817,24 @@
     <t>晕船 / 晕眩恶心的</t>
   </si>
   <si>
+    <t>秘境 / 私密独享感</t>
+  </si>
+  <si>
+    <t>安全平稳地</t>
+  </si>
+  <si>
+    <t>璀璨夺目的</t>
+  </si>
+  <si>
+    <t>平稳安心感</t>
+  </si>
+  <si>
+    <t>微妙精细的</t>
+  </si>
+  <si>
+    <t>才华横溢精湛的</t>
+  </si>
+  <si>
     <t>不稳定摇晃令人担心的</t>
   </si>
   <si>
@@ -776,6 +929,9 @@
   </si>
   <si>
     <t>宽慰的 / 松了一口气</t>
+  </si>
+  <si>
+    <t>赏心悦目的奖赏体验</t>
   </si>
   <si>
     <t>非常有成就感/物超所值的</t>
@@ -967,9 +1123,18 @@
     <t>review_2437be8aa60056f18e560577 :: Our flight over Kaua'i with our charming, skillful pilot was the best experience of our island vacation. She gave a most interesting and helpful account of what we could see below,...</t>
   </si>
   <si>
+    <t>review_48861d1a4276178379e27007 :: We had the privilege of doing the Grand Canyon West Rim Adventure Tours.  We will never forget this AMAZING experience!!!  From the welcoming staff to  the incredible views, this i...</t>
+  </si>
+  <si>
+    <t>review_8cbe628c5c47e65c0e97f867 :: We stayed in Talkeetna for two nights, planning on a flight seeing on our first day there. We were scheduled for the first morning flight. The morning was very overcast and the fli...</t>
+  </si>
+  <si>
     <t>review_641866daade55fe429557808 :: Unfortunately Denali was socked in with weather. Also the glaciers had degraded to the point of no landings. We were very sad. K2 offered us an option to Knik. It was UNBELIEVABLE!...</t>
   </si>
   <si>
+    <t>review_c4e918eedbed49349a333a93 :: This is expensive, but worth every penny. If you visit the Grand Canyon and can afford it, we recommend you do it. For us it was one, if not the, highlight on our extended US trip ...</t>
+  </si>
+  <si>
     <t>review_eda1a4bce0aac45015172f03 :: We heard so much about how beautiful Kauai was, but after driving around the entire island, we weren't that impressed. Mind you, we had just seen all the major sights of Maui, so w...</t>
   </si>
   <si>
@@ -1004,6 +1169,22 @@
   </si>
   <si>
     <t>review_b3611bb117be728e25d5ddec :: We had booked the 11 am tour online even before we reached Kauai. We called ahead and the person who answered told us we could come by 10:45 am or so. We reached round about then o...</t>
+  </si>
+  <si>
+    <t>review_0b5b314e6afb25f8dff5666d :: We had only one day in Kauai while visiting the islands on a cruise.  I had read these reviews and so booked the flight for our group of 4.  I am so glad I did!  They could not be ...</t>
+  </si>
+  <si>
+    <t>review_946bb8d70631840517ffae88 :: It was amazing!! Highly recommend! The views were immaculate &amp; the pilot was so knowledgeable! Would go again!...</t>
+  </si>
+  <si>
+    <t>review_6b4f55a23869141d6e9fcb5b :: We are long time Alaskans and have viewed Denali from the air as well as the road system on several occasions.  Our K2 Aviation flightseeing trip topped them all. 
+The phone reser...</t>
+  </si>
+  <si>
+    <t>review_1893bdcfa0517b11567fd56d :: I booked the Cessna tour for my wife and I on our babymoon in April. I recommend the private Cessna tour if you only have 2 people.  For only slightly more $$, you get a personal e...</t>
+  </si>
+  <si>
+    <t>review_5fe403d9e2633bea2fb1bc97 :: How often do you get a chance to fly in an open cockpit biplane? Our pilot, Harry, was friendly and very experienced. The plane is quite new, and in great shape, the intercom syste...</t>
   </si>
   <si>
     <t>review_fe566c581798d89f19f642e5 :: My husband and I were rained or otherwise "bad-weathered" out of every adventure we planned on Kauai.  Couldn't hike Kalalau due to the river crossing being flooded. 
@@ -1013,6 +1194,9 @@
     <t>review_69b44dac34b50350cfb373aa :: Steve, our pilot was sensational.   We were greeted by name, promptness, and courtesy.  They took our bags and explained the flight procedure.   Steve pointed out areas of interest...</t>
   </si>
   <si>
+    <t>review_d5b09587168814a8a6cba02a :: Planned a ride for my son's 12th birthday in April. I am a bit late getting around to writing my review and have since forgotten our pilots name, which is a shame because he was WO...</t>
+  </si>
+  <si>
     <t>review_bcedc98e43ad7edec05befa8 :: There isn't much to say here, except the experience was fantastic. Seeing the landscape from the air was breathtaking, and landing and taking off from the glacier was a hoot. Our p...</t>
   </si>
   <si>
@@ -1063,7 +1247,13 @@
     <t>review_b5268b40d3aafe7496fcb498 :: If you are visiting the Grand Canyon, the only way to take in it's full majesty is to do it by Helicopter. Maverick Helicopter were fantastic. You must take a flight with them, wel...</t>
   </si>
   <si>
+    <t>review_be59fcb99b0add1dc982d912 :: We booked a half hour flight with another couple that told us the gentleman was flying on the recommendation of his psychologist.  He got pretty nervous after takeoff, Pilot Fred t...</t>
+  </si>
+  <si>
     <t>review_c8c04aed9cd305332764808f :: I encouraged my husband to take the biplane flight/tour. I had no intention of going. My husband and the pilot Mark encouraged me to go along. The front seat holds two. I decided t...</t>
+  </si>
+  <si>
+    <t>review_9f9111190c4a6d851371d2f7 :: We want to express our appreciation to Chip Sonn, our K2 pilot for our fantastic late afternoon/evening flight excursion while recently visiting Talkeetna, Alaska.  As part of our ...</t>
   </si>
   <si>
     <t>review_ebb70b11c29e696fbd1d4b9d :: Both K2 and Talkeetna Air Taxi (TAT) get my highest recommendation. Follow along with the bouncing ball, kids, as our tale unfolds:
@@ -1073,13 +1263,29 @@
     <t>review_1a8c661361e1a55ed4a0ed52 :: The service provided by the Wings Over Kauai tours was very well done.  Ellen was very hospitable while waiting for our scheduled flight.  Capt. Josh has a very clear passion for a...</t>
   </si>
   <si>
+    <t>review_d1dfcb69be6315d42fc6e8f8 :: DISCLAIMER: I’m a tour professional living and working here in Alaska and not compensated in any way for this review. I do it because these operators are my FELLOW ALASKANS. 
+Ther...</t>
+  </si>
+  <si>
     <t>review_27ee31e44dec37dd44a492ba :: Eric, the pilot, is a amazing guy doing a great job! He said we are sharing his dream, actually he was making my dream come true by letting my little girl driving a little bit! Sou...</t>
   </si>
   <si>
+    <t>review_91b07376e836c82b2b2ff5cc :: We had the open cockpit biplane flight beginning of February after booking online from the UK.  Jill kindly offered to collect/shuttle us from the ABC Store at Anchor Cove Shopping...</t>
+  </si>
+  <si>
+    <t>review_af6c769cd16b044c81ee438f :: My husband &amp; I were visiting Kauai from New York.  We were extremely fortunate to fly in a comfortable but small plane to view the luscious island of Kauai.  When we arrived for ou...</t>
+  </si>
+  <si>
     <t>review_09687f3c5332ab59381de30a :: It was perfect and we would go again with this same company. A small fixed wing plane seating a pilot and 2 riders. Things to keep in mind if you pick this small plane-If you are v...</t>
   </si>
   <si>
+    <t>review_c47a8f0a85e514d042ad1889 :: Though TAT doesn't *need* more praise, my experience with them was simply so phenomenal that I have to give them yet another Excellent review. This is a top-notch company with some...</t>
+  </si>
+  <si>
     <t>review_02d9b6799d194eb3a407125d :: Just got back from Kauai - went on a 1 hour airplane tour over Kauai - very nice experience over the island of Kauai - pilot tells you the sites that you are going over; at the end...</t>
+  </si>
+  <si>
+    <t>review_e0d4177111a512725ecee24d :: I have to share my experience this morning. I took my Very First Flight Ever a couple of hours ago and did it through RedTail Aviation in a 6 person plane. I was so nervous before ...</t>
   </si>
   <si>
     <t>review_1758d760d6f52438c4d85cce :: Bruce the pilot was great with our 2 nervous flyers.  He gave a great talk while we were flying and patiently answered any/all questions.  All of us were raving about the tour long...</t>
@@ -1111,6 +1317,23 @@
     <t>review_b4defed8dabe04d3de367e4c :: Awesome service. Our pilot, Bruce, made a point to keep track of all our names and interacted with each of us by name throughout the flight. A very nice touch. We actually flew thr...</t>
   </si>
   <si>
+    <t>review_3fabab1c18329fdb94e0581c :: The day before my Air Ventures Hi flight, I had an amazing conversation with a helicopter tour across the street. I was the 1st for the next tour which required 6 passengers. No on...</t>
+  </si>
+  <si>
+    <t>review_168aab1a1f0b80f2400963aa :: This was a spectacular flight! We had a sunny day and Denali was out in all it's glory.
+Our pilot Stan started off with all the safety features and then after we were securely in o...</t>
+  </si>
+  <si>
+    <t>review_4b4ba93d00a26f2d30de6497 :: From the very beginning the flight was unbelievable. The sun was shining and the views were beyond spectacular!  A chance of a life time and well worth the price.
+Paul made us feel...</t>
+  </si>
+  <si>
+    <t>review_cce5c0d3468ee1bee4178621 :: What a wonderful way to start a week in Kauai with a flight over the island in a stable, roomyAir Ventures Hawaii Airvan plane with a super pilot who provided a wonderful, informat...</t>
+  </si>
+  <si>
+    <t>review_0cf8290af6a3504f8b5f33d9 :: We had a wonderful time on our flight with Wings Over Kauai! I had looked at helicopter tours as well, but we chose a fixed-wing flight because it's far safer (check out Kauai Unde...</t>
+  </si>
+  <si>
     <t>review_905ea7ae4640bfc3d91b8080 :: This trip around Mt Denali was breath taking and our pilot was awsome on knowledge and making sure we all had great views for pictures. The sky around the mountain was clear but th...</t>
   </si>
   <si>
@@ -1197,6 +1420,9 @@
   </si>
   <si>
     <t>review_0fd62b59dfddedcc4ce37b1b :: We arrived in good time and after  paying and being weighed for the correct distribution within the helicopter, we sat and waited for the 3 other passengers. The area you sit and w...</t>
+  </si>
+  <si>
+    <t>review_62065bd2615e8936538e71b3 :: You cannot go wrong snagging a flight to the Alaska Mountain Range and Denali up close. While it seems like a scary thing to do, I felt safe 100% of the time. The reward was the cl...</t>
   </si>
   <si>
     <t>review_20a5d0a4abc1952fcfbb43d0 :: Had a flight seeing tour with K2. We couldn't do the glacier landing due to weather conditions but nevermind, we still very much enjoyed that our. We saw dramatic landscape, glacie...</t>
@@ -1627,7 +1853,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:F138"/>
+  <dimension ref="A1:F164"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:6">
@@ -1655,10 +1881,10 @@
         <v>6</v>
       </c>
       <c r="B2" t="s">
-        <v>143</v>
+        <v>169</v>
       </c>
       <c r="C2" t="s">
-        <v>280</v>
+        <v>332</v>
       </c>
       <c r="D2">
         <v>12</v>
@@ -1667,7 +1893,7 @@
         <v>12</v>
       </c>
       <c r="F2" t="s">
-        <v>283</v>
+        <v>335</v>
       </c>
     </row>
     <row r="3" spans="1:6">
@@ -1675,10 +1901,10 @@
         <v>7</v>
       </c>
       <c r="B3" t="s">
-        <v>144</v>
+        <v>170</v>
       </c>
       <c r="C3" t="s">
-        <v>281</v>
+        <v>333</v>
       </c>
       <c r="D3">
         <v>10</v>
@@ -1687,7 +1913,7 @@
         <v>10</v>
       </c>
       <c r="F3" t="s">
-        <v>284</v>
+        <v>336</v>
       </c>
     </row>
     <row r="4" spans="1:6">
@@ -1695,10 +1921,10 @@
         <v>8</v>
       </c>
       <c r="B4" t="s">
-        <v>145</v>
+        <v>171</v>
       </c>
       <c r="C4" t="s">
-        <v>281</v>
+        <v>333</v>
       </c>
       <c r="D4">
         <v>10</v>
@@ -1707,7 +1933,7 @@
         <v>9</v>
       </c>
       <c r="F4" t="s">
-        <v>285</v>
+        <v>337</v>
       </c>
     </row>
     <row r="5" spans="1:6">
@@ -1715,10 +1941,10 @@
         <v>9</v>
       </c>
       <c r="B5" t="s">
-        <v>146</v>
+        <v>172</v>
       </c>
       <c r="C5" t="s">
-        <v>281</v>
+        <v>333</v>
       </c>
       <c r="D5">
         <v>9</v>
@@ -1727,7 +1953,7 @@
         <v>9</v>
       </c>
       <c r="F5" t="s">
-        <v>286</v>
+        <v>338</v>
       </c>
     </row>
     <row r="6" spans="1:6">
@@ -1735,10 +1961,10 @@
         <v>10</v>
       </c>
       <c r="B6" t="s">
-        <v>147</v>
+        <v>173</v>
       </c>
       <c r="C6" t="s">
-        <v>281</v>
+        <v>333</v>
       </c>
       <c r="D6">
         <v>9</v>
@@ -1747,7 +1973,7 @@
         <v>9</v>
       </c>
       <c r="F6" t="s">
-        <v>287</v>
+        <v>339</v>
       </c>
     </row>
     <row r="7" spans="1:6">
@@ -1755,10 +1981,10 @@
         <v>11</v>
       </c>
       <c r="B7" t="s">
-        <v>148</v>
+        <v>174</v>
       </c>
       <c r="C7" t="s">
-        <v>281</v>
+        <v>333</v>
       </c>
       <c r="D7">
         <v>9</v>
@@ -1767,7 +1993,7 @@
         <v>9</v>
       </c>
       <c r="F7" t="s">
-        <v>288</v>
+        <v>340</v>
       </c>
     </row>
     <row r="8" spans="1:6">
@@ -1775,10 +2001,10 @@
         <v>12</v>
       </c>
       <c r="B8" t="s">
-        <v>149</v>
+        <v>175</v>
       </c>
       <c r="C8" t="s">
-        <v>281</v>
+        <v>333</v>
       </c>
       <c r="D8">
         <v>8</v>
@@ -1787,7 +2013,7 @@
         <v>8</v>
       </c>
       <c r="F8" t="s">
-        <v>289</v>
+        <v>341</v>
       </c>
     </row>
     <row r="9" spans="1:6">
@@ -1795,10 +2021,10 @@
         <v>13</v>
       </c>
       <c r="B9" t="s">
-        <v>150</v>
+        <v>176</v>
       </c>
       <c r="C9" t="s">
-        <v>280</v>
+        <v>332</v>
       </c>
       <c r="D9">
         <v>8</v>
@@ -1807,7 +2033,7 @@
         <v>8</v>
       </c>
       <c r="F9" t="s">
-        <v>290</v>
+        <v>342</v>
       </c>
     </row>
     <row r="10" spans="1:6">
@@ -1815,10 +2041,10 @@
         <v>14</v>
       </c>
       <c r="B10" t="s">
-        <v>151</v>
+        <v>177</v>
       </c>
       <c r="C10" t="s">
-        <v>280</v>
+        <v>332</v>
       </c>
       <c r="D10">
         <v>7</v>
@@ -1827,7 +2053,7 @@
         <v>7</v>
       </c>
       <c r="F10" t="s">
-        <v>291</v>
+        <v>343</v>
       </c>
     </row>
     <row r="11" spans="1:6">
@@ -1835,10 +2061,10 @@
         <v>15</v>
       </c>
       <c r="B11" t="s">
-        <v>152</v>
+        <v>178</v>
       </c>
       <c r="C11" t="s">
-        <v>281</v>
+        <v>333</v>
       </c>
       <c r="D11">
         <v>7</v>
@@ -1847,7 +2073,7 @@
         <v>7</v>
       </c>
       <c r="F11" t="s">
-        <v>292</v>
+        <v>344</v>
       </c>
     </row>
     <row r="12" spans="1:6">
@@ -1855,10 +2081,10 @@
         <v>16</v>
       </c>
       <c r="B12" t="s">
-        <v>153</v>
+        <v>179</v>
       </c>
       <c r="C12" t="s">
-        <v>281</v>
+        <v>333</v>
       </c>
       <c r="D12">
         <v>7</v>
@@ -1867,7 +2093,7 @@
         <v>7</v>
       </c>
       <c r="F12" t="s">
-        <v>293</v>
+        <v>345</v>
       </c>
     </row>
     <row r="13" spans="1:6">
@@ -1875,10 +2101,10 @@
         <v>17</v>
       </c>
       <c r="B13" t="s">
-        <v>154</v>
+        <v>180</v>
       </c>
       <c r="C13" t="s">
-        <v>281</v>
+        <v>333</v>
       </c>
       <c r="D13">
         <v>7</v>
@@ -1887,7 +2113,7 @@
         <v>7</v>
       </c>
       <c r="F13" t="s">
-        <v>294</v>
+        <v>346</v>
       </c>
     </row>
     <row r="14" spans="1:6">
@@ -1895,10 +2121,10 @@
         <v>18</v>
       </c>
       <c r="B14" t="s">
-        <v>155</v>
+        <v>181</v>
       </c>
       <c r="C14" t="s">
-        <v>281</v>
+        <v>333</v>
       </c>
       <c r="D14">
         <v>7</v>
@@ -1907,7 +2133,7 @@
         <v>6</v>
       </c>
       <c r="F14" t="s">
-        <v>295</v>
+        <v>347</v>
       </c>
     </row>
     <row r="15" spans="1:6">
@@ -1915,10 +2141,10 @@
         <v>19</v>
       </c>
       <c r="B15" t="s">
-        <v>156</v>
+        <v>182</v>
       </c>
       <c r="C15" t="s">
-        <v>281</v>
+        <v>333</v>
       </c>
       <c r="D15">
         <v>7</v>
@@ -1927,7 +2153,7 @@
         <v>7</v>
       </c>
       <c r="F15" t="s">
-        <v>286</v>
+        <v>338</v>
       </c>
     </row>
     <row r="16" spans="1:6">
@@ -1935,10 +2161,10 @@
         <v>20</v>
       </c>
       <c r="B16" t="s">
-        <v>157</v>
+        <v>183</v>
       </c>
       <c r="C16" t="s">
-        <v>281</v>
+        <v>333</v>
       </c>
       <c r="D16">
         <v>6</v>
@@ -1947,7 +2173,7 @@
         <v>6</v>
       </c>
       <c r="F16" t="s">
-        <v>296</v>
+        <v>348</v>
       </c>
     </row>
     <row r="17" spans="1:6">
@@ -1955,10 +2181,10 @@
         <v>21</v>
       </c>
       <c r="B17" t="s">
-        <v>158</v>
+        <v>184</v>
       </c>
       <c r="C17" t="s">
-        <v>280</v>
+        <v>332</v>
       </c>
       <c r="D17">
         <v>6</v>
@@ -1967,7 +2193,7 @@
         <v>6</v>
       </c>
       <c r="F17" t="s">
-        <v>297</v>
+        <v>349</v>
       </c>
     </row>
     <row r="18" spans="1:6">
@@ -1975,10 +2201,10 @@
         <v>22</v>
       </c>
       <c r="B18" t="s">
-        <v>159</v>
+        <v>185</v>
       </c>
       <c r="C18" t="s">
-        <v>281</v>
+        <v>333</v>
       </c>
       <c r="D18">
         <v>6</v>
@@ -1987,7 +2213,7 @@
         <v>6</v>
       </c>
       <c r="F18" t="s">
-        <v>298</v>
+        <v>350</v>
       </c>
     </row>
     <row r="19" spans="1:6">
@@ -1995,10 +2221,10 @@
         <v>23</v>
       </c>
       <c r="B19" t="s">
-        <v>160</v>
+        <v>186</v>
       </c>
       <c r="C19" t="s">
-        <v>281</v>
+        <v>333</v>
       </c>
       <c r="D19">
         <v>6</v>
@@ -2007,7 +2233,7 @@
         <v>5</v>
       </c>
       <c r="F19" t="s">
-        <v>299</v>
+        <v>351</v>
       </c>
     </row>
     <row r="20" spans="1:6">
@@ -2015,10 +2241,10 @@
         <v>24</v>
       </c>
       <c r="B20" t="s">
-        <v>161</v>
+        <v>187</v>
       </c>
       <c r="C20" t="s">
-        <v>280</v>
+        <v>332</v>
       </c>
       <c r="D20">
         <v>6</v>
@@ -2027,7 +2253,7 @@
         <v>6</v>
       </c>
       <c r="F20" t="s">
-        <v>300</v>
+        <v>352</v>
       </c>
     </row>
     <row r="21" spans="1:6">
@@ -2035,10 +2261,10 @@
         <v>25</v>
       </c>
       <c r="B21" t="s">
-        <v>162</v>
+        <v>188</v>
       </c>
       <c r="C21" t="s">
-        <v>280</v>
+        <v>332</v>
       </c>
       <c r="D21">
         <v>6</v>
@@ -2047,7 +2273,7 @@
         <v>5</v>
       </c>
       <c r="F21" t="s">
-        <v>301</v>
+        <v>353</v>
       </c>
     </row>
     <row r="22" spans="1:6">
@@ -2055,10 +2281,10 @@
         <v>26</v>
       </c>
       <c r="B22" t="s">
-        <v>163</v>
+        <v>189</v>
       </c>
       <c r="C22" t="s">
-        <v>280</v>
+        <v>332</v>
       </c>
       <c r="D22">
         <v>6</v>
@@ -2067,7 +2293,7 @@
         <v>6</v>
       </c>
       <c r="F22" t="s">
-        <v>302</v>
+        <v>354</v>
       </c>
     </row>
     <row r="23" spans="1:6">
@@ -2075,10 +2301,10 @@
         <v>27</v>
       </c>
       <c r="B23" t="s">
-        <v>164</v>
+        <v>190</v>
       </c>
       <c r="C23" t="s">
-        <v>280</v>
+        <v>332</v>
       </c>
       <c r="D23">
         <v>6</v>
@@ -2087,7 +2313,7 @@
         <v>6</v>
       </c>
       <c r="F23" t="s">
-        <v>303</v>
+        <v>355</v>
       </c>
     </row>
     <row r="24" spans="1:6">
@@ -2095,10 +2321,10 @@
         <v>28</v>
       </c>
       <c r="B24" t="s">
-        <v>165</v>
+        <v>191</v>
       </c>
       <c r="C24" t="s">
-        <v>281</v>
+        <v>333</v>
       </c>
       <c r="D24">
         <v>6</v>
@@ -2107,7 +2333,7 @@
         <v>6</v>
       </c>
       <c r="F24" t="s">
-        <v>304</v>
+        <v>356</v>
       </c>
     </row>
     <row r="25" spans="1:6">
@@ -2115,10 +2341,10 @@
         <v>29</v>
       </c>
       <c r="B25" t="s">
-        <v>166</v>
+        <v>192</v>
       </c>
       <c r="C25" t="s">
-        <v>280</v>
+        <v>332</v>
       </c>
       <c r="D25">
         <v>5</v>
@@ -2127,7 +2353,7 @@
         <v>5</v>
       </c>
       <c r="F25" t="s">
-        <v>305</v>
+        <v>357</v>
       </c>
     </row>
     <row r="26" spans="1:6">
@@ -2135,10 +2361,10 @@
         <v>30</v>
       </c>
       <c r="B26" t="s">
-        <v>167</v>
+        <v>193</v>
       </c>
       <c r="C26" t="s">
-        <v>281</v>
+        <v>333</v>
       </c>
       <c r="D26">
         <v>5</v>
@@ -2147,7 +2373,7 @@
         <v>5</v>
       </c>
       <c r="F26" t="s">
-        <v>306</v>
+        <v>358</v>
       </c>
     </row>
     <row r="27" spans="1:6">
@@ -2155,10 +2381,10 @@
         <v>31</v>
       </c>
       <c r="B27" t="s">
-        <v>168</v>
+        <v>194</v>
       </c>
       <c r="C27" t="s">
-        <v>281</v>
+        <v>333</v>
       </c>
       <c r="D27">
         <v>5</v>
@@ -2167,7 +2393,7 @@
         <v>4</v>
       </c>
       <c r="F27" t="s">
-        <v>307</v>
+        <v>359</v>
       </c>
     </row>
     <row r="28" spans="1:6">
@@ -2175,10 +2401,10 @@
         <v>32</v>
       </c>
       <c r="B28" t="s">
-        <v>169</v>
+        <v>195</v>
       </c>
       <c r="C28" t="s">
-        <v>281</v>
+        <v>333</v>
       </c>
       <c r="D28">
         <v>5</v>
@@ -2187,7 +2413,7 @@
         <v>5</v>
       </c>
       <c r="F28" t="s">
-        <v>308</v>
+        <v>360</v>
       </c>
     </row>
     <row r="29" spans="1:6">
@@ -2195,10 +2421,10 @@
         <v>33</v>
       </c>
       <c r="B29" t="s">
-        <v>170</v>
+        <v>196</v>
       </c>
       <c r="C29" t="s">
-        <v>280</v>
+        <v>332</v>
       </c>
       <c r="D29">
         <v>5</v>
@@ -2207,7 +2433,7 @@
         <v>5</v>
       </c>
       <c r="F29" t="s">
-        <v>309</v>
+        <v>361</v>
       </c>
     </row>
     <row r="30" spans="1:6">
@@ -2215,10 +2441,10 @@
         <v>34</v>
       </c>
       <c r="B30" t="s">
-        <v>171</v>
+        <v>197</v>
       </c>
       <c r="C30" t="s">
-        <v>281</v>
+        <v>333</v>
       </c>
       <c r="D30">
         <v>5</v>
@@ -2227,7 +2453,7 @@
         <v>5</v>
       </c>
       <c r="F30" t="s">
-        <v>310</v>
+        <v>362</v>
       </c>
     </row>
     <row r="31" spans="1:6">
@@ -2235,10 +2461,10 @@
         <v>35</v>
       </c>
       <c r="B31" t="s">
-        <v>172</v>
+        <v>198</v>
       </c>
       <c r="C31" t="s">
-        <v>281</v>
+        <v>333</v>
       </c>
       <c r="D31">
         <v>5</v>
@@ -2247,7 +2473,7 @@
         <v>4</v>
       </c>
       <c r="F31" t="s">
-        <v>311</v>
+        <v>363</v>
       </c>
     </row>
     <row r="32" spans="1:6">
@@ -2255,10 +2481,10 @@
         <v>36</v>
       </c>
       <c r="B32" t="s">
-        <v>173</v>
+        <v>199</v>
       </c>
       <c r="C32" t="s">
-        <v>281</v>
+        <v>333</v>
       </c>
       <c r="D32">
         <v>5</v>
@@ -2267,7 +2493,7 @@
         <v>5</v>
       </c>
       <c r="F32" t="s">
-        <v>312</v>
+        <v>364</v>
       </c>
     </row>
     <row r="33" spans="1:6">
@@ -2275,10 +2501,10 @@
         <v>37</v>
       </c>
       <c r="B33" t="s">
-        <v>174</v>
+        <v>200</v>
       </c>
       <c r="C33" t="s">
-        <v>280</v>
+        <v>332</v>
       </c>
       <c r="D33">
         <v>5</v>
@@ -2287,7 +2513,7 @@
         <v>5</v>
       </c>
       <c r="F33" t="s">
-        <v>313</v>
+        <v>365</v>
       </c>
     </row>
     <row r="34" spans="1:6">
@@ -2295,10 +2521,10 @@
         <v>38</v>
       </c>
       <c r="B34" t="s">
-        <v>175</v>
+        <v>201</v>
       </c>
       <c r="C34" t="s">
-        <v>281</v>
+        <v>333</v>
       </c>
       <c r="D34">
         <v>4</v>
@@ -2307,7 +2533,7 @@
         <v>4</v>
       </c>
       <c r="F34" t="s">
-        <v>314</v>
+        <v>366</v>
       </c>
     </row>
     <row r="35" spans="1:6">
@@ -2315,10 +2541,10 @@
         <v>39</v>
       </c>
       <c r="B35" t="s">
-        <v>176</v>
+        <v>202</v>
       </c>
       <c r="C35" t="s">
-        <v>280</v>
+        <v>332</v>
       </c>
       <c r="D35">
         <v>4</v>
@@ -2327,7 +2553,7 @@
         <v>4</v>
       </c>
       <c r="F35" t="s">
-        <v>315</v>
+        <v>367</v>
       </c>
     </row>
     <row r="36" spans="1:6">
@@ -2335,10 +2561,10 @@
         <v>40</v>
       </c>
       <c r="B36" t="s">
-        <v>177</v>
+        <v>203</v>
       </c>
       <c r="C36" t="s">
-        <v>280</v>
+        <v>332</v>
       </c>
       <c r="D36">
         <v>4</v>
@@ -2347,7 +2573,7 @@
         <v>4</v>
       </c>
       <c r="F36" t="s">
-        <v>316</v>
+        <v>368</v>
       </c>
     </row>
     <row r="37" spans="1:6">
@@ -2355,10 +2581,10 @@
         <v>41</v>
       </c>
       <c r="B37" t="s">
-        <v>178</v>
+        <v>204</v>
       </c>
       <c r="C37" t="s">
-        <v>280</v>
+        <v>332</v>
       </c>
       <c r="D37">
         <v>4</v>
@@ -2367,7 +2593,7 @@
         <v>4</v>
       </c>
       <c r="F37" t="s">
-        <v>317</v>
+        <v>369</v>
       </c>
     </row>
     <row r="38" spans="1:6">
@@ -2375,19 +2601,19 @@
         <v>42</v>
       </c>
       <c r="B38" t="s">
-        <v>179</v>
+        <v>205</v>
       </c>
       <c r="C38" t="s">
-        <v>280</v>
+        <v>332</v>
       </c>
       <c r="D38">
         <v>4</v>
       </c>
       <c r="E38">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="F38" t="s">
-        <v>318</v>
+        <v>370</v>
       </c>
     </row>
     <row r="39" spans="1:6">
@@ -2395,10 +2621,10 @@
         <v>43</v>
       </c>
       <c r="B39" t="s">
-        <v>180</v>
+        <v>206</v>
       </c>
       <c r="C39" t="s">
-        <v>281</v>
+        <v>332</v>
       </c>
       <c r="D39">
         <v>4</v>
@@ -2407,7 +2633,7 @@
         <v>4</v>
       </c>
       <c r="F39" t="s">
-        <v>319</v>
+        <v>371</v>
       </c>
     </row>
     <row r="40" spans="1:6">
@@ -2415,10 +2641,10 @@
         <v>44</v>
       </c>
       <c r="B40" t="s">
-        <v>181</v>
+        <v>207</v>
       </c>
       <c r="C40" t="s">
-        <v>281</v>
+        <v>332</v>
       </c>
       <c r="D40">
         <v>4</v>
@@ -2427,7 +2653,7 @@
         <v>4</v>
       </c>
       <c r="F40" t="s">
-        <v>320</v>
+        <v>372</v>
       </c>
     </row>
     <row r="41" spans="1:6">
@@ -2435,10 +2661,10 @@
         <v>45</v>
       </c>
       <c r="B41" t="s">
-        <v>182</v>
+        <v>208</v>
       </c>
       <c r="C41" t="s">
-        <v>281</v>
+        <v>332</v>
       </c>
       <c r="D41">
         <v>4</v>
@@ -2447,7 +2673,7 @@
         <v>4</v>
       </c>
       <c r="F41" t="s">
-        <v>321</v>
+        <v>373</v>
       </c>
     </row>
     <row r="42" spans="1:6">
@@ -2455,10 +2681,10 @@
         <v>46</v>
       </c>
       <c r="B42" t="s">
-        <v>183</v>
+        <v>209</v>
       </c>
       <c r="C42" t="s">
-        <v>281</v>
+        <v>333</v>
       </c>
       <c r="D42">
         <v>4</v>
@@ -2467,7 +2693,7 @@
         <v>4</v>
       </c>
       <c r="F42" t="s">
-        <v>322</v>
+        <v>374</v>
       </c>
     </row>
     <row r="43" spans="1:6">
@@ -2475,19 +2701,19 @@
         <v>47</v>
       </c>
       <c r="B43" t="s">
-        <v>184</v>
+        <v>210</v>
       </c>
       <c r="C43" t="s">
-        <v>282</v>
+        <v>333</v>
       </c>
       <c r="D43">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="E43">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="F43" t="s">
-        <v>323</v>
+        <v>375</v>
       </c>
     </row>
     <row r="44" spans="1:6">
@@ -2495,19 +2721,19 @@
         <v>48</v>
       </c>
       <c r="B44" t="s">
-        <v>185</v>
+        <v>211</v>
       </c>
       <c r="C44" t="s">
-        <v>280</v>
+        <v>333</v>
       </c>
       <c r="D44">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="E44">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="F44" t="s">
-        <v>324</v>
+        <v>376</v>
       </c>
     </row>
     <row r="45" spans="1:6">
@@ -2515,19 +2741,19 @@
         <v>49</v>
       </c>
       <c r="B45" t="s">
-        <v>186</v>
+        <v>212</v>
       </c>
       <c r="C45" t="s">
-        <v>281</v>
+        <v>333</v>
       </c>
       <c r="D45">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="E45">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="F45" t="s">
-        <v>325</v>
+        <v>377</v>
       </c>
     </row>
     <row r="46" spans="1:6">
@@ -2535,10 +2761,10 @@
         <v>50</v>
       </c>
       <c r="B46" t="s">
-        <v>187</v>
+        <v>213</v>
       </c>
       <c r="C46" t="s">
-        <v>280</v>
+        <v>334</v>
       </c>
       <c r="D46">
         <v>3</v>
@@ -2547,7 +2773,7 @@
         <v>3</v>
       </c>
       <c r="F46" t="s">
-        <v>326</v>
+        <v>378</v>
       </c>
     </row>
     <row r="47" spans="1:6">
@@ -2555,10 +2781,10 @@
         <v>51</v>
       </c>
       <c r="B47" t="s">
-        <v>188</v>
+        <v>214</v>
       </c>
       <c r="C47" t="s">
-        <v>280</v>
+        <v>332</v>
       </c>
       <c r="D47">
         <v>3</v>
@@ -2567,7 +2793,7 @@
         <v>3</v>
       </c>
       <c r="F47" t="s">
-        <v>327</v>
+        <v>379</v>
       </c>
     </row>
     <row r="48" spans="1:6">
@@ -2575,10 +2801,10 @@
         <v>52</v>
       </c>
       <c r="B48" t="s">
-        <v>189</v>
+        <v>215</v>
       </c>
       <c r="C48" t="s">
-        <v>281</v>
+        <v>333</v>
       </c>
       <c r="D48">
         <v>3</v>
@@ -2587,7 +2813,7 @@
         <v>3</v>
       </c>
       <c r="F48" t="s">
-        <v>328</v>
+        <v>380</v>
       </c>
     </row>
     <row r="49" spans="1:6">
@@ -2595,10 +2821,10 @@
         <v>53</v>
       </c>
       <c r="B49" t="s">
-        <v>190</v>
+        <v>216</v>
       </c>
       <c r="C49" t="s">
-        <v>281</v>
+        <v>332</v>
       </c>
       <c r="D49">
         <v>3</v>
@@ -2607,7 +2833,7 @@
         <v>3</v>
       </c>
       <c r="F49" t="s">
-        <v>329</v>
+        <v>381</v>
       </c>
     </row>
     <row r="50" spans="1:6">
@@ -2615,10 +2841,10 @@
         <v>54</v>
       </c>
       <c r="B50" t="s">
-        <v>191</v>
+        <v>217</v>
       </c>
       <c r="C50" t="s">
-        <v>281</v>
+        <v>332</v>
       </c>
       <c r="D50">
         <v>3</v>
@@ -2627,7 +2853,7 @@
         <v>3</v>
       </c>
       <c r="F50" t="s">
-        <v>330</v>
+        <v>382</v>
       </c>
     </row>
     <row r="51" spans="1:6">
@@ -2635,10 +2861,10 @@
         <v>55</v>
       </c>
       <c r="B51" t="s">
-        <v>192</v>
+        <v>218</v>
       </c>
       <c r="C51" t="s">
-        <v>281</v>
+        <v>333</v>
       </c>
       <c r="D51">
         <v>3</v>
@@ -2647,7 +2873,7 @@
         <v>3</v>
       </c>
       <c r="F51" t="s">
-        <v>331</v>
+        <v>383</v>
       </c>
     </row>
     <row r="52" spans="1:6">
@@ -2655,19 +2881,19 @@
         <v>56</v>
       </c>
       <c r="B52" t="s">
-        <v>193</v>
+        <v>219</v>
       </c>
       <c r="C52" t="s">
-        <v>281</v>
+        <v>333</v>
       </c>
       <c r="D52">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="E52">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="F52" t="s">
-        <v>332</v>
+        <v>384</v>
       </c>
     </row>
     <row r="53" spans="1:6">
@@ -2675,19 +2901,19 @@
         <v>57</v>
       </c>
       <c r="B53" t="s">
-        <v>194</v>
+        <v>220</v>
       </c>
       <c r="C53" t="s">
-        <v>281</v>
+        <v>333</v>
       </c>
       <c r="D53">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="E53">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="F53" t="s">
-        <v>333</v>
+        <v>385</v>
       </c>
     </row>
     <row r="54" spans="1:6">
@@ -2695,19 +2921,19 @@
         <v>58</v>
       </c>
       <c r="B54" t="s">
-        <v>195</v>
+        <v>221</v>
       </c>
       <c r="C54" t="s">
-        <v>281</v>
+        <v>333</v>
       </c>
       <c r="D54">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="E54">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="F54" t="s">
-        <v>334</v>
+        <v>386</v>
       </c>
     </row>
     <row r="55" spans="1:6">
@@ -2715,19 +2941,19 @@
         <v>59</v>
       </c>
       <c r="B55" t="s">
-        <v>196</v>
+        <v>222</v>
       </c>
       <c r="C55" t="s">
-        <v>280</v>
+        <v>333</v>
       </c>
       <c r="D55">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="E55">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="F55" t="s">
-        <v>335</v>
+        <v>387</v>
       </c>
     </row>
     <row r="56" spans="1:6">
@@ -2735,19 +2961,19 @@
         <v>60</v>
       </c>
       <c r="B56" t="s">
-        <v>197</v>
+        <v>223</v>
       </c>
       <c r="C56" t="s">
-        <v>280</v>
+        <v>333</v>
       </c>
       <c r="D56">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="E56">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="F56" t="s">
-        <v>320</v>
+        <v>388</v>
       </c>
     </row>
     <row r="57" spans="1:6">
@@ -2755,19 +2981,19 @@
         <v>61</v>
       </c>
       <c r="B57" t="s">
-        <v>198</v>
+        <v>224</v>
       </c>
       <c r="C57" t="s">
-        <v>281</v>
+        <v>333</v>
       </c>
       <c r="D57">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="E57">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="F57" t="s">
-        <v>336</v>
+        <v>389</v>
       </c>
     </row>
     <row r="58" spans="1:6">
@@ -2775,19 +3001,19 @@
         <v>62</v>
       </c>
       <c r="B58" t="s">
-        <v>199</v>
+        <v>225</v>
       </c>
       <c r="C58" t="s">
-        <v>280</v>
+        <v>332</v>
       </c>
       <c r="D58">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="E58">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="F58" t="s">
-        <v>337</v>
+        <v>390</v>
       </c>
     </row>
     <row r="59" spans="1:6">
@@ -2795,19 +3021,19 @@
         <v>63</v>
       </c>
       <c r="B59" t="s">
-        <v>200</v>
+        <v>226</v>
       </c>
       <c r="C59" t="s">
-        <v>280</v>
+        <v>333</v>
       </c>
       <c r="D59">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="E59">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="F59" t="s">
-        <v>338</v>
+        <v>391</v>
       </c>
     </row>
     <row r="60" spans="1:6">
@@ -2815,19 +3041,19 @@
         <v>64</v>
       </c>
       <c r="B60" t="s">
-        <v>201</v>
+        <v>227</v>
       </c>
       <c r="C60" t="s">
-        <v>281</v>
+        <v>333</v>
       </c>
       <c r="D60">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="E60">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="F60" t="s">
-        <v>339</v>
+        <v>392</v>
       </c>
     </row>
     <row r="61" spans="1:6">
@@ -2835,10 +3061,10 @@
         <v>65</v>
       </c>
       <c r="B61" t="s">
-        <v>202</v>
+        <v>228</v>
       </c>
       <c r="C61" t="s">
-        <v>280</v>
+        <v>333</v>
       </c>
       <c r="D61">
         <v>2</v>
@@ -2847,7 +3073,7 @@
         <v>2</v>
       </c>
       <c r="F61" t="s">
-        <v>340</v>
+        <v>393</v>
       </c>
     </row>
     <row r="62" spans="1:6">
@@ -2855,10 +3081,10 @@
         <v>66</v>
       </c>
       <c r="B62" t="s">
-        <v>203</v>
+        <v>229</v>
       </c>
       <c r="C62" t="s">
-        <v>280</v>
+        <v>333</v>
       </c>
       <c r="D62">
         <v>2</v>
@@ -2867,7 +3093,7 @@
         <v>2</v>
       </c>
       <c r="F62" t="s">
-        <v>341</v>
+        <v>394</v>
       </c>
     </row>
     <row r="63" spans="1:6">
@@ -2875,10 +3101,10 @@
         <v>67</v>
       </c>
       <c r="B63" t="s">
-        <v>204</v>
+        <v>230</v>
       </c>
       <c r="C63" t="s">
-        <v>280</v>
+        <v>333</v>
       </c>
       <c r="D63">
         <v>2</v>
@@ -2887,7 +3113,7 @@
         <v>2</v>
       </c>
       <c r="F63" t="s">
-        <v>342</v>
+        <v>395</v>
       </c>
     </row>
     <row r="64" spans="1:6">
@@ -2895,10 +3121,10 @@
         <v>68</v>
       </c>
       <c r="B64" t="s">
-        <v>205</v>
+        <v>231</v>
       </c>
       <c r="C64" t="s">
-        <v>280</v>
+        <v>332</v>
       </c>
       <c r="D64">
         <v>2</v>
@@ -2907,7 +3133,7 @@
         <v>2</v>
       </c>
       <c r="F64" t="s">
-        <v>343</v>
+        <v>396</v>
       </c>
     </row>
     <row r="65" spans="1:6">
@@ -2915,10 +3141,10 @@
         <v>69</v>
       </c>
       <c r="B65" t="s">
-        <v>206</v>
+        <v>232</v>
       </c>
       <c r="C65" t="s">
-        <v>281</v>
+        <v>332</v>
       </c>
       <c r="D65">
         <v>2</v>
@@ -2927,7 +3153,7 @@
         <v>2</v>
       </c>
       <c r="F65" t="s">
-        <v>344</v>
+        <v>375</v>
       </c>
     </row>
     <row r="66" spans="1:6">
@@ -2935,10 +3161,10 @@
         <v>70</v>
       </c>
       <c r="B66" t="s">
-        <v>207</v>
+        <v>233</v>
       </c>
       <c r="C66" t="s">
-        <v>281</v>
+        <v>333</v>
       </c>
       <c r="D66">
         <v>2</v>
@@ -2947,7 +3173,7 @@
         <v>2</v>
       </c>
       <c r="F66" t="s">
-        <v>345</v>
+        <v>397</v>
       </c>
     </row>
     <row r="67" spans="1:6">
@@ -2955,10 +3181,10 @@
         <v>71</v>
       </c>
       <c r="B67" t="s">
-        <v>208</v>
+        <v>234</v>
       </c>
       <c r="C67" t="s">
-        <v>280</v>
+        <v>332</v>
       </c>
       <c r="D67">
         <v>2</v>
@@ -2967,7 +3193,7 @@
         <v>2</v>
       </c>
       <c r="F67" t="s">
-        <v>346</v>
+        <v>398</v>
       </c>
     </row>
     <row r="68" spans="1:6">
@@ -2975,10 +3201,10 @@
         <v>72</v>
       </c>
       <c r="B68" t="s">
-        <v>209</v>
+        <v>235</v>
       </c>
       <c r="C68" t="s">
-        <v>281</v>
+        <v>332</v>
       </c>
       <c r="D68">
         <v>2</v>
@@ -2987,7 +3213,7 @@
         <v>2</v>
       </c>
       <c r="F68" t="s">
-        <v>347</v>
+        <v>399</v>
       </c>
     </row>
     <row r="69" spans="1:6">
@@ -2995,10 +3221,10 @@
         <v>73</v>
       </c>
       <c r="B69" t="s">
-        <v>210</v>
+        <v>236</v>
       </c>
       <c r="C69" t="s">
-        <v>281</v>
+        <v>333</v>
       </c>
       <c r="D69">
         <v>2</v>
@@ -3007,7 +3233,7 @@
         <v>2</v>
       </c>
       <c r="F69" t="s">
-        <v>348</v>
+        <v>400</v>
       </c>
     </row>
     <row r="70" spans="1:6">
@@ -3015,10 +3241,10 @@
         <v>74</v>
       </c>
       <c r="B70" t="s">
-        <v>211</v>
+        <v>237</v>
       </c>
       <c r="C70" t="s">
-        <v>280</v>
+        <v>332</v>
       </c>
       <c r="D70">
         <v>2</v>
@@ -3027,7 +3253,7 @@
         <v>2</v>
       </c>
       <c r="F70" t="s">
-        <v>349</v>
+        <v>401</v>
       </c>
     </row>
     <row r="71" spans="1:6">
@@ -3035,10 +3261,10 @@
         <v>75</v>
       </c>
       <c r="B71" t="s">
-        <v>212</v>
+        <v>238</v>
       </c>
       <c r="C71" t="s">
-        <v>281</v>
+        <v>332</v>
       </c>
       <c r="D71">
         <v>2</v>
@@ -3047,7 +3273,7 @@
         <v>2</v>
       </c>
       <c r="F71" t="s">
-        <v>350</v>
+        <v>402</v>
       </c>
     </row>
     <row r="72" spans="1:6">
@@ -3055,10 +3281,10 @@
         <v>76</v>
       </c>
       <c r="B72" t="s">
-        <v>213</v>
+        <v>239</v>
       </c>
       <c r="C72" t="s">
-        <v>281</v>
+        <v>332</v>
       </c>
       <c r="D72">
         <v>2</v>
@@ -3067,7 +3293,7 @@
         <v>2</v>
       </c>
       <c r="F72" t="s">
-        <v>351</v>
+        <v>403</v>
       </c>
     </row>
     <row r="73" spans="1:6">
@@ -3075,10 +3301,10 @@
         <v>77</v>
       </c>
       <c r="B73" t="s">
-        <v>214</v>
+        <v>240</v>
       </c>
       <c r="C73" t="s">
-        <v>281</v>
+        <v>332</v>
       </c>
       <c r="D73">
         <v>2</v>
@@ -3087,7 +3313,7 @@
         <v>2</v>
       </c>
       <c r="F73" t="s">
-        <v>352</v>
+        <v>404</v>
       </c>
     </row>
     <row r="74" spans="1:6">
@@ -3095,10 +3321,10 @@
         <v>78</v>
       </c>
       <c r="B74" t="s">
-        <v>215</v>
+        <v>241</v>
       </c>
       <c r="C74" t="s">
-        <v>281</v>
+        <v>333</v>
       </c>
       <c r="D74">
         <v>2</v>
@@ -3107,7 +3333,7 @@
         <v>2</v>
       </c>
       <c r="F74" t="s">
-        <v>353</v>
+        <v>405</v>
       </c>
     </row>
     <row r="75" spans="1:6">
@@ -3115,10 +3341,10 @@
         <v>79</v>
       </c>
       <c r="B75" t="s">
-        <v>216</v>
+        <v>242</v>
       </c>
       <c r="C75" t="s">
-        <v>281</v>
+        <v>333</v>
       </c>
       <c r="D75">
         <v>2</v>
@@ -3127,7 +3353,7 @@
         <v>2</v>
       </c>
       <c r="F75" t="s">
-        <v>354</v>
+        <v>406</v>
       </c>
     </row>
     <row r="76" spans="1:6">
@@ -3135,10 +3361,10 @@
         <v>80</v>
       </c>
       <c r="B76" t="s">
-        <v>217</v>
+        <v>243</v>
       </c>
       <c r="C76" t="s">
-        <v>281</v>
+        <v>333</v>
       </c>
       <c r="D76">
         <v>2</v>
@@ -3147,7 +3373,7 @@
         <v>2</v>
       </c>
       <c r="F76" t="s">
-        <v>355</v>
+        <v>407</v>
       </c>
     </row>
     <row r="77" spans="1:6">
@@ -3155,10 +3381,10 @@
         <v>81</v>
       </c>
       <c r="B77" t="s">
-        <v>218</v>
+        <v>244</v>
       </c>
       <c r="C77" t="s">
-        <v>281</v>
+        <v>332</v>
       </c>
       <c r="D77">
         <v>2</v>
@@ -3167,7 +3393,7 @@
         <v>2</v>
       </c>
       <c r="F77" t="s">
-        <v>356</v>
+        <v>408</v>
       </c>
     </row>
     <row r="78" spans="1:6">
@@ -3175,10 +3401,10 @@
         <v>82</v>
       </c>
       <c r="B78" t="s">
-        <v>219</v>
+        <v>245</v>
       </c>
       <c r="C78" t="s">
-        <v>281</v>
+        <v>333</v>
       </c>
       <c r="D78">
         <v>2</v>
@@ -3187,7 +3413,7 @@
         <v>2</v>
       </c>
       <c r="F78" t="s">
-        <v>357</v>
+        <v>409</v>
       </c>
     </row>
     <row r="79" spans="1:6">
@@ -3195,10 +3421,10 @@
         <v>83</v>
       </c>
       <c r="B79" t="s">
-        <v>220</v>
+        <v>246</v>
       </c>
       <c r="C79" t="s">
-        <v>281</v>
+        <v>333</v>
       </c>
       <c r="D79">
         <v>2</v>
@@ -3207,7 +3433,7 @@
         <v>2</v>
       </c>
       <c r="F79" t="s">
-        <v>358</v>
+        <v>410</v>
       </c>
     </row>
     <row r="80" spans="1:6">
@@ -3215,10 +3441,10 @@
         <v>84</v>
       </c>
       <c r="B80" t="s">
-        <v>221</v>
+        <v>247</v>
       </c>
       <c r="C80" t="s">
-        <v>280</v>
+        <v>333</v>
       </c>
       <c r="D80">
         <v>2</v>
@@ -3227,7 +3453,7 @@
         <v>2</v>
       </c>
       <c r="F80" t="s">
-        <v>359</v>
+        <v>411</v>
       </c>
     </row>
     <row r="81" spans="1:6">
@@ -3235,19 +3461,19 @@
         <v>85</v>
       </c>
       <c r="B81" t="s">
-        <v>222</v>
+        <v>248</v>
       </c>
       <c r="C81" t="s">
-        <v>281</v>
+        <v>333</v>
       </c>
       <c r="D81">
         <v>2</v>
       </c>
       <c r="E81">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="F81" t="s">
-        <v>360</v>
+        <v>412</v>
       </c>
     </row>
     <row r="82" spans="1:6">
@@ -3255,10 +3481,10 @@
         <v>86</v>
       </c>
       <c r="B82" t="s">
-        <v>223</v>
+        <v>249</v>
       </c>
       <c r="C82" t="s">
-        <v>281</v>
+        <v>333</v>
       </c>
       <c r="D82">
         <v>2</v>
@@ -3267,7 +3493,7 @@
         <v>2</v>
       </c>
       <c r="F82" t="s">
-        <v>295</v>
+        <v>368</v>
       </c>
     </row>
     <row r="83" spans="1:6">
@@ -3275,19 +3501,19 @@
         <v>87</v>
       </c>
       <c r="B83" t="s">
-        <v>224</v>
+        <v>250</v>
       </c>
       <c r="C83" t="s">
-        <v>281</v>
+        <v>332</v>
       </c>
       <c r="D83">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="E83">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="F83" t="s">
-        <v>361</v>
+        <v>356</v>
       </c>
     </row>
     <row r="84" spans="1:6">
@@ -3295,19 +3521,19 @@
         <v>88</v>
       </c>
       <c r="B84" t="s">
-        <v>225</v>
+        <v>251</v>
       </c>
       <c r="C84" t="s">
-        <v>280</v>
+        <v>332</v>
       </c>
       <c r="D84">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="E84">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="F84" t="s">
-        <v>362</v>
+        <v>413</v>
       </c>
     </row>
     <row r="85" spans="1:6">
@@ -3315,19 +3541,19 @@
         <v>89</v>
       </c>
       <c r="B85" t="s">
-        <v>226</v>
+        <v>252</v>
       </c>
       <c r="C85" t="s">
-        <v>280</v>
+        <v>333</v>
       </c>
       <c r="D85">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="E85">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="F85" t="s">
-        <v>363</v>
+        <v>414</v>
       </c>
     </row>
     <row r="86" spans="1:6">
@@ -3335,19 +3561,19 @@
         <v>90</v>
       </c>
       <c r="B86" t="s">
-        <v>227</v>
+        <v>253</v>
       </c>
       <c r="C86" t="s">
-        <v>280</v>
+        <v>333</v>
       </c>
       <c r="D86">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="E86">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="F86" t="s">
-        <v>364</v>
+        <v>415</v>
       </c>
     </row>
     <row r="87" spans="1:6">
@@ -3355,19 +3581,19 @@
         <v>91</v>
       </c>
       <c r="B87" t="s">
-        <v>228</v>
+        <v>254</v>
       </c>
       <c r="C87" t="s">
-        <v>281</v>
+        <v>333</v>
       </c>
       <c r="D87">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="E87">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="F87" t="s">
-        <v>365</v>
+        <v>339</v>
       </c>
     </row>
     <row r="88" spans="1:6">
@@ -3375,19 +3601,19 @@
         <v>92</v>
       </c>
       <c r="B88" t="s">
-        <v>229</v>
+        <v>255</v>
       </c>
       <c r="C88" t="s">
-        <v>280</v>
+        <v>333</v>
       </c>
       <c r="D88">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="E88">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="F88" t="s">
-        <v>366</v>
+        <v>416</v>
       </c>
     </row>
     <row r="89" spans="1:6">
@@ -3395,19 +3621,19 @@
         <v>93</v>
       </c>
       <c r="B89" t="s">
-        <v>230</v>
+        <v>256</v>
       </c>
       <c r="C89" t="s">
-        <v>281</v>
+        <v>333</v>
       </c>
       <c r="D89">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="E89">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="F89" t="s">
-        <v>367</v>
+        <v>417</v>
       </c>
     </row>
     <row r="90" spans="1:6">
@@ -3415,19 +3641,19 @@
         <v>94</v>
       </c>
       <c r="B90" t="s">
-        <v>231</v>
+        <v>257</v>
       </c>
       <c r="C90" t="s">
-        <v>280</v>
+        <v>333</v>
       </c>
       <c r="D90">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="E90">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="F90" t="s">
-        <v>368</v>
+        <v>418</v>
       </c>
     </row>
     <row r="91" spans="1:6">
@@ -3435,19 +3661,19 @@
         <v>95</v>
       </c>
       <c r="B91" t="s">
-        <v>232</v>
+        <v>258</v>
       </c>
       <c r="C91" t="s">
-        <v>280</v>
+        <v>333</v>
       </c>
       <c r="D91">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="E91">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="F91" t="s">
-        <v>369</v>
+        <v>419</v>
       </c>
     </row>
     <row r="92" spans="1:6">
@@ -3455,19 +3681,19 @@
         <v>96</v>
       </c>
       <c r="B92" t="s">
-        <v>233</v>
+        <v>259</v>
       </c>
       <c r="C92" t="s">
-        <v>280</v>
+        <v>333</v>
       </c>
       <c r="D92">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="E92">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="F92" t="s">
-        <v>370</v>
+        <v>420</v>
       </c>
     </row>
     <row r="93" spans="1:6">
@@ -3475,19 +3701,19 @@
         <v>97</v>
       </c>
       <c r="B93" t="s">
-        <v>234</v>
+        <v>260</v>
       </c>
       <c r="C93" t="s">
-        <v>280</v>
+        <v>333</v>
       </c>
       <c r="D93">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="E93">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="F93" t="s">
-        <v>371</v>
+        <v>421</v>
       </c>
     </row>
     <row r="94" spans="1:6">
@@ -3495,19 +3721,19 @@
         <v>98</v>
       </c>
       <c r="B94" t="s">
-        <v>235</v>
+        <v>261</v>
       </c>
       <c r="C94" t="s">
-        <v>280</v>
+        <v>333</v>
       </c>
       <c r="D94">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="E94">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="F94" t="s">
-        <v>372</v>
+        <v>422</v>
       </c>
     </row>
     <row r="95" spans="1:6">
@@ -3515,19 +3741,19 @@
         <v>99</v>
       </c>
       <c r="B95" t="s">
-        <v>236</v>
+        <v>262</v>
       </c>
       <c r="C95" t="s">
-        <v>280</v>
+        <v>333</v>
       </c>
       <c r="D95">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="E95">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="F95" t="s">
-        <v>373</v>
+        <v>423</v>
       </c>
     </row>
     <row r="96" spans="1:6">
@@ -3535,19 +3761,19 @@
         <v>100</v>
       </c>
       <c r="B96" t="s">
-        <v>237</v>
+        <v>263</v>
       </c>
       <c r="C96" t="s">
-        <v>281</v>
+        <v>333</v>
       </c>
       <c r="D96">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="E96">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="F96" t="s">
-        <v>374</v>
+        <v>424</v>
       </c>
     </row>
     <row r="97" spans="1:6">
@@ -3555,19 +3781,19 @@
         <v>101</v>
       </c>
       <c r="B97" t="s">
-        <v>238</v>
+        <v>264</v>
       </c>
       <c r="C97" t="s">
-        <v>281</v>
+        <v>333</v>
       </c>
       <c r="D97">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="E97">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="F97" t="s">
-        <v>375</v>
+        <v>425</v>
       </c>
     </row>
     <row r="98" spans="1:6">
@@ -3575,19 +3801,19 @@
         <v>102</v>
       </c>
       <c r="B98" t="s">
-        <v>239</v>
+        <v>265</v>
       </c>
       <c r="C98" t="s">
-        <v>281</v>
+        <v>333</v>
       </c>
       <c r="D98">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="E98">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="F98" t="s">
-        <v>376</v>
+        <v>426</v>
       </c>
     </row>
     <row r="99" spans="1:6">
@@ -3595,19 +3821,19 @@
         <v>103</v>
       </c>
       <c r="B99" t="s">
-        <v>240</v>
+        <v>266</v>
       </c>
       <c r="C99" t="s">
-        <v>281</v>
+        <v>332</v>
       </c>
       <c r="D99">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="E99">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="F99" t="s">
-        <v>377</v>
+        <v>427</v>
       </c>
     </row>
     <row r="100" spans="1:6">
@@ -3615,19 +3841,19 @@
         <v>104</v>
       </c>
       <c r="B100" t="s">
-        <v>241</v>
+        <v>267</v>
       </c>
       <c r="C100" t="s">
-        <v>280</v>
+        <v>333</v>
       </c>
       <c r="D100">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="E100">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="F100" t="s">
-        <v>378</v>
+        <v>428</v>
       </c>
     </row>
     <row r="101" spans="1:6">
@@ -3635,19 +3861,19 @@
         <v>105</v>
       </c>
       <c r="B101" t="s">
-        <v>242</v>
+        <v>268</v>
       </c>
       <c r="C101" t="s">
-        <v>280</v>
+        <v>333</v>
       </c>
       <c r="D101">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="E101">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="F101" t="s">
-        <v>379</v>
+        <v>429</v>
       </c>
     </row>
     <row r="102" spans="1:6">
@@ -3655,19 +3881,19 @@
         <v>106</v>
       </c>
       <c r="B102" t="s">
-        <v>243</v>
+        <v>269</v>
       </c>
       <c r="C102" t="s">
-        <v>281</v>
+        <v>333</v>
       </c>
       <c r="D102">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="E102">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="F102" t="s">
-        <v>380</v>
+        <v>430</v>
       </c>
     </row>
     <row r="103" spans="1:6">
@@ -3675,19 +3901,19 @@
         <v>107</v>
       </c>
       <c r="B103" t="s">
-        <v>244</v>
+        <v>270</v>
       </c>
       <c r="C103" t="s">
-        <v>281</v>
+        <v>333</v>
       </c>
       <c r="D103">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="E103">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="F103" t="s">
-        <v>381</v>
+        <v>431</v>
       </c>
     </row>
     <row r="104" spans="1:6">
@@ -3695,19 +3921,19 @@
         <v>108</v>
       </c>
       <c r="B104" t="s">
-        <v>245</v>
+        <v>271</v>
       </c>
       <c r="C104" t="s">
-        <v>280</v>
+        <v>333</v>
       </c>
       <c r="D104">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="E104">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="F104" t="s">
-        <v>374</v>
+        <v>343</v>
       </c>
     </row>
     <row r="105" spans="1:6">
@@ -3715,19 +3941,19 @@
         <v>109</v>
       </c>
       <c r="B105" t="s">
-        <v>246</v>
+        <v>272</v>
       </c>
       <c r="C105" t="s">
-        <v>280</v>
+        <v>333</v>
       </c>
       <c r="D105">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="E105">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="F105" t="s">
-        <v>382</v>
+        <v>432</v>
       </c>
     </row>
     <row r="106" spans="1:6">
@@ -3735,19 +3961,19 @@
         <v>110</v>
       </c>
       <c r="B106" t="s">
-        <v>247</v>
+        <v>273</v>
       </c>
       <c r="C106" t="s">
-        <v>280</v>
+        <v>333</v>
       </c>
       <c r="D106">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="E106">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="F106" t="s">
-        <v>383</v>
+        <v>433</v>
       </c>
     </row>
     <row r="107" spans="1:6">
@@ -3755,19 +3981,19 @@
         <v>111</v>
       </c>
       <c r="B107" t="s">
-        <v>248</v>
+        <v>274</v>
       </c>
       <c r="C107" t="s">
-        <v>281</v>
+        <v>333</v>
       </c>
       <c r="D107">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="E107">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="F107" t="s">
-        <v>384</v>
+        <v>347</v>
       </c>
     </row>
     <row r="108" spans="1:6">
@@ -3775,10 +4001,10 @@
         <v>112</v>
       </c>
       <c r="B108" t="s">
-        <v>249</v>
+        <v>275</v>
       </c>
       <c r="C108" t="s">
-        <v>280</v>
+        <v>333</v>
       </c>
       <c r="D108">
         <v>1</v>
@@ -3787,7 +4013,7 @@
         <v>1</v>
       </c>
       <c r="F108" t="s">
-        <v>385</v>
+        <v>434</v>
       </c>
     </row>
     <row r="109" spans="1:6">
@@ -3795,10 +4021,10 @@
         <v>113</v>
       </c>
       <c r="B109" t="s">
-        <v>250</v>
+        <v>276</v>
       </c>
       <c r="C109" t="s">
-        <v>281</v>
+        <v>332</v>
       </c>
       <c r="D109">
         <v>1</v>
@@ -3807,7 +4033,7 @@
         <v>1</v>
       </c>
       <c r="F109" t="s">
-        <v>386</v>
+        <v>435</v>
       </c>
     </row>
     <row r="110" spans="1:6">
@@ -3815,10 +4041,10 @@
         <v>114</v>
       </c>
       <c r="B110" t="s">
-        <v>251</v>
+        <v>277</v>
       </c>
       <c r="C110" t="s">
-        <v>280</v>
+        <v>332</v>
       </c>
       <c r="D110">
         <v>1</v>
@@ -3827,7 +4053,7 @@
         <v>1</v>
       </c>
       <c r="F110" t="s">
-        <v>336</v>
+        <v>436</v>
       </c>
     </row>
     <row r="111" spans="1:6">
@@ -3835,10 +4061,10 @@
         <v>115</v>
       </c>
       <c r="B111" t="s">
-        <v>252</v>
+        <v>278</v>
       </c>
       <c r="C111" t="s">
-        <v>281</v>
+        <v>332</v>
       </c>
       <c r="D111">
         <v>1</v>
@@ -3847,7 +4073,7 @@
         <v>1</v>
       </c>
       <c r="F111" t="s">
-        <v>387</v>
+        <v>437</v>
       </c>
     </row>
     <row r="112" spans="1:6">
@@ -3855,10 +4081,10 @@
         <v>116</v>
       </c>
       <c r="B112" t="s">
-        <v>253</v>
+        <v>279</v>
       </c>
       <c r="C112" t="s">
-        <v>280</v>
+        <v>333</v>
       </c>
       <c r="D112">
         <v>1</v>
@@ -3867,7 +4093,7 @@
         <v>1</v>
       </c>
       <c r="F112" t="s">
-        <v>388</v>
+        <v>438</v>
       </c>
     </row>
     <row r="113" spans="1:6">
@@ -3875,10 +4101,10 @@
         <v>117</v>
       </c>
       <c r="B113" t="s">
-        <v>254</v>
+        <v>280</v>
       </c>
       <c r="C113" t="s">
-        <v>281</v>
+        <v>332</v>
       </c>
       <c r="D113">
         <v>1</v>
@@ -3887,7 +4113,7 @@
         <v>1</v>
       </c>
       <c r="F113" t="s">
-        <v>389</v>
+        <v>439</v>
       </c>
     </row>
     <row r="114" spans="1:6">
@@ -3895,10 +4121,10 @@
         <v>118</v>
       </c>
       <c r="B114" t="s">
-        <v>255</v>
+        <v>281</v>
       </c>
       <c r="C114" t="s">
-        <v>280</v>
+        <v>333</v>
       </c>
       <c r="D114">
         <v>1</v>
@@ -3907,7 +4133,7 @@
         <v>1</v>
       </c>
       <c r="F114" t="s">
-        <v>390</v>
+        <v>440</v>
       </c>
     </row>
     <row r="115" spans="1:6">
@@ -3915,10 +4141,10 @@
         <v>119</v>
       </c>
       <c r="B115" t="s">
-        <v>256</v>
+        <v>282</v>
       </c>
       <c r="C115" t="s">
-        <v>280</v>
+        <v>332</v>
       </c>
       <c r="D115">
         <v>1</v>
@@ -3927,7 +4153,7 @@
         <v>1</v>
       </c>
       <c r="F115" t="s">
-        <v>368</v>
+        <v>441</v>
       </c>
     </row>
     <row r="116" spans="1:6">
@@ -3935,10 +4161,10 @@
         <v>120</v>
       </c>
       <c r="B116" t="s">
-        <v>257</v>
+        <v>283</v>
       </c>
       <c r="C116" t="s">
-        <v>281</v>
+        <v>332</v>
       </c>
       <c r="D116">
         <v>1</v>
@@ -3947,7 +4173,7 @@
         <v>1</v>
       </c>
       <c r="F116" t="s">
-        <v>391</v>
+        <v>442</v>
       </c>
     </row>
     <row r="117" spans="1:6">
@@ -3955,10 +4181,10 @@
         <v>121</v>
       </c>
       <c r="B117" t="s">
-        <v>258</v>
+        <v>284</v>
       </c>
       <c r="C117" t="s">
-        <v>281</v>
+        <v>332</v>
       </c>
       <c r="D117">
         <v>1</v>
@@ -3967,7 +4193,7 @@
         <v>1</v>
       </c>
       <c r="F117" t="s">
-        <v>392</v>
+        <v>443</v>
       </c>
     </row>
     <row r="118" spans="1:6">
@@ -3975,10 +4201,10 @@
         <v>122</v>
       </c>
       <c r="B118" t="s">
-        <v>259</v>
+        <v>285</v>
       </c>
       <c r="C118" t="s">
-        <v>281</v>
+        <v>332</v>
       </c>
       <c r="D118">
         <v>1</v>
@@ -3987,7 +4213,7 @@
         <v>1</v>
       </c>
       <c r="F118" t="s">
-        <v>393</v>
+        <v>444</v>
       </c>
     </row>
     <row r="119" spans="1:6">
@@ -3995,10 +4221,10 @@
         <v>123</v>
       </c>
       <c r="B119" t="s">
-        <v>260</v>
+        <v>286</v>
       </c>
       <c r="C119" t="s">
-        <v>281</v>
+        <v>332</v>
       </c>
       <c r="D119">
         <v>1</v>
@@ -4007,7 +4233,7 @@
         <v>1</v>
       </c>
       <c r="F119" t="s">
-        <v>394</v>
+        <v>445</v>
       </c>
     </row>
     <row r="120" spans="1:6">
@@ -4015,10 +4241,10 @@
         <v>124</v>
       </c>
       <c r="B120" t="s">
-        <v>261</v>
+        <v>287</v>
       </c>
       <c r="C120" t="s">
-        <v>280</v>
+        <v>332</v>
       </c>
       <c r="D120">
         <v>1</v>
@@ -4027,7 +4253,7 @@
         <v>1</v>
       </c>
       <c r="F120" t="s">
-        <v>316</v>
+        <v>446</v>
       </c>
     </row>
     <row r="121" spans="1:6">
@@ -4035,10 +4261,10 @@
         <v>125</v>
       </c>
       <c r="B121" t="s">
-        <v>262</v>
+        <v>288</v>
       </c>
       <c r="C121" t="s">
-        <v>280</v>
+        <v>333</v>
       </c>
       <c r="D121">
         <v>1</v>
@@ -4047,7 +4273,7 @@
         <v>1</v>
       </c>
       <c r="F121" t="s">
-        <v>395</v>
+        <v>447</v>
       </c>
     </row>
     <row r="122" spans="1:6">
@@ -4055,10 +4281,10 @@
         <v>126</v>
       </c>
       <c r="B122" t="s">
-        <v>263</v>
+        <v>289</v>
       </c>
       <c r="C122" t="s">
-        <v>280</v>
+        <v>333</v>
       </c>
       <c r="D122">
         <v>1</v>
@@ -4067,7 +4293,7 @@
         <v>1</v>
       </c>
       <c r="F122" t="s">
-        <v>396</v>
+        <v>448</v>
       </c>
     </row>
     <row r="123" spans="1:6">
@@ -4075,10 +4301,10 @@
         <v>127</v>
       </c>
       <c r="B123" t="s">
-        <v>264</v>
+        <v>290</v>
       </c>
       <c r="C123" t="s">
-        <v>280</v>
+        <v>333</v>
       </c>
       <c r="D123">
         <v>1</v>
@@ -4087,7 +4313,7 @@
         <v>1</v>
       </c>
       <c r="F123" t="s">
-        <v>397</v>
+        <v>449</v>
       </c>
     </row>
     <row r="124" spans="1:6">
@@ -4095,10 +4321,10 @@
         <v>128</v>
       </c>
       <c r="B124" t="s">
-        <v>265</v>
+        <v>291</v>
       </c>
       <c r="C124" t="s">
-        <v>281</v>
+        <v>333</v>
       </c>
       <c r="D124">
         <v>1</v>
@@ -4107,7 +4333,7 @@
         <v>1</v>
       </c>
       <c r="F124" t="s">
-        <v>296</v>
+        <v>450</v>
       </c>
     </row>
     <row r="125" spans="1:6">
@@ -4115,10 +4341,10 @@
         <v>129</v>
       </c>
       <c r="B125" t="s">
-        <v>266</v>
+        <v>292</v>
       </c>
       <c r="C125" t="s">
-        <v>281</v>
+        <v>332</v>
       </c>
       <c r="D125">
         <v>1</v>
@@ -4127,7 +4353,7 @@
         <v>1</v>
       </c>
       <c r="F125" t="s">
-        <v>398</v>
+        <v>451</v>
       </c>
     </row>
     <row r="126" spans="1:6">
@@ -4135,10 +4361,10 @@
         <v>130</v>
       </c>
       <c r="B126" t="s">
-        <v>267</v>
+        <v>293</v>
       </c>
       <c r="C126" t="s">
-        <v>281</v>
+        <v>332</v>
       </c>
       <c r="D126">
         <v>1</v>
@@ -4147,7 +4373,7 @@
         <v>1</v>
       </c>
       <c r="F126" t="s">
-        <v>399</v>
+        <v>452</v>
       </c>
     </row>
     <row r="127" spans="1:6">
@@ -4155,10 +4381,10 @@
         <v>131</v>
       </c>
       <c r="B127" t="s">
-        <v>268</v>
+        <v>294</v>
       </c>
       <c r="C127" t="s">
-        <v>281</v>
+        <v>333</v>
       </c>
       <c r="D127">
         <v>1</v>
@@ -4167,7 +4393,7 @@
         <v>1</v>
       </c>
       <c r="F127" t="s">
-        <v>400</v>
+        <v>453</v>
       </c>
     </row>
     <row r="128" spans="1:6">
@@ -4175,10 +4401,10 @@
         <v>132</v>
       </c>
       <c r="B128" t="s">
-        <v>269</v>
+        <v>295</v>
       </c>
       <c r="C128" t="s">
-        <v>280</v>
+        <v>333</v>
       </c>
       <c r="D128">
         <v>1</v>
@@ -4187,7 +4413,7 @@
         <v>1</v>
       </c>
       <c r="F128" t="s">
-        <v>401</v>
+        <v>454</v>
       </c>
     </row>
     <row r="129" spans="1:6">
@@ -4195,10 +4421,10 @@
         <v>133</v>
       </c>
       <c r="B129" t="s">
-        <v>270</v>
+        <v>296</v>
       </c>
       <c r="C129" t="s">
-        <v>281</v>
+        <v>332</v>
       </c>
       <c r="D129">
         <v>1</v>
@@ -4207,7 +4433,7 @@
         <v>1</v>
       </c>
       <c r="F129" t="s">
-        <v>402</v>
+        <v>447</v>
       </c>
     </row>
     <row r="130" spans="1:6">
@@ -4215,10 +4441,10 @@
         <v>134</v>
       </c>
       <c r="B130" t="s">
-        <v>271</v>
+        <v>297</v>
       </c>
       <c r="C130" t="s">
-        <v>281</v>
+        <v>332</v>
       </c>
       <c r="D130">
         <v>1</v>
@@ -4227,7 +4453,7 @@
         <v>1</v>
       </c>
       <c r="F130" t="s">
-        <v>403</v>
+        <v>455</v>
       </c>
     </row>
     <row r="131" spans="1:6">
@@ -4235,10 +4461,10 @@
         <v>135</v>
       </c>
       <c r="B131" t="s">
-        <v>272</v>
+        <v>298</v>
       </c>
       <c r="C131" t="s">
-        <v>281</v>
+        <v>332</v>
       </c>
       <c r="D131">
         <v>1</v>
@@ -4247,7 +4473,7 @@
         <v>1</v>
       </c>
       <c r="F131" t="s">
-        <v>404</v>
+        <v>456</v>
       </c>
     </row>
     <row r="132" spans="1:6">
@@ -4255,10 +4481,10 @@
         <v>136</v>
       </c>
       <c r="B132" t="s">
-        <v>273</v>
+        <v>299</v>
       </c>
       <c r="C132" t="s">
-        <v>281</v>
+        <v>333</v>
       </c>
       <c r="D132">
         <v>1</v>
@@ -4267,7 +4493,7 @@
         <v>1</v>
       </c>
       <c r="F132" t="s">
-        <v>405</v>
+        <v>457</v>
       </c>
     </row>
     <row r="133" spans="1:6">
@@ -4275,10 +4501,10 @@
         <v>137</v>
       </c>
       <c r="B133" t="s">
-        <v>274</v>
+        <v>300</v>
       </c>
       <c r="C133" t="s">
-        <v>281</v>
+        <v>332</v>
       </c>
       <c r="D133">
         <v>1</v>
@@ -4287,7 +4513,7 @@
         <v>1</v>
       </c>
       <c r="F133" t="s">
-        <v>406</v>
+        <v>458</v>
       </c>
     </row>
     <row r="134" spans="1:6">
@@ -4295,10 +4521,10 @@
         <v>138</v>
       </c>
       <c r="B134" t="s">
-        <v>275</v>
+        <v>301</v>
       </c>
       <c r="C134" t="s">
-        <v>280</v>
+        <v>333</v>
       </c>
       <c r="D134">
         <v>1</v>
@@ -4307,7 +4533,7 @@
         <v>1</v>
       </c>
       <c r="F134" t="s">
-        <v>407</v>
+        <v>459</v>
       </c>
     </row>
     <row r="135" spans="1:6">
@@ -4315,10 +4541,10 @@
         <v>139</v>
       </c>
       <c r="B135" t="s">
-        <v>276</v>
+        <v>302</v>
       </c>
       <c r="C135" t="s">
-        <v>281</v>
+        <v>332</v>
       </c>
       <c r="D135">
         <v>1</v>
@@ -4327,7 +4553,7 @@
         <v>1</v>
       </c>
       <c r="F135" t="s">
-        <v>408</v>
+        <v>397</v>
       </c>
     </row>
     <row r="136" spans="1:6">
@@ -4335,10 +4561,10 @@
         <v>140</v>
       </c>
       <c r="B136" t="s">
-        <v>277</v>
+        <v>303</v>
       </c>
       <c r="C136" t="s">
-        <v>281</v>
+        <v>333</v>
       </c>
       <c r="D136">
         <v>1</v>
@@ -4347,7 +4573,7 @@
         <v>1</v>
       </c>
       <c r="F136" t="s">
-        <v>409</v>
+        <v>460</v>
       </c>
     </row>
     <row r="137" spans="1:6">
@@ -4355,10 +4581,10 @@
         <v>141</v>
       </c>
       <c r="B137" t="s">
-        <v>278</v>
+        <v>304</v>
       </c>
       <c r="C137" t="s">
-        <v>281</v>
+        <v>332</v>
       </c>
       <c r="D137">
         <v>1</v>
@@ -4367,7 +4593,7 @@
         <v>1</v>
       </c>
       <c r="F137" t="s">
-        <v>410</v>
+        <v>461</v>
       </c>
     </row>
     <row r="138" spans="1:6">
@@ -4375,10 +4601,10 @@
         <v>142</v>
       </c>
       <c r="B138" t="s">
-        <v>279</v>
+        <v>305</v>
       </c>
       <c r="C138" t="s">
-        <v>280</v>
+        <v>332</v>
       </c>
       <c r="D138">
         <v>1</v>
@@ -4387,7 +4613,527 @@
         <v>1</v>
       </c>
       <c r="F138" t="s">
-        <v>411</v>
+        <v>462</v>
+      </c>
+    </row>
+    <row r="139" spans="1:6">
+      <c r="A139" t="s">
+        <v>143</v>
+      </c>
+      <c r="B139" t="s">
+        <v>306</v>
+      </c>
+      <c r="C139" t="s">
+        <v>333</v>
+      </c>
+      <c r="D139">
+        <v>1</v>
+      </c>
+      <c r="E139">
+        <v>1</v>
+      </c>
+      <c r="F139" t="s">
+        <v>463</v>
+      </c>
+    </row>
+    <row r="140" spans="1:6">
+      <c r="A140" t="s">
+        <v>144</v>
+      </c>
+      <c r="B140" t="s">
+        <v>307</v>
+      </c>
+      <c r="C140" t="s">
+        <v>332</v>
+      </c>
+      <c r="D140">
+        <v>1</v>
+      </c>
+      <c r="E140">
+        <v>1</v>
+      </c>
+      <c r="F140" t="s">
+        <v>464</v>
+      </c>
+    </row>
+    <row r="141" spans="1:6">
+      <c r="A141" t="s">
+        <v>145</v>
+      </c>
+      <c r="B141" t="s">
+        <v>308</v>
+      </c>
+      <c r="C141" t="s">
+        <v>332</v>
+      </c>
+      <c r="D141">
+        <v>1</v>
+      </c>
+      <c r="E141">
+        <v>1</v>
+      </c>
+      <c r="F141" t="s">
+        <v>441</v>
+      </c>
+    </row>
+    <row r="142" spans="1:6">
+      <c r="A142" t="s">
+        <v>146</v>
+      </c>
+      <c r="B142" t="s">
+        <v>309</v>
+      </c>
+      <c r="C142" t="s">
+        <v>333</v>
+      </c>
+      <c r="D142">
+        <v>1</v>
+      </c>
+      <c r="E142">
+        <v>1</v>
+      </c>
+      <c r="F142" t="s">
+        <v>465</v>
+      </c>
+    </row>
+    <row r="143" spans="1:6">
+      <c r="A143" t="s">
+        <v>147</v>
+      </c>
+      <c r="B143" t="s">
+        <v>310</v>
+      </c>
+      <c r="C143" t="s">
+        <v>333</v>
+      </c>
+      <c r="D143">
+        <v>1</v>
+      </c>
+      <c r="E143">
+        <v>1</v>
+      </c>
+      <c r="F143" t="s">
+        <v>466</v>
+      </c>
+    </row>
+    <row r="144" spans="1:6">
+      <c r="A144" t="s">
+        <v>148</v>
+      </c>
+      <c r="B144" t="s">
+        <v>311</v>
+      </c>
+      <c r="C144" t="s">
+        <v>333</v>
+      </c>
+      <c r="D144">
+        <v>1</v>
+      </c>
+      <c r="E144">
+        <v>1</v>
+      </c>
+      <c r="F144" t="s">
+        <v>467</v>
+      </c>
+    </row>
+    <row r="145" spans="1:6">
+      <c r="A145" t="s">
+        <v>149</v>
+      </c>
+      <c r="B145" t="s">
+        <v>312</v>
+      </c>
+      <c r="C145" t="s">
+        <v>333</v>
+      </c>
+      <c r="D145">
+        <v>1</v>
+      </c>
+      <c r="E145">
+        <v>1</v>
+      </c>
+      <c r="F145" t="s">
+        <v>468</v>
+      </c>
+    </row>
+    <row r="146" spans="1:6">
+      <c r="A146" t="s">
+        <v>150</v>
+      </c>
+      <c r="B146" t="s">
+        <v>313</v>
+      </c>
+      <c r="C146" t="s">
+        <v>332</v>
+      </c>
+      <c r="D146">
+        <v>1</v>
+      </c>
+      <c r="E146">
+        <v>1</v>
+      </c>
+      <c r="F146" t="s">
+        <v>371</v>
+      </c>
+    </row>
+    <row r="147" spans="1:6">
+      <c r="A147" t="s">
+        <v>151</v>
+      </c>
+      <c r="B147" t="s">
+        <v>314</v>
+      </c>
+      <c r="C147" t="s">
+        <v>332</v>
+      </c>
+      <c r="D147">
+        <v>1</v>
+      </c>
+      <c r="E147">
+        <v>1</v>
+      </c>
+      <c r="F147" t="s">
+        <v>469</v>
+      </c>
+    </row>
+    <row r="148" spans="1:6">
+      <c r="A148" t="s">
+        <v>152</v>
+      </c>
+      <c r="B148" t="s">
+        <v>315</v>
+      </c>
+      <c r="C148" t="s">
+        <v>332</v>
+      </c>
+      <c r="D148">
+        <v>1</v>
+      </c>
+      <c r="E148">
+        <v>1</v>
+      </c>
+      <c r="F148" t="s">
+        <v>470</v>
+      </c>
+    </row>
+    <row r="149" spans="1:6">
+      <c r="A149" t="s">
+        <v>153</v>
+      </c>
+      <c r="B149" t="s">
+        <v>316</v>
+      </c>
+      <c r="C149" t="s">
+        <v>332</v>
+      </c>
+      <c r="D149">
+        <v>1</v>
+      </c>
+      <c r="E149">
+        <v>1</v>
+      </c>
+      <c r="F149" t="s">
+        <v>471</v>
+      </c>
+    </row>
+    <row r="150" spans="1:6">
+      <c r="A150" t="s">
+        <v>154</v>
+      </c>
+      <c r="B150" t="s">
+        <v>317</v>
+      </c>
+      <c r="C150" t="s">
+        <v>333</v>
+      </c>
+      <c r="D150">
+        <v>1</v>
+      </c>
+      <c r="E150">
+        <v>1</v>
+      </c>
+      <c r="F150" t="s">
+        <v>348</v>
+      </c>
+    </row>
+    <row r="151" spans="1:6">
+      <c r="A151" t="s">
+        <v>155</v>
+      </c>
+      <c r="B151" t="s">
+        <v>318</v>
+      </c>
+      <c r="C151" t="s">
+        <v>333</v>
+      </c>
+      <c r="D151">
+        <v>1</v>
+      </c>
+      <c r="E151">
+        <v>1</v>
+      </c>
+      <c r="F151" t="s">
+        <v>472</v>
+      </c>
+    </row>
+    <row r="152" spans="1:6">
+      <c r="A152" t="s">
+        <v>156</v>
+      </c>
+      <c r="B152" t="s">
+        <v>319</v>
+      </c>
+      <c r="C152" t="s">
+        <v>333</v>
+      </c>
+      <c r="D152">
+        <v>1</v>
+      </c>
+      <c r="E152">
+        <v>1</v>
+      </c>
+      <c r="F152" t="s">
+        <v>473</v>
+      </c>
+    </row>
+    <row r="153" spans="1:6">
+      <c r="A153" t="s">
+        <v>157</v>
+      </c>
+      <c r="B153" t="s">
+        <v>320</v>
+      </c>
+      <c r="C153" t="s">
+        <v>333</v>
+      </c>
+      <c r="D153">
+        <v>1</v>
+      </c>
+      <c r="E153">
+        <v>1</v>
+      </c>
+      <c r="F153" t="s">
+        <v>474</v>
+      </c>
+    </row>
+    <row r="154" spans="1:6">
+      <c r="A154" t="s">
+        <v>158</v>
+      </c>
+      <c r="B154" t="s">
+        <v>321</v>
+      </c>
+      <c r="C154" t="s">
+        <v>332</v>
+      </c>
+      <c r="D154">
+        <v>1</v>
+      </c>
+      <c r="E154">
+        <v>1</v>
+      </c>
+      <c r="F154" t="s">
+        <v>475</v>
+      </c>
+    </row>
+    <row r="155" spans="1:6">
+      <c r="A155" t="s">
+        <v>159</v>
+      </c>
+      <c r="B155" t="s">
+        <v>322</v>
+      </c>
+      <c r="C155" t="s">
+        <v>333</v>
+      </c>
+      <c r="D155">
+        <v>1</v>
+      </c>
+      <c r="E155">
+        <v>1</v>
+      </c>
+      <c r="F155" t="s">
+        <v>476</v>
+      </c>
+    </row>
+    <row r="156" spans="1:6">
+      <c r="A156" t="s">
+        <v>160</v>
+      </c>
+      <c r="B156" t="s">
+        <v>323</v>
+      </c>
+      <c r="C156" t="s">
+        <v>333</v>
+      </c>
+      <c r="D156">
+        <v>1</v>
+      </c>
+      <c r="E156">
+        <v>1</v>
+      </c>
+      <c r="F156" t="s">
+        <v>477</v>
+      </c>
+    </row>
+    <row r="157" spans="1:6">
+      <c r="A157" t="s">
+        <v>161</v>
+      </c>
+      <c r="B157" t="s">
+        <v>324</v>
+      </c>
+      <c r="C157" t="s">
+        <v>333</v>
+      </c>
+      <c r="D157">
+        <v>1</v>
+      </c>
+      <c r="E157">
+        <v>1</v>
+      </c>
+      <c r="F157" t="s">
+        <v>478</v>
+      </c>
+    </row>
+    <row r="158" spans="1:6">
+      <c r="A158" t="s">
+        <v>162</v>
+      </c>
+      <c r="B158" t="s">
+        <v>325</v>
+      </c>
+      <c r="C158" t="s">
+        <v>333</v>
+      </c>
+      <c r="D158">
+        <v>1</v>
+      </c>
+      <c r="E158">
+        <v>1</v>
+      </c>
+      <c r="F158" t="s">
+        <v>479</v>
+      </c>
+    </row>
+    <row r="159" spans="1:6">
+      <c r="A159" t="s">
+        <v>163</v>
+      </c>
+      <c r="B159" t="s">
+        <v>326</v>
+      </c>
+      <c r="C159" t="s">
+        <v>333</v>
+      </c>
+      <c r="D159">
+        <v>1</v>
+      </c>
+      <c r="E159">
+        <v>1</v>
+      </c>
+      <c r="F159" t="s">
+        <v>480</v>
+      </c>
+    </row>
+    <row r="160" spans="1:6">
+      <c r="A160" t="s">
+        <v>164</v>
+      </c>
+      <c r="B160" t="s">
+        <v>327</v>
+      </c>
+      <c r="C160" t="s">
+        <v>332</v>
+      </c>
+      <c r="D160">
+        <v>1</v>
+      </c>
+      <c r="E160">
+        <v>1</v>
+      </c>
+      <c r="F160" t="s">
+        <v>481</v>
+      </c>
+    </row>
+    <row r="161" spans="1:6">
+      <c r="A161" t="s">
+        <v>165</v>
+      </c>
+      <c r="B161" t="s">
+        <v>328</v>
+      </c>
+      <c r="C161" t="s">
+        <v>333</v>
+      </c>
+      <c r="D161">
+        <v>1</v>
+      </c>
+      <c r="E161">
+        <v>1</v>
+      </c>
+      <c r="F161" t="s">
+        <v>482</v>
+      </c>
+    </row>
+    <row r="162" spans="1:6">
+      <c r="A162" t="s">
+        <v>166</v>
+      </c>
+      <c r="B162" t="s">
+        <v>329</v>
+      </c>
+      <c r="C162" t="s">
+        <v>333</v>
+      </c>
+      <c r="D162">
+        <v>1</v>
+      </c>
+      <c r="E162">
+        <v>1</v>
+      </c>
+      <c r="F162" t="s">
+        <v>483</v>
+      </c>
+    </row>
+    <row r="163" spans="1:6">
+      <c r="A163" t="s">
+        <v>167</v>
+      </c>
+      <c r="B163" t="s">
+        <v>330</v>
+      </c>
+      <c r="C163" t="s">
+        <v>333</v>
+      </c>
+      <c r="D163">
+        <v>1</v>
+      </c>
+      <c r="E163">
+        <v>1</v>
+      </c>
+      <c r="F163" t="s">
+        <v>484</v>
+      </c>
+    </row>
+    <row r="164" spans="1:6">
+      <c r="A164" t="s">
+        <v>168</v>
+      </c>
+      <c r="B164" t="s">
+        <v>331</v>
+      </c>
+      <c r="C164" t="s">
+        <v>332</v>
+      </c>
+      <c r="D164">
+        <v>1</v>
+      </c>
+      <c r="E164">
+        <v>1</v>
+      </c>
+      <c r="F164" t="s">
+        <v>485</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
feat(ai): recover laughing, soaring, glowing -ing emotion terms into clean_emotion_words_2000_reviews
</commit_message>
<xml_diff>
--- a/data/derived_outputs/clean_emotion_words_2000_reviews.xlsx
+++ b/data/derived_outputs/clean_emotion_words_2000_reviews.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="658" uniqueCount="486">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="678" uniqueCount="501">
   <si>
     <t>word</t>
   </si>
@@ -190,6 +190,9 @@
     <t>improvement</t>
   </si>
   <si>
+    <t>laughing</t>
+  </si>
+  <si>
     <t>lush</t>
   </si>
   <si>
@@ -208,6 +211,9 @@
     <t>superbly</t>
   </si>
   <si>
+    <t>wondering</t>
+  </si>
+  <si>
     <t>worthy</t>
   </si>
   <si>
@@ -262,6 +268,9 @@
     <t>happiness</t>
   </si>
   <si>
+    <t>hesitating</t>
+  </si>
+  <si>
     <t>honesty</t>
   </si>
   <si>
@@ -379,6 +388,9 @@
     <t>desperate</t>
   </si>
   <si>
+    <t>dreaming</t>
+  </si>
+  <si>
     <t>embarrassed</t>
   </si>
   <si>
@@ -394,6 +406,9 @@
     <t>frightening</t>
   </si>
   <si>
+    <t>gushing</t>
+  </si>
+  <si>
     <t>hilarious</t>
   </si>
   <si>
@@ -679,6 +694,9 @@
     <t>体验改善 / 提升</t>
   </si>
   <si>
+    <t>欢声笑语 / 开心大笑</t>
+  </si>
+  <si>
     <t>郁郁葱葱宜人的</t>
   </si>
   <si>
@@ -697,6 +715,9 @@
     <t>出类拔萃完美地</t>
   </si>
   <si>
+    <t>心生好奇 / 纳闷想知道</t>
+  </si>
+  <si>
     <t>非常值的 / 值得的</t>
   </si>
   <si>
@@ -751,6 +772,9 @@
     <t>幸福快乐感</t>
   </si>
   <si>
+    <t>犹豫顾虑（心理活动）</t>
+  </si>
+  <si>
     <t>真诚 / 诚信解说</t>
   </si>
   <si>
@@ -868,6 +892,9 @@
     <t>感到绝望迫切的</t>
   </si>
   <si>
+    <t>梦寐以求 / 心驰神往</t>
+  </si>
+  <si>
     <t>感到尴尬难堪的</t>
   </si>
   <si>
@@ -881,6 +908,9 @@
   </si>
   <si>
     <t>令人惊恐吓人的</t>
+  </si>
+  <si>
+    <t>滔滔不绝赞赞称道的</t>
   </si>
   <si>
     <t>爆笑幽默搞笑的</t>
@@ -1181,6 +1211,9 @@
 The phone reser...</t>
   </si>
   <si>
+    <t>review_297816c223f0885e99c4fc19 :: For a first timer, nothing tops a fly over the spectacular sights of this island. And AirVenture did it best thanks to their exceptional ground and air staff. Our pilot Eric, who c...</t>
+  </si>
+  <si>
     <t>review_1893bdcfa0517b11567fd56d :: I booked the Cessna tour for my wife and I on our babymoon in April. I recommend the private Cessna tour if you only have 2 people.  For only slightly more $$, you get a personal e...</t>
   </si>
   <si>
@@ -1200,6 +1233,9 @@
     <t>review_bcedc98e43ad7edec05befa8 :: There isn't much to say here, except the experience was fantastic. Seeing the landscape from the air was breathtaking, and landing and taking off from the glacier was a hoot. Our p...</t>
   </si>
   <si>
+    <t>review_81b92c127ddb88bab681a2dd :: I do not have enough words to describe all the beauty and nature we saw on this flight. We were greeted with a friendly, Aloha and given the ground rules for the flight. Bruce our ...</t>
+  </si>
+  <si>
     <t>review_d38fb233c92c34b779e4871c :: Wow - what an experience! I had the opportunity to take two separate flights - one in their Cessna and one in their incredible cherry red biplane (the only one on the island). 
 On...</t>
   </si>
@@ -1251,6 +1287,9 @@
   </si>
   <si>
     <t>review_c8c04aed9cd305332764808f :: I encouraged my husband to take the biplane flight/tour. I had no intention of going. My husband and the pilot Mark encouraged me to go along. The front seat holds two. I decided t...</t>
+  </si>
+  <si>
+    <t>review_feb2301965baf7cd372cbd1f :: It's Alyssa Jacey, the singer/songwriter you hosted on the private helicopter tour! I have been MEANING to review this and my only excuse is that I went on tour! I've opened for Br...</t>
   </si>
   <si>
     <t>review_9f9111190c4a6d851371d2f7 :: We want to express our appreciation to Chip Sonn, our K2 pilot for our fantastic late afternoon/evening flight excursion while recently visiting Talkeetna, Alaska.  As part of our ...</t>
@@ -1365,6 +1404,9 @@
     <t>review_93002c7973ba2bb5ce9edb94 :: My husband and I were desperate to take a flight over Kauai but were concerned we wouldn't be able to because of our children being so young (3yrs and 1yr). We stumbled across Wing...</t>
   </si>
   <si>
+    <t>review_66a4fcc5850ed47eb61fb160 :: Booked 4 on the Grand Denali flight. The weather was great, and the views were unbelievable. Our pilot, Sean, did a great job of making sure everyone got a good view and told us lo...</t>
+  </si>
+  <si>
     <t>review_46ddfd4445283a6a81911504 :: Booked the Grand Canyon Discovery Tour and very unimpressed with how short the flight time was (less than ten minutes total) with a short photo op stop on a ridge in the canyon.  O...</t>
   </si>
   <si>
@@ -1378,6 +1420,9 @@
   </si>
   <si>
     <t>review_ad4c129d7431549c0c82f1a8 :: Three of us signed up for the plane ride about a month in advance. There were really high winds that day (40 mph+), but the company didn't cancel so we went for the ride. 15 minute...</t>
+  </si>
+  <si>
+    <t>review_6d89a83a7e6c40e34fc3fabb :: From start to finish, our flightseeing tour from Talkeetna to Mt. McKinley, landing on Ruth Glacier was jaw-droppingly wonderful. I've lived in Alaska for almost 40 years and thoug...</t>
   </si>
   <si>
     <t>review_af9c2e4c708b6ef1ddffbdef :: We booked this as part of a Viator package to see Alcatraz and it completely blew us away.  We were a party of 4 - two adults, a ten year old and a 4 year old.  Despite a total fea...</t>
@@ -1853,7 +1898,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:F164"/>
+  <dimension ref="A1:F169"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:6">
@@ -1881,10 +1926,10 @@
         <v>6</v>
       </c>
       <c r="B2" t="s">
-        <v>169</v>
+        <v>174</v>
       </c>
       <c r="C2" t="s">
-        <v>332</v>
+        <v>342</v>
       </c>
       <c r="D2">
         <v>12</v>
@@ -1893,7 +1938,7 @@
         <v>12</v>
       </c>
       <c r="F2" t="s">
-        <v>335</v>
+        <v>345</v>
       </c>
     </row>
     <row r="3" spans="1:6">
@@ -1901,10 +1946,10 @@
         <v>7</v>
       </c>
       <c r="B3" t="s">
-        <v>170</v>
+        <v>175</v>
       </c>
       <c r="C3" t="s">
-        <v>333</v>
+        <v>343</v>
       </c>
       <c r="D3">
         <v>10</v>
@@ -1913,7 +1958,7 @@
         <v>10</v>
       </c>
       <c r="F3" t="s">
-        <v>336</v>
+        <v>346</v>
       </c>
     </row>
     <row r="4" spans="1:6">
@@ -1921,10 +1966,10 @@
         <v>8</v>
       </c>
       <c r="B4" t="s">
-        <v>171</v>
+        <v>176</v>
       </c>
       <c r="C4" t="s">
-        <v>333</v>
+        <v>343</v>
       </c>
       <c r="D4">
         <v>10</v>
@@ -1933,7 +1978,7 @@
         <v>9</v>
       </c>
       <c r="F4" t="s">
-        <v>337</v>
+        <v>347</v>
       </c>
     </row>
     <row r="5" spans="1:6">
@@ -1941,10 +1986,10 @@
         <v>9</v>
       </c>
       <c r="B5" t="s">
-        <v>172</v>
+        <v>177</v>
       </c>
       <c r="C5" t="s">
-        <v>333</v>
+        <v>343</v>
       </c>
       <c r="D5">
         <v>9</v>
@@ -1953,7 +1998,7 @@
         <v>9</v>
       </c>
       <c r="F5" t="s">
-        <v>338</v>
+        <v>348</v>
       </c>
     </row>
     <row r="6" spans="1:6">
@@ -1961,10 +2006,10 @@
         <v>10</v>
       </c>
       <c r="B6" t="s">
-        <v>173</v>
+        <v>178</v>
       </c>
       <c r="C6" t="s">
-        <v>333</v>
+        <v>343</v>
       </c>
       <c r="D6">
         <v>9</v>
@@ -1973,7 +2018,7 @@
         <v>9</v>
       </c>
       <c r="F6" t="s">
-        <v>339</v>
+        <v>349</v>
       </c>
     </row>
     <row r="7" spans="1:6">
@@ -1981,10 +2026,10 @@
         <v>11</v>
       </c>
       <c r="B7" t="s">
-        <v>174</v>
+        <v>179</v>
       </c>
       <c r="C7" t="s">
-        <v>333</v>
+        <v>343</v>
       </c>
       <c r="D7">
         <v>9</v>
@@ -1993,7 +2038,7 @@
         <v>9</v>
       </c>
       <c r="F7" t="s">
-        <v>340</v>
+        <v>350</v>
       </c>
     </row>
     <row r="8" spans="1:6">
@@ -2001,10 +2046,10 @@
         <v>12</v>
       </c>
       <c r="B8" t="s">
-        <v>175</v>
+        <v>180</v>
       </c>
       <c r="C8" t="s">
-        <v>333</v>
+        <v>343</v>
       </c>
       <c r="D8">
         <v>8</v>
@@ -2013,7 +2058,7 @@
         <v>8</v>
       </c>
       <c r="F8" t="s">
-        <v>341</v>
+        <v>351</v>
       </c>
     </row>
     <row r="9" spans="1:6">
@@ -2021,10 +2066,10 @@
         <v>13</v>
       </c>
       <c r="B9" t="s">
-        <v>176</v>
+        <v>181</v>
       </c>
       <c r="C9" t="s">
-        <v>332</v>
+        <v>342</v>
       </c>
       <c r="D9">
         <v>8</v>
@@ -2033,7 +2078,7 @@
         <v>8</v>
       </c>
       <c r="F9" t="s">
-        <v>342</v>
+        <v>352</v>
       </c>
     </row>
     <row r="10" spans="1:6">
@@ -2041,10 +2086,10 @@
         <v>14</v>
       </c>
       <c r="B10" t="s">
-        <v>177</v>
+        <v>182</v>
       </c>
       <c r="C10" t="s">
-        <v>332</v>
+        <v>342</v>
       </c>
       <c r="D10">
         <v>7</v>
@@ -2053,7 +2098,7 @@
         <v>7</v>
       </c>
       <c r="F10" t="s">
-        <v>343</v>
+        <v>353</v>
       </c>
     </row>
     <row r="11" spans="1:6">
@@ -2061,10 +2106,10 @@
         <v>15</v>
       </c>
       <c r="B11" t="s">
-        <v>178</v>
+        <v>183</v>
       </c>
       <c r="C11" t="s">
-        <v>333</v>
+        <v>343</v>
       </c>
       <c r="D11">
         <v>7</v>
@@ -2073,7 +2118,7 @@
         <v>7</v>
       </c>
       <c r="F11" t="s">
-        <v>344</v>
+        <v>354</v>
       </c>
     </row>
     <row r="12" spans="1:6">
@@ -2081,10 +2126,10 @@
         <v>16</v>
       </c>
       <c r="B12" t="s">
-        <v>179</v>
+        <v>184</v>
       </c>
       <c r="C12" t="s">
-        <v>333</v>
+        <v>343</v>
       </c>
       <c r="D12">
         <v>7</v>
@@ -2093,7 +2138,7 @@
         <v>7</v>
       </c>
       <c r="F12" t="s">
-        <v>345</v>
+        <v>355</v>
       </c>
     </row>
     <row r="13" spans="1:6">
@@ -2101,10 +2146,10 @@
         <v>17</v>
       </c>
       <c r="B13" t="s">
-        <v>180</v>
+        <v>185</v>
       </c>
       <c r="C13" t="s">
-        <v>333</v>
+        <v>343</v>
       </c>
       <c r="D13">
         <v>7</v>
@@ -2113,7 +2158,7 @@
         <v>7</v>
       </c>
       <c r="F13" t="s">
-        <v>346</v>
+        <v>356</v>
       </c>
     </row>
     <row r="14" spans="1:6">
@@ -2121,10 +2166,10 @@
         <v>18</v>
       </c>
       <c r="B14" t="s">
-        <v>181</v>
+        <v>186</v>
       </c>
       <c r="C14" t="s">
-        <v>333</v>
+        <v>343</v>
       </c>
       <c r="D14">
         <v>7</v>
@@ -2133,7 +2178,7 @@
         <v>6</v>
       </c>
       <c r="F14" t="s">
-        <v>347</v>
+        <v>357</v>
       </c>
     </row>
     <row r="15" spans="1:6">
@@ -2141,10 +2186,10 @@
         <v>19</v>
       </c>
       <c r="B15" t="s">
-        <v>182</v>
+        <v>187</v>
       </c>
       <c r="C15" t="s">
-        <v>333</v>
+        <v>343</v>
       </c>
       <c r="D15">
         <v>7</v>
@@ -2153,7 +2198,7 @@
         <v>7</v>
       </c>
       <c r="F15" t="s">
-        <v>338</v>
+        <v>348</v>
       </c>
     </row>
     <row r="16" spans="1:6">
@@ -2161,10 +2206,10 @@
         <v>20</v>
       </c>
       <c r="B16" t="s">
-        <v>183</v>
+        <v>188</v>
       </c>
       <c r="C16" t="s">
-        <v>333</v>
+        <v>343</v>
       </c>
       <c r="D16">
         <v>6</v>
@@ -2173,7 +2218,7 @@
         <v>6</v>
       </c>
       <c r="F16" t="s">
-        <v>348</v>
+        <v>358</v>
       </c>
     </row>
     <row r="17" spans="1:6">
@@ -2181,10 +2226,10 @@
         <v>21</v>
       </c>
       <c r="B17" t="s">
-        <v>184</v>
+        <v>189</v>
       </c>
       <c r="C17" t="s">
-        <v>332</v>
+        <v>342</v>
       </c>
       <c r="D17">
         <v>6</v>
@@ -2193,7 +2238,7 @@
         <v>6</v>
       </c>
       <c r="F17" t="s">
-        <v>349</v>
+        <v>359</v>
       </c>
     </row>
     <row r="18" spans="1:6">
@@ -2201,10 +2246,10 @@
         <v>22</v>
       </c>
       <c r="B18" t="s">
-        <v>185</v>
+        <v>190</v>
       </c>
       <c r="C18" t="s">
-        <v>333</v>
+        <v>343</v>
       </c>
       <c r="D18">
         <v>6</v>
@@ -2213,7 +2258,7 @@
         <v>6</v>
       </c>
       <c r="F18" t="s">
-        <v>350</v>
+        <v>360</v>
       </c>
     </row>
     <row r="19" spans="1:6">
@@ -2221,10 +2266,10 @@
         <v>23</v>
       </c>
       <c r="B19" t="s">
-        <v>186</v>
+        <v>191</v>
       </c>
       <c r="C19" t="s">
-        <v>333</v>
+        <v>343</v>
       </c>
       <c r="D19">
         <v>6</v>
@@ -2233,7 +2278,7 @@
         <v>5</v>
       </c>
       <c r="F19" t="s">
-        <v>351</v>
+        <v>361</v>
       </c>
     </row>
     <row r="20" spans="1:6">
@@ -2241,10 +2286,10 @@
         <v>24</v>
       </c>
       <c r="B20" t="s">
-        <v>187</v>
+        <v>192</v>
       </c>
       <c r="C20" t="s">
-        <v>332</v>
+        <v>342</v>
       </c>
       <c r="D20">
         <v>6</v>
@@ -2253,7 +2298,7 @@
         <v>6</v>
       </c>
       <c r="F20" t="s">
-        <v>352</v>
+        <v>362</v>
       </c>
     </row>
     <row r="21" spans="1:6">
@@ -2261,10 +2306,10 @@
         <v>25</v>
       </c>
       <c r="B21" t="s">
-        <v>188</v>
+        <v>193</v>
       </c>
       <c r="C21" t="s">
-        <v>332</v>
+        <v>342</v>
       </c>
       <c r="D21">
         <v>6</v>
@@ -2273,7 +2318,7 @@
         <v>5</v>
       </c>
       <c r="F21" t="s">
-        <v>353</v>
+        <v>363</v>
       </c>
     </row>
     <row r="22" spans="1:6">
@@ -2281,10 +2326,10 @@
         <v>26</v>
       </c>
       <c r="B22" t="s">
-        <v>189</v>
+        <v>194</v>
       </c>
       <c r="C22" t="s">
-        <v>332</v>
+        <v>342</v>
       </c>
       <c r="D22">
         <v>6</v>
@@ -2293,7 +2338,7 @@
         <v>6</v>
       </c>
       <c r="F22" t="s">
-        <v>354</v>
+        <v>364</v>
       </c>
     </row>
     <row r="23" spans="1:6">
@@ -2301,10 +2346,10 @@
         <v>27</v>
       </c>
       <c r="B23" t="s">
-        <v>190</v>
+        <v>195</v>
       </c>
       <c r="C23" t="s">
-        <v>332</v>
+        <v>342</v>
       </c>
       <c r="D23">
         <v>6</v>
@@ -2313,7 +2358,7 @@
         <v>6</v>
       </c>
       <c r="F23" t="s">
-        <v>355</v>
+        <v>365</v>
       </c>
     </row>
     <row r="24" spans="1:6">
@@ -2321,10 +2366,10 @@
         <v>28</v>
       </c>
       <c r="B24" t="s">
-        <v>191</v>
+        <v>196</v>
       </c>
       <c r="C24" t="s">
-        <v>333</v>
+        <v>343</v>
       </c>
       <c r="D24">
         <v>6</v>
@@ -2333,7 +2378,7 @@
         <v>6</v>
       </c>
       <c r="F24" t="s">
-        <v>356</v>
+        <v>366</v>
       </c>
     </row>
     <row r="25" spans="1:6">
@@ -2341,10 +2386,10 @@
         <v>29</v>
       </c>
       <c r="B25" t="s">
-        <v>192</v>
+        <v>197</v>
       </c>
       <c r="C25" t="s">
-        <v>332</v>
+        <v>342</v>
       </c>
       <c r="D25">
         <v>5</v>
@@ -2353,7 +2398,7 @@
         <v>5</v>
       </c>
       <c r="F25" t="s">
-        <v>357</v>
+        <v>367</v>
       </c>
     </row>
     <row r="26" spans="1:6">
@@ -2361,10 +2406,10 @@
         <v>30</v>
       </c>
       <c r="B26" t="s">
-        <v>193</v>
+        <v>198</v>
       </c>
       <c r="C26" t="s">
-        <v>333</v>
+        <v>343</v>
       </c>
       <c r="D26">
         <v>5</v>
@@ -2373,7 +2418,7 @@
         <v>5</v>
       </c>
       <c r="F26" t="s">
-        <v>358</v>
+        <v>368</v>
       </c>
     </row>
     <row r="27" spans="1:6">
@@ -2381,10 +2426,10 @@
         <v>31</v>
       </c>
       <c r="B27" t="s">
-        <v>194</v>
+        <v>199</v>
       </c>
       <c r="C27" t="s">
-        <v>333</v>
+        <v>343</v>
       </c>
       <c r="D27">
         <v>5</v>
@@ -2393,7 +2438,7 @@
         <v>4</v>
       </c>
       <c r="F27" t="s">
-        <v>359</v>
+        <v>369</v>
       </c>
     </row>
     <row r="28" spans="1:6">
@@ -2401,10 +2446,10 @@
         <v>32</v>
       </c>
       <c r="B28" t="s">
-        <v>195</v>
+        <v>200</v>
       </c>
       <c r="C28" t="s">
-        <v>333</v>
+        <v>343</v>
       </c>
       <c r="D28">
         <v>5</v>
@@ -2413,7 +2458,7 @@
         <v>5</v>
       </c>
       <c r="F28" t="s">
-        <v>360</v>
+        <v>370</v>
       </c>
     </row>
     <row r="29" spans="1:6">
@@ -2421,10 +2466,10 @@
         <v>33</v>
       </c>
       <c r="B29" t="s">
-        <v>196</v>
+        <v>201</v>
       </c>
       <c r="C29" t="s">
-        <v>332</v>
+        <v>342</v>
       </c>
       <c r="D29">
         <v>5</v>
@@ -2433,7 +2478,7 @@
         <v>5</v>
       </c>
       <c r="F29" t="s">
-        <v>361</v>
+        <v>371</v>
       </c>
     </row>
     <row r="30" spans="1:6">
@@ -2441,10 +2486,10 @@
         <v>34</v>
       </c>
       <c r="B30" t="s">
-        <v>197</v>
+        <v>202</v>
       </c>
       <c r="C30" t="s">
-        <v>333</v>
+        <v>343</v>
       </c>
       <c r="D30">
         <v>5</v>
@@ -2453,7 +2498,7 @@
         <v>5</v>
       </c>
       <c r="F30" t="s">
-        <v>362</v>
+        <v>372</v>
       </c>
     </row>
     <row r="31" spans="1:6">
@@ -2461,10 +2506,10 @@
         <v>35</v>
       </c>
       <c r="B31" t="s">
-        <v>198</v>
+        <v>203</v>
       </c>
       <c r="C31" t="s">
-        <v>333</v>
+        <v>343</v>
       </c>
       <c r="D31">
         <v>5</v>
@@ -2473,7 +2518,7 @@
         <v>4</v>
       </c>
       <c r="F31" t="s">
-        <v>363</v>
+        <v>373</v>
       </c>
     </row>
     <row r="32" spans="1:6">
@@ -2481,10 +2526,10 @@
         <v>36</v>
       </c>
       <c r="B32" t="s">
-        <v>199</v>
+        <v>204</v>
       </c>
       <c r="C32" t="s">
-        <v>333</v>
+        <v>343</v>
       </c>
       <c r="D32">
         <v>5</v>
@@ -2493,7 +2538,7 @@
         <v>5</v>
       </c>
       <c r="F32" t="s">
-        <v>364</v>
+        <v>374</v>
       </c>
     </row>
     <row r="33" spans="1:6">
@@ -2501,10 +2546,10 @@
         <v>37</v>
       </c>
       <c r="B33" t="s">
-        <v>200</v>
+        <v>205</v>
       </c>
       <c r="C33" t="s">
-        <v>332</v>
+        <v>342</v>
       </c>
       <c r="D33">
         <v>5</v>
@@ -2513,7 +2558,7 @@
         <v>5</v>
       </c>
       <c r="F33" t="s">
-        <v>365</v>
+        <v>375</v>
       </c>
     </row>
     <row r="34" spans="1:6">
@@ -2521,10 +2566,10 @@
         <v>38</v>
       </c>
       <c r="B34" t="s">
-        <v>201</v>
+        <v>206</v>
       </c>
       <c r="C34" t="s">
-        <v>333</v>
+        <v>343</v>
       </c>
       <c r="D34">
         <v>4</v>
@@ -2533,7 +2578,7 @@
         <v>4</v>
       </c>
       <c r="F34" t="s">
-        <v>366</v>
+        <v>376</v>
       </c>
     </row>
     <row r="35" spans="1:6">
@@ -2541,10 +2586,10 @@
         <v>39</v>
       </c>
       <c r="B35" t="s">
-        <v>202</v>
+        <v>207</v>
       </c>
       <c r="C35" t="s">
-        <v>332</v>
+        <v>342</v>
       </c>
       <c r="D35">
         <v>4</v>
@@ -2553,7 +2598,7 @@
         <v>4</v>
       </c>
       <c r="F35" t="s">
-        <v>367</v>
+        <v>377</v>
       </c>
     </row>
     <row r="36" spans="1:6">
@@ -2561,10 +2606,10 @@
         <v>40</v>
       </c>
       <c r="B36" t="s">
-        <v>203</v>
+        <v>208</v>
       </c>
       <c r="C36" t="s">
-        <v>332</v>
+        <v>342</v>
       </c>
       <c r="D36">
         <v>4</v>
@@ -2573,7 +2618,7 @@
         <v>4</v>
       </c>
       <c r="F36" t="s">
-        <v>368</v>
+        <v>378</v>
       </c>
     </row>
     <row r="37" spans="1:6">
@@ -2581,10 +2626,10 @@
         <v>41</v>
       </c>
       <c r="B37" t="s">
-        <v>204</v>
+        <v>209</v>
       </c>
       <c r="C37" t="s">
-        <v>332</v>
+        <v>342</v>
       </c>
       <c r="D37">
         <v>4</v>
@@ -2593,7 +2638,7 @@
         <v>4</v>
       </c>
       <c r="F37" t="s">
-        <v>369</v>
+        <v>379</v>
       </c>
     </row>
     <row r="38" spans="1:6">
@@ -2601,10 +2646,10 @@
         <v>42</v>
       </c>
       <c r="B38" t="s">
-        <v>205</v>
+        <v>210</v>
       </c>
       <c r="C38" t="s">
-        <v>332</v>
+        <v>342</v>
       </c>
       <c r="D38">
         <v>4</v>
@@ -2613,7 +2658,7 @@
         <v>3</v>
       </c>
       <c r="F38" t="s">
-        <v>370</v>
+        <v>380</v>
       </c>
     </row>
     <row r="39" spans="1:6">
@@ -2621,10 +2666,10 @@
         <v>43</v>
       </c>
       <c r="B39" t="s">
-        <v>206</v>
+        <v>211</v>
       </c>
       <c r="C39" t="s">
-        <v>332</v>
+        <v>342</v>
       </c>
       <c r="D39">
         <v>4</v>
@@ -2633,7 +2678,7 @@
         <v>4</v>
       </c>
       <c r="F39" t="s">
-        <v>371</v>
+        <v>381</v>
       </c>
     </row>
     <row r="40" spans="1:6">
@@ -2641,10 +2686,10 @@
         <v>44</v>
       </c>
       <c r="B40" t="s">
-        <v>207</v>
+        <v>212</v>
       </c>
       <c r="C40" t="s">
-        <v>332</v>
+        <v>342</v>
       </c>
       <c r="D40">
         <v>4</v>
@@ -2653,7 +2698,7 @@
         <v>4</v>
       </c>
       <c r="F40" t="s">
-        <v>372</v>
+        <v>382</v>
       </c>
     </row>
     <row r="41" spans="1:6">
@@ -2661,10 +2706,10 @@
         <v>45</v>
       </c>
       <c r="B41" t="s">
-        <v>208</v>
+        <v>213</v>
       </c>
       <c r="C41" t="s">
-        <v>332</v>
+        <v>342</v>
       </c>
       <c r="D41">
         <v>4</v>
@@ -2673,7 +2718,7 @@
         <v>4</v>
       </c>
       <c r="F41" t="s">
-        <v>373</v>
+        <v>383</v>
       </c>
     </row>
     <row r="42" spans="1:6">
@@ -2681,10 +2726,10 @@
         <v>46</v>
       </c>
       <c r="B42" t="s">
-        <v>209</v>
+        <v>214</v>
       </c>
       <c r="C42" t="s">
-        <v>333</v>
+        <v>343</v>
       </c>
       <c r="D42">
         <v>4</v>
@@ -2693,7 +2738,7 @@
         <v>4</v>
       </c>
       <c r="F42" t="s">
-        <v>374</v>
+        <v>384</v>
       </c>
     </row>
     <row r="43" spans="1:6">
@@ -2701,10 +2746,10 @@
         <v>47</v>
       </c>
       <c r="B43" t="s">
-        <v>210</v>
+        <v>215</v>
       </c>
       <c r="C43" t="s">
-        <v>333</v>
+        <v>343</v>
       </c>
       <c r="D43">
         <v>4</v>
@@ -2713,7 +2758,7 @@
         <v>4</v>
       </c>
       <c r="F43" t="s">
-        <v>375</v>
+        <v>385</v>
       </c>
     </row>
     <row r="44" spans="1:6">
@@ -2721,10 +2766,10 @@
         <v>48</v>
       </c>
       <c r="B44" t="s">
-        <v>211</v>
+        <v>216</v>
       </c>
       <c r="C44" t="s">
-        <v>333</v>
+        <v>343</v>
       </c>
       <c r="D44">
         <v>4</v>
@@ -2733,7 +2778,7 @@
         <v>4</v>
       </c>
       <c r="F44" t="s">
-        <v>376</v>
+        <v>386</v>
       </c>
     </row>
     <row r="45" spans="1:6">
@@ -2741,10 +2786,10 @@
         <v>49</v>
       </c>
       <c r="B45" t="s">
-        <v>212</v>
+        <v>217</v>
       </c>
       <c r="C45" t="s">
-        <v>333</v>
+        <v>343</v>
       </c>
       <c r="D45">
         <v>4</v>
@@ -2753,7 +2798,7 @@
         <v>4</v>
       </c>
       <c r="F45" t="s">
-        <v>377</v>
+        <v>387</v>
       </c>
     </row>
     <row r="46" spans="1:6">
@@ -2761,10 +2806,10 @@
         <v>50</v>
       </c>
       <c r="B46" t="s">
-        <v>213</v>
+        <v>218</v>
       </c>
       <c r="C46" t="s">
-        <v>334</v>
+        <v>344</v>
       </c>
       <c r="D46">
         <v>3</v>
@@ -2773,7 +2818,7 @@
         <v>3</v>
       </c>
       <c r="F46" t="s">
-        <v>378</v>
+        <v>388</v>
       </c>
     </row>
     <row r="47" spans="1:6">
@@ -2781,10 +2826,10 @@
         <v>51</v>
       </c>
       <c r="B47" t="s">
-        <v>214</v>
+        <v>219</v>
       </c>
       <c r="C47" t="s">
-        <v>332</v>
+        <v>342</v>
       </c>
       <c r="D47">
         <v>3</v>
@@ -2793,7 +2838,7 @@
         <v>3</v>
       </c>
       <c r="F47" t="s">
-        <v>379</v>
+        <v>389</v>
       </c>
     </row>
     <row r="48" spans="1:6">
@@ -2801,10 +2846,10 @@
         <v>52</v>
       </c>
       <c r="B48" t="s">
-        <v>215</v>
+        <v>220</v>
       </c>
       <c r="C48" t="s">
-        <v>333</v>
+        <v>343</v>
       </c>
       <c r="D48">
         <v>3</v>
@@ -2813,7 +2858,7 @@
         <v>3</v>
       </c>
       <c r="F48" t="s">
-        <v>380</v>
+        <v>390</v>
       </c>
     </row>
     <row r="49" spans="1:6">
@@ -2821,10 +2866,10 @@
         <v>53</v>
       </c>
       <c r="B49" t="s">
-        <v>216</v>
+        <v>221</v>
       </c>
       <c r="C49" t="s">
-        <v>332</v>
+        <v>342</v>
       </c>
       <c r="D49">
         <v>3</v>
@@ -2833,7 +2878,7 @@
         <v>3</v>
       </c>
       <c r="F49" t="s">
-        <v>381</v>
+        <v>391</v>
       </c>
     </row>
     <row r="50" spans="1:6">
@@ -2841,10 +2886,10 @@
         <v>54</v>
       </c>
       <c r="B50" t="s">
-        <v>217</v>
+        <v>222</v>
       </c>
       <c r="C50" t="s">
-        <v>332</v>
+        <v>342</v>
       </c>
       <c r="D50">
         <v>3</v>
@@ -2853,7 +2898,7 @@
         <v>3</v>
       </c>
       <c r="F50" t="s">
-        <v>382</v>
+        <v>392</v>
       </c>
     </row>
     <row r="51" spans="1:6">
@@ -2861,10 +2906,10 @@
         <v>55</v>
       </c>
       <c r="B51" t="s">
-        <v>218</v>
+        <v>223</v>
       </c>
       <c r="C51" t="s">
-        <v>333</v>
+        <v>343</v>
       </c>
       <c r="D51">
         <v>3</v>
@@ -2873,7 +2918,7 @@
         <v>3</v>
       </c>
       <c r="F51" t="s">
-        <v>383</v>
+        <v>393</v>
       </c>
     </row>
     <row r="52" spans="1:6">
@@ -2881,10 +2926,10 @@
         <v>56</v>
       </c>
       <c r="B52" t="s">
-        <v>219</v>
+        <v>224</v>
       </c>
       <c r="C52" t="s">
-        <v>333</v>
+        <v>343</v>
       </c>
       <c r="D52">
         <v>3</v>
@@ -2893,7 +2938,7 @@
         <v>3</v>
       </c>
       <c r="F52" t="s">
-        <v>384</v>
+        <v>394</v>
       </c>
     </row>
     <row r="53" spans="1:6">
@@ -2901,10 +2946,10 @@
         <v>57</v>
       </c>
       <c r="B53" t="s">
-        <v>220</v>
+        <v>225</v>
       </c>
       <c r="C53" t="s">
-        <v>333</v>
+        <v>343</v>
       </c>
       <c r="D53">
         <v>3</v>
@@ -2913,7 +2958,7 @@
         <v>3</v>
       </c>
       <c r="F53" t="s">
-        <v>385</v>
+        <v>395</v>
       </c>
     </row>
     <row r="54" spans="1:6">
@@ -2921,10 +2966,10 @@
         <v>58</v>
       </c>
       <c r="B54" t="s">
-        <v>221</v>
+        <v>226</v>
       </c>
       <c r="C54" t="s">
-        <v>333</v>
+        <v>342</v>
       </c>
       <c r="D54">
         <v>3</v>
@@ -2933,7 +2978,7 @@
         <v>3</v>
       </c>
       <c r="F54" t="s">
-        <v>386</v>
+        <v>396</v>
       </c>
     </row>
     <row r="55" spans="1:6">
@@ -2941,10 +2986,10 @@
         <v>59</v>
       </c>
       <c r="B55" t="s">
-        <v>222</v>
+        <v>227</v>
       </c>
       <c r="C55" t="s">
-        <v>333</v>
+        <v>343</v>
       </c>
       <c r="D55">
         <v>3</v>
@@ -2953,7 +2998,7 @@
         <v>3</v>
       </c>
       <c r="F55" t="s">
-        <v>387</v>
+        <v>397</v>
       </c>
     </row>
     <row r="56" spans="1:6">
@@ -2961,10 +3006,10 @@
         <v>60</v>
       </c>
       <c r="B56" t="s">
-        <v>223</v>
+        <v>228</v>
       </c>
       <c r="C56" t="s">
-        <v>333</v>
+        <v>343</v>
       </c>
       <c r="D56">
         <v>3</v>
@@ -2973,7 +3018,7 @@
         <v>3</v>
       </c>
       <c r="F56" t="s">
-        <v>388</v>
+        <v>398</v>
       </c>
     </row>
     <row r="57" spans="1:6">
@@ -2981,10 +3026,10 @@
         <v>61</v>
       </c>
       <c r="B57" t="s">
-        <v>224</v>
+        <v>229</v>
       </c>
       <c r="C57" t="s">
-        <v>333</v>
+        <v>343</v>
       </c>
       <c r="D57">
         <v>3</v>
@@ -2993,7 +3038,7 @@
         <v>3</v>
       </c>
       <c r="F57" t="s">
-        <v>389</v>
+        <v>399</v>
       </c>
     </row>
     <row r="58" spans="1:6">
@@ -3001,10 +3046,10 @@
         <v>62</v>
       </c>
       <c r="B58" t="s">
-        <v>225</v>
+        <v>230</v>
       </c>
       <c r="C58" t="s">
-        <v>332</v>
+        <v>343</v>
       </c>
       <c r="D58">
         <v>3</v>
@@ -3013,7 +3058,7 @@
         <v>3</v>
       </c>
       <c r="F58" t="s">
-        <v>390</v>
+        <v>400</v>
       </c>
     </row>
     <row r="59" spans="1:6">
@@ -3021,10 +3066,10 @@
         <v>63</v>
       </c>
       <c r="B59" t="s">
-        <v>226</v>
+        <v>231</v>
       </c>
       <c r="C59" t="s">
-        <v>333</v>
+        <v>342</v>
       </c>
       <c r="D59">
         <v>3</v>
@@ -3033,7 +3078,7 @@
         <v>3</v>
       </c>
       <c r="F59" t="s">
-        <v>391</v>
+        <v>401</v>
       </c>
     </row>
     <row r="60" spans="1:6">
@@ -3041,10 +3086,10 @@
         <v>64</v>
       </c>
       <c r="B60" t="s">
-        <v>227</v>
+        <v>232</v>
       </c>
       <c r="C60" t="s">
-        <v>333</v>
+        <v>343</v>
       </c>
       <c r="D60">
         <v>3</v>
@@ -3053,7 +3098,7 @@
         <v>3</v>
       </c>
       <c r="F60" t="s">
-        <v>392</v>
+        <v>402</v>
       </c>
     </row>
     <row r="61" spans="1:6">
@@ -3061,19 +3106,19 @@
         <v>65</v>
       </c>
       <c r="B61" t="s">
-        <v>228</v>
+        <v>233</v>
       </c>
       <c r="C61" t="s">
-        <v>333</v>
+        <v>342</v>
       </c>
       <c r="D61">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="E61">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="F61" t="s">
-        <v>393</v>
+        <v>403</v>
       </c>
     </row>
     <row r="62" spans="1:6">
@@ -3081,19 +3126,19 @@
         <v>66</v>
       </c>
       <c r="B62" t="s">
-        <v>229</v>
+        <v>234</v>
       </c>
       <c r="C62" t="s">
-        <v>333</v>
+        <v>343</v>
       </c>
       <c r="D62">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="E62">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="F62" t="s">
-        <v>394</v>
+        <v>404</v>
       </c>
     </row>
     <row r="63" spans="1:6">
@@ -3101,10 +3146,10 @@
         <v>67</v>
       </c>
       <c r="B63" t="s">
-        <v>230</v>
+        <v>235</v>
       </c>
       <c r="C63" t="s">
-        <v>333</v>
+        <v>343</v>
       </c>
       <c r="D63">
         <v>2</v>
@@ -3113,7 +3158,7 @@
         <v>2</v>
       </c>
       <c r="F63" t="s">
-        <v>395</v>
+        <v>405</v>
       </c>
     </row>
     <row r="64" spans="1:6">
@@ -3121,10 +3166,10 @@
         <v>68</v>
       </c>
       <c r="B64" t="s">
-        <v>231</v>
+        <v>236</v>
       </c>
       <c r="C64" t="s">
-        <v>332</v>
+        <v>343</v>
       </c>
       <c r="D64">
         <v>2</v>
@@ -3133,7 +3178,7 @@
         <v>2</v>
       </c>
       <c r="F64" t="s">
-        <v>396</v>
+        <v>406</v>
       </c>
     </row>
     <row r="65" spans="1:6">
@@ -3141,10 +3186,10 @@
         <v>69</v>
       </c>
       <c r="B65" t="s">
-        <v>232</v>
+        <v>237</v>
       </c>
       <c r="C65" t="s">
-        <v>332</v>
+        <v>343</v>
       </c>
       <c r="D65">
         <v>2</v>
@@ -3153,7 +3198,7 @@
         <v>2</v>
       </c>
       <c r="F65" t="s">
-        <v>375</v>
+        <v>407</v>
       </c>
     </row>
     <row r="66" spans="1:6">
@@ -3161,10 +3206,10 @@
         <v>70</v>
       </c>
       <c r="B66" t="s">
-        <v>233</v>
+        <v>238</v>
       </c>
       <c r="C66" t="s">
-        <v>333</v>
+        <v>342</v>
       </c>
       <c r="D66">
         <v>2</v>
@@ -3173,7 +3218,7 @@
         <v>2</v>
       </c>
       <c r="F66" t="s">
-        <v>397</v>
+        <v>408</v>
       </c>
     </row>
     <row r="67" spans="1:6">
@@ -3181,10 +3226,10 @@
         <v>71</v>
       </c>
       <c r="B67" t="s">
-        <v>234</v>
+        <v>239</v>
       </c>
       <c r="C67" t="s">
-        <v>332</v>
+        <v>342</v>
       </c>
       <c r="D67">
         <v>2</v>
@@ -3193,7 +3238,7 @@
         <v>2</v>
       </c>
       <c r="F67" t="s">
-        <v>398</v>
+        <v>385</v>
       </c>
     </row>
     <row r="68" spans="1:6">
@@ -3201,10 +3246,10 @@
         <v>72</v>
       </c>
       <c r="B68" t="s">
-        <v>235</v>
+        <v>240</v>
       </c>
       <c r="C68" t="s">
-        <v>332</v>
+        <v>343</v>
       </c>
       <c r="D68">
         <v>2</v>
@@ -3213,7 +3258,7 @@
         <v>2</v>
       </c>
       <c r="F68" t="s">
-        <v>399</v>
+        <v>409</v>
       </c>
     </row>
     <row r="69" spans="1:6">
@@ -3221,10 +3266,10 @@
         <v>73</v>
       </c>
       <c r="B69" t="s">
-        <v>236</v>
+        <v>241</v>
       </c>
       <c r="C69" t="s">
-        <v>333</v>
+        <v>342</v>
       </c>
       <c r="D69">
         <v>2</v>
@@ -3233,7 +3278,7 @@
         <v>2</v>
       </c>
       <c r="F69" t="s">
-        <v>400</v>
+        <v>410</v>
       </c>
     </row>
     <row r="70" spans="1:6">
@@ -3241,10 +3286,10 @@
         <v>74</v>
       </c>
       <c r="B70" t="s">
-        <v>237</v>
+        <v>242</v>
       </c>
       <c r="C70" t="s">
-        <v>332</v>
+        <v>342</v>
       </c>
       <c r="D70">
         <v>2</v>
@@ -3253,7 +3298,7 @@
         <v>2</v>
       </c>
       <c r="F70" t="s">
-        <v>401</v>
+        <v>411</v>
       </c>
     </row>
     <row r="71" spans="1:6">
@@ -3261,10 +3306,10 @@
         <v>75</v>
       </c>
       <c r="B71" t="s">
-        <v>238</v>
+        <v>243</v>
       </c>
       <c r="C71" t="s">
-        <v>332</v>
+        <v>343</v>
       </c>
       <c r="D71">
         <v>2</v>
@@ -3273,7 +3318,7 @@
         <v>2</v>
       </c>
       <c r="F71" t="s">
-        <v>402</v>
+        <v>412</v>
       </c>
     </row>
     <row r="72" spans="1:6">
@@ -3281,10 +3326,10 @@
         <v>76</v>
       </c>
       <c r="B72" t="s">
-        <v>239</v>
+        <v>244</v>
       </c>
       <c r="C72" t="s">
-        <v>332</v>
+        <v>342</v>
       </c>
       <c r="D72">
         <v>2</v>
@@ -3293,7 +3338,7 @@
         <v>2</v>
       </c>
       <c r="F72" t="s">
-        <v>403</v>
+        <v>413</v>
       </c>
     </row>
     <row r="73" spans="1:6">
@@ -3301,10 +3346,10 @@
         <v>77</v>
       </c>
       <c r="B73" t="s">
-        <v>240</v>
+        <v>245</v>
       </c>
       <c r="C73" t="s">
-        <v>332</v>
+        <v>342</v>
       </c>
       <c r="D73">
         <v>2</v>
@@ -3313,7 +3358,7 @@
         <v>2</v>
       </c>
       <c r="F73" t="s">
-        <v>404</v>
+        <v>414</v>
       </c>
     </row>
     <row r="74" spans="1:6">
@@ -3321,10 +3366,10 @@
         <v>78</v>
       </c>
       <c r="B74" t="s">
-        <v>241</v>
+        <v>246</v>
       </c>
       <c r="C74" t="s">
-        <v>333</v>
+        <v>342</v>
       </c>
       <c r="D74">
         <v>2</v>
@@ -3333,7 +3378,7 @@
         <v>2</v>
       </c>
       <c r="F74" t="s">
-        <v>405</v>
+        <v>415</v>
       </c>
     </row>
     <row r="75" spans="1:6">
@@ -3341,10 +3386,10 @@
         <v>79</v>
       </c>
       <c r="B75" t="s">
-        <v>242</v>
+        <v>247</v>
       </c>
       <c r="C75" t="s">
-        <v>333</v>
+        <v>342</v>
       </c>
       <c r="D75">
         <v>2</v>
@@ -3353,7 +3398,7 @@
         <v>2</v>
       </c>
       <c r="F75" t="s">
-        <v>406</v>
+        <v>416</v>
       </c>
     </row>
     <row r="76" spans="1:6">
@@ -3361,10 +3406,10 @@
         <v>80</v>
       </c>
       <c r="B76" t="s">
-        <v>243</v>
+        <v>248</v>
       </c>
       <c r="C76" t="s">
-        <v>333</v>
+        <v>343</v>
       </c>
       <c r="D76">
         <v>2</v>
@@ -3373,7 +3418,7 @@
         <v>2</v>
       </c>
       <c r="F76" t="s">
-        <v>407</v>
+        <v>417</v>
       </c>
     </row>
     <row r="77" spans="1:6">
@@ -3381,10 +3426,10 @@
         <v>81</v>
       </c>
       <c r="B77" t="s">
-        <v>244</v>
+        <v>249</v>
       </c>
       <c r="C77" t="s">
-        <v>332</v>
+        <v>343</v>
       </c>
       <c r="D77">
         <v>2</v>
@@ -3393,7 +3438,7 @@
         <v>2</v>
       </c>
       <c r="F77" t="s">
-        <v>408</v>
+        <v>418</v>
       </c>
     </row>
     <row r="78" spans="1:6">
@@ -3401,10 +3446,10 @@
         <v>82</v>
       </c>
       <c r="B78" t="s">
-        <v>245</v>
+        <v>250</v>
       </c>
       <c r="C78" t="s">
-        <v>333</v>
+        <v>343</v>
       </c>
       <c r="D78">
         <v>2</v>
@@ -3413,7 +3458,7 @@
         <v>2</v>
       </c>
       <c r="F78" t="s">
-        <v>409</v>
+        <v>419</v>
       </c>
     </row>
     <row r="79" spans="1:6">
@@ -3421,10 +3466,10 @@
         <v>83</v>
       </c>
       <c r="B79" t="s">
-        <v>246</v>
+        <v>251</v>
       </c>
       <c r="C79" t="s">
-        <v>333</v>
+        <v>342</v>
       </c>
       <c r="D79">
         <v>2</v>
@@ -3433,7 +3478,7 @@
         <v>2</v>
       </c>
       <c r="F79" t="s">
-        <v>410</v>
+        <v>420</v>
       </c>
     </row>
     <row r="80" spans="1:6">
@@ -3441,10 +3486,10 @@
         <v>84</v>
       </c>
       <c r="B80" t="s">
-        <v>247</v>
+        <v>252</v>
       </c>
       <c r="C80" t="s">
-        <v>333</v>
+        <v>342</v>
       </c>
       <c r="D80">
         <v>2</v>
@@ -3453,7 +3498,7 @@
         <v>2</v>
       </c>
       <c r="F80" t="s">
-        <v>411</v>
+        <v>421</v>
       </c>
     </row>
     <row r="81" spans="1:6">
@@ -3461,19 +3506,19 @@
         <v>85</v>
       </c>
       <c r="B81" t="s">
-        <v>248</v>
+        <v>253</v>
       </c>
       <c r="C81" t="s">
-        <v>333</v>
+        <v>343</v>
       </c>
       <c r="D81">
         <v>2</v>
       </c>
       <c r="E81">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="F81" t="s">
-        <v>412</v>
+        <v>422</v>
       </c>
     </row>
     <row r="82" spans="1:6">
@@ -3481,10 +3526,10 @@
         <v>86</v>
       </c>
       <c r="B82" t="s">
-        <v>249</v>
+        <v>254</v>
       </c>
       <c r="C82" t="s">
-        <v>333</v>
+        <v>343</v>
       </c>
       <c r="D82">
         <v>2</v>
@@ -3493,7 +3538,7 @@
         <v>2</v>
       </c>
       <c r="F82" t="s">
-        <v>368</v>
+        <v>423</v>
       </c>
     </row>
     <row r="83" spans="1:6">
@@ -3501,10 +3546,10 @@
         <v>87</v>
       </c>
       <c r="B83" t="s">
-        <v>250</v>
+        <v>255</v>
       </c>
       <c r="C83" t="s">
-        <v>332</v>
+        <v>343</v>
       </c>
       <c r="D83">
         <v>2</v>
@@ -3513,7 +3558,7 @@
         <v>2</v>
       </c>
       <c r="F83" t="s">
-        <v>356</v>
+        <v>424</v>
       </c>
     </row>
     <row r="84" spans="1:6">
@@ -3521,19 +3566,19 @@
         <v>88</v>
       </c>
       <c r="B84" t="s">
-        <v>251</v>
+        <v>256</v>
       </c>
       <c r="C84" t="s">
-        <v>332</v>
+        <v>343</v>
       </c>
       <c r="D84">
         <v>2</v>
       </c>
       <c r="E84">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="F84" t="s">
-        <v>413</v>
+        <v>425</v>
       </c>
     </row>
     <row r="85" spans="1:6">
@@ -3541,10 +3586,10 @@
         <v>89</v>
       </c>
       <c r="B85" t="s">
-        <v>252</v>
+        <v>257</v>
       </c>
       <c r="C85" t="s">
-        <v>333</v>
+        <v>343</v>
       </c>
       <c r="D85">
         <v>2</v>
@@ -3553,7 +3598,7 @@
         <v>2</v>
       </c>
       <c r="F85" t="s">
-        <v>414</v>
+        <v>378</v>
       </c>
     </row>
     <row r="86" spans="1:6">
@@ -3561,10 +3606,10 @@
         <v>90</v>
       </c>
       <c r="B86" t="s">
-        <v>253</v>
+        <v>258</v>
       </c>
       <c r="C86" t="s">
-        <v>333</v>
+        <v>342</v>
       </c>
       <c r="D86">
         <v>2</v>
@@ -3573,7 +3618,7 @@
         <v>2</v>
       </c>
       <c r="F86" t="s">
-        <v>415</v>
+        <v>366</v>
       </c>
     </row>
     <row r="87" spans="1:6">
@@ -3581,10 +3626,10 @@
         <v>91</v>
       </c>
       <c r="B87" t="s">
-        <v>254</v>
+        <v>259</v>
       </c>
       <c r="C87" t="s">
-        <v>333</v>
+        <v>342</v>
       </c>
       <c r="D87">
         <v>2</v>
@@ -3593,7 +3638,7 @@
         <v>2</v>
       </c>
       <c r="F87" t="s">
-        <v>339</v>
+        <v>426</v>
       </c>
     </row>
     <row r="88" spans="1:6">
@@ -3601,10 +3646,10 @@
         <v>92</v>
       </c>
       <c r="B88" t="s">
-        <v>255</v>
+        <v>260</v>
       </c>
       <c r="C88" t="s">
-        <v>333</v>
+        <v>343</v>
       </c>
       <c r="D88">
         <v>2</v>
@@ -3613,7 +3658,7 @@
         <v>2</v>
       </c>
       <c r="F88" t="s">
-        <v>416</v>
+        <v>427</v>
       </c>
     </row>
     <row r="89" spans="1:6">
@@ -3621,10 +3666,10 @@
         <v>93</v>
       </c>
       <c r="B89" t="s">
-        <v>256</v>
+        <v>261</v>
       </c>
       <c r="C89" t="s">
-        <v>333</v>
+        <v>343</v>
       </c>
       <c r="D89">
         <v>2</v>
@@ -3633,7 +3678,7 @@
         <v>2</v>
       </c>
       <c r="F89" t="s">
-        <v>417</v>
+        <v>428</v>
       </c>
     </row>
     <row r="90" spans="1:6">
@@ -3641,10 +3686,10 @@
         <v>94</v>
       </c>
       <c r="B90" t="s">
-        <v>257</v>
+        <v>262</v>
       </c>
       <c r="C90" t="s">
-        <v>333</v>
+        <v>343</v>
       </c>
       <c r="D90">
         <v>2</v>
@@ -3653,7 +3698,7 @@
         <v>2</v>
       </c>
       <c r="F90" t="s">
-        <v>418</v>
+        <v>349</v>
       </c>
     </row>
     <row r="91" spans="1:6">
@@ -3661,10 +3706,10 @@
         <v>95</v>
       </c>
       <c r="B91" t="s">
-        <v>258</v>
+        <v>263</v>
       </c>
       <c r="C91" t="s">
-        <v>333</v>
+        <v>343</v>
       </c>
       <c r="D91">
         <v>2</v>
@@ -3673,7 +3718,7 @@
         <v>2</v>
       </c>
       <c r="F91" t="s">
-        <v>419</v>
+        <v>429</v>
       </c>
     </row>
     <row r="92" spans="1:6">
@@ -3681,10 +3726,10 @@
         <v>96</v>
       </c>
       <c r="B92" t="s">
-        <v>259</v>
+        <v>264</v>
       </c>
       <c r="C92" t="s">
-        <v>333</v>
+        <v>343</v>
       </c>
       <c r="D92">
         <v>2</v>
@@ -3693,7 +3738,7 @@
         <v>2</v>
       </c>
       <c r="F92" t="s">
-        <v>420</v>
+        <v>430</v>
       </c>
     </row>
     <row r="93" spans="1:6">
@@ -3701,10 +3746,10 @@
         <v>97</v>
       </c>
       <c r="B93" t="s">
-        <v>260</v>
+        <v>265</v>
       </c>
       <c r="C93" t="s">
-        <v>333</v>
+        <v>343</v>
       </c>
       <c r="D93">
         <v>2</v>
@@ -3713,7 +3758,7 @@
         <v>2</v>
       </c>
       <c r="F93" t="s">
-        <v>421</v>
+        <v>431</v>
       </c>
     </row>
     <row r="94" spans="1:6">
@@ -3721,10 +3766,10 @@
         <v>98</v>
       </c>
       <c r="B94" t="s">
-        <v>261</v>
+        <v>266</v>
       </c>
       <c r="C94" t="s">
-        <v>333</v>
+        <v>343</v>
       </c>
       <c r="D94">
         <v>2</v>
@@ -3733,7 +3778,7 @@
         <v>2</v>
       </c>
       <c r="F94" t="s">
-        <v>422</v>
+        <v>432</v>
       </c>
     </row>
     <row r="95" spans="1:6">
@@ -3741,10 +3786,10 @@
         <v>99</v>
       </c>
       <c r="B95" t="s">
-        <v>262</v>
+        <v>267</v>
       </c>
       <c r="C95" t="s">
-        <v>333</v>
+        <v>343</v>
       </c>
       <c r="D95">
         <v>2</v>
@@ -3753,7 +3798,7 @@
         <v>2</v>
       </c>
       <c r="F95" t="s">
-        <v>423</v>
+        <v>433</v>
       </c>
     </row>
     <row r="96" spans="1:6">
@@ -3761,10 +3806,10 @@
         <v>100</v>
       </c>
       <c r="B96" t="s">
-        <v>263</v>
+        <v>268</v>
       </c>
       <c r="C96" t="s">
-        <v>333</v>
+        <v>343</v>
       </c>
       <c r="D96">
         <v>2</v>
@@ -3773,7 +3818,7 @@
         <v>2</v>
       </c>
       <c r="F96" t="s">
-        <v>424</v>
+        <v>434</v>
       </c>
     </row>
     <row r="97" spans="1:6">
@@ -3781,10 +3826,10 @@
         <v>101</v>
       </c>
       <c r="B97" t="s">
-        <v>264</v>
+        <v>269</v>
       </c>
       <c r="C97" t="s">
-        <v>333</v>
+        <v>343</v>
       </c>
       <c r="D97">
         <v>2</v>
@@ -3793,7 +3838,7 @@
         <v>2</v>
       </c>
       <c r="F97" t="s">
-        <v>425</v>
+        <v>435</v>
       </c>
     </row>
     <row r="98" spans="1:6">
@@ -3801,10 +3846,10 @@
         <v>102</v>
       </c>
       <c r="B98" t="s">
-        <v>265</v>
+        <v>270</v>
       </c>
       <c r="C98" t="s">
-        <v>333</v>
+        <v>343</v>
       </c>
       <c r="D98">
         <v>2</v>
@@ -3813,7 +3858,7 @@
         <v>2</v>
       </c>
       <c r="F98" t="s">
-        <v>426</v>
+        <v>436</v>
       </c>
     </row>
     <row r="99" spans="1:6">
@@ -3821,10 +3866,10 @@
         <v>103</v>
       </c>
       <c r="B99" t="s">
-        <v>266</v>
+        <v>271</v>
       </c>
       <c r="C99" t="s">
-        <v>332</v>
+        <v>343</v>
       </c>
       <c r="D99">
         <v>2</v>
@@ -3833,7 +3878,7 @@
         <v>2</v>
       </c>
       <c r="F99" t="s">
-        <v>427</v>
+        <v>437</v>
       </c>
     </row>
     <row r="100" spans="1:6">
@@ -3841,10 +3886,10 @@
         <v>104</v>
       </c>
       <c r="B100" t="s">
-        <v>267</v>
+        <v>272</v>
       </c>
       <c r="C100" t="s">
-        <v>333</v>
+        <v>343</v>
       </c>
       <c r="D100">
         <v>2</v>
@@ -3853,7 +3898,7 @@
         <v>2</v>
       </c>
       <c r="F100" t="s">
-        <v>428</v>
+        <v>438</v>
       </c>
     </row>
     <row r="101" spans="1:6">
@@ -3861,10 +3906,10 @@
         <v>105</v>
       </c>
       <c r="B101" t="s">
-        <v>268</v>
+        <v>273</v>
       </c>
       <c r="C101" t="s">
-        <v>333</v>
+        <v>343</v>
       </c>
       <c r="D101">
         <v>2</v>
@@ -3873,7 +3918,7 @@
         <v>2</v>
       </c>
       <c r="F101" t="s">
-        <v>429</v>
+        <v>439</v>
       </c>
     </row>
     <row r="102" spans="1:6">
@@ -3881,10 +3926,10 @@
         <v>106</v>
       </c>
       <c r="B102" t="s">
-        <v>269</v>
+        <v>274</v>
       </c>
       <c r="C102" t="s">
-        <v>333</v>
+        <v>342</v>
       </c>
       <c r="D102">
         <v>2</v>
@@ -3893,7 +3938,7 @@
         <v>2</v>
       </c>
       <c r="F102" t="s">
-        <v>430</v>
+        <v>440</v>
       </c>
     </row>
     <row r="103" spans="1:6">
@@ -3901,10 +3946,10 @@
         <v>107</v>
       </c>
       <c r="B103" t="s">
-        <v>270</v>
+        <v>275</v>
       </c>
       <c r="C103" t="s">
-        <v>333</v>
+        <v>343</v>
       </c>
       <c r="D103">
         <v>2</v>
@@ -3913,7 +3958,7 @@
         <v>2</v>
       </c>
       <c r="F103" t="s">
-        <v>431</v>
+        <v>441</v>
       </c>
     </row>
     <row r="104" spans="1:6">
@@ -3921,10 +3966,10 @@
         <v>108</v>
       </c>
       <c r="B104" t="s">
-        <v>271</v>
+        <v>276</v>
       </c>
       <c r="C104" t="s">
-        <v>333</v>
+        <v>343</v>
       </c>
       <c r="D104">
         <v>2</v>
@@ -3933,7 +3978,7 @@
         <v>2</v>
       </c>
       <c r="F104" t="s">
-        <v>343</v>
+        <v>442</v>
       </c>
     </row>
     <row r="105" spans="1:6">
@@ -3941,10 +3986,10 @@
         <v>109</v>
       </c>
       <c r="B105" t="s">
-        <v>272</v>
+        <v>277</v>
       </c>
       <c r="C105" t="s">
-        <v>333</v>
+        <v>343</v>
       </c>
       <c r="D105">
         <v>2</v>
@@ -3953,7 +3998,7 @@
         <v>2</v>
       </c>
       <c r="F105" t="s">
-        <v>432</v>
+        <v>443</v>
       </c>
     </row>
     <row r="106" spans="1:6">
@@ -3961,10 +4006,10 @@
         <v>110</v>
       </c>
       <c r="B106" t="s">
-        <v>273</v>
+        <v>278</v>
       </c>
       <c r="C106" t="s">
-        <v>333</v>
+        <v>343</v>
       </c>
       <c r="D106">
         <v>2</v>
@@ -3973,7 +4018,7 @@
         <v>2</v>
       </c>
       <c r="F106" t="s">
-        <v>433</v>
+        <v>444</v>
       </c>
     </row>
     <row r="107" spans="1:6">
@@ -3981,10 +4026,10 @@
         <v>111</v>
       </c>
       <c r="B107" t="s">
-        <v>274</v>
+        <v>279</v>
       </c>
       <c r="C107" t="s">
-        <v>333</v>
+        <v>343</v>
       </c>
       <c r="D107">
         <v>2</v>
@@ -3993,7 +4038,7 @@
         <v>2</v>
       </c>
       <c r="F107" t="s">
-        <v>347</v>
+        <v>353</v>
       </c>
     </row>
     <row r="108" spans="1:6">
@@ -4001,19 +4046,19 @@
         <v>112</v>
       </c>
       <c r="B108" t="s">
-        <v>275</v>
+        <v>280</v>
       </c>
       <c r="C108" t="s">
-        <v>333</v>
+        <v>343</v>
       </c>
       <c r="D108">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="E108">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="F108" t="s">
-        <v>434</v>
+        <v>445</v>
       </c>
     </row>
     <row r="109" spans="1:6">
@@ -4021,19 +4066,19 @@
         <v>113</v>
       </c>
       <c r="B109" t="s">
-        <v>276</v>
+        <v>281</v>
       </c>
       <c r="C109" t="s">
-        <v>332</v>
+        <v>343</v>
       </c>
       <c r="D109">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="E109">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="F109" t="s">
-        <v>435</v>
+        <v>446</v>
       </c>
     </row>
     <row r="110" spans="1:6">
@@ -4041,19 +4086,19 @@
         <v>114</v>
       </c>
       <c r="B110" t="s">
-        <v>277</v>
+        <v>282</v>
       </c>
       <c r="C110" t="s">
-        <v>332</v>
+        <v>343</v>
       </c>
       <c r="D110">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="E110">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="F110" t="s">
-        <v>436</v>
+        <v>357</v>
       </c>
     </row>
     <row r="111" spans="1:6">
@@ -4061,10 +4106,10 @@
         <v>115</v>
       </c>
       <c r="B111" t="s">
-        <v>278</v>
+        <v>283</v>
       </c>
       <c r="C111" t="s">
-        <v>332</v>
+        <v>343</v>
       </c>
       <c r="D111">
         <v>1</v>
@@ -4073,7 +4118,7 @@
         <v>1</v>
       </c>
       <c r="F111" t="s">
-        <v>437</v>
+        <v>447</v>
       </c>
     </row>
     <row r="112" spans="1:6">
@@ -4081,10 +4126,10 @@
         <v>116</v>
       </c>
       <c r="B112" t="s">
-        <v>279</v>
+        <v>284</v>
       </c>
       <c r="C112" t="s">
-        <v>333</v>
+        <v>342</v>
       </c>
       <c r="D112">
         <v>1</v>
@@ -4093,7 +4138,7 @@
         <v>1</v>
       </c>
       <c r="F112" t="s">
-        <v>438</v>
+        <v>448</v>
       </c>
     </row>
     <row r="113" spans="1:6">
@@ -4101,10 +4146,10 @@
         <v>117</v>
       </c>
       <c r="B113" t="s">
-        <v>280</v>
+        <v>285</v>
       </c>
       <c r="C113" t="s">
-        <v>332</v>
+        <v>342</v>
       </c>
       <c r="D113">
         <v>1</v>
@@ -4113,7 +4158,7 @@
         <v>1</v>
       </c>
       <c r="F113" t="s">
-        <v>439</v>
+        <v>449</v>
       </c>
     </row>
     <row r="114" spans="1:6">
@@ -4121,10 +4166,10 @@
         <v>118</v>
       </c>
       <c r="B114" t="s">
-        <v>281</v>
+        <v>286</v>
       </c>
       <c r="C114" t="s">
-        <v>333</v>
+        <v>342</v>
       </c>
       <c r="D114">
         <v>1</v>
@@ -4133,7 +4178,7 @@
         <v>1</v>
       </c>
       <c r="F114" t="s">
-        <v>440</v>
+        <v>450</v>
       </c>
     </row>
     <row r="115" spans="1:6">
@@ -4141,10 +4186,10 @@
         <v>119</v>
       </c>
       <c r="B115" t="s">
-        <v>282</v>
+        <v>287</v>
       </c>
       <c r="C115" t="s">
-        <v>332</v>
+        <v>343</v>
       </c>
       <c r="D115">
         <v>1</v>
@@ -4153,7 +4198,7 @@
         <v>1</v>
       </c>
       <c r="F115" t="s">
-        <v>441</v>
+        <v>451</v>
       </c>
     </row>
     <row r="116" spans="1:6">
@@ -4161,10 +4206,10 @@
         <v>120</v>
       </c>
       <c r="B116" t="s">
-        <v>283</v>
+        <v>288</v>
       </c>
       <c r="C116" t="s">
-        <v>332</v>
+        <v>342</v>
       </c>
       <c r="D116">
         <v>1</v>
@@ -4173,7 +4218,7 @@
         <v>1</v>
       </c>
       <c r="F116" t="s">
-        <v>442</v>
+        <v>452</v>
       </c>
     </row>
     <row r="117" spans="1:6">
@@ -4181,10 +4226,10 @@
         <v>121</v>
       </c>
       <c r="B117" t="s">
-        <v>284</v>
+        <v>289</v>
       </c>
       <c r="C117" t="s">
-        <v>332</v>
+        <v>343</v>
       </c>
       <c r="D117">
         <v>1</v>
@@ -4193,7 +4238,7 @@
         <v>1</v>
       </c>
       <c r="F117" t="s">
-        <v>443</v>
+        <v>453</v>
       </c>
     </row>
     <row r="118" spans="1:6">
@@ -4201,10 +4246,10 @@
         <v>122</v>
       </c>
       <c r="B118" t="s">
-        <v>285</v>
+        <v>290</v>
       </c>
       <c r="C118" t="s">
-        <v>332</v>
+        <v>342</v>
       </c>
       <c r="D118">
         <v>1</v>
@@ -4213,7 +4258,7 @@
         <v>1</v>
       </c>
       <c r="F118" t="s">
-        <v>444</v>
+        <v>454</v>
       </c>
     </row>
     <row r="119" spans="1:6">
@@ -4221,10 +4266,10 @@
         <v>123</v>
       </c>
       <c r="B119" t="s">
-        <v>286</v>
+        <v>291</v>
       </c>
       <c r="C119" t="s">
-        <v>332</v>
+        <v>342</v>
       </c>
       <c r="D119">
         <v>1</v>
@@ -4233,7 +4278,7 @@
         <v>1</v>
       </c>
       <c r="F119" t="s">
-        <v>445</v>
+        <v>455</v>
       </c>
     </row>
     <row r="120" spans="1:6">
@@ -4241,10 +4286,10 @@
         <v>124</v>
       </c>
       <c r="B120" t="s">
-        <v>287</v>
+        <v>292</v>
       </c>
       <c r="C120" t="s">
-        <v>332</v>
+        <v>342</v>
       </c>
       <c r="D120">
         <v>1</v>
@@ -4253,7 +4298,7 @@
         <v>1</v>
       </c>
       <c r="F120" t="s">
-        <v>446</v>
+        <v>456</v>
       </c>
     </row>
     <row r="121" spans="1:6">
@@ -4261,10 +4306,10 @@
         <v>125</v>
       </c>
       <c r="B121" t="s">
-        <v>288</v>
+        <v>293</v>
       </c>
       <c r="C121" t="s">
-        <v>333</v>
+        <v>342</v>
       </c>
       <c r="D121">
         <v>1</v>
@@ -4273,7 +4318,7 @@
         <v>1</v>
       </c>
       <c r="F121" t="s">
-        <v>447</v>
+        <v>457</v>
       </c>
     </row>
     <row r="122" spans="1:6">
@@ -4281,10 +4326,10 @@
         <v>126</v>
       </c>
       <c r="B122" t="s">
-        <v>289</v>
+        <v>294</v>
       </c>
       <c r="C122" t="s">
-        <v>333</v>
+        <v>342</v>
       </c>
       <c r="D122">
         <v>1</v>
@@ -4293,7 +4338,7 @@
         <v>1</v>
       </c>
       <c r="F122" t="s">
-        <v>448</v>
+        <v>458</v>
       </c>
     </row>
     <row r="123" spans="1:6">
@@ -4301,10 +4346,10 @@
         <v>127</v>
       </c>
       <c r="B123" t="s">
-        <v>290</v>
+        <v>295</v>
       </c>
       <c r="C123" t="s">
-        <v>333</v>
+        <v>342</v>
       </c>
       <c r="D123">
         <v>1</v>
@@ -4313,7 +4358,7 @@
         <v>1</v>
       </c>
       <c r="F123" t="s">
-        <v>449</v>
+        <v>459</v>
       </c>
     </row>
     <row r="124" spans="1:6">
@@ -4321,10 +4366,10 @@
         <v>128</v>
       </c>
       <c r="B124" t="s">
-        <v>291</v>
+        <v>296</v>
       </c>
       <c r="C124" t="s">
-        <v>333</v>
+        <v>342</v>
       </c>
       <c r="D124">
         <v>1</v>
@@ -4333,7 +4378,7 @@
         <v>1</v>
       </c>
       <c r="F124" t="s">
-        <v>450</v>
+        <v>460</v>
       </c>
     </row>
     <row r="125" spans="1:6">
@@ -4341,10 +4386,10 @@
         <v>129</v>
       </c>
       <c r="B125" t="s">
-        <v>292</v>
+        <v>297</v>
       </c>
       <c r="C125" t="s">
-        <v>332</v>
+        <v>343</v>
       </c>
       <c r="D125">
         <v>1</v>
@@ -4353,7 +4398,7 @@
         <v>1</v>
       </c>
       <c r="F125" t="s">
-        <v>451</v>
+        <v>461</v>
       </c>
     </row>
     <row r="126" spans="1:6">
@@ -4361,10 +4406,10 @@
         <v>130</v>
       </c>
       <c r="B126" t="s">
-        <v>293</v>
+        <v>298</v>
       </c>
       <c r="C126" t="s">
-        <v>332</v>
+        <v>343</v>
       </c>
       <c r="D126">
         <v>1</v>
@@ -4373,7 +4418,7 @@
         <v>1</v>
       </c>
       <c r="F126" t="s">
-        <v>452</v>
+        <v>462</v>
       </c>
     </row>
     <row r="127" spans="1:6">
@@ -4381,10 +4426,10 @@
         <v>131</v>
       </c>
       <c r="B127" t="s">
-        <v>294</v>
+        <v>299</v>
       </c>
       <c r="C127" t="s">
-        <v>333</v>
+        <v>343</v>
       </c>
       <c r="D127">
         <v>1</v>
@@ -4393,7 +4438,7 @@
         <v>1</v>
       </c>
       <c r="F127" t="s">
-        <v>453</v>
+        <v>463</v>
       </c>
     </row>
     <row r="128" spans="1:6">
@@ -4401,10 +4446,10 @@
         <v>132</v>
       </c>
       <c r="B128" t="s">
-        <v>295</v>
+        <v>300</v>
       </c>
       <c r="C128" t="s">
-        <v>333</v>
+        <v>343</v>
       </c>
       <c r="D128">
         <v>1</v>
@@ -4413,7 +4458,7 @@
         <v>1</v>
       </c>
       <c r="F128" t="s">
-        <v>454</v>
+        <v>464</v>
       </c>
     </row>
     <row r="129" spans="1:6">
@@ -4421,10 +4466,10 @@
         <v>133</v>
       </c>
       <c r="B129" t="s">
-        <v>296</v>
+        <v>301</v>
       </c>
       <c r="C129" t="s">
-        <v>332</v>
+        <v>343</v>
       </c>
       <c r="D129">
         <v>1</v>
@@ -4433,7 +4478,7 @@
         <v>1</v>
       </c>
       <c r="F129" t="s">
-        <v>447</v>
+        <v>465</v>
       </c>
     </row>
     <row r="130" spans="1:6">
@@ -4441,10 +4486,10 @@
         <v>134</v>
       </c>
       <c r="B130" t="s">
-        <v>297</v>
+        <v>302</v>
       </c>
       <c r="C130" t="s">
-        <v>332</v>
+        <v>342</v>
       </c>
       <c r="D130">
         <v>1</v>
@@ -4453,7 +4498,7 @@
         <v>1</v>
       </c>
       <c r="F130" t="s">
-        <v>455</v>
+        <v>466</v>
       </c>
     </row>
     <row r="131" spans="1:6">
@@ -4461,10 +4506,10 @@
         <v>135</v>
       </c>
       <c r="B131" t="s">
-        <v>298</v>
+        <v>303</v>
       </c>
       <c r="C131" t="s">
-        <v>332</v>
+        <v>342</v>
       </c>
       <c r="D131">
         <v>1</v>
@@ -4473,7 +4518,7 @@
         <v>1</v>
       </c>
       <c r="F131" t="s">
-        <v>456</v>
+        <v>467</v>
       </c>
     </row>
     <row r="132" spans="1:6">
@@ -4481,10 +4526,10 @@
         <v>136</v>
       </c>
       <c r="B132" t="s">
-        <v>299</v>
+        <v>304</v>
       </c>
       <c r="C132" t="s">
-        <v>333</v>
+        <v>343</v>
       </c>
       <c r="D132">
         <v>1</v>
@@ -4493,7 +4538,7 @@
         <v>1</v>
       </c>
       <c r="F132" t="s">
-        <v>457</v>
+        <v>468</v>
       </c>
     </row>
     <row r="133" spans="1:6">
@@ -4501,10 +4546,10 @@
         <v>137</v>
       </c>
       <c r="B133" t="s">
-        <v>300</v>
+        <v>305</v>
       </c>
       <c r="C133" t="s">
-        <v>332</v>
+        <v>343</v>
       </c>
       <c r="D133">
         <v>1</v>
@@ -4513,7 +4558,7 @@
         <v>1</v>
       </c>
       <c r="F133" t="s">
-        <v>458</v>
+        <v>469</v>
       </c>
     </row>
     <row r="134" spans="1:6">
@@ -4521,10 +4566,10 @@
         <v>138</v>
       </c>
       <c r="B134" t="s">
-        <v>301</v>
+        <v>306</v>
       </c>
       <c r="C134" t="s">
-        <v>333</v>
+        <v>342</v>
       </c>
       <c r="D134">
         <v>1</v>
@@ -4533,7 +4578,7 @@
         <v>1</v>
       </c>
       <c r="F134" t="s">
-        <v>459</v>
+        <v>461</v>
       </c>
     </row>
     <row r="135" spans="1:6">
@@ -4541,10 +4586,10 @@
         <v>139</v>
       </c>
       <c r="B135" t="s">
-        <v>302</v>
+        <v>307</v>
       </c>
       <c r="C135" t="s">
-        <v>332</v>
+        <v>342</v>
       </c>
       <c r="D135">
         <v>1</v>
@@ -4553,7 +4598,7 @@
         <v>1</v>
       </c>
       <c r="F135" t="s">
-        <v>397</v>
+        <v>470</v>
       </c>
     </row>
     <row r="136" spans="1:6">
@@ -4561,10 +4606,10 @@
         <v>140</v>
       </c>
       <c r="B136" t="s">
-        <v>303</v>
+        <v>308</v>
       </c>
       <c r="C136" t="s">
-        <v>333</v>
+        <v>342</v>
       </c>
       <c r="D136">
         <v>1</v>
@@ -4573,7 +4618,7 @@
         <v>1</v>
       </c>
       <c r="F136" t="s">
-        <v>460</v>
+        <v>471</v>
       </c>
     </row>
     <row r="137" spans="1:6">
@@ -4581,10 +4626,10 @@
         <v>141</v>
       </c>
       <c r="B137" t="s">
-        <v>304</v>
+        <v>309</v>
       </c>
       <c r="C137" t="s">
-        <v>332</v>
+        <v>343</v>
       </c>
       <c r="D137">
         <v>1</v>
@@ -4593,7 +4638,7 @@
         <v>1</v>
       </c>
       <c r="F137" t="s">
-        <v>461</v>
+        <v>472</v>
       </c>
     </row>
     <row r="138" spans="1:6">
@@ -4601,10 +4646,10 @@
         <v>142</v>
       </c>
       <c r="B138" t="s">
-        <v>305</v>
+        <v>310</v>
       </c>
       <c r="C138" t="s">
-        <v>332</v>
+        <v>342</v>
       </c>
       <c r="D138">
         <v>1</v>
@@ -4613,7 +4658,7 @@
         <v>1</v>
       </c>
       <c r="F138" t="s">
-        <v>462</v>
+        <v>473</v>
       </c>
     </row>
     <row r="139" spans="1:6">
@@ -4621,10 +4666,10 @@
         <v>143</v>
       </c>
       <c r="B139" t="s">
-        <v>306</v>
+        <v>311</v>
       </c>
       <c r="C139" t="s">
-        <v>333</v>
+        <v>343</v>
       </c>
       <c r="D139">
         <v>1</v>
@@ -4633,7 +4678,7 @@
         <v>1</v>
       </c>
       <c r="F139" t="s">
-        <v>463</v>
+        <v>474</v>
       </c>
     </row>
     <row r="140" spans="1:6">
@@ -4641,10 +4686,10 @@
         <v>144</v>
       </c>
       <c r="B140" t="s">
-        <v>307</v>
+        <v>312</v>
       </c>
       <c r="C140" t="s">
-        <v>332</v>
+        <v>342</v>
       </c>
       <c r="D140">
         <v>1</v>
@@ -4653,7 +4698,7 @@
         <v>1</v>
       </c>
       <c r="F140" t="s">
-        <v>464</v>
+        <v>409</v>
       </c>
     </row>
     <row r="141" spans="1:6">
@@ -4661,10 +4706,10 @@
         <v>145</v>
       </c>
       <c r="B141" t="s">
-        <v>308</v>
+        <v>313</v>
       </c>
       <c r="C141" t="s">
-        <v>332</v>
+        <v>343</v>
       </c>
       <c r="D141">
         <v>1</v>
@@ -4673,7 +4718,7 @@
         <v>1</v>
       </c>
       <c r="F141" t="s">
-        <v>441</v>
+        <v>475</v>
       </c>
     </row>
     <row r="142" spans="1:6">
@@ -4681,10 +4726,10 @@
         <v>146</v>
       </c>
       <c r="B142" t="s">
-        <v>309</v>
+        <v>314</v>
       </c>
       <c r="C142" t="s">
-        <v>333</v>
+        <v>342</v>
       </c>
       <c r="D142">
         <v>1</v>
@@ -4693,7 +4738,7 @@
         <v>1</v>
       </c>
       <c r="F142" t="s">
-        <v>465</v>
+        <v>476</v>
       </c>
     </row>
     <row r="143" spans="1:6">
@@ -4701,10 +4746,10 @@
         <v>147</v>
       </c>
       <c r="B143" t="s">
-        <v>310</v>
+        <v>315</v>
       </c>
       <c r="C143" t="s">
-        <v>333</v>
+        <v>342</v>
       </c>
       <c r="D143">
         <v>1</v>
@@ -4713,7 +4758,7 @@
         <v>1</v>
       </c>
       <c r="F143" t="s">
-        <v>466</v>
+        <v>477</v>
       </c>
     </row>
     <row r="144" spans="1:6">
@@ -4721,10 +4766,10 @@
         <v>148</v>
       </c>
       <c r="B144" t="s">
-        <v>311</v>
+        <v>316</v>
       </c>
       <c r="C144" t="s">
-        <v>333</v>
+        <v>343</v>
       </c>
       <c r="D144">
         <v>1</v>
@@ -4733,7 +4778,7 @@
         <v>1</v>
       </c>
       <c r="F144" t="s">
-        <v>467</v>
+        <v>478</v>
       </c>
     </row>
     <row r="145" spans="1:6">
@@ -4741,10 +4786,10 @@
         <v>149</v>
       </c>
       <c r="B145" t="s">
-        <v>312</v>
+        <v>317</v>
       </c>
       <c r="C145" t="s">
-        <v>333</v>
+        <v>342</v>
       </c>
       <c r="D145">
         <v>1</v>
@@ -4753,7 +4798,7 @@
         <v>1</v>
       </c>
       <c r="F145" t="s">
-        <v>468</v>
+        <v>479</v>
       </c>
     </row>
     <row r="146" spans="1:6">
@@ -4761,10 +4806,10 @@
         <v>150</v>
       </c>
       <c r="B146" t="s">
-        <v>313</v>
+        <v>318</v>
       </c>
       <c r="C146" t="s">
-        <v>332</v>
+        <v>342</v>
       </c>
       <c r="D146">
         <v>1</v>
@@ -4773,7 +4818,7 @@
         <v>1</v>
       </c>
       <c r="F146" t="s">
-        <v>371</v>
+        <v>454</v>
       </c>
     </row>
     <row r="147" spans="1:6">
@@ -4781,10 +4826,10 @@
         <v>151</v>
       </c>
       <c r="B147" t="s">
-        <v>314</v>
+        <v>319</v>
       </c>
       <c r="C147" t="s">
-        <v>332</v>
+        <v>343</v>
       </c>
       <c r="D147">
         <v>1</v>
@@ -4793,7 +4838,7 @@
         <v>1</v>
       </c>
       <c r="F147" t="s">
-        <v>469</v>
+        <v>480</v>
       </c>
     </row>
     <row r="148" spans="1:6">
@@ -4801,10 +4846,10 @@
         <v>152</v>
       </c>
       <c r="B148" t="s">
-        <v>315</v>
+        <v>320</v>
       </c>
       <c r="C148" t="s">
-        <v>332</v>
+        <v>343</v>
       </c>
       <c r="D148">
         <v>1</v>
@@ -4813,7 +4858,7 @@
         <v>1</v>
       </c>
       <c r="F148" t="s">
-        <v>470</v>
+        <v>481</v>
       </c>
     </row>
     <row r="149" spans="1:6">
@@ -4821,10 +4866,10 @@
         <v>153</v>
       </c>
       <c r="B149" t="s">
-        <v>316</v>
+        <v>321</v>
       </c>
       <c r="C149" t="s">
-        <v>332</v>
+        <v>343</v>
       </c>
       <c r="D149">
         <v>1</v>
@@ -4833,7 +4878,7 @@
         <v>1</v>
       </c>
       <c r="F149" t="s">
-        <v>471</v>
+        <v>482</v>
       </c>
     </row>
     <row r="150" spans="1:6">
@@ -4841,10 +4886,10 @@
         <v>154</v>
       </c>
       <c r="B150" t="s">
-        <v>317</v>
+        <v>322</v>
       </c>
       <c r="C150" t="s">
-        <v>333</v>
+        <v>343</v>
       </c>
       <c r="D150">
         <v>1</v>
@@ -4853,7 +4898,7 @@
         <v>1</v>
       </c>
       <c r="F150" t="s">
-        <v>348</v>
+        <v>483</v>
       </c>
     </row>
     <row r="151" spans="1:6">
@@ -4861,10 +4906,10 @@
         <v>155</v>
       </c>
       <c r="B151" t="s">
-        <v>318</v>
+        <v>323</v>
       </c>
       <c r="C151" t="s">
-        <v>333</v>
+        <v>342</v>
       </c>
       <c r="D151">
         <v>1</v>
@@ -4873,7 +4918,7 @@
         <v>1</v>
       </c>
       <c r="F151" t="s">
-        <v>472</v>
+        <v>381</v>
       </c>
     </row>
     <row r="152" spans="1:6">
@@ -4881,10 +4926,10 @@
         <v>156</v>
       </c>
       <c r="B152" t="s">
-        <v>319</v>
+        <v>324</v>
       </c>
       <c r="C152" t="s">
-        <v>333</v>
+        <v>342</v>
       </c>
       <c r="D152">
         <v>1</v>
@@ -4893,7 +4938,7 @@
         <v>1</v>
       </c>
       <c r="F152" t="s">
-        <v>473</v>
+        <v>484</v>
       </c>
     </row>
     <row r="153" spans="1:6">
@@ -4901,10 +4946,10 @@
         <v>157</v>
       </c>
       <c r="B153" t="s">
-        <v>320</v>
+        <v>325</v>
       </c>
       <c r="C153" t="s">
-        <v>333</v>
+        <v>342</v>
       </c>
       <c r="D153">
         <v>1</v>
@@ -4913,7 +4958,7 @@
         <v>1</v>
       </c>
       <c r="F153" t="s">
-        <v>474</v>
+        <v>485</v>
       </c>
     </row>
     <row r="154" spans="1:6">
@@ -4921,10 +4966,10 @@
         <v>158</v>
       </c>
       <c r="B154" t="s">
-        <v>321</v>
+        <v>326</v>
       </c>
       <c r="C154" t="s">
-        <v>332</v>
+        <v>342</v>
       </c>
       <c r="D154">
         <v>1</v>
@@ -4933,7 +4978,7 @@
         <v>1</v>
       </c>
       <c r="F154" t="s">
-        <v>475</v>
+        <v>486</v>
       </c>
     </row>
     <row r="155" spans="1:6">
@@ -4941,10 +4986,10 @@
         <v>159</v>
       </c>
       <c r="B155" t="s">
-        <v>322</v>
+        <v>327</v>
       </c>
       <c r="C155" t="s">
-        <v>333</v>
+        <v>343</v>
       </c>
       <c r="D155">
         <v>1</v>
@@ -4953,7 +4998,7 @@
         <v>1</v>
       </c>
       <c r="F155" t="s">
-        <v>476</v>
+        <v>358</v>
       </c>
     </row>
     <row r="156" spans="1:6">
@@ -4961,10 +5006,10 @@
         <v>160</v>
       </c>
       <c r="B156" t="s">
-        <v>323</v>
+        <v>328</v>
       </c>
       <c r="C156" t="s">
-        <v>333</v>
+        <v>343</v>
       </c>
       <c r="D156">
         <v>1</v>
@@ -4973,7 +5018,7 @@
         <v>1</v>
       </c>
       <c r="F156" t="s">
-        <v>477</v>
+        <v>487</v>
       </c>
     </row>
     <row r="157" spans="1:6">
@@ -4981,10 +5026,10 @@
         <v>161</v>
       </c>
       <c r="B157" t="s">
-        <v>324</v>
+        <v>329</v>
       </c>
       <c r="C157" t="s">
-        <v>333</v>
+        <v>343</v>
       </c>
       <c r="D157">
         <v>1</v>
@@ -4993,7 +5038,7 @@
         <v>1</v>
       </c>
       <c r="F157" t="s">
-        <v>478</v>
+        <v>488</v>
       </c>
     </row>
     <row r="158" spans="1:6">
@@ -5001,10 +5046,10 @@
         <v>162</v>
       </c>
       <c r="B158" t="s">
-        <v>325</v>
+        <v>330</v>
       </c>
       <c r="C158" t="s">
-        <v>333</v>
+        <v>343</v>
       </c>
       <c r="D158">
         <v>1</v>
@@ -5013,7 +5058,7 @@
         <v>1</v>
       </c>
       <c r="F158" t="s">
-        <v>479</v>
+        <v>489</v>
       </c>
     </row>
     <row r="159" spans="1:6">
@@ -5021,10 +5066,10 @@
         <v>163</v>
       </c>
       <c r="B159" t="s">
-        <v>326</v>
+        <v>331</v>
       </c>
       <c r="C159" t="s">
-        <v>333</v>
+        <v>342</v>
       </c>
       <c r="D159">
         <v>1</v>
@@ -5033,7 +5078,7 @@
         <v>1</v>
       </c>
       <c r="F159" t="s">
-        <v>480</v>
+        <v>490</v>
       </c>
     </row>
     <row r="160" spans="1:6">
@@ -5041,10 +5086,10 @@
         <v>164</v>
       </c>
       <c r="B160" t="s">
-        <v>327</v>
+        <v>332</v>
       </c>
       <c r="C160" t="s">
-        <v>332</v>
+        <v>343</v>
       </c>
       <c r="D160">
         <v>1</v>
@@ -5053,7 +5098,7 @@
         <v>1</v>
       </c>
       <c r="F160" t="s">
-        <v>481</v>
+        <v>491</v>
       </c>
     </row>
     <row r="161" spans="1:6">
@@ -5061,10 +5106,10 @@
         <v>165</v>
       </c>
       <c r="B161" t="s">
-        <v>328</v>
+        <v>333</v>
       </c>
       <c r="C161" t="s">
-        <v>333</v>
+        <v>343</v>
       </c>
       <c r="D161">
         <v>1</v>
@@ -5073,7 +5118,7 @@
         <v>1</v>
       </c>
       <c r="F161" t="s">
-        <v>482</v>
+        <v>492</v>
       </c>
     </row>
     <row r="162" spans="1:6">
@@ -5081,10 +5126,10 @@
         <v>166</v>
       </c>
       <c r="B162" t="s">
-        <v>329</v>
+        <v>334</v>
       </c>
       <c r="C162" t="s">
-        <v>333</v>
+        <v>343</v>
       </c>
       <c r="D162">
         <v>1</v>
@@ -5093,7 +5138,7 @@
         <v>1</v>
       </c>
       <c r="F162" t="s">
-        <v>483</v>
+        <v>493</v>
       </c>
     </row>
     <row r="163" spans="1:6">
@@ -5101,10 +5146,10 @@
         <v>167</v>
       </c>
       <c r="B163" t="s">
-        <v>330</v>
+        <v>335</v>
       </c>
       <c r="C163" t="s">
-        <v>333</v>
+        <v>343</v>
       </c>
       <c r="D163">
         <v>1</v>
@@ -5113,7 +5158,7 @@
         <v>1</v>
       </c>
       <c r="F163" t="s">
-        <v>484</v>
+        <v>494</v>
       </c>
     </row>
     <row r="164" spans="1:6">
@@ -5121,10 +5166,10 @@
         <v>168</v>
       </c>
       <c r="B164" t="s">
-        <v>331</v>
+        <v>336</v>
       </c>
       <c r="C164" t="s">
-        <v>332</v>
+        <v>343</v>
       </c>
       <c r="D164">
         <v>1</v>
@@ -5133,7 +5178,107 @@
         <v>1</v>
       </c>
       <c r="F164" t="s">
-        <v>485</v>
+        <v>495</v>
+      </c>
+    </row>
+    <row r="165" spans="1:6">
+      <c r="A165" t="s">
+        <v>169</v>
+      </c>
+      <c r="B165" t="s">
+        <v>337</v>
+      </c>
+      <c r="C165" t="s">
+        <v>342</v>
+      </c>
+      <c r="D165">
+        <v>1</v>
+      </c>
+      <c r="E165">
+        <v>1</v>
+      </c>
+      <c r="F165" t="s">
+        <v>496</v>
+      </c>
+    </row>
+    <row r="166" spans="1:6">
+      <c r="A166" t="s">
+        <v>170</v>
+      </c>
+      <c r="B166" t="s">
+        <v>338</v>
+      </c>
+      <c r="C166" t="s">
+        <v>343</v>
+      </c>
+      <c r="D166">
+        <v>1</v>
+      </c>
+      <c r="E166">
+        <v>1</v>
+      </c>
+      <c r="F166" t="s">
+        <v>497</v>
+      </c>
+    </row>
+    <row r="167" spans="1:6">
+      <c r="A167" t="s">
+        <v>171</v>
+      </c>
+      <c r="B167" t="s">
+        <v>339</v>
+      </c>
+      <c r="C167" t="s">
+        <v>343</v>
+      </c>
+      <c r="D167">
+        <v>1</v>
+      </c>
+      <c r="E167">
+        <v>1</v>
+      </c>
+      <c r="F167" t="s">
+        <v>498</v>
+      </c>
+    </row>
+    <row r="168" spans="1:6">
+      <c r="A168" t="s">
+        <v>172</v>
+      </c>
+      <c r="B168" t="s">
+        <v>340</v>
+      </c>
+      <c r="C168" t="s">
+        <v>343</v>
+      </c>
+      <c r="D168">
+        <v>1</v>
+      </c>
+      <c r="E168">
+        <v>1</v>
+      </c>
+      <c r="F168" t="s">
+        <v>499</v>
+      </c>
+    </row>
+    <row r="169" spans="1:6">
+      <c r="A169" t="s">
+        <v>173</v>
+      </c>
+      <c r="B169" t="s">
+        <v>341</v>
+      </c>
+      <c r="C169" t="s">
+        <v>342</v>
+      </c>
+      <c r="D169">
+        <v>1</v>
+      </c>
+      <c r="E169">
+        <v>1</v>
+      </c>
+      <c r="F169" t="s">
+        <v>500</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
feat(ai): recover compliment, cute, hesitating, incomprehensible, leery into clean_emotion_words_2000_reviews
</commit_message>
<xml_diff>
--- a/data/derived_outputs/clean_emotion_words_2000_reviews.xlsx
+++ b/data/derived_outputs/clean_emotion_words_2000_reviews.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="678" uniqueCount="501">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="694" uniqueCount="512">
   <si>
     <t>word</t>
   </si>
@@ -241,12 +241,18 @@
     <t>captivated</t>
   </si>
   <si>
+    <t>compliment</t>
+  </si>
+  <si>
     <t>cordial</t>
   </si>
   <si>
     <t>curiosity</t>
   </si>
   <si>
+    <t>cute</t>
+  </si>
+  <si>
     <t>discouraged</t>
   </si>
   <si>
@@ -286,6 +292,9 @@
     <t>improving</t>
   </si>
   <si>
+    <t>incomprehensible</t>
+  </si>
+  <si>
     <t>indulge</t>
   </si>
   <si>
@@ -295,6 +304,9 @@
     <t>kindly</t>
   </si>
   <si>
+    <t>leery</t>
+  </si>
+  <si>
     <t>luscious</t>
   </si>
   <si>
@@ -745,12 +757,18 @@
     <t>被深深吸引着迷的</t>
   </si>
   <si>
+    <t>赞美 / 赞赏评价</t>
+  </si>
+  <si>
     <t>热情亲切礼貌的</t>
   </si>
   <si>
     <t>好奇心 / 探索欲</t>
   </si>
   <si>
+    <t>可爱宜人的</t>
+  </si>
+  <si>
     <t>感到灰心气馁的</t>
   </si>
   <si>
@@ -790,6 +808,9 @@
     <t>不断改善令人满意的</t>
   </si>
   <si>
+    <t>难以理解令人困惑的</t>
+  </si>
+  <si>
     <t>尽情享受 / 犒劳自己</t>
   </si>
   <si>
@@ -797,6 +818,9 @@
   </si>
   <si>
     <t>体贴友善地</t>
+  </si>
+  <si>
+    <t>提防警惕 / 顾虑重重的</t>
   </si>
   <si>
     <t>秀美令人心旷神怡的</t>
@@ -1261,6 +1285,9 @@
     <t>review_53fcd6e518ab4f8fb6d54d7d :: Unforgettable!  Views stunning, excellent pilot. We were captivated by all of it...views of Denali and surrounding mountains, glaciers, moose, sheep, trumpet swans. Landing on glac...</t>
   </si>
   <si>
+    <t>review_6d89a83a7e6c40e34fc3fabb :: From start to finish, our flightseeing tour from Talkeetna to Mt. McKinley, landing on Ruth Glacier was jaw-droppingly wonderful. I've lived in Alaska for almost 40 years and thoug...</t>
+  </si>
+  <si>
     <t>review_a6425ff1171e21e3392aa88c :: The personnel at Air Ventures cordial, helpful and polite.  I would recommend their services to anyone wanting to get a great aerial view of the Island of Kawaii.
 Our pilot, rob, ...</t>
   </si>
@@ -1268,6 +1295,9 @@
     <t>review_49cf9647abacf6af128bd5f4 :: Everything about Talkeetna Air Taxi oozes experience and professionalism.  From the initial decision process on which flight to take, to the actual flight itself, I could not have ...</t>
   </si>
   <si>
+    <t>review_57b73b29bbe868d4692cb554 :: Our original reservation fell during a cloudy evening, so the company advised delaying (without any fees) until the next morning.  It turned out to be the clearest day in weeks.  O...</t>
+  </si>
+  <si>
     <t>review_8fc23fecb45ba0ee94242f62 :: We are a family with 4 children ages 12 to 19 and spent a week on Kauai.  We really wanted to do an air tour with our kids but the cost of a helicopter flight would have been well ...</t>
   </si>
   <si>
@@ -1306,10 +1336,17 @@
 Ther...</t>
   </si>
   <si>
+    <t>review_c765b5e7676ff96bb64c9185 :: We did the Denali experience with a landing on the Eldridge Glacier and I can confidently say it was in the top 5 experiences of my life. I felt like a child again soaring past she...</t>
+  </si>
+  <si>
     <t>review_27ee31e44dec37dd44a492ba :: Eric, the pilot, is a amazing guy doing a great job! He said we are sharing his dream, actually he was making my dream come true by letting my little girl driving a little bit! Sou...</t>
   </si>
   <si>
     <t>review_91b07376e836c82b2b2ff5cc :: We had the open cockpit biplane flight beginning of February after booking online from the UK.  Jill kindly offered to collect/shuttle us from the ABC Store at Anchor Cove Shopping...</t>
+  </si>
+  <si>
+    <t>review_2c936441bbc2f31d7558ce47 :: Words cannot describe how amazing this tour is.
+From the office staff, to the ground crew, to the pilot; these people are fantastic.  The pilot went over all the emergency necessi...</t>
   </si>
   <si>
     <t>review_af6c769cd16b044c81ee438f :: My husband &amp; I were visiting Kauai from New York.  We were extremely fortunate to fly in a comfortable but small plane to view the luscious island of Kauai.  When we arrived for ou...</t>
@@ -1420,9 +1457,6 @@
   </si>
   <si>
     <t>review_ad4c129d7431549c0c82f1a8 :: Three of us signed up for the plane ride about a month in advance. There were really high winds that day (40 mph+), but the company didn't cancel so we went for the ride. 15 minute...</t>
-  </si>
-  <si>
-    <t>review_6d89a83a7e6c40e34fc3fabb :: From start to finish, our flightseeing tour from Talkeetna to Mt. McKinley, landing on Ruth Glacier was jaw-droppingly wonderful. I've lived in Alaska for almost 40 years and thoug...</t>
   </si>
   <si>
     <t>review_af9c2e4c708b6ef1ddffbdef :: We booked this as part of a Viator package to see Alcatraz and it completely blew us away.  We were a party of 4 - two adults, a ten year old and a 4 year old.  Despite a total fea...</t>
@@ -1898,7 +1932,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:F169"/>
+  <dimension ref="A1:F173"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:6">
@@ -1926,10 +1960,10 @@
         <v>6</v>
       </c>
       <c r="B2" t="s">
-        <v>174</v>
+        <v>178</v>
       </c>
       <c r="C2" t="s">
-        <v>342</v>
+        <v>350</v>
       </c>
       <c r="D2">
         <v>12</v>
@@ -1938,7 +1972,7 @@
         <v>12</v>
       </c>
       <c r="F2" t="s">
-        <v>345</v>
+        <v>353</v>
       </c>
     </row>
     <row r="3" spans="1:6">
@@ -1946,10 +1980,10 @@
         <v>7</v>
       </c>
       <c r="B3" t="s">
-        <v>175</v>
+        <v>179</v>
       </c>
       <c r="C3" t="s">
-        <v>343</v>
+        <v>351</v>
       </c>
       <c r="D3">
         <v>10</v>
@@ -1958,7 +1992,7 @@
         <v>10</v>
       </c>
       <c r="F3" t="s">
-        <v>346</v>
+        <v>354</v>
       </c>
     </row>
     <row r="4" spans="1:6">
@@ -1966,10 +2000,10 @@
         <v>8</v>
       </c>
       <c r="B4" t="s">
-        <v>176</v>
+        <v>180</v>
       </c>
       <c r="C4" t="s">
-        <v>343</v>
+        <v>351</v>
       </c>
       <c r="D4">
         <v>10</v>
@@ -1978,7 +2012,7 @@
         <v>9</v>
       </c>
       <c r="F4" t="s">
-        <v>347</v>
+        <v>355</v>
       </c>
     </row>
     <row r="5" spans="1:6">
@@ -1986,10 +2020,10 @@
         <v>9</v>
       </c>
       <c r="B5" t="s">
-        <v>177</v>
+        <v>181</v>
       </c>
       <c r="C5" t="s">
-        <v>343</v>
+        <v>351</v>
       </c>
       <c r="D5">
         <v>9</v>
@@ -1998,7 +2032,7 @@
         <v>9</v>
       </c>
       <c r="F5" t="s">
-        <v>348</v>
+        <v>356</v>
       </c>
     </row>
     <row r="6" spans="1:6">
@@ -2006,10 +2040,10 @@
         <v>10</v>
       </c>
       <c r="B6" t="s">
-        <v>178</v>
+        <v>182</v>
       </c>
       <c r="C6" t="s">
-        <v>343</v>
+        <v>351</v>
       </c>
       <c r="D6">
         <v>9</v>
@@ -2018,7 +2052,7 @@
         <v>9</v>
       </c>
       <c r="F6" t="s">
-        <v>349</v>
+        <v>357</v>
       </c>
     </row>
     <row r="7" spans="1:6">
@@ -2026,10 +2060,10 @@
         <v>11</v>
       </c>
       <c r="B7" t="s">
-        <v>179</v>
+        <v>183</v>
       </c>
       <c r="C7" t="s">
-        <v>343</v>
+        <v>351</v>
       </c>
       <c r="D7">
         <v>9</v>
@@ -2038,7 +2072,7 @@
         <v>9</v>
       </c>
       <c r="F7" t="s">
-        <v>350</v>
+        <v>358</v>
       </c>
     </row>
     <row r="8" spans="1:6">
@@ -2046,10 +2080,10 @@
         <v>12</v>
       </c>
       <c r="B8" t="s">
-        <v>180</v>
+        <v>184</v>
       </c>
       <c r="C8" t="s">
-        <v>343</v>
+        <v>351</v>
       </c>
       <c r="D8">
         <v>8</v>
@@ -2058,7 +2092,7 @@
         <v>8</v>
       </c>
       <c r="F8" t="s">
-        <v>351</v>
+        <v>359</v>
       </c>
     </row>
     <row r="9" spans="1:6">
@@ -2066,10 +2100,10 @@
         <v>13</v>
       </c>
       <c r="B9" t="s">
-        <v>181</v>
+        <v>185</v>
       </c>
       <c r="C9" t="s">
-        <v>342</v>
+        <v>350</v>
       </c>
       <c r="D9">
         <v>8</v>
@@ -2078,7 +2112,7 @@
         <v>8</v>
       </c>
       <c r="F9" t="s">
-        <v>352</v>
+        <v>360</v>
       </c>
     </row>
     <row r="10" spans="1:6">
@@ -2086,10 +2120,10 @@
         <v>14</v>
       </c>
       <c r="B10" t="s">
-        <v>182</v>
+        <v>186</v>
       </c>
       <c r="C10" t="s">
-        <v>342</v>
+        <v>350</v>
       </c>
       <c r="D10">
         <v>7</v>
@@ -2098,7 +2132,7 @@
         <v>7</v>
       </c>
       <c r="F10" t="s">
-        <v>353</v>
+        <v>361</v>
       </c>
     </row>
     <row r="11" spans="1:6">
@@ -2106,10 +2140,10 @@
         <v>15</v>
       </c>
       <c r="B11" t="s">
-        <v>183</v>
+        <v>187</v>
       </c>
       <c r="C11" t="s">
-        <v>343</v>
+        <v>351</v>
       </c>
       <c r="D11">
         <v>7</v>
@@ -2118,7 +2152,7 @@
         <v>7</v>
       </c>
       <c r="F11" t="s">
-        <v>354</v>
+        <v>362</v>
       </c>
     </row>
     <row r="12" spans="1:6">
@@ -2126,10 +2160,10 @@
         <v>16</v>
       </c>
       <c r="B12" t="s">
-        <v>184</v>
+        <v>188</v>
       </c>
       <c r="C12" t="s">
-        <v>343</v>
+        <v>351</v>
       </c>
       <c r="D12">
         <v>7</v>
@@ -2138,7 +2172,7 @@
         <v>7</v>
       </c>
       <c r="F12" t="s">
-        <v>355</v>
+        <v>363</v>
       </c>
     </row>
     <row r="13" spans="1:6">
@@ -2146,10 +2180,10 @@
         <v>17</v>
       </c>
       <c r="B13" t="s">
-        <v>185</v>
+        <v>189</v>
       </c>
       <c r="C13" t="s">
-        <v>343</v>
+        <v>351</v>
       </c>
       <c r="D13">
         <v>7</v>
@@ -2158,7 +2192,7 @@
         <v>7</v>
       </c>
       <c r="F13" t="s">
-        <v>356</v>
+        <v>364</v>
       </c>
     </row>
     <row r="14" spans="1:6">
@@ -2166,10 +2200,10 @@
         <v>18</v>
       </c>
       <c r="B14" t="s">
-        <v>186</v>
+        <v>190</v>
       </c>
       <c r="C14" t="s">
-        <v>343</v>
+        <v>351</v>
       </c>
       <c r="D14">
         <v>7</v>
@@ -2178,7 +2212,7 @@
         <v>6</v>
       </c>
       <c r="F14" t="s">
-        <v>357</v>
+        <v>365</v>
       </c>
     </row>
     <row r="15" spans="1:6">
@@ -2186,10 +2220,10 @@
         <v>19</v>
       </c>
       <c r="B15" t="s">
-        <v>187</v>
+        <v>191</v>
       </c>
       <c r="C15" t="s">
-        <v>343</v>
+        <v>351</v>
       </c>
       <c r="D15">
         <v>7</v>
@@ -2198,7 +2232,7 @@
         <v>7</v>
       </c>
       <c r="F15" t="s">
-        <v>348</v>
+        <v>356</v>
       </c>
     </row>
     <row r="16" spans="1:6">
@@ -2206,10 +2240,10 @@
         <v>20</v>
       </c>
       <c r="B16" t="s">
-        <v>188</v>
+        <v>192</v>
       </c>
       <c r="C16" t="s">
-        <v>343</v>
+        <v>351</v>
       </c>
       <c r="D16">
         <v>6</v>
@@ -2218,7 +2252,7 @@
         <v>6</v>
       </c>
       <c r="F16" t="s">
-        <v>358</v>
+        <v>366</v>
       </c>
     </row>
     <row r="17" spans="1:6">
@@ -2226,10 +2260,10 @@
         <v>21</v>
       </c>
       <c r="B17" t="s">
-        <v>189</v>
+        <v>193</v>
       </c>
       <c r="C17" t="s">
-        <v>342</v>
+        <v>350</v>
       </c>
       <c r="D17">
         <v>6</v>
@@ -2238,7 +2272,7 @@
         <v>6</v>
       </c>
       <c r="F17" t="s">
-        <v>359</v>
+        <v>367</v>
       </c>
     </row>
     <row r="18" spans="1:6">
@@ -2246,10 +2280,10 @@
         <v>22</v>
       </c>
       <c r="B18" t="s">
-        <v>190</v>
+        <v>194</v>
       </c>
       <c r="C18" t="s">
-        <v>343</v>
+        <v>351</v>
       </c>
       <c r="D18">
         <v>6</v>
@@ -2258,7 +2292,7 @@
         <v>6</v>
       </c>
       <c r="F18" t="s">
-        <v>360</v>
+        <v>368</v>
       </c>
     </row>
     <row r="19" spans="1:6">
@@ -2266,10 +2300,10 @@
         <v>23</v>
       </c>
       <c r="B19" t="s">
-        <v>191</v>
+        <v>195</v>
       </c>
       <c r="C19" t="s">
-        <v>343</v>
+        <v>351</v>
       </c>
       <c r="D19">
         <v>6</v>
@@ -2278,7 +2312,7 @@
         <v>5</v>
       </c>
       <c r="F19" t="s">
-        <v>361</v>
+        <v>369</v>
       </c>
     </row>
     <row r="20" spans="1:6">
@@ -2286,10 +2320,10 @@
         <v>24</v>
       </c>
       <c r="B20" t="s">
-        <v>192</v>
+        <v>196</v>
       </c>
       <c r="C20" t="s">
-        <v>342</v>
+        <v>350</v>
       </c>
       <c r="D20">
         <v>6</v>
@@ -2298,7 +2332,7 @@
         <v>6</v>
       </c>
       <c r="F20" t="s">
-        <v>362</v>
+        <v>370</v>
       </c>
     </row>
     <row r="21" spans="1:6">
@@ -2306,10 +2340,10 @@
         <v>25</v>
       </c>
       <c r="B21" t="s">
-        <v>193</v>
+        <v>197</v>
       </c>
       <c r="C21" t="s">
-        <v>342</v>
+        <v>350</v>
       </c>
       <c r="D21">
         <v>6</v>
@@ -2318,7 +2352,7 @@
         <v>5</v>
       </c>
       <c r="F21" t="s">
-        <v>363</v>
+        <v>371</v>
       </c>
     </row>
     <row r="22" spans="1:6">
@@ -2326,10 +2360,10 @@
         <v>26</v>
       </c>
       <c r="B22" t="s">
-        <v>194</v>
+        <v>198</v>
       </c>
       <c r="C22" t="s">
-        <v>342</v>
+        <v>350</v>
       </c>
       <c r="D22">
         <v>6</v>
@@ -2338,7 +2372,7 @@
         <v>6</v>
       </c>
       <c r="F22" t="s">
-        <v>364</v>
+        <v>372</v>
       </c>
     </row>
     <row r="23" spans="1:6">
@@ -2346,10 +2380,10 @@
         <v>27</v>
       </c>
       <c r="B23" t="s">
-        <v>195</v>
+        <v>199</v>
       </c>
       <c r="C23" t="s">
-        <v>342</v>
+        <v>350</v>
       </c>
       <c r="D23">
         <v>6</v>
@@ -2358,7 +2392,7 @@
         <v>6</v>
       </c>
       <c r="F23" t="s">
-        <v>365</v>
+        <v>373</v>
       </c>
     </row>
     <row r="24" spans="1:6">
@@ -2366,10 +2400,10 @@
         <v>28</v>
       </c>
       <c r="B24" t="s">
-        <v>196</v>
+        <v>200</v>
       </c>
       <c r="C24" t="s">
-        <v>343</v>
+        <v>351</v>
       </c>
       <c r="D24">
         <v>6</v>
@@ -2378,7 +2412,7 @@
         <v>6</v>
       </c>
       <c r="F24" t="s">
-        <v>366</v>
+        <v>374</v>
       </c>
     </row>
     <row r="25" spans="1:6">
@@ -2386,10 +2420,10 @@
         <v>29</v>
       </c>
       <c r="B25" t="s">
-        <v>197</v>
+        <v>201</v>
       </c>
       <c r="C25" t="s">
-        <v>342</v>
+        <v>350</v>
       </c>
       <c r="D25">
         <v>5</v>
@@ -2398,7 +2432,7 @@
         <v>5</v>
       </c>
       <c r="F25" t="s">
-        <v>367</v>
+        <v>375</v>
       </c>
     </row>
     <row r="26" spans="1:6">
@@ -2406,10 +2440,10 @@
         <v>30</v>
       </c>
       <c r="B26" t="s">
-        <v>198</v>
+        <v>202</v>
       </c>
       <c r="C26" t="s">
-        <v>343</v>
+        <v>351</v>
       </c>
       <c r="D26">
         <v>5</v>
@@ -2418,7 +2452,7 @@
         <v>5</v>
       </c>
       <c r="F26" t="s">
-        <v>368</v>
+        <v>376</v>
       </c>
     </row>
     <row r="27" spans="1:6">
@@ -2426,10 +2460,10 @@
         <v>31</v>
       </c>
       <c r="B27" t="s">
-        <v>199</v>
+        <v>203</v>
       </c>
       <c r="C27" t="s">
-        <v>343</v>
+        <v>351</v>
       </c>
       <c r="D27">
         <v>5</v>
@@ -2438,7 +2472,7 @@
         <v>4</v>
       </c>
       <c r="F27" t="s">
-        <v>369</v>
+        <v>377</v>
       </c>
     </row>
     <row r="28" spans="1:6">
@@ -2446,10 +2480,10 @@
         <v>32</v>
       </c>
       <c r="B28" t="s">
-        <v>200</v>
+        <v>204</v>
       </c>
       <c r="C28" t="s">
-        <v>343</v>
+        <v>351</v>
       </c>
       <c r="D28">
         <v>5</v>
@@ -2458,7 +2492,7 @@
         <v>5</v>
       </c>
       <c r="F28" t="s">
-        <v>370</v>
+        <v>378</v>
       </c>
     </row>
     <row r="29" spans="1:6">
@@ -2466,10 +2500,10 @@
         <v>33</v>
       </c>
       <c r="B29" t="s">
-        <v>201</v>
+        <v>205</v>
       </c>
       <c r="C29" t="s">
-        <v>342</v>
+        <v>350</v>
       </c>
       <c r="D29">
         <v>5</v>
@@ -2478,7 +2512,7 @@
         <v>5</v>
       </c>
       <c r="F29" t="s">
-        <v>371</v>
+        <v>379</v>
       </c>
     </row>
     <row r="30" spans="1:6">
@@ -2486,10 +2520,10 @@
         <v>34</v>
       </c>
       <c r="B30" t="s">
-        <v>202</v>
+        <v>206</v>
       </c>
       <c r="C30" t="s">
-        <v>343</v>
+        <v>351</v>
       </c>
       <c r="D30">
         <v>5</v>
@@ -2498,7 +2532,7 @@
         <v>5</v>
       </c>
       <c r="F30" t="s">
-        <v>372</v>
+        <v>380</v>
       </c>
     </row>
     <row r="31" spans="1:6">
@@ -2506,10 +2540,10 @@
         <v>35</v>
       </c>
       <c r="B31" t="s">
-        <v>203</v>
+        <v>207</v>
       </c>
       <c r="C31" t="s">
-        <v>343</v>
+        <v>351</v>
       </c>
       <c r="D31">
         <v>5</v>
@@ -2518,7 +2552,7 @@
         <v>4</v>
       </c>
       <c r="F31" t="s">
-        <v>373</v>
+        <v>381</v>
       </c>
     </row>
     <row r="32" spans="1:6">
@@ -2526,10 +2560,10 @@
         <v>36</v>
       </c>
       <c r="B32" t="s">
-        <v>204</v>
+        <v>208</v>
       </c>
       <c r="C32" t="s">
-        <v>343</v>
+        <v>351</v>
       </c>
       <c r="D32">
         <v>5</v>
@@ -2538,7 +2572,7 @@
         <v>5</v>
       </c>
       <c r="F32" t="s">
-        <v>374</v>
+        <v>382</v>
       </c>
     </row>
     <row r="33" spans="1:6">
@@ -2546,10 +2580,10 @@
         <v>37</v>
       </c>
       <c r="B33" t="s">
-        <v>205</v>
+        <v>209</v>
       </c>
       <c r="C33" t="s">
-        <v>342</v>
+        <v>350</v>
       </c>
       <c r="D33">
         <v>5</v>
@@ -2558,7 +2592,7 @@
         <v>5</v>
       </c>
       <c r="F33" t="s">
-        <v>375</v>
+        <v>383</v>
       </c>
     </row>
     <row r="34" spans="1:6">
@@ -2566,10 +2600,10 @@
         <v>38</v>
       </c>
       <c r="B34" t="s">
-        <v>206</v>
+        <v>210</v>
       </c>
       <c r="C34" t="s">
-        <v>343</v>
+        <v>351</v>
       </c>
       <c r="D34">
         <v>4</v>
@@ -2578,7 +2612,7 @@
         <v>4</v>
       </c>
       <c r="F34" t="s">
-        <v>376</v>
+        <v>384</v>
       </c>
     </row>
     <row r="35" spans="1:6">
@@ -2586,10 +2620,10 @@
         <v>39</v>
       </c>
       <c r="B35" t="s">
-        <v>207</v>
+        <v>211</v>
       </c>
       <c r="C35" t="s">
-        <v>342</v>
+        <v>350</v>
       </c>
       <c r="D35">
         <v>4</v>
@@ -2598,7 +2632,7 @@
         <v>4</v>
       </c>
       <c r="F35" t="s">
-        <v>377</v>
+        <v>385</v>
       </c>
     </row>
     <row r="36" spans="1:6">
@@ -2606,10 +2640,10 @@
         <v>40</v>
       </c>
       <c r="B36" t="s">
-        <v>208</v>
+        <v>212</v>
       </c>
       <c r="C36" t="s">
-        <v>342</v>
+        <v>350</v>
       </c>
       <c r="D36">
         <v>4</v>
@@ -2618,7 +2652,7 @@
         <v>4</v>
       </c>
       <c r="F36" t="s">
-        <v>378</v>
+        <v>386</v>
       </c>
     </row>
     <row r="37" spans="1:6">
@@ -2626,10 +2660,10 @@
         <v>41</v>
       </c>
       <c r="B37" t="s">
-        <v>209</v>
+        <v>213</v>
       </c>
       <c r="C37" t="s">
-        <v>342</v>
+        <v>350</v>
       </c>
       <c r="D37">
         <v>4</v>
@@ -2638,7 +2672,7 @@
         <v>4</v>
       </c>
       <c r="F37" t="s">
-        <v>379</v>
+        <v>387</v>
       </c>
     </row>
     <row r="38" spans="1:6">
@@ -2646,10 +2680,10 @@
         <v>42</v>
       </c>
       <c r="B38" t="s">
-        <v>210</v>
+        <v>214</v>
       </c>
       <c r="C38" t="s">
-        <v>342</v>
+        <v>350</v>
       </c>
       <c r="D38">
         <v>4</v>
@@ -2658,7 +2692,7 @@
         <v>3</v>
       </c>
       <c r="F38" t="s">
-        <v>380</v>
+        <v>388</v>
       </c>
     </row>
     <row r="39" spans="1:6">
@@ -2666,10 +2700,10 @@
         <v>43</v>
       </c>
       <c r="B39" t="s">
-        <v>211</v>
+        <v>215</v>
       </c>
       <c r="C39" t="s">
-        <v>342</v>
+        <v>350</v>
       </c>
       <c r="D39">
         <v>4</v>
@@ -2678,7 +2712,7 @@
         <v>4</v>
       </c>
       <c r="F39" t="s">
-        <v>381</v>
+        <v>389</v>
       </c>
     </row>
     <row r="40" spans="1:6">
@@ -2686,10 +2720,10 @@
         <v>44</v>
       </c>
       <c r="B40" t="s">
-        <v>212</v>
+        <v>216</v>
       </c>
       <c r="C40" t="s">
-        <v>342</v>
+        <v>350</v>
       </c>
       <c r="D40">
         <v>4</v>
@@ -2698,7 +2732,7 @@
         <v>4</v>
       </c>
       <c r="F40" t="s">
-        <v>382</v>
+        <v>390</v>
       </c>
     </row>
     <row r="41" spans="1:6">
@@ -2706,10 +2740,10 @@
         <v>45</v>
       </c>
       <c r="B41" t="s">
-        <v>213</v>
+        <v>217</v>
       </c>
       <c r="C41" t="s">
-        <v>342</v>
+        <v>350</v>
       </c>
       <c r="D41">
         <v>4</v>
@@ -2718,7 +2752,7 @@
         <v>4</v>
       </c>
       <c r="F41" t="s">
-        <v>383</v>
+        <v>391</v>
       </c>
     </row>
     <row r="42" spans="1:6">
@@ -2726,10 +2760,10 @@
         <v>46</v>
       </c>
       <c r="B42" t="s">
-        <v>214</v>
+        <v>218</v>
       </c>
       <c r="C42" t="s">
-        <v>343</v>
+        <v>351</v>
       </c>
       <c r="D42">
         <v>4</v>
@@ -2738,7 +2772,7 @@
         <v>4</v>
       </c>
       <c r="F42" t="s">
-        <v>384</v>
+        <v>392</v>
       </c>
     </row>
     <row r="43" spans="1:6">
@@ -2746,10 +2780,10 @@
         <v>47</v>
       </c>
       <c r="B43" t="s">
-        <v>215</v>
+        <v>219</v>
       </c>
       <c r="C43" t="s">
-        <v>343</v>
+        <v>351</v>
       </c>
       <c r="D43">
         <v>4</v>
@@ -2758,7 +2792,7 @@
         <v>4</v>
       </c>
       <c r="F43" t="s">
-        <v>385</v>
+        <v>393</v>
       </c>
     </row>
     <row r="44" spans="1:6">
@@ -2766,10 +2800,10 @@
         <v>48</v>
       </c>
       <c r="B44" t="s">
-        <v>216</v>
+        <v>220</v>
       </c>
       <c r="C44" t="s">
-        <v>343</v>
+        <v>351</v>
       </c>
       <c r="D44">
         <v>4</v>
@@ -2778,7 +2812,7 @@
         <v>4</v>
       </c>
       <c r="F44" t="s">
-        <v>386</v>
+        <v>394</v>
       </c>
     </row>
     <row r="45" spans="1:6">
@@ -2786,10 +2820,10 @@
         <v>49</v>
       </c>
       <c r="B45" t="s">
-        <v>217</v>
+        <v>221</v>
       </c>
       <c r="C45" t="s">
-        <v>343</v>
+        <v>351</v>
       </c>
       <c r="D45">
         <v>4</v>
@@ -2798,7 +2832,7 @@
         <v>4</v>
       </c>
       <c r="F45" t="s">
-        <v>387</v>
+        <v>395</v>
       </c>
     </row>
     <row r="46" spans="1:6">
@@ -2806,10 +2840,10 @@
         <v>50</v>
       </c>
       <c r="B46" t="s">
-        <v>218</v>
+        <v>222</v>
       </c>
       <c r="C46" t="s">
-        <v>344</v>
+        <v>352</v>
       </c>
       <c r="D46">
         <v>3</v>
@@ -2818,7 +2852,7 @@
         <v>3</v>
       </c>
       <c r="F46" t="s">
-        <v>388</v>
+        <v>396</v>
       </c>
     </row>
     <row r="47" spans="1:6">
@@ -2826,10 +2860,10 @@
         <v>51</v>
       </c>
       <c r="B47" t="s">
-        <v>219</v>
+        <v>223</v>
       </c>
       <c r="C47" t="s">
-        <v>342</v>
+        <v>350</v>
       </c>
       <c r="D47">
         <v>3</v>
@@ -2838,7 +2872,7 @@
         <v>3</v>
       </c>
       <c r="F47" t="s">
-        <v>389</v>
+        <v>397</v>
       </c>
     </row>
     <row r="48" spans="1:6">
@@ -2846,10 +2880,10 @@
         <v>52</v>
       </c>
       <c r="B48" t="s">
-        <v>220</v>
+        <v>224</v>
       </c>
       <c r="C48" t="s">
-        <v>343</v>
+        <v>351</v>
       </c>
       <c r="D48">
         <v>3</v>
@@ -2858,7 +2892,7 @@
         <v>3</v>
       </c>
       <c r="F48" t="s">
-        <v>390</v>
+        <v>398</v>
       </c>
     </row>
     <row r="49" spans="1:6">
@@ -2866,10 +2900,10 @@
         <v>53</v>
       </c>
       <c r="B49" t="s">
-        <v>221</v>
+        <v>225</v>
       </c>
       <c r="C49" t="s">
-        <v>342</v>
+        <v>350</v>
       </c>
       <c r="D49">
         <v>3</v>
@@ -2878,7 +2912,7 @@
         <v>3</v>
       </c>
       <c r="F49" t="s">
-        <v>391</v>
+        <v>399</v>
       </c>
     </row>
     <row r="50" spans="1:6">
@@ -2886,10 +2920,10 @@
         <v>54</v>
       </c>
       <c r="B50" t="s">
-        <v>222</v>
+        <v>226</v>
       </c>
       <c r="C50" t="s">
-        <v>342</v>
+        <v>350</v>
       </c>
       <c r="D50">
         <v>3</v>
@@ -2898,7 +2932,7 @@
         <v>3</v>
       </c>
       <c r="F50" t="s">
-        <v>392</v>
+        <v>400</v>
       </c>
     </row>
     <row r="51" spans="1:6">
@@ -2906,10 +2940,10 @@
         <v>55</v>
       </c>
       <c r="B51" t="s">
-        <v>223</v>
+        <v>227</v>
       </c>
       <c r="C51" t="s">
-        <v>343</v>
+        <v>351</v>
       </c>
       <c r="D51">
         <v>3</v>
@@ -2918,7 +2952,7 @@
         <v>3</v>
       </c>
       <c r="F51" t="s">
-        <v>393</v>
+        <v>401</v>
       </c>
     </row>
     <row r="52" spans="1:6">
@@ -2926,10 +2960,10 @@
         <v>56</v>
       </c>
       <c r="B52" t="s">
-        <v>224</v>
+        <v>228</v>
       </c>
       <c r="C52" t="s">
-        <v>343</v>
+        <v>351</v>
       </c>
       <c r="D52">
         <v>3</v>
@@ -2938,7 +2972,7 @@
         <v>3</v>
       </c>
       <c r="F52" t="s">
-        <v>394</v>
+        <v>402</v>
       </c>
     </row>
     <row r="53" spans="1:6">
@@ -2946,10 +2980,10 @@
         <v>57</v>
       </c>
       <c r="B53" t="s">
-        <v>225</v>
+        <v>229</v>
       </c>
       <c r="C53" t="s">
-        <v>343</v>
+        <v>351</v>
       </c>
       <c r="D53">
         <v>3</v>
@@ -2958,7 +2992,7 @@
         <v>3</v>
       </c>
       <c r="F53" t="s">
-        <v>395</v>
+        <v>403</v>
       </c>
     </row>
     <row r="54" spans="1:6">
@@ -2966,10 +3000,10 @@
         <v>58</v>
       </c>
       <c r="B54" t="s">
-        <v>226</v>
+        <v>230</v>
       </c>
       <c r="C54" t="s">
-        <v>342</v>
+        <v>350</v>
       </c>
       <c r="D54">
         <v>3</v>
@@ -2978,7 +3012,7 @@
         <v>3</v>
       </c>
       <c r="F54" t="s">
-        <v>396</v>
+        <v>404</v>
       </c>
     </row>
     <row r="55" spans="1:6">
@@ -2986,10 +3020,10 @@
         <v>59</v>
       </c>
       <c r="B55" t="s">
-        <v>227</v>
+        <v>231</v>
       </c>
       <c r="C55" t="s">
-        <v>343</v>
+        <v>351</v>
       </c>
       <c r="D55">
         <v>3</v>
@@ -2998,7 +3032,7 @@
         <v>3</v>
       </c>
       <c r="F55" t="s">
-        <v>397</v>
+        <v>405</v>
       </c>
     </row>
     <row r="56" spans="1:6">
@@ -3006,10 +3040,10 @@
         <v>60</v>
       </c>
       <c r="B56" t="s">
-        <v>228</v>
+        <v>232</v>
       </c>
       <c r="C56" t="s">
-        <v>343</v>
+        <v>351</v>
       </c>
       <c r="D56">
         <v>3</v>
@@ -3018,7 +3052,7 @@
         <v>3</v>
       </c>
       <c r="F56" t="s">
-        <v>398</v>
+        <v>406</v>
       </c>
     </row>
     <row r="57" spans="1:6">
@@ -3026,10 +3060,10 @@
         <v>61</v>
       </c>
       <c r="B57" t="s">
-        <v>229</v>
+        <v>233</v>
       </c>
       <c r="C57" t="s">
-        <v>343</v>
+        <v>351</v>
       </c>
       <c r="D57">
         <v>3</v>
@@ -3038,7 +3072,7 @@
         <v>3</v>
       </c>
       <c r="F57" t="s">
-        <v>399</v>
+        <v>407</v>
       </c>
     </row>
     <row r="58" spans="1:6">
@@ -3046,10 +3080,10 @@
         <v>62</v>
       </c>
       <c r="B58" t="s">
-        <v>230</v>
+        <v>234</v>
       </c>
       <c r="C58" t="s">
-        <v>343</v>
+        <v>351</v>
       </c>
       <c r="D58">
         <v>3</v>
@@ -3058,7 +3092,7 @@
         <v>3</v>
       </c>
       <c r="F58" t="s">
-        <v>400</v>
+        <v>408</v>
       </c>
     </row>
     <row r="59" spans="1:6">
@@ -3066,10 +3100,10 @@
         <v>63</v>
       </c>
       <c r="B59" t="s">
-        <v>231</v>
+        <v>235</v>
       </c>
       <c r="C59" t="s">
-        <v>342</v>
+        <v>350</v>
       </c>
       <c r="D59">
         <v>3</v>
@@ -3078,7 +3112,7 @@
         <v>3</v>
       </c>
       <c r="F59" t="s">
-        <v>401</v>
+        <v>409</v>
       </c>
     </row>
     <row r="60" spans="1:6">
@@ -3086,10 +3120,10 @@
         <v>64</v>
       </c>
       <c r="B60" t="s">
-        <v>232</v>
+        <v>236</v>
       </c>
       <c r="C60" t="s">
-        <v>343</v>
+        <v>351</v>
       </c>
       <c r="D60">
         <v>3</v>
@@ -3098,7 +3132,7 @@
         <v>3</v>
       </c>
       <c r="F60" t="s">
-        <v>402</v>
+        <v>410</v>
       </c>
     </row>
     <row r="61" spans="1:6">
@@ -3106,10 +3140,10 @@
         <v>65</v>
       </c>
       <c r="B61" t="s">
-        <v>233</v>
+        <v>237</v>
       </c>
       <c r="C61" t="s">
-        <v>342</v>
+        <v>350</v>
       </c>
       <c r="D61">
         <v>3</v>
@@ -3118,7 +3152,7 @@
         <v>3</v>
       </c>
       <c r="F61" t="s">
-        <v>403</v>
+        <v>411</v>
       </c>
     </row>
     <row r="62" spans="1:6">
@@ -3126,10 +3160,10 @@
         <v>66</v>
       </c>
       <c r="B62" t="s">
-        <v>234</v>
+        <v>238</v>
       </c>
       <c r="C62" t="s">
-        <v>343</v>
+        <v>351</v>
       </c>
       <c r="D62">
         <v>3</v>
@@ -3138,7 +3172,7 @@
         <v>3</v>
       </c>
       <c r="F62" t="s">
-        <v>404</v>
+        <v>412</v>
       </c>
     </row>
     <row r="63" spans="1:6">
@@ -3146,10 +3180,10 @@
         <v>67</v>
       </c>
       <c r="B63" t="s">
-        <v>235</v>
+        <v>239</v>
       </c>
       <c r="C63" t="s">
-        <v>343</v>
+        <v>351</v>
       </c>
       <c r="D63">
         <v>2</v>
@@ -3158,7 +3192,7 @@
         <v>2</v>
       </c>
       <c r="F63" t="s">
-        <v>405</v>
+        <v>413</v>
       </c>
     </row>
     <row r="64" spans="1:6">
@@ -3166,10 +3200,10 @@
         <v>68</v>
       </c>
       <c r="B64" t="s">
-        <v>236</v>
+        <v>240</v>
       </c>
       <c r="C64" t="s">
-        <v>343</v>
+        <v>351</v>
       </c>
       <c r="D64">
         <v>2</v>
@@ -3178,7 +3212,7 @@
         <v>2</v>
       </c>
       <c r="F64" t="s">
-        <v>406</v>
+        <v>414</v>
       </c>
     </row>
     <row r="65" spans="1:6">
@@ -3186,10 +3220,10 @@
         <v>69</v>
       </c>
       <c r="B65" t="s">
-        <v>237</v>
+        <v>241</v>
       </c>
       <c r="C65" t="s">
-        <v>343</v>
+        <v>351</v>
       </c>
       <c r="D65">
         <v>2</v>
@@ -3198,7 +3232,7 @@
         <v>2</v>
       </c>
       <c r="F65" t="s">
-        <v>407</v>
+        <v>415</v>
       </c>
     </row>
     <row r="66" spans="1:6">
@@ -3206,10 +3240,10 @@
         <v>70</v>
       </c>
       <c r="B66" t="s">
-        <v>238</v>
+        <v>242</v>
       </c>
       <c r="C66" t="s">
-        <v>342</v>
+        <v>350</v>
       </c>
       <c r="D66">
         <v>2</v>
@@ -3218,7 +3252,7 @@
         <v>2</v>
       </c>
       <c r="F66" t="s">
-        <v>408</v>
+        <v>416</v>
       </c>
     </row>
     <row r="67" spans="1:6">
@@ -3226,10 +3260,10 @@
         <v>71</v>
       </c>
       <c r="B67" t="s">
-        <v>239</v>
+        <v>243</v>
       </c>
       <c r="C67" t="s">
-        <v>342</v>
+        <v>350</v>
       </c>
       <c r="D67">
         <v>2</v>
@@ -3238,7 +3272,7 @@
         <v>2</v>
       </c>
       <c r="F67" t="s">
-        <v>385</v>
+        <v>393</v>
       </c>
     </row>
     <row r="68" spans="1:6">
@@ -3246,10 +3280,10 @@
         <v>72</v>
       </c>
       <c r="B68" t="s">
-        <v>240</v>
+        <v>244</v>
       </c>
       <c r="C68" t="s">
-        <v>343</v>
+        <v>351</v>
       </c>
       <c r="D68">
         <v>2</v>
@@ -3258,7 +3292,7 @@
         <v>2</v>
       </c>
       <c r="F68" t="s">
-        <v>409</v>
+        <v>417</v>
       </c>
     </row>
     <row r="69" spans="1:6">
@@ -3266,10 +3300,10 @@
         <v>73</v>
       </c>
       <c r="B69" t="s">
-        <v>241</v>
+        <v>245</v>
       </c>
       <c r="C69" t="s">
-        <v>342</v>
+        <v>350</v>
       </c>
       <c r="D69">
         <v>2</v>
@@ -3278,7 +3312,7 @@
         <v>2</v>
       </c>
       <c r="F69" t="s">
-        <v>410</v>
+        <v>418</v>
       </c>
     </row>
     <row r="70" spans="1:6">
@@ -3286,10 +3320,10 @@
         <v>74</v>
       </c>
       <c r="B70" t="s">
-        <v>242</v>
+        <v>246</v>
       </c>
       <c r="C70" t="s">
-        <v>342</v>
+        <v>350</v>
       </c>
       <c r="D70">
         <v>2</v>
@@ -3298,7 +3332,7 @@
         <v>2</v>
       </c>
       <c r="F70" t="s">
-        <v>411</v>
+        <v>419</v>
       </c>
     </row>
     <row r="71" spans="1:6">
@@ -3306,10 +3340,10 @@
         <v>75</v>
       </c>
       <c r="B71" t="s">
-        <v>243</v>
+        <v>247</v>
       </c>
       <c r="C71" t="s">
-        <v>343</v>
+        <v>351</v>
       </c>
       <c r="D71">
         <v>2</v>
@@ -3318,7 +3352,7 @@
         <v>2</v>
       </c>
       <c r="F71" t="s">
-        <v>412</v>
+        <v>420</v>
       </c>
     </row>
     <row r="72" spans="1:6">
@@ -3326,10 +3360,10 @@
         <v>76</v>
       </c>
       <c r="B72" t="s">
-        <v>244</v>
+        <v>248</v>
       </c>
       <c r="C72" t="s">
-        <v>342</v>
+        <v>351</v>
       </c>
       <c r="D72">
         <v>2</v>
@@ -3338,7 +3372,7 @@
         <v>2</v>
       </c>
       <c r="F72" t="s">
-        <v>413</v>
+        <v>421</v>
       </c>
     </row>
     <row r="73" spans="1:6">
@@ -3346,10 +3380,10 @@
         <v>77</v>
       </c>
       <c r="B73" t="s">
-        <v>245</v>
+        <v>249</v>
       </c>
       <c r="C73" t="s">
-        <v>342</v>
+        <v>350</v>
       </c>
       <c r="D73">
         <v>2</v>
@@ -3358,7 +3392,7 @@
         <v>2</v>
       </c>
       <c r="F73" t="s">
-        <v>414</v>
+        <v>422</v>
       </c>
     </row>
     <row r="74" spans="1:6">
@@ -3366,10 +3400,10 @@
         <v>78</v>
       </c>
       <c r="B74" t="s">
-        <v>246</v>
+        <v>250</v>
       </c>
       <c r="C74" t="s">
-        <v>342</v>
+        <v>351</v>
       </c>
       <c r="D74">
         <v>2</v>
@@ -3378,7 +3412,7 @@
         <v>2</v>
       </c>
       <c r="F74" t="s">
-        <v>415</v>
+        <v>423</v>
       </c>
     </row>
     <row r="75" spans="1:6">
@@ -3386,10 +3420,10 @@
         <v>79</v>
       </c>
       <c r="B75" t="s">
-        <v>247</v>
+        <v>251</v>
       </c>
       <c r="C75" t="s">
-        <v>342</v>
+        <v>350</v>
       </c>
       <c r="D75">
         <v>2</v>
@@ -3398,7 +3432,7 @@
         <v>2</v>
       </c>
       <c r="F75" t="s">
-        <v>416</v>
+        <v>424</v>
       </c>
     </row>
     <row r="76" spans="1:6">
@@ -3406,10 +3440,10 @@
         <v>80</v>
       </c>
       <c r="B76" t="s">
-        <v>248</v>
+        <v>252</v>
       </c>
       <c r="C76" t="s">
-        <v>343</v>
+        <v>350</v>
       </c>
       <c r="D76">
         <v>2</v>
@@ -3418,7 +3452,7 @@
         <v>2</v>
       </c>
       <c r="F76" t="s">
-        <v>417</v>
+        <v>425</v>
       </c>
     </row>
     <row r="77" spans="1:6">
@@ -3426,10 +3460,10 @@
         <v>81</v>
       </c>
       <c r="B77" t="s">
-        <v>249</v>
+        <v>253</v>
       </c>
       <c r="C77" t="s">
-        <v>343</v>
+        <v>350</v>
       </c>
       <c r="D77">
         <v>2</v>
@@ -3438,7 +3472,7 @@
         <v>2</v>
       </c>
       <c r="F77" t="s">
-        <v>418</v>
+        <v>426</v>
       </c>
     </row>
     <row r="78" spans="1:6">
@@ -3446,10 +3480,10 @@
         <v>82</v>
       </c>
       <c r="B78" t="s">
-        <v>250</v>
+        <v>254</v>
       </c>
       <c r="C78" t="s">
-        <v>343</v>
+        <v>351</v>
       </c>
       <c r="D78">
         <v>2</v>
@@ -3458,7 +3492,7 @@
         <v>2</v>
       </c>
       <c r="F78" t="s">
-        <v>419</v>
+        <v>427</v>
       </c>
     </row>
     <row r="79" spans="1:6">
@@ -3466,10 +3500,10 @@
         <v>83</v>
       </c>
       <c r="B79" t="s">
-        <v>251</v>
+        <v>255</v>
       </c>
       <c r="C79" t="s">
-        <v>342</v>
+        <v>351</v>
       </c>
       <c r="D79">
         <v>2</v>
@@ -3478,7 +3512,7 @@
         <v>2</v>
       </c>
       <c r="F79" t="s">
-        <v>420</v>
+        <v>428</v>
       </c>
     </row>
     <row r="80" spans="1:6">
@@ -3486,10 +3520,10 @@
         <v>84</v>
       </c>
       <c r="B80" t="s">
-        <v>252</v>
+        <v>256</v>
       </c>
       <c r="C80" t="s">
-        <v>342</v>
+        <v>351</v>
       </c>
       <c r="D80">
         <v>2</v>
@@ -3498,7 +3532,7 @@
         <v>2</v>
       </c>
       <c r="F80" t="s">
-        <v>421</v>
+        <v>429</v>
       </c>
     </row>
     <row r="81" spans="1:6">
@@ -3506,10 +3540,10 @@
         <v>85</v>
       </c>
       <c r="B81" t="s">
-        <v>253</v>
+        <v>257</v>
       </c>
       <c r="C81" t="s">
-        <v>343</v>
+        <v>350</v>
       </c>
       <c r="D81">
         <v>2</v>
@@ -3518,7 +3552,7 @@
         <v>2</v>
       </c>
       <c r="F81" t="s">
-        <v>422</v>
+        <v>430</v>
       </c>
     </row>
     <row r="82" spans="1:6">
@@ -3526,10 +3560,10 @@
         <v>86</v>
       </c>
       <c r="B82" t="s">
-        <v>254</v>
+        <v>258</v>
       </c>
       <c r="C82" t="s">
-        <v>343</v>
+        <v>350</v>
       </c>
       <c r="D82">
         <v>2</v>
@@ -3538,7 +3572,7 @@
         <v>2</v>
       </c>
       <c r="F82" t="s">
-        <v>423</v>
+        <v>431</v>
       </c>
     </row>
     <row r="83" spans="1:6">
@@ -3546,10 +3580,10 @@
         <v>87</v>
       </c>
       <c r="B83" t="s">
-        <v>255</v>
+        <v>259</v>
       </c>
       <c r="C83" t="s">
-        <v>343</v>
+        <v>351</v>
       </c>
       <c r="D83">
         <v>2</v>
@@ -3558,7 +3592,7 @@
         <v>2</v>
       </c>
       <c r="F83" t="s">
-        <v>424</v>
+        <v>432</v>
       </c>
     </row>
     <row r="84" spans="1:6">
@@ -3566,19 +3600,19 @@
         <v>88</v>
       </c>
       <c r="B84" t="s">
-        <v>256</v>
+        <v>260</v>
       </c>
       <c r="C84" t="s">
-        <v>343</v>
+        <v>351</v>
       </c>
       <c r="D84">
         <v>2</v>
       </c>
       <c r="E84">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="F84" t="s">
-        <v>425</v>
+        <v>433</v>
       </c>
     </row>
     <row r="85" spans="1:6">
@@ -3586,10 +3620,10 @@
         <v>89</v>
       </c>
       <c r="B85" t="s">
-        <v>257</v>
+        <v>261</v>
       </c>
       <c r="C85" t="s">
-        <v>343</v>
+        <v>351</v>
       </c>
       <c r="D85">
         <v>2</v>
@@ -3598,7 +3632,7 @@
         <v>2</v>
       </c>
       <c r="F85" t="s">
-        <v>378</v>
+        <v>434</v>
       </c>
     </row>
     <row r="86" spans="1:6">
@@ -3606,19 +3640,19 @@
         <v>90</v>
       </c>
       <c r="B86" t="s">
-        <v>258</v>
+        <v>262</v>
       </c>
       <c r="C86" t="s">
-        <v>342</v>
+        <v>351</v>
       </c>
       <c r="D86">
         <v>2</v>
       </c>
       <c r="E86">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="F86" t="s">
-        <v>366</v>
+        <v>435</v>
       </c>
     </row>
     <row r="87" spans="1:6">
@@ -3626,10 +3660,10 @@
         <v>91</v>
       </c>
       <c r="B87" t="s">
-        <v>259</v>
+        <v>263</v>
       </c>
       <c r="C87" t="s">
-        <v>342</v>
+        <v>351</v>
       </c>
       <c r="D87">
         <v>2</v>
@@ -3638,7 +3672,7 @@
         <v>2</v>
       </c>
       <c r="F87" t="s">
-        <v>426</v>
+        <v>386</v>
       </c>
     </row>
     <row r="88" spans="1:6">
@@ -3646,10 +3680,10 @@
         <v>92</v>
       </c>
       <c r="B88" t="s">
-        <v>260</v>
+        <v>264</v>
       </c>
       <c r="C88" t="s">
-        <v>343</v>
+        <v>351</v>
       </c>
       <c r="D88">
         <v>2</v>
@@ -3658,7 +3692,7 @@
         <v>2</v>
       </c>
       <c r="F88" t="s">
-        <v>427</v>
+        <v>436</v>
       </c>
     </row>
     <row r="89" spans="1:6">
@@ -3666,10 +3700,10 @@
         <v>93</v>
       </c>
       <c r="B89" t="s">
-        <v>261</v>
+        <v>265</v>
       </c>
       <c r="C89" t="s">
-        <v>343</v>
+        <v>350</v>
       </c>
       <c r="D89">
         <v>2</v>
@@ -3678,7 +3712,7 @@
         <v>2</v>
       </c>
       <c r="F89" t="s">
-        <v>428</v>
+        <v>374</v>
       </c>
     </row>
     <row r="90" spans="1:6">
@@ -3686,10 +3720,10 @@
         <v>94</v>
       </c>
       <c r="B90" t="s">
-        <v>262</v>
+        <v>266</v>
       </c>
       <c r="C90" t="s">
-        <v>343</v>
+        <v>350</v>
       </c>
       <c r="D90">
         <v>2</v>
@@ -3698,7 +3732,7 @@
         <v>2</v>
       </c>
       <c r="F90" t="s">
-        <v>349</v>
+        <v>437</v>
       </c>
     </row>
     <row r="91" spans="1:6">
@@ -3706,10 +3740,10 @@
         <v>95</v>
       </c>
       <c r="B91" t="s">
-        <v>263</v>
+        <v>267</v>
       </c>
       <c r="C91" t="s">
-        <v>343</v>
+        <v>351</v>
       </c>
       <c r="D91">
         <v>2</v>
@@ -3718,7 +3752,7 @@
         <v>2</v>
       </c>
       <c r="F91" t="s">
-        <v>429</v>
+        <v>438</v>
       </c>
     </row>
     <row r="92" spans="1:6">
@@ -3726,10 +3760,10 @@
         <v>96</v>
       </c>
       <c r="B92" t="s">
-        <v>264</v>
+        <v>268</v>
       </c>
       <c r="C92" t="s">
-        <v>343</v>
+        <v>350</v>
       </c>
       <c r="D92">
         <v>2</v>
@@ -3738,7 +3772,7 @@
         <v>2</v>
       </c>
       <c r="F92" t="s">
-        <v>430</v>
+        <v>439</v>
       </c>
     </row>
     <row r="93" spans="1:6">
@@ -3746,10 +3780,10 @@
         <v>97</v>
       </c>
       <c r="B93" t="s">
-        <v>265</v>
+        <v>269</v>
       </c>
       <c r="C93" t="s">
-        <v>343</v>
+        <v>351</v>
       </c>
       <c r="D93">
         <v>2</v>
@@ -3758,7 +3792,7 @@
         <v>2</v>
       </c>
       <c r="F93" t="s">
-        <v>431</v>
+        <v>440</v>
       </c>
     </row>
     <row r="94" spans="1:6">
@@ -3766,10 +3800,10 @@
         <v>98</v>
       </c>
       <c r="B94" t="s">
-        <v>266</v>
+        <v>270</v>
       </c>
       <c r="C94" t="s">
-        <v>343</v>
+        <v>351</v>
       </c>
       <c r="D94">
         <v>2</v>
@@ -3778,7 +3812,7 @@
         <v>2</v>
       </c>
       <c r="F94" t="s">
-        <v>432</v>
+        <v>357</v>
       </c>
     </row>
     <row r="95" spans="1:6">
@@ -3786,10 +3820,10 @@
         <v>99</v>
       </c>
       <c r="B95" t="s">
-        <v>267</v>
+        <v>271</v>
       </c>
       <c r="C95" t="s">
-        <v>343</v>
+        <v>351</v>
       </c>
       <c r="D95">
         <v>2</v>
@@ -3798,7 +3832,7 @@
         <v>2</v>
       </c>
       <c r="F95" t="s">
-        <v>433</v>
+        <v>441</v>
       </c>
     </row>
     <row r="96" spans="1:6">
@@ -3806,10 +3840,10 @@
         <v>100</v>
       </c>
       <c r="B96" t="s">
-        <v>268</v>
+        <v>272</v>
       </c>
       <c r="C96" t="s">
-        <v>343</v>
+        <v>351</v>
       </c>
       <c r="D96">
         <v>2</v>
@@ -3818,7 +3852,7 @@
         <v>2</v>
       </c>
       <c r="F96" t="s">
-        <v>434</v>
+        <v>442</v>
       </c>
     </row>
     <row r="97" spans="1:6">
@@ -3826,10 +3860,10 @@
         <v>101</v>
       </c>
       <c r="B97" t="s">
-        <v>269</v>
+        <v>273</v>
       </c>
       <c r="C97" t="s">
-        <v>343</v>
+        <v>351</v>
       </c>
       <c r="D97">
         <v>2</v>
@@ -3838,7 +3872,7 @@
         <v>2</v>
       </c>
       <c r="F97" t="s">
-        <v>435</v>
+        <v>443</v>
       </c>
     </row>
     <row r="98" spans="1:6">
@@ -3846,10 +3880,10 @@
         <v>102</v>
       </c>
       <c r="B98" t="s">
-        <v>270</v>
+        <v>274</v>
       </c>
       <c r="C98" t="s">
-        <v>343</v>
+        <v>351</v>
       </c>
       <c r="D98">
         <v>2</v>
@@ -3858,7 +3892,7 @@
         <v>2</v>
       </c>
       <c r="F98" t="s">
-        <v>436</v>
+        <v>444</v>
       </c>
     </row>
     <row r="99" spans="1:6">
@@ -3866,10 +3900,10 @@
         <v>103</v>
       </c>
       <c r="B99" t="s">
-        <v>271</v>
+        <v>275</v>
       </c>
       <c r="C99" t="s">
-        <v>343</v>
+        <v>351</v>
       </c>
       <c r="D99">
         <v>2</v>
@@ -3878,7 +3912,7 @@
         <v>2</v>
       </c>
       <c r="F99" t="s">
-        <v>437</v>
+        <v>445</v>
       </c>
     </row>
     <row r="100" spans="1:6">
@@ -3886,10 +3920,10 @@
         <v>104</v>
       </c>
       <c r="B100" t="s">
-        <v>272</v>
+        <v>276</v>
       </c>
       <c r="C100" t="s">
-        <v>343</v>
+        <v>351</v>
       </c>
       <c r="D100">
         <v>2</v>
@@ -3898,7 +3932,7 @@
         <v>2</v>
       </c>
       <c r="F100" t="s">
-        <v>438</v>
+        <v>446</v>
       </c>
     </row>
     <row r="101" spans="1:6">
@@ -3906,10 +3940,10 @@
         <v>105</v>
       </c>
       <c r="B101" t="s">
-        <v>273</v>
+        <v>277</v>
       </c>
       <c r="C101" t="s">
-        <v>343</v>
+        <v>351</v>
       </c>
       <c r="D101">
         <v>2</v>
@@ -3918,7 +3952,7 @@
         <v>2</v>
       </c>
       <c r="F101" t="s">
-        <v>439</v>
+        <v>447</v>
       </c>
     </row>
     <row r="102" spans="1:6">
@@ -3926,10 +3960,10 @@
         <v>106</v>
       </c>
       <c r="B102" t="s">
-        <v>274</v>
+        <v>278</v>
       </c>
       <c r="C102" t="s">
-        <v>342</v>
+        <v>351</v>
       </c>
       <c r="D102">
         <v>2</v>
@@ -3938,7 +3972,7 @@
         <v>2</v>
       </c>
       <c r="F102" t="s">
-        <v>440</v>
+        <v>448</v>
       </c>
     </row>
     <row r="103" spans="1:6">
@@ -3946,10 +3980,10 @@
         <v>107</v>
       </c>
       <c r="B103" t="s">
-        <v>275</v>
+        <v>279</v>
       </c>
       <c r="C103" t="s">
-        <v>343</v>
+        <v>351</v>
       </c>
       <c r="D103">
         <v>2</v>
@@ -3958,7 +3992,7 @@
         <v>2</v>
       </c>
       <c r="F103" t="s">
-        <v>441</v>
+        <v>449</v>
       </c>
     </row>
     <row r="104" spans="1:6">
@@ -3966,10 +4000,10 @@
         <v>108</v>
       </c>
       <c r="B104" t="s">
-        <v>276</v>
+        <v>280</v>
       </c>
       <c r="C104" t="s">
-        <v>343</v>
+        <v>351</v>
       </c>
       <c r="D104">
         <v>2</v>
@@ -3978,7 +4012,7 @@
         <v>2</v>
       </c>
       <c r="F104" t="s">
-        <v>442</v>
+        <v>450</v>
       </c>
     </row>
     <row r="105" spans="1:6">
@@ -3986,10 +4020,10 @@
         <v>109</v>
       </c>
       <c r="B105" t="s">
-        <v>277</v>
+        <v>281</v>
       </c>
       <c r="C105" t="s">
-        <v>343</v>
+        <v>351</v>
       </c>
       <c r="D105">
         <v>2</v>
@@ -3998,7 +4032,7 @@
         <v>2</v>
       </c>
       <c r="F105" t="s">
-        <v>443</v>
+        <v>451</v>
       </c>
     </row>
     <row r="106" spans="1:6">
@@ -4006,10 +4040,10 @@
         <v>110</v>
       </c>
       <c r="B106" t="s">
-        <v>278</v>
+        <v>282</v>
       </c>
       <c r="C106" t="s">
-        <v>343</v>
+        <v>350</v>
       </c>
       <c r="D106">
         <v>2</v>
@@ -4018,7 +4052,7 @@
         <v>2</v>
       </c>
       <c r="F106" t="s">
-        <v>444</v>
+        <v>452</v>
       </c>
     </row>
     <row r="107" spans="1:6">
@@ -4026,10 +4060,10 @@
         <v>111</v>
       </c>
       <c r="B107" t="s">
-        <v>279</v>
+        <v>283</v>
       </c>
       <c r="C107" t="s">
-        <v>343</v>
+        <v>351</v>
       </c>
       <c r="D107">
         <v>2</v>
@@ -4038,7 +4072,7 @@
         <v>2</v>
       </c>
       <c r="F107" t="s">
-        <v>353</v>
+        <v>453</v>
       </c>
     </row>
     <row r="108" spans="1:6">
@@ -4046,10 +4080,10 @@
         <v>112</v>
       </c>
       <c r="B108" t="s">
-        <v>280</v>
+        <v>284</v>
       </c>
       <c r="C108" t="s">
-        <v>343</v>
+        <v>351</v>
       </c>
       <c r="D108">
         <v>2</v>
@@ -4058,7 +4092,7 @@
         <v>2</v>
       </c>
       <c r="F108" t="s">
-        <v>445</v>
+        <v>454</v>
       </c>
     </row>
     <row r="109" spans="1:6">
@@ -4066,10 +4100,10 @@
         <v>113</v>
       </c>
       <c r="B109" t="s">
-        <v>281</v>
+        <v>285</v>
       </c>
       <c r="C109" t="s">
-        <v>343</v>
+        <v>351</v>
       </c>
       <c r="D109">
         <v>2</v>
@@ -4078,7 +4112,7 @@
         <v>2</v>
       </c>
       <c r="F109" t="s">
-        <v>446</v>
+        <v>455</v>
       </c>
     </row>
     <row r="110" spans="1:6">
@@ -4086,10 +4120,10 @@
         <v>114</v>
       </c>
       <c r="B110" t="s">
-        <v>282</v>
+        <v>286</v>
       </c>
       <c r="C110" t="s">
-        <v>343</v>
+        <v>351</v>
       </c>
       <c r="D110">
         <v>2</v>
@@ -4098,7 +4132,7 @@
         <v>2</v>
       </c>
       <c r="F110" t="s">
-        <v>357</v>
+        <v>456</v>
       </c>
     </row>
     <row r="111" spans="1:6">
@@ -4106,19 +4140,19 @@
         <v>115</v>
       </c>
       <c r="B111" t="s">
-        <v>283</v>
+        <v>287</v>
       </c>
       <c r="C111" t="s">
-        <v>343</v>
+        <v>351</v>
       </c>
       <c r="D111">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="E111">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="F111" t="s">
-        <v>447</v>
+        <v>361</v>
       </c>
     </row>
     <row r="112" spans="1:6">
@@ -4126,19 +4160,19 @@
         <v>116</v>
       </c>
       <c r="B112" t="s">
-        <v>284</v>
+        <v>288</v>
       </c>
       <c r="C112" t="s">
-        <v>342</v>
+        <v>351</v>
       </c>
       <c r="D112">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="E112">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="F112" t="s">
-        <v>448</v>
+        <v>457</v>
       </c>
     </row>
     <row r="113" spans="1:6">
@@ -4146,19 +4180,19 @@
         <v>117</v>
       </c>
       <c r="B113" t="s">
-        <v>285</v>
+        <v>289</v>
       </c>
       <c r="C113" t="s">
-        <v>342</v>
+        <v>351</v>
       </c>
       <c r="D113">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="E113">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="F113" t="s">
-        <v>449</v>
+        <v>458</v>
       </c>
     </row>
     <row r="114" spans="1:6">
@@ -4166,19 +4200,19 @@
         <v>118</v>
       </c>
       <c r="B114" t="s">
-        <v>286</v>
+        <v>290</v>
       </c>
       <c r="C114" t="s">
-        <v>342</v>
+        <v>351</v>
       </c>
       <c r="D114">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="E114">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="F114" t="s">
-        <v>450</v>
+        <v>365</v>
       </c>
     </row>
     <row r="115" spans="1:6">
@@ -4186,10 +4220,10 @@
         <v>119</v>
       </c>
       <c r="B115" t="s">
-        <v>287</v>
+        <v>291</v>
       </c>
       <c r="C115" t="s">
-        <v>343</v>
+        <v>351</v>
       </c>
       <c r="D115">
         <v>1</v>
@@ -4198,7 +4232,7 @@
         <v>1</v>
       </c>
       <c r="F115" t="s">
-        <v>451</v>
+        <v>459</v>
       </c>
     </row>
     <row r="116" spans="1:6">
@@ -4206,10 +4240,10 @@
         <v>120</v>
       </c>
       <c r="B116" t="s">
-        <v>288</v>
+        <v>292</v>
       </c>
       <c r="C116" t="s">
-        <v>342</v>
+        <v>350</v>
       </c>
       <c r="D116">
         <v>1</v>
@@ -4218,7 +4252,7 @@
         <v>1</v>
       </c>
       <c r="F116" t="s">
-        <v>452</v>
+        <v>460</v>
       </c>
     </row>
     <row r="117" spans="1:6">
@@ -4226,10 +4260,10 @@
         <v>121</v>
       </c>
       <c r="B117" t="s">
-        <v>289</v>
+        <v>293</v>
       </c>
       <c r="C117" t="s">
-        <v>343</v>
+        <v>350</v>
       </c>
       <c r="D117">
         <v>1</v>
@@ -4238,7 +4272,7 @@
         <v>1</v>
       </c>
       <c r="F117" t="s">
-        <v>453</v>
+        <v>461</v>
       </c>
     </row>
     <row r="118" spans="1:6">
@@ -4246,10 +4280,10 @@
         <v>122</v>
       </c>
       <c r="B118" t="s">
-        <v>290</v>
+        <v>294</v>
       </c>
       <c r="C118" t="s">
-        <v>342</v>
+        <v>350</v>
       </c>
       <c r="D118">
         <v>1</v>
@@ -4258,7 +4292,7 @@
         <v>1</v>
       </c>
       <c r="F118" t="s">
-        <v>454</v>
+        <v>462</v>
       </c>
     </row>
     <row r="119" spans="1:6">
@@ -4266,10 +4300,10 @@
         <v>123</v>
       </c>
       <c r="B119" t="s">
-        <v>291</v>
+        <v>295</v>
       </c>
       <c r="C119" t="s">
-        <v>342</v>
+        <v>351</v>
       </c>
       <c r="D119">
         <v>1</v>
@@ -4278,7 +4312,7 @@
         <v>1</v>
       </c>
       <c r="F119" t="s">
-        <v>455</v>
+        <v>463</v>
       </c>
     </row>
     <row r="120" spans="1:6">
@@ -4286,10 +4320,10 @@
         <v>124</v>
       </c>
       <c r="B120" t="s">
-        <v>292</v>
+        <v>296</v>
       </c>
       <c r="C120" t="s">
-        <v>342</v>
+        <v>350</v>
       </c>
       <c r="D120">
         <v>1</v>
@@ -4298,7 +4332,7 @@
         <v>1</v>
       </c>
       <c r="F120" t="s">
-        <v>456</v>
+        <v>464</v>
       </c>
     </row>
     <row r="121" spans="1:6">
@@ -4306,10 +4340,10 @@
         <v>125</v>
       </c>
       <c r="B121" t="s">
-        <v>293</v>
+        <v>297</v>
       </c>
       <c r="C121" t="s">
-        <v>342</v>
+        <v>351</v>
       </c>
       <c r="D121">
         <v>1</v>
@@ -4318,7 +4352,7 @@
         <v>1</v>
       </c>
       <c r="F121" t="s">
-        <v>457</v>
+        <v>465</v>
       </c>
     </row>
     <row r="122" spans="1:6">
@@ -4326,10 +4360,10 @@
         <v>126</v>
       </c>
       <c r="B122" t="s">
-        <v>294</v>
+        <v>298</v>
       </c>
       <c r="C122" t="s">
-        <v>342</v>
+        <v>350</v>
       </c>
       <c r="D122">
         <v>1</v>
@@ -4338,7 +4372,7 @@
         <v>1</v>
       </c>
       <c r="F122" t="s">
-        <v>458</v>
+        <v>466</v>
       </c>
     </row>
     <row r="123" spans="1:6">
@@ -4346,10 +4380,10 @@
         <v>127</v>
       </c>
       <c r="B123" t="s">
-        <v>295</v>
+        <v>299</v>
       </c>
       <c r="C123" t="s">
-        <v>342</v>
+        <v>350</v>
       </c>
       <c r="D123">
         <v>1</v>
@@ -4358,7 +4392,7 @@
         <v>1</v>
       </c>
       <c r="F123" t="s">
-        <v>459</v>
+        <v>467</v>
       </c>
     </row>
     <row r="124" spans="1:6">
@@ -4366,10 +4400,10 @@
         <v>128</v>
       </c>
       <c r="B124" t="s">
-        <v>296</v>
+        <v>300</v>
       </c>
       <c r="C124" t="s">
-        <v>342</v>
+        <v>350</v>
       </c>
       <c r="D124">
         <v>1</v>
@@ -4378,7 +4412,7 @@
         <v>1</v>
       </c>
       <c r="F124" t="s">
-        <v>460</v>
+        <v>468</v>
       </c>
     </row>
     <row r="125" spans="1:6">
@@ -4386,10 +4420,10 @@
         <v>129</v>
       </c>
       <c r="B125" t="s">
-        <v>297</v>
+        <v>301</v>
       </c>
       <c r="C125" t="s">
-        <v>343</v>
+        <v>350</v>
       </c>
       <c r="D125">
         <v>1</v>
@@ -4398,7 +4432,7 @@
         <v>1</v>
       </c>
       <c r="F125" t="s">
-        <v>461</v>
+        <v>469</v>
       </c>
     </row>
     <row r="126" spans="1:6">
@@ -4406,10 +4440,10 @@
         <v>130</v>
       </c>
       <c r="B126" t="s">
-        <v>298</v>
+        <v>302</v>
       </c>
       <c r="C126" t="s">
-        <v>343</v>
+        <v>350</v>
       </c>
       <c r="D126">
         <v>1</v>
@@ -4418,7 +4452,7 @@
         <v>1</v>
       </c>
       <c r="F126" t="s">
-        <v>462</v>
+        <v>470</v>
       </c>
     </row>
     <row r="127" spans="1:6">
@@ -4426,10 +4460,10 @@
         <v>131</v>
       </c>
       <c r="B127" t="s">
-        <v>299</v>
+        <v>303</v>
       </c>
       <c r="C127" t="s">
-        <v>343</v>
+        <v>350</v>
       </c>
       <c r="D127">
         <v>1</v>
@@ -4438,7 +4472,7 @@
         <v>1</v>
       </c>
       <c r="F127" t="s">
-        <v>463</v>
+        <v>471</v>
       </c>
     </row>
     <row r="128" spans="1:6">
@@ -4446,10 +4480,10 @@
         <v>132</v>
       </c>
       <c r="B128" t="s">
-        <v>300</v>
+        <v>304</v>
       </c>
       <c r="C128" t="s">
-        <v>343</v>
+        <v>350</v>
       </c>
       <c r="D128">
         <v>1</v>
@@ -4458,7 +4492,7 @@
         <v>1</v>
       </c>
       <c r="F128" t="s">
-        <v>464</v>
+        <v>472</v>
       </c>
     </row>
     <row r="129" spans="1:6">
@@ -4466,10 +4500,10 @@
         <v>133</v>
       </c>
       <c r="B129" t="s">
-        <v>301</v>
+        <v>305</v>
       </c>
       <c r="C129" t="s">
-        <v>343</v>
+        <v>351</v>
       </c>
       <c r="D129">
         <v>1</v>
@@ -4478,7 +4512,7 @@
         <v>1</v>
       </c>
       <c r="F129" t="s">
-        <v>465</v>
+        <v>473</v>
       </c>
     </row>
     <row r="130" spans="1:6">
@@ -4486,10 +4520,10 @@
         <v>134</v>
       </c>
       <c r="B130" t="s">
-        <v>302</v>
+        <v>306</v>
       </c>
       <c r="C130" t="s">
-        <v>342</v>
+        <v>351</v>
       </c>
       <c r="D130">
         <v>1</v>
@@ -4498,7 +4532,7 @@
         <v>1</v>
       </c>
       <c r="F130" t="s">
-        <v>466</v>
+        <v>420</v>
       </c>
     </row>
     <row r="131" spans="1:6">
@@ -4506,10 +4540,10 @@
         <v>135</v>
       </c>
       <c r="B131" t="s">
-        <v>303</v>
+        <v>307</v>
       </c>
       <c r="C131" t="s">
-        <v>342</v>
+        <v>351</v>
       </c>
       <c r="D131">
         <v>1</v>
@@ -4518,7 +4552,7 @@
         <v>1</v>
       </c>
       <c r="F131" t="s">
-        <v>467</v>
+        <v>474</v>
       </c>
     </row>
     <row r="132" spans="1:6">
@@ -4526,10 +4560,10 @@
         <v>136</v>
       </c>
       <c r="B132" t="s">
-        <v>304</v>
+        <v>308</v>
       </c>
       <c r="C132" t="s">
-        <v>343</v>
+        <v>351</v>
       </c>
       <c r="D132">
         <v>1</v>
@@ -4538,7 +4572,7 @@
         <v>1</v>
       </c>
       <c r="F132" t="s">
-        <v>468</v>
+        <v>475</v>
       </c>
     </row>
     <row r="133" spans="1:6">
@@ -4546,10 +4580,10 @@
         <v>137</v>
       </c>
       <c r="B133" t="s">
-        <v>305</v>
+        <v>309</v>
       </c>
       <c r="C133" t="s">
-        <v>343</v>
+        <v>351</v>
       </c>
       <c r="D133">
         <v>1</v>
@@ -4558,7 +4592,7 @@
         <v>1</v>
       </c>
       <c r="F133" t="s">
-        <v>469</v>
+        <v>476</v>
       </c>
     </row>
     <row r="134" spans="1:6">
@@ -4566,10 +4600,10 @@
         <v>138</v>
       </c>
       <c r="B134" t="s">
-        <v>306</v>
+        <v>310</v>
       </c>
       <c r="C134" t="s">
-        <v>342</v>
+        <v>350</v>
       </c>
       <c r="D134">
         <v>1</v>
@@ -4578,7 +4612,7 @@
         <v>1</v>
       </c>
       <c r="F134" t="s">
-        <v>461</v>
+        <v>477</v>
       </c>
     </row>
     <row r="135" spans="1:6">
@@ -4586,10 +4620,10 @@
         <v>139</v>
       </c>
       <c r="B135" t="s">
-        <v>307</v>
+        <v>311</v>
       </c>
       <c r="C135" t="s">
-        <v>342</v>
+        <v>350</v>
       </c>
       <c r="D135">
         <v>1</v>
@@ -4598,7 +4632,7 @@
         <v>1</v>
       </c>
       <c r="F135" t="s">
-        <v>470</v>
+        <v>478</v>
       </c>
     </row>
     <row r="136" spans="1:6">
@@ -4606,10 +4640,10 @@
         <v>140</v>
       </c>
       <c r="B136" t="s">
-        <v>308</v>
+        <v>312</v>
       </c>
       <c r="C136" t="s">
-        <v>342</v>
+        <v>351</v>
       </c>
       <c r="D136">
         <v>1</v>
@@ -4618,7 +4652,7 @@
         <v>1</v>
       </c>
       <c r="F136" t="s">
-        <v>471</v>
+        <v>479</v>
       </c>
     </row>
     <row r="137" spans="1:6">
@@ -4626,10 +4660,10 @@
         <v>141</v>
       </c>
       <c r="B137" t="s">
-        <v>309</v>
+        <v>313</v>
       </c>
       <c r="C137" t="s">
-        <v>343</v>
+        <v>351</v>
       </c>
       <c r="D137">
         <v>1</v>
@@ -4638,7 +4672,7 @@
         <v>1</v>
       </c>
       <c r="F137" t="s">
-        <v>472</v>
+        <v>480</v>
       </c>
     </row>
     <row r="138" spans="1:6">
@@ -4646,10 +4680,10 @@
         <v>142</v>
       </c>
       <c r="B138" t="s">
-        <v>310</v>
+        <v>314</v>
       </c>
       <c r="C138" t="s">
-        <v>342</v>
+        <v>350</v>
       </c>
       <c r="D138">
         <v>1</v>
@@ -4666,10 +4700,10 @@
         <v>143</v>
       </c>
       <c r="B139" t="s">
-        <v>311</v>
+        <v>315</v>
       </c>
       <c r="C139" t="s">
-        <v>343</v>
+        <v>350</v>
       </c>
       <c r="D139">
         <v>1</v>
@@ -4678,7 +4712,7 @@
         <v>1</v>
       </c>
       <c r="F139" t="s">
-        <v>474</v>
+        <v>481</v>
       </c>
     </row>
     <row r="140" spans="1:6">
@@ -4686,10 +4720,10 @@
         <v>144</v>
       </c>
       <c r="B140" t="s">
-        <v>312</v>
+        <v>316</v>
       </c>
       <c r="C140" t="s">
-        <v>342</v>
+        <v>350</v>
       </c>
       <c r="D140">
         <v>1</v>
@@ -4698,7 +4732,7 @@
         <v>1</v>
       </c>
       <c r="F140" t="s">
-        <v>409</v>
+        <v>482</v>
       </c>
     </row>
     <row r="141" spans="1:6">
@@ -4706,10 +4740,10 @@
         <v>145</v>
       </c>
       <c r="B141" t="s">
-        <v>313</v>
+        <v>317</v>
       </c>
       <c r="C141" t="s">
-        <v>343</v>
+        <v>351</v>
       </c>
       <c r="D141">
         <v>1</v>
@@ -4718,7 +4752,7 @@
         <v>1</v>
       </c>
       <c r="F141" t="s">
-        <v>475</v>
+        <v>483</v>
       </c>
     </row>
     <row r="142" spans="1:6">
@@ -4726,10 +4760,10 @@
         <v>146</v>
       </c>
       <c r="B142" t="s">
-        <v>314</v>
+        <v>318</v>
       </c>
       <c r="C142" t="s">
-        <v>342</v>
+        <v>350</v>
       </c>
       <c r="D142">
         <v>1</v>
@@ -4738,7 +4772,7 @@
         <v>1</v>
       </c>
       <c r="F142" t="s">
-        <v>476</v>
+        <v>484</v>
       </c>
     </row>
     <row r="143" spans="1:6">
@@ -4746,10 +4780,10 @@
         <v>147</v>
       </c>
       <c r="B143" t="s">
-        <v>315</v>
+        <v>319</v>
       </c>
       <c r="C143" t="s">
-        <v>342</v>
+        <v>351</v>
       </c>
       <c r="D143">
         <v>1</v>
@@ -4758,7 +4792,7 @@
         <v>1</v>
       </c>
       <c r="F143" t="s">
-        <v>477</v>
+        <v>485</v>
       </c>
     </row>
     <row r="144" spans="1:6">
@@ -4766,10 +4800,10 @@
         <v>148</v>
       </c>
       <c r="B144" t="s">
-        <v>316</v>
+        <v>320</v>
       </c>
       <c r="C144" t="s">
-        <v>343</v>
+        <v>350</v>
       </c>
       <c r="D144">
         <v>1</v>
@@ -4778,7 +4812,7 @@
         <v>1</v>
       </c>
       <c r="F144" t="s">
-        <v>478</v>
+        <v>417</v>
       </c>
     </row>
     <row r="145" spans="1:6">
@@ -4786,10 +4820,10 @@
         <v>149</v>
       </c>
       <c r="B145" t="s">
-        <v>317</v>
+        <v>321</v>
       </c>
       <c r="C145" t="s">
-        <v>342</v>
+        <v>351</v>
       </c>
       <c r="D145">
         <v>1</v>
@@ -4798,7 +4832,7 @@
         <v>1</v>
       </c>
       <c r="F145" t="s">
-        <v>479</v>
+        <v>486</v>
       </c>
     </row>
     <row r="146" spans="1:6">
@@ -4806,10 +4840,10 @@
         <v>150</v>
       </c>
       <c r="B146" t="s">
-        <v>318</v>
+        <v>322</v>
       </c>
       <c r="C146" t="s">
-        <v>342</v>
+        <v>350</v>
       </c>
       <c r="D146">
         <v>1</v>
@@ -4818,7 +4852,7 @@
         <v>1</v>
       </c>
       <c r="F146" t="s">
-        <v>454</v>
+        <v>487</v>
       </c>
     </row>
     <row r="147" spans="1:6">
@@ -4826,10 +4860,10 @@
         <v>151</v>
       </c>
       <c r="B147" t="s">
-        <v>319</v>
+        <v>323</v>
       </c>
       <c r="C147" t="s">
-        <v>343</v>
+        <v>350</v>
       </c>
       <c r="D147">
         <v>1</v>
@@ -4838,7 +4872,7 @@
         <v>1</v>
       </c>
       <c r="F147" t="s">
-        <v>480</v>
+        <v>488</v>
       </c>
     </row>
     <row r="148" spans="1:6">
@@ -4846,10 +4880,10 @@
         <v>152</v>
       </c>
       <c r="B148" t="s">
-        <v>320</v>
+        <v>324</v>
       </c>
       <c r="C148" t="s">
-        <v>343</v>
+        <v>351</v>
       </c>
       <c r="D148">
         <v>1</v>
@@ -4858,7 +4892,7 @@
         <v>1</v>
       </c>
       <c r="F148" t="s">
-        <v>481</v>
+        <v>489</v>
       </c>
     </row>
     <row r="149" spans="1:6">
@@ -4866,10 +4900,10 @@
         <v>153</v>
       </c>
       <c r="B149" t="s">
-        <v>321</v>
+        <v>325</v>
       </c>
       <c r="C149" t="s">
-        <v>343</v>
+        <v>350</v>
       </c>
       <c r="D149">
         <v>1</v>
@@ -4878,7 +4912,7 @@
         <v>1</v>
       </c>
       <c r="F149" t="s">
-        <v>482</v>
+        <v>490</v>
       </c>
     </row>
     <row r="150" spans="1:6">
@@ -4886,10 +4920,10 @@
         <v>154</v>
       </c>
       <c r="B150" t="s">
-        <v>322</v>
+        <v>326</v>
       </c>
       <c r="C150" t="s">
-        <v>343</v>
+        <v>350</v>
       </c>
       <c r="D150">
         <v>1</v>
@@ -4898,7 +4932,7 @@
         <v>1</v>
       </c>
       <c r="F150" t="s">
-        <v>483</v>
+        <v>466</v>
       </c>
     </row>
     <row r="151" spans="1:6">
@@ -4906,10 +4940,10 @@
         <v>155</v>
       </c>
       <c r="B151" t="s">
-        <v>323</v>
+        <v>327</v>
       </c>
       <c r="C151" t="s">
-        <v>342</v>
+        <v>351</v>
       </c>
       <c r="D151">
         <v>1</v>
@@ -4918,7 +4952,7 @@
         <v>1</v>
       </c>
       <c r="F151" t="s">
-        <v>381</v>
+        <v>491</v>
       </c>
     </row>
     <row r="152" spans="1:6">
@@ -4926,10 +4960,10 @@
         <v>156</v>
       </c>
       <c r="B152" t="s">
-        <v>324</v>
+        <v>328</v>
       </c>
       <c r="C152" t="s">
-        <v>342</v>
+        <v>351</v>
       </c>
       <c r="D152">
         <v>1</v>
@@ -4938,7 +4972,7 @@
         <v>1</v>
       </c>
       <c r="F152" t="s">
-        <v>484</v>
+        <v>492</v>
       </c>
     </row>
     <row r="153" spans="1:6">
@@ -4946,10 +4980,10 @@
         <v>157</v>
       </c>
       <c r="B153" t="s">
-        <v>325</v>
+        <v>329</v>
       </c>
       <c r="C153" t="s">
-        <v>342</v>
+        <v>351</v>
       </c>
       <c r="D153">
         <v>1</v>
@@ -4958,7 +4992,7 @@
         <v>1</v>
       </c>
       <c r="F153" t="s">
-        <v>485</v>
+        <v>493</v>
       </c>
     </row>
     <row r="154" spans="1:6">
@@ -4966,10 +5000,10 @@
         <v>158</v>
       </c>
       <c r="B154" t="s">
-        <v>326</v>
+        <v>330</v>
       </c>
       <c r="C154" t="s">
-        <v>342</v>
+        <v>351</v>
       </c>
       <c r="D154">
         <v>1</v>
@@ -4978,7 +5012,7 @@
         <v>1</v>
       </c>
       <c r="F154" t="s">
-        <v>486</v>
+        <v>494</v>
       </c>
     </row>
     <row r="155" spans="1:6">
@@ -4986,10 +5020,10 @@
         <v>159</v>
       </c>
       <c r="B155" t="s">
-        <v>327</v>
+        <v>331</v>
       </c>
       <c r="C155" t="s">
-        <v>343</v>
+        <v>350</v>
       </c>
       <c r="D155">
         <v>1</v>
@@ -4998,7 +5032,7 @@
         <v>1</v>
       </c>
       <c r="F155" t="s">
-        <v>358</v>
+        <v>389</v>
       </c>
     </row>
     <row r="156" spans="1:6">
@@ -5006,10 +5040,10 @@
         <v>160</v>
       </c>
       <c r="B156" t="s">
-        <v>328</v>
+        <v>332</v>
       </c>
       <c r="C156" t="s">
-        <v>343</v>
+        <v>350</v>
       </c>
       <c r="D156">
         <v>1</v>
@@ -5018,7 +5052,7 @@
         <v>1</v>
       </c>
       <c r="F156" t="s">
-        <v>487</v>
+        <v>495</v>
       </c>
     </row>
     <row r="157" spans="1:6">
@@ -5026,10 +5060,10 @@
         <v>161</v>
       </c>
       <c r="B157" t="s">
-        <v>329</v>
+        <v>333</v>
       </c>
       <c r="C157" t="s">
-        <v>343</v>
+        <v>350</v>
       </c>
       <c r="D157">
         <v>1</v>
@@ -5038,7 +5072,7 @@
         <v>1</v>
       </c>
       <c r="F157" t="s">
-        <v>488</v>
+        <v>496</v>
       </c>
     </row>
     <row r="158" spans="1:6">
@@ -5046,10 +5080,10 @@
         <v>162</v>
       </c>
       <c r="B158" t="s">
-        <v>330</v>
+        <v>334</v>
       </c>
       <c r="C158" t="s">
-        <v>343</v>
+        <v>350</v>
       </c>
       <c r="D158">
         <v>1</v>
@@ -5058,7 +5092,7 @@
         <v>1</v>
       </c>
       <c r="F158" t="s">
-        <v>489</v>
+        <v>497</v>
       </c>
     </row>
     <row r="159" spans="1:6">
@@ -5066,10 +5100,10 @@
         <v>163</v>
       </c>
       <c r="B159" t="s">
-        <v>331</v>
+        <v>335</v>
       </c>
       <c r="C159" t="s">
-        <v>342</v>
+        <v>351</v>
       </c>
       <c r="D159">
         <v>1</v>
@@ -5078,7 +5112,7 @@
         <v>1</v>
       </c>
       <c r="F159" t="s">
-        <v>490</v>
+        <v>366</v>
       </c>
     </row>
     <row r="160" spans="1:6">
@@ -5086,10 +5120,10 @@
         <v>164</v>
       </c>
       <c r="B160" t="s">
-        <v>332</v>
+        <v>336</v>
       </c>
       <c r="C160" t="s">
-        <v>343</v>
+        <v>351</v>
       </c>
       <c r="D160">
         <v>1</v>
@@ -5098,7 +5132,7 @@
         <v>1</v>
       </c>
       <c r="F160" t="s">
-        <v>491</v>
+        <v>498</v>
       </c>
     </row>
     <row r="161" spans="1:6">
@@ -5106,10 +5140,10 @@
         <v>165</v>
       </c>
       <c r="B161" t="s">
-        <v>333</v>
+        <v>337</v>
       </c>
       <c r="C161" t="s">
-        <v>343</v>
+        <v>351</v>
       </c>
       <c r="D161">
         <v>1</v>
@@ -5118,7 +5152,7 @@
         <v>1</v>
       </c>
       <c r="F161" t="s">
-        <v>492</v>
+        <v>499</v>
       </c>
     </row>
     <row r="162" spans="1:6">
@@ -5126,10 +5160,10 @@
         <v>166</v>
       </c>
       <c r="B162" t="s">
-        <v>334</v>
+        <v>338</v>
       </c>
       <c r="C162" t="s">
-        <v>343</v>
+        <v>351</v>
       </c>
       <c r="D162">
         <v>1</v>
@@ -5138,7 +5172,7 @@
         <v>1</v>
       </c>
       <c r="F162" t="s">
-        <v>493</v>
+        <v>500</v>
       </c>
     </row>
     <row r="163" spans="1:6">
@@ -5146,10 +5180,10 @@
         <v>167</v>
       </c>
       <c r="B163" t="s">
-        <v>335</v>
+        <v>339</v>
       </c>
       <c r="C163" t="s">
-        <v>343</v>
+        <v>350</v>
       </c>
       <c r="D163">
         <v>1</v>
@@ -5158,7 +5192,7 @@
         <v>1</v>
       </c>
       <c r="F163" t="s">
-        <v>494</v>
+        <v>501</v>
       </c>
     </row>
     <row r="164" spans="1:6">
@@ -5166,10 +5200,10 @@
         <v>168</v>
       </c>
       <c r="B164" t="s">
-        <v>336</v>
+        <v>340</v>
       </c>
       <c r="C164" t="s">
-        <v>343</v>
+        <v>351</v>
       </c>
       <c r="D164">
         <v>1</v>
@@ -5178,7 +5212,7 @@
         <v>1</v>
       </c>
       <c r="F164" t="s">
-        <v>495</v>
+        <v>502</v>
       </c>
     </row>
     <row r="165" spans="1:6">
@@ -5186,10 +5220,10 @@
         <v>169</v>
       </c>
       <c r="B165" t="s">
-        <v>337</v>
+        <v>341</v>
       </c>
       <c r="C165" t="s">
-        <v>342</v>
+        <v>351</v>
       </c>
       <c r="D165">
         <v>1</v>
@@ -5198,7 +5232,7 @@
         <v>1</v>
       </c>
       <c r="F165" t="s">
-        <v>496</v>
+        <v>503</v>
       </c>
     </row>
     <row r="166" spans="1:6">
@@ -5206,10 +5240,10 @@
         <v>170</v>
       </c>
       <c r="B166" t="s">
-        <v>338</v>
+        <v>342</v>
       </c>
       <c r="C166" t="s">
-        <v>343</v>
+        <v>351</v>
       </c>
       <c r="D166">
         <v>1</v>
@@ -5218,7 +5252,7 @@
         <v>1</v>
       </c>
       <c r="F166" t="s">
-        <v>497</v>
+        <v>504</v>
       </c>
     </row>
     <row r="167" spans="1:6">
@@ -5226,10 +5260,10 @@
         <v>171</v>
       </c>
       <c r="B167" t="s">
-        <v>339</v>
+        <v>343</v>
       </c>
       <c r="C167" t="s">
-        <v>343</v>
+        <v>351</v>
       </c>
       <c r="D167">
         <v>1</v>
@@ -5238,7 +5272,7 @@
         <v>1</v>
       </c>
       <c r="F167" t="s">
-        <v>498</v>
+        <v>505</v>
       </c>
     </row>
     <row r="168" spans="1:6">
@@ -5246,10 +5280,10 @@
         <v>172</v>
       </c>
       <c r="B168" t="s">
-        <v>340</v>
+        <v>344</v>
       </c>
       <c r="C168" t="s">
-        <v>343</v>
+        <v>351</v>
       </c>
       <c r="D168">
         <v>1</v>
@@ -5258,7 +5292,7 @@
         <v>1</v>
       </c>
       <c r="F168" t="s">
-        <v>499</v>
+        <v>506</v>
       </c>
     </row>
     <row r="169" spans="1:6">
@@ -5266,10 +5300,10 @@
         <v>173</v>
       </c>
       <c r="B169" t="s">
-        <v>341</v>
+        <v>345</v>
       </c>
       <c r="C169" t="s">
-        <v>342</v>
+        <v>350</v>
       </c>
       <c r="D169">
         <v>1</v>
@@ -5278,7 +5312,87 @@
         <v>1</v>
       </c>
       <c r="F169" t="s">
-        <v>500</v>
+        <v>507</v>
+      </c>
+    </row>
+    <row r="170" spans="1:6">
+      <c r="A170" t="s">
+        <v>174</v>
+      </c>
+      <c r="B170" t="s">
+        <v>346</v>
+      </c>
+      <c r="C170" t="s">
+        <v>351</v>
+      </c>
+      <c r="D170">
+        <v>1</v>
+      </c>
+      <c r="E170">
+        <v>1</v>
+      </c>
+      <c r="F170" t="s">
+        <v>508</v>
+      </c>
+    </row>
+    <row r="171" spans="1:6">
+      <c r="A171" t="s">
+        <v>175</v>
+      </c>
+      <c r="B171" t="s">
+        <v>347</v>
+      </c>
+      <c r="C171" t="s">
+        <v>351</v>
+      </c>
+      <c r="D171">
+        <v>1</v>
+      </c>
+      <c r="E171">
+        <v>1</v>
+      </c>
+      <c r="F171" t="s">
+        <v>509</v>
+      </c>
+    </row>
+    <row r="172" spans="1:6">
+      <c r="A172" t="s">
+        <v>176</v>
+      </c>
+      <c r="B172" t="s">
+        <v>348</v>
+      </c>
+      <c r="C172" t="s">
+        <v>351</v>
+      </c>
+      <c r="D172">
+        <v>1</v>
+      </c>
+      <c r="E172">
+        <v>1</v>
+      </c>
+      <c r="F172" t="s">
+        <v>510</v>
+      </c>
+    </row>
+    <row r="173" spans="1:6">
+      <c r="A173" t="s">
+        <v>177</v>
+      </c>
+      <c r="B173" t="s">
+        <v>349</v>
+      </c>
+      <c r="C173" t="s">
+        <v>350</v>
+      </c>
+      <c r="D173">
+        <v>1</v>
+      </c>
+      <c r="E173">
+        <v>1</v>
+      </c>
+      <c r="F173" t="s">
+        <v>511</v>
       </c>
     </row>
   </sheetData>

</xml_diff>